<commit_message>
Auto-refresh: casino gaming market data update 2026-03-16 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -842,7 +842,7 @@
         <v>100.63</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.19914064</v>
+        <v>0.199141</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -975,19 +975,19 @@
         <v>6.042</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8.52</v>
+        <v>8.398999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.5478725</v>
+        <v>3.6184447</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>9.823980000000001</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>7.094</v>
+        <v>6.994</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>1.22</v>
@@ -1034,16 +1034,16 @@
         <v>6.011</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11.061</v>
+        <v>11.05</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.294895</v>
+        <v>16.325756</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>11.609365</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>11.562</v>
+        <v>11.55</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>9.800000000000001</v>
@@ -1078,7 +1078,7 @@
         <v>57.77</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.32997328</v>
+        <v>0.329973</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1198,7 +1198,7 @@
         <v>18.18</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>-0.025723448</v>
+        <v>-0.0257234</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>32.22</v>
@@ -1216,7 +1216,7 @@
         <v>5.157</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>50.5</v>
+        <v>51.94286</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>22.35407</v>
@@ -1381,7 +1381,7 @@
         <v>5.61</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.3577814</v>
+        <v>0.357781</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>10.15</v>
@@ -1440,7 +1440,7 @@
         <v>13.98</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>-0.023060856</v>
+        <v>-0.0230609</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>20.61</v>
@@ -1501,7 +1501,7 @@
         <v>98.43000000000001</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>-0.019719183</v>
+        <v>-0.0197192</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>113.88</v>
@@ -1809,13 +1809,13 @@
         <v>0.0379939</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>10.29</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="G21" s="3" t="n">
         <v>6.505</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.336</v>
+        <v>-0.314</v>
       </c>
       <c r="I21" s="6" t="n">
         <v>0.184</v>
@@ -1880,7 +1880,7 @@
         <v>0.093</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.596</v>
+        <v>0.594</v>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
@@ -1891,7 +1891,7 @@
         <v>-6.2926826</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>12.968</v>
+        <v>12.945</v>
       </c>
       <c r="N22" s="7" t="n">
         <v>9.300000000000001</v>
@@ -2434,7 +2434,7 @@
         <v>100.63</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.19914064</v>
+        <v>0.199141</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.177</v>
@@ -2622,7 +2622,7 @@
         <v>57.77</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.32997328</v>
+        <v>0.329973</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.068</v>
@@ -2716,7 +2716,7 @@
         <v>18.18</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>-0.025723448</v>
+        <v>-0.0257234</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>-0.22</v>
@@ -2857,7 +2857,7 @@
         <v>5.61</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.3577814</v>
+        <v>0.357781</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>-0.253</v>
@@ -2904,7 +2904,7 @@
         <v>13.98</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-0.023060856</v>
+        <v>-0.0230609</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.059</v>
@@ -2951,7 +2951,7 @@
         <v>98.43000000000001</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.019719183</v>
+        <v>-0.0197192</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>0.028</v>
@@ -3206,7 +3206,7 @@
         <v>-0.205</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.336</v>
+        <v>-0.314</v>
       </c>
       <c r="L21" s="8" t="n">
         <v>1.206</v>
@@ -3650,7 +3650,7 @@
         <v>1.1629317</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>-1.74</v>
+        <v>-1.75</v>
       </c>
       <c r="N3" s="3" t="n">
         <v>10.80017</v>
@@ -3843,19 +3843,19 @@
         <v>6.042</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.5478725</v>
+        <v>3.6184447</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>9.823980000000001</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>7.094</v>
+        <v>6.994</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>2.082</v>
+        <v>2.053</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>2.343297</v>
@@ -3864,7 +3864,7 @@
         <v>1.4766403</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>22.56</v>
+        <v>22.12</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>8.147410000000001</v>
@@ -3896,19 +3896,19 @@
         <v>6.011</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.294895</v>
+        <v>16.325756</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>11.609365</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>11.562</v>
+        <v>11.55</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.781</v>
+        <v>3.777</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>5.941959</v>
@@ -3917,7 +3917,7 @@
         <v>2.0542798</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>5.29</v>
+        <v>5.28</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>7.42504</v>
@@ -4025,7 +4025,7 @@
         <v>0.48263726</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-2.42</v>
+        <v>-2.34</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>0.925</v>
@@ -4057,7 +4057,7 @@
         <v>5.38</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>50.5</v>
+        <v>51.94286</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>22.35407</v>
@@ -4078,7 +4078,7 @@
         <v>4.1709666</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>0.81327474</v>
@@ -4408,7 +4408,7 @@
         <v>1.9130899</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.43</v>
       </c>
       <c r="N17" s="3" t="n">
         <v>0.99</v>
@@ -4571,7 +4571,7 @@
         <v>0.25303388</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>-13.26</v>
+        <v>-13.39</v>
       </c>
       <c r="N20" s="3" t="n">
         <v>-1.49</v>
@@ -4664,13 +4664,13 @@
         <v>-6.2926826</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>12.968</v>
+        <v>12.945</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>9.300000000000001</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1.97</v>
+        <v>1.966</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>6.564885</v>
@@ -4679,7 +4679,7 @@
         <v>0.30820388</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.09</v>
       </c>
       <c r="N22" s="3" t="n">
         <v>-0.41</v>
@@ -7053,7 +7053,7 @@
         <v>0.68579</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -7369,13 +7369,13 @@
         <v>21</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>28.680185</v>
+        <v>28.690083</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>36.99057</v>
+        <v>37.003334</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>21.818075</v>
+        <v>21.825605</v>
       </c>
       <c r="J11" s="4" t="n">
         <v>0.578</v>
@@ -7685,7 +7685,7 @@
         <v>0.64761</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
       <c r="P16" s="5" t="n">
         <v>0.221</v>
@@ -8714,7 +8714,7 @@
         <v>6.011</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>16.294895</v>
+        <v>16.325756</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.067</v>
@@ -8729,7 +8729,7 @@
         <v>-0.23</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>11.562</v>
+        <v>11.55</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>9.800000000000001</v>
@@ -8758,7 +8758,7 @@
         <v>6.042</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3.5478725</v>
+        <v>3.6184447</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.02</v>
@@ -8773,10 +8773,10 @@
         <v>-0.07099999999999999</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>7.094</v>
+        <v>6.994</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>64.3</v>
@@ -8999,7 +8999,7 @@
         <v>0.032</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>12.968</v>
+        <v>12.945</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>9.300000000000001</v>
@@ -9136,7 +9136,7 @@
         <v>5.38</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>50.5</v>
+        <v>51.94286</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -11340,7 +11340,7 @@
         <v>1237.26</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>1234.13</v>
+        <v>1234.12</v>
       </c>
       <c r="D14" s="13" t="n">
         <v>1047.95</v>
@@ -11580,7 +11580,7 @@
         <v>1120.5</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>1240.57</v>
+        <v>1240.56</v>
       </c>
       <c r="D29" s="13" t="n">
         <v>996.5599999999999</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-21 16:14
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -679,7 +679,7 @@
         <v>48.099</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.013044</v>
+        <v>22.523405</v>
       </c>
       <c r="L2" s="7" t="n">
         <v>14.086344</v>
@@ -857,16 +857,16 @@
         <v>10.426</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>19.75</v>
+        <v>19.746</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.88816</v>
+        <v>31.840765</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>16.826635</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>11.288</v>
+        <v>11.286</v>
       </c>
       <c r="N5" s="7" t="n">
         <v>9.1</v>
@@ -919,10 +919,10 @@
         <v>39.176</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.452053</v>
+        <v>46.539474</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.072357</v>
+        <v>15.095321</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.638</v>
@@ -978,7 +978,7 @@
         <v>8.476000000000001</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6811988</v>
+        <v>3.593085</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>9.949173</v>
@@ -1034,16 +1034,16 @@
         <v>5.915</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>6.815</v>
+        <v>6.814</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>19.173334</v>
+        <v>18.435898</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>17.504938</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>8.374000000000001</v>
+        <v>8.372999999999999</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>7.3</v>
@@ -1093,16 +1093,16 @@
         <v>5.836</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>10.88</v>
+        <v>10.878</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.613096</v>
+        <v>15.827978</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>11.276708</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>11.373</v>
+        <v>11.371</v>
       </c>
       <c r="N9" s="7" t="n">
         <v>9.6</v>
@@ -1137,7 +1137,7 @@
         <v>19.61</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-0.406297</v>
+        <v>-0.4062972000000001</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1152,7 +1152,7 @@
         <v>5.804</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>5.593</v>
+        <v>5.587</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>54.47222</v>
@@ -1161,7 +1161,7 @@
         <v>23.874111</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>11.021</v>
+        <v>11.009</v>
       </c>
       <c r="N10" s="7" t="n">
         <v>9.6</v>
@@ -1196,7 +1196,7 @@
         <v>26.76</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-0.0247814</v>
+        <v>-0.02478135</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>31.58</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69</v>
+        <v>66.77419</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>27.661594</v>
@@ -1440,7 +1440,7 @@
         <v>13.67</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-0.0346045</v>
+        <v>-0.034604504</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>20.61</v>
@@ -1455,7 +1455,7 @@
         <v>1.826</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12.314</v>
+        <v>12.313</v>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
@@ -1466,7 +1466,7 @@
         <v>7.8539295</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>17.051</v>
+        <v>17.049</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>10.8</v>
@@ -1501,7 +1501,7 @@
         <v>96.5</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.0112705</v>
+        <v>-0.011270477</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>113.88</v>
@@ -1519,7 +1519,7 @@
         <v>1.643</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>17.970205</v>
+        <v>17.771639</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>16.232128</v>
@@ -1867,7 +1867,7 @@
         <v>2.32</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>-0.0607288</v>
+        <v>-0.06072878399999999</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>4.95</v>
@@ -2671,7 +2671,7 @@
         <v>19.61</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.406297</v>
+        <v>-0.4062972000000001</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>-0.159</v>
@@ -2718,7 +2718,7 @@
         <v>26.76</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>-0.0247814</v>
+        <v>-0.02478135</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.136</v>
@@ -2906,7 +2906,7 @@
         <v>13.67</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-0.0346045</v>
+        <v>-0.034604504</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.079</v>
@@ -2953,7 +2953,7 @@
         <v>96.5</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.0112705</v>
+        <v>-0.011270477</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>0.008</v>
@@ -3237,7 +3237,7 @@
         <v>2.32</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.0607288</v>
+        <v>-0.06072878399999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-0.07200000000000001</v>
@@ -3576,7 +3576,7 @@
         <v>35.788</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.013044</v>
+        <v>22.523405</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>14.086344</v>
@@ -3597,7 +3597,7 @@
         <v>2.7493122</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>2.3</v>
+        <v>2.35</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>3.75754</v>
@@ -3652,7 +3652,7 @@
         <v>1.1214118</v>
       </c>
       <c r="M3" s="3" t="n">
-        <v>-1.72</v>
+        <v>-1.75</v>
       </c>
       <c r="N3" s="3" t="n">
         <v>10.80017</v>
@@ -3739,19 +3739,19 @@
         <v>10.426</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.88816</v>
+        <v>31.840765</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>16.826635</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>11.288</v>
+        <v>11.286</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>9.1</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2.767</v>
+        <v>2.766</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>-37.194942</v>
@@ -3760,7 +3760,7 @@
         <v>1.4606829</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>3.04</v>
+        <v>3.14</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>5.94177</v>
@@ -3792,10 +3792,10 @@
         <v>9.673999999999999</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.452053</v>
+        <v>46.539474</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.072357</v>
+        <v>15.095321</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.638</v>
@@ -3813,10 +3813,10 @@
         <v>0.5516078</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>2.34668</v>
+        <v>2.34311</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>9.407</v>
@@ -3845,7 +3845,7 @@
         <v>6.119</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6811988</v>
+        <v>3.593085</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>9.949173</v>
@@ -3866,7 +3866,7 @@
         <v>1.4954581</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>22.02</v>
+        <v>22.56</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>8.147410000000001</v>
@@ -3898,13 +3898,13 @@
         <v>5.915</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>19.173334</v>
+        <v>18.435898</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>17.504938</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>8.374000000000001</v>
+        <v>8.372999999999999</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>7.3</v>
@@ -3919,7 +3919,7 @@
         <v>2.940419</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3</v>
+        <v>3.12</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>3.28593</v>
@@ -3951,19 +3951,19 @@
         <v>5.836</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.613096</v>
+        <v>15.827978</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>11.276708</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>11.373</v>
+        <v>11.371</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>9.6</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.719</v>
+        <v>3.718</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>5.7716966</v>
@@ -3972,7 +3972,7 @@
         <v>1.9944898</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>5.04</v>
+        <v>5.29</v>
       </c>
       <c r="N9" s="3" t="n">
         <v>7.42504</v>
@@ -4010,13 +4010,13 @@
         <v>23.874111</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>11.021</v>
+        <v>11.009</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>9.6</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>4.336</v>
+        <v>4.331</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>5.199397</v>
@@ -4080,7 +4080,7 @@
         <v>0.4755292</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-2.36</v>
+        <v>-2.42</v>
       </c>
       <c r="N11" s="3" t="n">
         <v>0.925</v>
@@ -4165,7 +4165,7 @@
         <v>4.819</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69</v>
+        <v>66.77419</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>27.661594</v>
@@ -4192,7 +4192,7 @@
         <v>4.2476387</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="N13" s="3" t="n">
         <v>0.7483300000000001</v>
@@ -4285,7 +4285,7 @@
         <v>7.8539295</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>17.051</v>
+        <v>17.049</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>10.8</v>
@@ -4332,7 +4332,7 @@
         <v>1.726</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>17.970205</v>
+        <v>17.771639</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>16.232128</v>
@@ -4353,7 +4353,7 @@
         <v>3.1662657</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>5.37</v>
+        <v>5.43</v>
       </c>
       <c r="N16" s="3" t="n">
         <v>5.945</v>
@@ -4410,7 +4410,7 @@
         <v>1.740646</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="N17" s="3" t="n">
         <v>0.99</v>
@@ -4518,7 +4518,7 @@
         <v>1.0893636</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>-0.22</v>
+        <v>-0.23</v>
       </c>
       <c r="N19" s="3" t="n">
         <v>1.21</v>
@@ -4683,7 +4683,7 @@
         <v>0.27761704</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>-1.05</v>
+        <v>-1.12</v>
       </c>
       <c r="N22" s="3" t="n">
         <v>-0.41</v>
@@ -6877,7 +6877,7 @@
         <v>0.41693002</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>1.94</v>
+        <v>1.98</v>
       </c>
       <c r="P2" s="5" t="n">
         <v>0.4255</v>
@@ -6930,7 +6930,7 @@
         <v>0.18823999</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>0.91029</v>
+        <v>0.9117</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -7046,10 +7046,10 @@
         <v>0.27027</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.68558997</v>
+        <v>0.68557</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>0.97</v>
+        <v>1</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -7163,7 +7163,7 @@
         <v>0.73223996</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.89</v>
+        <v>0.91</v>
       </c>
       <c r="P7" s="5" t="n">
         <v>0.0319</v>
@@ -7216,10 +7216,10 @@
         <v>0.07935</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>0.88903</v>
+        <v>0.88882005</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>1.74</v>
+        <v>1.81</v>
       </c>
       <c r="P8" s="5" t="n">
         <v>0.32369998</v>
@@ -7275,7 +7275,7 @@
         <v>0.81711</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="P9" s="5" t="n">
         <v>0.0828</v>
@@ -7447,7 +7447,7 @@
         <v>0.19124001</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>1.59</v>
+        <v>1.63</v>
       </c>
       <c r="P12" s="5" t="n">
         <v>0.2831</v>
@@ -7497,7 +7497,7 @@
         <v>0.0498</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>0.07047</v>
+        <v>0.07084</v>
       </c>
       <c r="N13" s="5" t="n">
         <v>0.93144995</v>
@@ -7679,7 +7679,7 @@
         <v>0.64762</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>1.23</v>
+        <v>1.24</v>
       </c>
       <c r="P16" s="5" t="n">
         <v>0.221</v>
@@ -7787,10 +7787,10 @@
         <v>0.028099999</v>
       </c>
       <c r="M18" s="5" t="n">
-        <v>0.17495</v>
+        <v>0.13798</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.76093</v>
+        <v>0.76087</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         <v>0.68561995</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>3.67</v>
+        <v>3.81</v>
       </c>
       <c r="P19" s="5" t="n">
         <v>4.5455</v>
@@ -8464,7 +8464,7 @@
         <v>35.788</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.013044</v>
+        <v>22.523405</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -8554,7 +8554,7 @@
         <v>10.426</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>32.88816</v>
+        <v>31.840765</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -8571,7 +8571,7 @@
         <v>-0.183</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>11.288</v>
+        <v>11.286</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>9.1</v>
@@ -8646,7 +8646,7 @@
         <v>9.673999999999999</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>48.452053</v>
+        <v>46.539474</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -8708,7 +8708,7 @@
         <v>6.119</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6811988</v>
+        <v>3.593085</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -8752,7 +8752,7 @@
         <v>5.836</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.613096</v>
+        <v>15.827978</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8767,7 +8767,7 @@
         <v>-0.252</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.373</v>
+        <v>11.371</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>9.6</v>
@@ -8796,7 +8796,7 @@
         <v>1.726</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.970205</v>
+        <v>17.771639</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.041</v>
@@ -8840,7 +8840,7 @@
         <v>5.915</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>19.173334</v>
+        <v>18.435898</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8855,7 +8855,7 @@
         <v>-0.068</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.374000000000001</v>
+        <v>8.372999999999999</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>7.3</v>
@@ -8901,7 +8901,7 @@
         <v>-0.079</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.051</v>
+        <v>17.049</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>10.8</v>
@@ -9145,7 +9145,7 @@
         <v>-0.159</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>11.021</v>
+        <v>11.009</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>9.6</v>
@@ -9174,7 +9174,7 @@
         <v>4.819</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>69</v>
+        <v>66.77419</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -10418,7 +10418,7 @@
         <v>0.18823999</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.91029</v>
+        <v>0.9117</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>1.72</v>
@@ -10472,7 +10472,7 @@
         <v>0.27027</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.68558997</v>
+        <v>0.68557</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>3.24</v>
@@ -10553,7 +10553,7 @@
         <v>0.07935</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.88903</v>
+        <v>0.88882005</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>3.89</v>
@@ -10685,7 +10685,7 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.07047</v>
+        <v>0.07084</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>0.93144995</v>
@@ -10820,10 +10820,10 @@
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0.17495</v>
+        <v>0.13798</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.76093</v>
+        <v>0.76087</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>3.68</v>
@@ -12087,8 +12087,12 @@
       <c r="B61" s="13" t="n">
         <v>1045.61</v>
       </c>
-      <c r="C61" s="13" t="n"/>
-      <c r="D61" s="13" t="n"/>
+      <c r="C61" s="13" t="n">
+        <v>1163.17</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <v>893.28</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-21 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -1158,7 +1158,7 @@
         <v>54.47222</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.874111</v>
+        <v>23.848154</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>11.009</v>
@@ -4007,7 +4007,7 @@
         <v>54.47222</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.874111</v>
+        <v>23.848154</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>11.009</v>
@@ -4019,7 +4019,7 @@
         <v>4.331</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.199397</v>
+        <v>5.193744</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>4.499046</v>
@@ -4028,10 +4028,10 @@
         <v>0.36</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.8213919</v>
+        <v>0.8222859</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>3.7715912</v>
+        <v>3.7756963</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-22 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -781,7 +781,7 @@
         <v>23.67</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.0497792</v>
+        <v>-0.049779196</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -842,7 +842,7 @@
         <v>99.98</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.0308259</v>
+        <v>-0.030825903</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -1019,7 +1019,7 @@
         <v>57.52</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-0.0390912</v>
+        <v>-0.039091215</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>83.73</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.0466811</v>
+        <v>-0.046013675</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>118.46</v>
@@ -1090,16 +1090,16 @@
         <v>-0.293</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.836</v>
+        <v>5.838</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>10.878</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.827978</v>
+        <v>15.833649</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>11.276708</v>
+        <v>11.280748</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>11.371</v>
@@ -1158,7 +1158,7 @@
         <v>54.47222</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.848154</v>
+        <v>23.858448</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>11.009</v>
@@ -1381,7 +1381,7 @@
         <v>5.46</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.7272719999999999</v>
+        <v>-0.7272720300000001</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>10.15</v>
@@ -1682,7 +1682,7 @@
         <v>26.2</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.0374724</v>
+        <v>-0.03747246</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>32.74</v>
@@ -1806,7 +1806,7 @@
         <v>6.11</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.0671756</v>
+        <v>-0.067175584</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>9.949999999999999</v>
@@ -2389,7 +2389,7 @@
         <v>23.67</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.0497792</v>
+        <v>-0.049779196</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.336</v>
@@ -2436,7 +2436,7 @@
         <v>99.98</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.0308259</v>
+        <v>-0.030825903</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.183</v>
@@ -2577,7 +2577,7 @@
         <v>57.52</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>-0.0390912</v>
+        <v>-0.039091215</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.068</v>
@@ -2621,10 +2621,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>83.73</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.0466811</v>
+        <v>-0.046013675</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.252</v>
@@ -2636,10 +2636,10 @@
         <v>-2.8</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.117</v>
+        <v>-0.116</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.171</v>
+        <v>-0.17</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>-0.293</v>
@@ -2859,7 +2859,7 @@
         <v>5.46</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.7272719999999999</v>
+        <v>-0.7272720300000001</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>-0.273</v>
@@ -3094,7 +3094,7 @@
         <v>26.2</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.0374724</v>
+        <v>-0.03747246</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-0.032</v>
@@ -3190,7 +3190,7 @@
         <v>6.11</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.0671756</v>
+        <v>-0.067175584</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-0.319</v>
@@ -3945,16 +3945,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>83.73</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.836</v>
+        <v>5.838</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>15.827978</v>
+        <v>15.833649</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>11.276708</v>
+        <v>11.280748</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>11.371</v>
@@ -3966,10 +3966,10 @@
         <v>3.718</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>5.7716966</v>
+        <v>5.7737646</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>1.9944898</v>
+        <v>1.9952044</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>5.29</v>
@@ -4007,7 +4007,7 @@
         <v>54.47222</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.848154</v>
+        <v>23.858448</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>11.009</v>
@@ -4019,7 +4019,7 @@
         <v>4.331</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.193744</v>
+        <v>5.1959863</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>4.499046</v>
@@ -4028,10 +4028,10 @@
         <v>0.36</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.8222859</v>
+        <v>0.8219311</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>3.7756963</v>
+        <v>3.7740672</v>
       </c>
     </row>
     <row r="11">
@@ -6967,7 +6967,7 @@
         <v>34</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>36.11471</v>
+        <v>36.17353</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>76</v>
@@ -6976,7 +6976,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.526</v>
+        <v>0.528</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -7237,7 +7237,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>83.73</v>
+        <v>83.76000000000001</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -7307,16 +7307,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.87972</v>
+        <v>28.826334</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.234634</v>
+        <v>37.165802</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.962032</v>
+        <v>21.921434</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.473</v>
+        <v>0.47</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -8749,10 +8749,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>5.836</v>
+        <v>5.838</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>15.827978</v>
+        <v>15.833649</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -11221,7 +11221,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1269.24</v>
+        <v>1269.23</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1219.65</v>
@@ -11237,7 +11237,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1274.55</v>
+        <v>1274.54</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1221.89</v>
@@ -11269,7 +11269,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1259.54</v>
+        <v>1259.53</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1237.34</v>
@@ -11317,7 +11317,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1208.45</v>
+        <v>1208.44</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1241.38</v>
@@ -11429,7 +11429,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1158.88</v>
+        <v>1158.87</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1225.88</v>
@@ -11445,7 +11445,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1163.97</v>
+        <v>1163.96</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1232.28</v>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1142.68</v>
+        <v>1142.67</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1243.8</v>
@@ -11621,7 +11621,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1115.8</v>
+        <v>1115.79</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1235.21</v>
@@ -11653,7 +11653,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1114.71</v>
+        <v>1114.7</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1237.89</v>
@@ -11845,7 +11845,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1088.52</v>
+        <v>1088.51</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1226.93</v>
@@ -11861,7 +11861,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1083.59</v>
+        <v>1083.58</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1227.63</v>
@@ -11877,7 +11877,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1079.45</v>
+        <v>1079.44</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1216.81</v>
@@ -11893,7 +11893,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1095.38</v>
+        <v>1095.37</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1225.39</v>
@@ -11909,7 +11909,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1093.13</v>
+        <v>1093.12</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1218.56</v>
@@ -11925,7 +11925,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1061.18</v>
+        <v>1061.17</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1202.59</v>
@@ -11957,7 +11957,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1062.16</v>
+        <v>1062.15</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1211.17</v>
@@ -12021,7 +12021,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1056.95</v>
+        <v>1056.94</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1196.6</v>
@@ -12037,7 +12037,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1069.59</v>
+        <v>1069.58</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1199.74</v>
@@ -12069,7 +12069,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1074.29</v>
+        <v>1074.28</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1180.09</v>
@@ -12085,7 +12085,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1045.61</v>
+        <v>1045.62</v>
       </c>
       <c r="C61" s="13" t="n">
         <v>1163.17</v>
@@ -12101,7 +12101,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1045.61</v>
+        <v>1045.62</v>
       </c>
     </row>
     <row r="64">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-22 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -7307,13 +7307,13 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.826334</v>
+        <v>28.819672</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.165802</v>
+        <v>37.15721</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.921434</v>
+        <v>21.916367</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>0.47</v>
@@ -11432,7 +11432,7 @@
         <v>1158.87</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>1225.88</v>
+        <v>1225.87</v>
       </c>
       <c r="D20" s="13" t="n">
         <v>1016.19</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-23 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.77</v>
+        <v>54</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.034762897</v>
+        <v>0.0202154</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,34 +670,34 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.233</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>37.032</v>
+        <v>36.511</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>48.099</v>
+        <v>48.818</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.306385</v>
+        <v>22.978724</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>14.576026</v>
+        <v>14.371104</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>10.611</v>
+        <v>10.77</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O2" s="8" t="n">
         <v>0.888</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.347</v>
+        <v>0.328</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.156</v>
+        <v>-0.168</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>111.03</v>
+        <v>109.38</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>0.059345493</v>
+        <v>0.0436027</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.6459999999999999</v>
+        <v>-0.6509999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>19.462</v>
+        <v>19.173</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.054</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>10.280394</v>
+        <v>10.127618</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.097</v>
@@ -755,10 +755,10 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>-0.55</v>
+        <v>-0.556</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>-0.491</v>
+        <v>-0.499</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>24.44</v>
+        <v>23.96</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.03251691</v>
+        <v>0.0122518</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,13 +790,13 @@
         <v>21.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.499</v>
+        <v>-0.509</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>12.166</v>
+        <v>11.927</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>12.431</v>
+        <v>12.562</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
@@ -804,22 +804,22 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>12.557159</v>
+        <v>12.310537</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>45.556</v>
+        <v>46.034</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.397</v>
+        <v>-0.409</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.315</v>
+        <v>-0.328</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>104.03</v>
+        <v>101.13</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.040508056</v>
+        <v>0.0115022</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,22 +851,22 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.228</v>
+        <v>-0.249</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.849</v>
+        <v>10.546</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>19.746</v>
+        <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>33.130573</v>
+        <v>32.207005</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.508251</v>
+        <v>17.02018</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>11.286</v>
+        <v>11.354</v>
       </c>
       <c r="N5" s="7" t="n">
         <v>9.1</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.237</v>
+        <v>0.202</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>-0.149</v>
+        <v>-0.173</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.72</v>
+        <v>36.95</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.066440554</v>
+        <v>0.04467069999999999</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,34 +910,34 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.08</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.317</v>
+        <v>10.106</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>39.176</v>
+        <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.63158</v>
+        <v>48.618423</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.098263</v>
+        <v>15.769639</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>16.638</v>
+        <v>16.81</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>1.396</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.163</v>
+        <v>0.14</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.034</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.55</v>
+        <v>81.94</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.043054595</v>
+        <v>0.0108562</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,19 +969,19 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.08900000000000001</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.383</v>
+        <v>6.186</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.476000000000001</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.747784</v>
+        <v>3.6320925</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.377531</v>
+        <v>10.057183</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.058</v>
@@ -993,10 +993,10 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.233</v>
+        <v>0.195</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>-0.017</v>
+        <v>-0.047</v>
       </c>
     </row>
     <row r="8">
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>59.98</v>
+        <v>58.08</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.042767715</v>
+        <v>0.9735770000000001</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1028,22 +1028,22 @@
         <v>35.09</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.131</v>
+        <v>-0.158</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.168</v>
+        <v>5.972</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>6.814</v>
+        <v>6.847</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>19.22436</v>
+        <v>18.615385</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>18.253584</v>
+        <v>17.675362</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>8.372999999999999</v>
+        <v>8.413</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>7.3</v>
@@ -1052,10 +1052,10 @@
         <v>1.453</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0.403</v>
+        <v>0.359</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.028</v>
+        <v>-0.059</v>
       </c>
     </row>
     <row r="9">
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.87</v>
+        <v>84.62</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.025191028</v>
+        <v>0.0102674</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>118.46</v>
@@ -1087,19 +1087,19 @@
         <v>80.23999999999999</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.275</v>
+        <v>-0.286</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.985</v>
+        <v>5.898</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>10.878</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.232515</v>
+        <v>15.99622</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>11.564921</v>
+        <v>11.396572</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>11.371</v>
@@ -1111,10 +1111,10 @@
         <v>0.66</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>-0.242</v>
+        <v>-0.253</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>-0.233</v>
+        <v>-0.244</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.82</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>0.010708776</v>
+        <v>19.53</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>-0.4079550000000001</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1146,154 +1146,154 @@
         <v>15.725</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.385</v>
+        <v>-0.394</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.866</v>
+        <v>5.78</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>5.587</v>
+        <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>55.055553</v>
+        <v>54.25</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>24.113943</v>
+        <v>23.811478</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>11.009</v>
+        <v>10.962</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>2.002</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.138</v>
+        <v>-0.151</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.15</v>
+        <v>-0.163</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>27.18</v>
+        <v>10.68</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.015508184</v>
+        <v>0.0210325</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>31.58</v>
+        <v>14.38</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>17.86</v>
+        <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.139</v>
+        <v>-0.257</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.547</v>
+        <v>5.4</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>30.363</v>
-      </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>4.993</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>25.428574</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>29.378378</v>
+        <v>12.312517</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>8.688000000000001</v>
+        <v>10.175</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>1.977</v>
-      </c>
-      <c r="P11" s="9" t="n">
-        <v>-0.034</v>
-      </c>
-      <c r="Q11" s="4" t="n">
-        <v>0.153</v>
+        <v>1.1</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="Q11" s="9" t="n">
+        <v>-0.078</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.77</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>0.02963675</v>
+        <v>26.44</v>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>-0.0119581</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>14.38</v>
+        <v>31.58</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>5.59</v>
+        <v>17.86</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.251</v>
+        <v>-0.163</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.446</v>
+        <v>5.397</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>4.882</v>
-      </c>
-      <c r="K12" s="7" t="n">
-        <v>25.642859</v>
+        <v>30.298</v>
+      </c>
+      <c r="K12" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>12.416274</v>
+        <v>28.583784</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>9.948</v>
+        <v>8.669</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>0.5479999999999999</v>
-      </c>
-      <c r="Q12" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>1.977</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0.122</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.4</v>
+        <v>21.75</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.033816369</v>
+        <v>0.0507246</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.055</v>
+        <v>-0.04</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4.982</v>
+        <v>5.063</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.03225999999999</v>
+        <v>70.16128999999999</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>28.59701</v>
+        <v>29.064718</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.887</v>
+        <v>0.9179999999999999</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.108</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.23</v>
+        <v>13.05</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>0.034401844</v>
+        <v>0.0203284</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.288</v>
+        <v>-0.297</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.441</v>
+        <v>2.408</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.928</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>12.277966</v>
+        <v>12.110919</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.721</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="9" t="n">
-        <v>-0.016</v>
+        <v>-0.03</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>-0.12</v>
+        <v>-0.132</v>
       </c>
     </row>
     <row r="15">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.47</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.014413931</v>
+        <v>0.183146</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,22 +1451,22 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.461</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.253</v>
+        <v>2.225</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12.751</v>
+        <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.040652</v>
+        <v>11.891304</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.961752</v>
+        <v>6.8754005</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>10.572</v>
+        <v>10.582</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>8.4</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.006</v>
+        <v>-0.018</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>-0.262</v>
+        <v>-0.272</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.76</v>
+        <v>14.44</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.079370885</v>
+        <v>0.0563277</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,13 +1510,13 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.284</v>
+        <v>-0.299</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.97</v>
+        <v>1.928</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>12.313</v>
+        <v>12.411</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
@@ -1524,22 +1524,22 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.477302999999999</v>
+        <v>8.296322999999999</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>17.049</v>
+        <v>17.184</v>
       </c>
       <c r="N16" s="7" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="O16" s="8" t="n">
         <v>1.364</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>-0.15</v>
+        <v>-0.168</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.006</v>
+        <v>-0.028</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>99.19</v>
+        <v>98.26000000000001</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.027875674</v>
+        <v>0.0182384</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,34 +1571,34 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.129</v>
+        <v>-0.137</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.774</v>
+        <v>1.757</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.643</v>
+        <v>1.674</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>18.267036</v>
+        <v>18.095766</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.684608</v>
+        <v>16.528175</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>8.614000000000001</v>
+        <v>8.779</v>
       </c>
       <c r="N17" s="7" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>1.376</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.238</v>
+        <v>0.226</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
     </row>
     <row r="18">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>0.045253844</v>
+        <v>0.0375275</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1630,13 +1630,13 @@
         <v>4.51</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>-0.655</v>
+        <v>-0.6579999999999999</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.218</v>
+        <v>1.209</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0.866</v>
+        <v>0.908</v>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
@@ -1644,10 +1644,10 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.7828283</v>
+        <v>4.7474747</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>-7.181</v>
+        <v>-7.528</v>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="9" t="n">
-        <v>-0.5710000000000001</v>
+        <v>-0.574</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-0.5639999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.33</v>
+        <v>11.26</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.037545774</v>
+        <v>0.0311355</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,34 +1693,34 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.154</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.214</v>
+        <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.883333</v>
+        <v>18.766666</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>12.235025</v>
+        <v>12.159433</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>6.422</v>
+        <v>6.569</v>
       </c>
       <c r="N19" s="7" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="O19" s="8" t="n">
         <v>1.07</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0.114</v>
+        <v>0.107</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>-0.004</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.58</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.014503784</v>
+        <v>0.610686</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,13 +1752,13 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.195</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.702</v>
+        <v>0.696</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.149</v>
+        <v>1.153</v>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
@@ -1766,10 +1766,10 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.966942</v>
+        <v>21.785124</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>9.414</v>
+        <v>9.449</v>
       </c>
       <c r="N20" s="7" t="n">
         <v>7.2</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>-0.016</v>
+        <v>-0.024</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>-0.017</v>
+        <v>-0.026</v>
       </c>
     </row>
     <row r="21">
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>12.34</v>
+        <v>12.11</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0.02491696</v>
+        <v>0.581393</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,10 +1813,10 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.416</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.607</v>
+        <v>0.595</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>6.095</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-8.281879</v>
+        <v>-14.950617</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>18.843</v>
@@ -1841,10 +1841,10 @@
         </is>
       </c>
       <c r="P21" s="9" t="n">
-        <v>-0.296</v>
+        <v>-0.31</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>-0.258</v>
+        <v>-0.272</v>
       </c>
     </row>
     <row r="22">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0.054009805</v>
+        <v>0.06382979999999999</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,13 +1876,13 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.353</v>
+        <v>-0.347</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.174</v>
+        <v>0.176</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.496</v>
+        <v>0.507</v>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.596294</v>
+        <v>8.676384000000001</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>6.676</v>
+        <v>6.818</v>
       </c>
       <c r="N22" s="7" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>1.206</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>-0.296</v>
+        <v>-0.29</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>-0.282</v>
+        <v>-0.275</v>
       </c>
     </row>
     <row r="23">
@@ -2152,28 +2152,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.77</v>
+        <v>54</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.034762897</v>
+        <v>0.0202154</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.168</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.347</v>
+        <v>0.328</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>53.7</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.051</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.031</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.233</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2199,28 +2199,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>111.03</v>
+        <v>109.38</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.059345493</v>
+        <v>0.0436027</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.491</v>
+        <v>-0.499</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.55</v>
+        <v>-0.556</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-56</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.228</v>
+        <v>-0.24</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.517</v>
+        <v>-0.524</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.6459999999999999</v>
+        <v>-0.6509999999999999</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2246,28 +2246,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>24.44</v>
+        <v>23.96</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.03251691</v>
+        <v>0.0122518</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.315</v>
+        <v>-0.328</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.397</v>
+        <v>-0.409</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-35.6</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.1</v>
+        <v>-0.118</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.316</v>
+        <v>-0.329</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.499</v>
+        <v>-0.509</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2293,28 +2293,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>104.03</v>
+        <v>101.13</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.040508056</v>
+        <v>0.0115022</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.173</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.237</v>
+        <v>0.202</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>35.3</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.053</v>
+        <v>-0.08</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.09</v>
+        <v>-0.115</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.228</v>
+        <v>-0.249</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2340,28 +2340,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.72</v>
+        <v>36.95</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.066440554</v>
+        <v>0.04467069999999999</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.034</v>
+        <v>0.013</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.163</v>
+        <v>0.14</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>11.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.064</v>
+        <v>0.043</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.073</v>
+        <v>0.051</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.08</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,28 +2387,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.55</v>
+        <v>81.94</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.043054595</v>
+        <v>0.0108562</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.047</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.233</v>
+        <v>0.195</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>20.7</v>
+        <v>20.6</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.008</v>
+        <v>-0.024</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.021</v>
+        <v>-0.01</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.08900000000000001</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2434,28 +2434,28 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>59.98</v>
+        <v>58.08</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.042767715</v>
+        <v>0.9735770000000001</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.059</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.403</v>
+        <v>0.359</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>39.5</v>
+        <v>39.4</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.058</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.022</v>
+        <v>-0.011</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.131</v>
+        <v>-0.158</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>1.453</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.87</v>
+        <v>84.62</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.025191028</v>
+        <v>0.0102674</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.244</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>-0.242</v>
+        <v>-0.253</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>-2.8</v>
+        <v>-2.9</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.107</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.162</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.275</v>
+        <v>-0.286</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>0.66</v>
@@ -2528,28 +2528,28 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.82</v>
+        <v>19.53</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.010708776</v>
+        <v>-0.4079550000000001</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.163</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.138</v>
+        <v>-0.151</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-27.9</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.078</v>
+        <v>0.063</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-0.191</v>
+        <v>-0.203</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-0.385</v>
+        <v>-0.394</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>2.002</v>
@@ -2561,95 +2561,95 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>27.18</v>
+        <v>10.68</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.015508184</v>
+        <v>0.0210325</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.153</v>
+        <v>-0.078</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>-0.034</v>
+        <v>0.535</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>-23</v>
+        <v>27.9</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.159</v>
+        <v>0.062</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.102</v>
+        <v>-0.049</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.139</v>
+        <v>-0.257</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>1.977</v>
+        <v>1.1</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>6358500</v>
+        <v>1926430</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.77</v>
+        <v>26.44</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.02963675</v>
+        <v>-0.0119581</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>0.122</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.5479999999999999</v>
+        <v>-0.06</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>27.9</v>
+        <v>-23.1</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.128</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.04099999999999999</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.251</v>
+        <v>-0.163</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>1.1</v>
+        <v>1.977</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1926430</v>
+        <v>6358500</v>
       </c>
     </row>
     <row r="13">
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.4</v>
+        <v>21.75</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.033816369</v>
+        <v>0.0507246</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.108</v>
+        <v>0.126</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.887</v>
+        <v>0.9179999999999999</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>51.1</v>
+        <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.138</v>
+        <v>0.156</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.17</v>
+        <v>0.19</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.055</v>
+        <v>-0.04</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2716,28 +2716,28 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.23</v>
+        <v>13.05</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.034401844</v>
+        <v>0.0203284</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.12</v>
+        <v>-0.132</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.016</v>
+        <v>-0.03</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.04</v>
+        <v>-0.053</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.144</v>
+        <v>-0.155</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.288</v>
+        <v>-0.297</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2763,28 +2763,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.47</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.014413931</v>
+        <v>0.183146</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.272</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.018</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>9.300000000000001</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.091</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.294</v>
+        <v>-0.303</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.461</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2810,28 +2810,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.76</v>
+        <v>14.44</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.079370885</v>
+        <v>0.0563277</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.028</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.168</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.2</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.048</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.091</v>
+        <v>-0.111</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.284</v>
+        <v>-0.299</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2857,28 +2857,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>99.19</v>
+        <v>98.26000000000001</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.027875674</v>
+        <v>0.0182384</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.238</v>
+        <v>0.226</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.7</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.045</v>
+        <v>0.036</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.032</v>
+        <v>0.022</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.129</v>
+        <v>-0.137</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2904,28 +2904,28 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.045253844</v>
+        <v>0.0375275</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.5710000000000001</v>
+        <v>-0.574</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-31.1</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.342</v>
+        <v>-0.347</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.536</v>
+        <v>-0.54</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.655</v>
+        <v>-0.6579999999999999</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>1.993</v>
@@ -2951,28 +2951,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.33</v>
+        <v>11.26</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.037545774</v>
+        <v>0.0311355</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.004</v>
+        <v>-0.01</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.114</v>
+        <v>0.107</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.2</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0.003</v>
+        <v>-0.003</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.012</v>
+        <v>0.005</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.154</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -2998,28 +2998,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.58</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.014503784</v>
+        <v>0.610686</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.026</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-0.016</v>
+        <v>-0.024</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.049</v>
+        <v>-0.057</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.019</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.195</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3045,28 +3045,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>12.34</v>
+        <v>12.11</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.02491696</v>
+        <v>0.581393</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.258</v>
+        <v>-0.272</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.31</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>38.7</v>
+        <v>38.6</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.166</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.07200000000000001</v>
+        <v>-0.08900000000000001</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.416</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.054009805</v>
+        <v>0.06382979999999999</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.282</v>
+        <v>-0.275</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.29</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>5</v>
+        <v>5.1</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.231</v>
+        <v>-0.224</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.248</v>
+        <v>-0.241</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.353</v>
+        <v>-0.347</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3200,7 +3200,7 @@
         <v>-0.239</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>-293.6</v>
+        <v>-288.9</v>
       </c>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
@@ -3342,31 +3342,31 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.77</v>
+        <v>54</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>37.032</v>
+        <v>36.511</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.306385</v>
+        <v>22.978724</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>14.576026</v>
+        <v>14.371104</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>10.611</v>
+        <v>10.77</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>3.695</v>
+        <v>3.75</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.24703</v>
+        <v>22.920204</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.8448865</v>
+        <v>2.8048906</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>111.03</v>
+        <v>109.38</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>19.462</v>
+        <v>19.173</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>10.280394</v>
+        <v>10.127618</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.097</v>
@@ -3418,10 +3418,10 @@
         <v>1.834</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.1525784</v>
+        <v>2.1205893</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1879625</v>
+        <v>1.1703084</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>24.44</v>
+        <v>23.96</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>12.166</v>
+        <v>11.927</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,22 +3461,22 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12.557159</v>
+        <v>12.310537</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>45.556</v>
+        <v>46.034</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>2.053</v>
+        <v>2.075</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>19.153605</v>
+        <v>18.777428</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>2.0093336</v>
+        <v>1.9698704</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,31 +3505,31 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>104.03</v>
+        <v>101.13</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.849</v>
+        <v>10.546</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>33.130573</v>
+        <v>32.207005</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.508251</v>
+        <v>17.02018</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>11.286</v>
+        <v>11.354</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>9.1</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2.766</v>
+        <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-38.701637</v>
+        <v>-37.62277</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.5198523</v>
+        <v>1.477484</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,31 +3558,31 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.72</v>
+        <v>36.95</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.317</v>
+        <v>10.106</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.63158</v>
+        <v>48.618423</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.098263</v>
+        <v>15.769639</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>16.638</v>
+        <v>16.81</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>11.5</v>
+        <v>11.6</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>2.234</v>
+        <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>4.0097804</v>
+        <v>3.9279263</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5882569</v>
+        <v>0.57624847</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.55</v>
+        <v>81.94</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.383</v>
+        <v>6.186</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.747784</v>
+        <v>3.6320925</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.377531</v>
+        <v>10.057183</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.058</v>
@@ -3632,10 +3632,10 @@
         <v>2.071</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4753344</v>
+        <v>2.3989227</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5598445</v>
+        <v>1.5116932</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,31 +3664,31 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>59.98</v>
+        <v>58.08</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.168</v>
+        <v>5.972</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>19.22436</v>
+        <v>18.615385</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>18.253584</v>
+        <v>17.675362</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>8.372999999999999</v>
+        <v>8.413</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>7.3</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.388</v>
+        <v>3.404</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.791714</v>
+        <v>16.259798</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>3.066174</v>
+        <v>2.9690464</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>3.12</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.87</v>
+        <v>84.62</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.985</v>
+        <v>5.898</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.232515</v>
+        <v>15.99622</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>11.564921</v>
+        <v>11.396572</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>11.371</v>
@@ -3738,10 +3738,10 @@
         <v>3.718</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>5.9192114</v>
+        <v>5.8330464</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.0454657</v>
+        <v>2.01569</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>5.29</v>
@@ -3770,148 +3770,148 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.82</v>
+        <v>19.53</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.866</v>
+        <v>5.78</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>55.055553</v>
+        <v>54.25</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>24.113943</v>
+        <v>23.811478</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>11.009</v>
+        <v>10.962</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>4.331</v>
+        <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.251629</v>
+        <v>5.1857567</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.5472255</v>
+        <v>4.480692</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>0.8219311</v>
+        <v>0.82019275</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>3.7740672</v>
+        <v>3.7660851</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>27.18</v>
+        <v>10.68</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.547</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>5.4</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>25.428574</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>29.378378</v>
+        <v>12.312517</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>8.688000000000001</v>
+        <v>10.175</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>7.3</v>
+        <v>7.9</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2.643</v>
+        <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.5714451</v>
+        <v>7.2505093</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>0.4829038</v>
+        <v>2.3049138</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>-2.42</v>
+        <v>0.42</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.925</v>
+        <v>0.86741</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>17.293</v>
+        <v>1.473</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.77</v>
+        <v>26.44</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.446</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>25.642859</v>
+        <v>5.397</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>12.416274</v>
+        <v>28.583784</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>9.948</v>
+        <v>8.669</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>2.084</v>
+        <v>2.638</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.311609</v>
+        <v>1.5289425</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>2.324337</v>
+        <v>0.46984276</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.42</v>
+        <v>-2.42</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.86741</v>
+        <v>0.925</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>1.473</v>
+        <v>17.293</v>
       </c>
     </row>
     <row r="13">
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.4</v>
+        <v>21.75</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>4.982</v>
+        <v>5.063</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.03225999999999</v>
+        <v>70.16128999999999</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>28.59701</v>
+        <v>29.064718</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.528173</v>
+        <v>14.765783</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.3912787</v>
+        <v>4.4630985</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.23</v>
+        <v>13.05</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.441</v>
+        <v>2.408</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>12.277966</v>
+        <v>12.110919</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.721</v>
@@ -4013,10 +4013,10 @@
         <v>2.361</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.8251119</v>
+        <v>2.7866752</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.9722474</v>
+        <v>0.9590196</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4045,31 +4045,31 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.47</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.253</v>
+        <v>2.225</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.040652</v>
+        <v>11.891304</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.961752</v>
+        <v>6.8754005</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>10.572</v>
+        <v>10.582</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>8.4</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>2.47</v>
+        <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7357255</v>
+        <v>-1.7141961</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.4363681</v>
+        <v>0.43095556</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.76</v>
+        <v>14.44</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.97</v>
+        <v>1.928</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,22 +4109,22 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.477302999999999</v>
+        <v>8.296322999999999</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17.049</v>
+        <v>17.184</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>1.769</v>
+        <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1.0156949</v>
+        <v>0.9940111</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.2830736</v>
+        <v>0.27703032</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,31 +4153,31 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>99.19</v>
+        <v>98.26000000000001</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.774</v>
+        <v>1.757</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>18.267036</v>
+        <v>18.095766</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.684608</v>
+        <v>16.528175</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>8.614000000000001</v>
+        <v>8.779</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>3.014</v>
+        <v>3.071</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2872672</v>
+        <v>3.2564461</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.2545276</v>
+        <v>3.2240133</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.218</v>
+        <v>1.209</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4217,10 +4217,10 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.7828283</v>
+        <v>4.7474747</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-7.181</v>
+        <v>-7.528</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
@@ -4228,13 +4228,13 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1.293</v>
+        <v>1.356</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.6099967</v>
+        <v>1.5980958</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.8194169</v>
+        <v>1.8059682</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4263,31 +4263,31 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.33</v>
+        <v>11.26</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.883333</v>
+        <v>18.766666</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>12.235025</v>
+        <v>12.159433</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>6.422</v>
+        <v>6.569</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.912</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.4574306</v>
+        <v>3.4360697</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.7083203</v>
+        <v>0.70394415</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4316,10 +4316,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.58</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.702</v>
+        <v>0.696</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4327,22 +4327,22 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.966942</v>
+        <v>21.785124</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>9.414</v>
+        <v>9.449</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>7.2</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1.81</v>
+        <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6536021</v>
+        <v>1.6399155</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1051636</v>
+        <v>1.0960162</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4371,10 +4371,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>12.34</v>
+        <v>12.11</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.607</v>
+        <v>0.595</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-8.281879</v>
+        <v>-14.950617</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>18.843</v>
@@ -4394,16 +4394,16 @@
         <v>2.447</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>1.162506</v>
+        <v>1.1408384</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.24355991</v>
+        <v>0.23902032</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-12.58</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>-1.49</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>10.615</v>
@@ -4426,10 +4426,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.174</v>
+        <v>0.176</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -4437,22 +4437,22 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.596294</v>
+        <v>8.676384000000001</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>6.676</v>
+        <v>6.818</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1.631</v>
+        <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.679934</v>
+        <v>-10.779436</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.57304716</v>
+        <v>0.5783861</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -5251,121 +5251,121 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>11.486</v>
+        <v>2.343</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.042</v>
+        <v>0.178</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.5</v>
+        <v>0.51058</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.1893</v>
+        <v>0.23518999</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.043709997</v>
+        <v>0.09804</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.30427998</v>
+        <v>0.20945999</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.10840999</v>
+        <v>0.32813</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0.04044</v>
+        <v>0.23642</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>3.495</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>0.6929999999999999</v>
+        <v>0.491</v>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N11" s="6" t="n">
-        <v>25.622</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>0.887</v>
+        <v>0.478</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>695.117</v>
+        <v>9.69</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>0.8</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2.343</v>
+        <v>11.486</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.178</v>
+        <v>0.042</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.51058</v>
+        <v>0.5</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.23518999</v>
+        <v>0.1893</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09804</v>
+        <v>-0.043709997</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.20945999</v>
+        <v>0.30427998</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.32813</v>
+        <v>-0.10840999</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0.23642</v>
+        <v>0.04044</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>3.495</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0.6929999999999999</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0.07199999999999999</v>
+        <v>25.622</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>0.478</v>
+        <v>0.887</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>9.69</v>
+        <v>695.117</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>1.75</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13">
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>54.77</v>
+        <v>54</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.276</v>
+        <v>0.294</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>1.8</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>111.03</v>
+        <v>109.38</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.9159999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>24.44</v>
+        <v>23.96</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>104.03</v>
+        <v>101.13</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.363</v>
+        <v>0.402</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.24</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.72</v>
+        <v>36.95</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.131</v>
+        <v>0.155</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>84.55</v>
+        <v>81.94</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6554,7 +6554,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.117</v>
+        <v>0.153</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.32</v>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>59.98</v>
+        <v>58.08</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         <v>59</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.223</v>
+        <v>0.263</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>3.89</v>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>85.87</v>
+        <v>84.62</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.578</v>
+        <v>0.601</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>2.68</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>19.82</v>
+        <v>19.53</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6713,16 +6713,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.997198</v>
+        <v>28.926596</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.386097</v>
+        <v>37.29507</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>22.051369</v>
+        <v>21.99768</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.463</v>
+        <v>0.481</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -6748,115 +6748,115 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>27.18</v>
+        <v>10.68</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>strong_buy</t>
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1.82353</v>
+        <v>1.25</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>31.95778</v>
+        <v>17.375</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.176</v>
+        <v>0.627</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>3.8</v>
+        <v>4.92</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0.1713</v>
+        <v>0.1039</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>0.010570001</v>
+        <v>0.68889</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>1.11968</v>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.19124001</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>1.63</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>0</v>
+        <v>0.2831</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>10.77</v>
+        <v>26.44</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1.25</v>
+        <v>1.82353</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>17.375</v>
+        <v>31.95778</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.613</v>
+        <v>0.209</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.92</v>
+        <v>3.8</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0.1039</v>
+        <v>0.1713</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.010570001</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.19124001</v>
-      </c>
-      <c r="O12" s="5" t="n">
-        <v>1.63</v>
+        <v>1.11968</v>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="P12" s="5" t="n">
-        <v>0.2831</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.4</v>
+        <v>21.75</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6894,7 +6894,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.159</v>
+        <v>0.14</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>13.23</v>
+        <v>13.05</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6952,7 +6952,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.367</v>
+        <v>0.385</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.42</v>
@@ -6985,7 +6985,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.47</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
         <v>6.3</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.674</v>
+        <v>0.695</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.08</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.76</v>
+        <v>14.44</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7066,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.295</v>
+        <v>0.323</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>99.19</v>
+        <v>98.26000000000001</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7126,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.096</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.53</v>
@@ -7159,7 +7159,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4.74</v>
+        <v>4.7</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -7182,7 +7182,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1.482</v>
+        <v>1.503</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>1.77</v>
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.33</v>
+        <v>11.26</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.368</v>
+        <v>0.377</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.68</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.58</v>
+        <v>26.36</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.147</v>
+        <v>0.157</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>2.5</v>
@@ -7331,7 +7331,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>12.34</v>
+        <v>12.11</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7354,7 +7354,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0.27</v>
+        <v>0.294</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>9.16</v>
@@ -7389,7 +7389,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7412,7 +7412,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.07</v>
+        <v>1.051</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7695,10 +7695,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>37.032</v>
+        <v>36.511</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.306385</v>
+        <v>22.978724</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7710,16 +7710,16 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.168</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10.611</v>
+        <v>10.77</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>82</v>
+        <v>86.09999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -7739,7 +7739,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.547</v>
+        <v>5.397</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7756,13 +7756,13 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.153</v>
+        <v>0.122</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>8.688000000000001</v>
+        <v>8.669</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="L4" s="7" t="n">
         <v>45</v>
@@ -7771,12 +7771,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>WYNN</t>
+          <t>MLCO</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Wynn Resorts</t>
+          <t>Melco Resorts</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -7785,16 +7785,16 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10.849</v>
+        <v>2.225</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>33.130573</v>
+        <v>11.891304</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.015</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.24510999</v>
+        <v>0.23358</v>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
@@ -7802,27 +7802,27 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.272</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>11.286</v>
+        <v>10.582</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>9.1</v>
+        <v>8.4</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>41.7</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>MLCO</t>
+          <t>MGM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Melco Resorts</t>
+          <t>MGM Resorts International</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -7831,44 +7831,42 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.253</v>
+        <v>10.106</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>12.040652</v>
+        <v>48.618423</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.06</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.23358</v>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.13426</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-0.262</v>
+        <v>0.013</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>10.572</v>
+        <v>16.81</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>8.4</v>
+        <v>11.6</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>40</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MGM</t>
+          <t>WYNN</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>MGM Resorts International</t>
+          <t>Wynn Resorts</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -7877,31 +7875,33 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.317</v>
+        <v>10.546</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.63158</v>
+        <v>32.207005</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.06</v>
+        <v>0.015</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.13426</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>0.1489</v>
+        <v>0.24510999</v>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.034</v>
+        <v>-0.173</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>16.638</v>
+        <v>11.354</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>11.5</v>
+        <v>9.1</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>37.5</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="9">
@@ -7939,10 +7939,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.383</v>
+        <v>6.186</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.747784</v>
+        <v>3.6320925</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7954,7 +7954,7 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.047</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>7.058</v>
@@ -7963,7 +7963,7 @@
         <v>5.9</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>71.40000000000001</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
@@ -7983,10 +7983,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>5.985</v>
+        <v>5.898</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.232515</v>
+        <v>15.99622</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -7998,7 +7998,7 @@
         <v>0.35709</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.244</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>11.371</v>
@@ -8027,10 +8027,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.774</v>
+        <v>1.757</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>18.267036</v>
+        <v>18.095766</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.041</v>
@@ -8042,13 +8042,13 @@
         <v>0.19214001</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.036</v>
+        <v>0.026</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.614000000000001</v>
+        <v>8.779</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>62.7</v>
@@ -8071,10 +8071,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>6.168</v>
+        <v>5.972</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>19.22436</v>
+        <v>18.615385</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8086,10 +8086,10 @@
         <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.059</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.372999999999999</v>
+        <v>8.413</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>7.3</v>
@@ -8115,7 +8115,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.97</v>
+        <v>1.928</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8132,16 +8132,16 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.028</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.049</v>
+        <v>17.184</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>54.3</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="15">
@@ -8161,7 +8161,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.702</v>
+        <v>0.696</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8178,16 +8178,16 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.026</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>9.414</v>
+        <v>9.449</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>7.2</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>34.3</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.607</v>
+        <v>0.595</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8224,7 +8224,7 @@
         <v>-1.1563</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.258</v>
+        <v>-0.272</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>18.843</v>
@@ -8317,10 +8317,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.446</v>
+        <v>5.4</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.642859</v>
+        <v>25.428574</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8332,13 +8332,13 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.078</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>9.948</v>
+        <v>10.175</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="L20" s="7" t="n">
         <v>66.7</v>
@@ -8361,10 +8361,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.866</v>
+        <v>5.78</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>55.055553</v>
+        <v>54.25</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8376,13 +8376,13 @@
         <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.163</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>11.009</v>
+        <v>10.962</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>9.6</v>
+        <v>9.5</v>
       </c>
       <c r="L21" s="7" t="n">
         <v>58.3</v>
@@ -8405,10 +8405,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>4.982</v>
+        <v>5.063</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>69.03225999999999</v>
+        <v>70.16128999999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8420,7 +8420,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.108</v>
+        <v>0.126</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8453,7 +8453,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>12.166</v>
+        <v>11.927</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8470,13 +8470,13 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.315</v>
+        <v>-0.328</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>45.556</v>
+        <v>46.034</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>19.5</v>
+        <v>19.7</v>
       </c>
       <c r="L23" s="7" t="n">
         <v>52</v>
@@ -8499,7 +8499,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>19.462</v>
+        <v>19.173</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8516,7 +8516,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.491</v>
+        <v>-0.499</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>14.097</v>
@@ -8545,7 +8545,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.218</v>
+        <v>1.209</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8562,10 +8562,10 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-7.181</v>
+        <v>-7.528</v>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
@@ -8611,10 +8611,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.883333</v>
+        <v>18.766666</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8626,13 +8626,13 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.004</v>
+        <v>-0.01</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>6.422</v>
+        <v>6.569</v>
       </c>
       <c r="K28" s="7" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="L28" s="7" t="n">
         <v>69.5</v>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.441</v>
+        <v>2.408</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8672,7 +8672,7 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.12</v>
+        <v>-0.132</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>6.721</v>
@@ -8701,7 +8701,7 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.174</v>
+        <v>0.176</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
@@ -8720,13 +8720,13 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.282</v>
+        <v>-0.275</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>6.676</v>
+        <v>6.818</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="L30" s="7" t="n">
         <v>20.8</v>
@@ -9761,55 +9761,55 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.010570001</v>
+        <v>0.68889</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>1.11968</v>
+        <v>0.19124001</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>3.8</v>
+        <v>4.92</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.1713</v>
+        <v>0.1039</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>30537844</v>
+        <v>16337061</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.010570001</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.19124001</v>
+        <v>1.11968</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4.92</v>
+        <v>3.8</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.1039</v>
+        <v>0.1713</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>16337061</v>
+        <v>30537844</v>
       </c>
     </row>
     <row r="13">
@@ -10196,7 +10196,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1267.17</v>
+        <v>1267.92</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1213.06</v>
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1273.07</v>
+        <v>1273.82</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1212.93</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.7</v>
+        <v>1263.51</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1257.63</v>
+        <v>1258.49</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1250.32</v>
+        <v>1251.13</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1255.31</v>
+        <v>1256.04</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1255.92</v>
+        <v>1256.72</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1241.2</v>
+        <v>1241.94</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1194.25</v>
+        <v>1194.87</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1219</v>
+        <v>1219.59</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1190.56</v>
+        <v>1191.13</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1186.19</v>
+        <v>1186.74</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1178.42</v>
+        <v>1178.93</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1176.06</v>
+        <v>1176.59</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1194.85</v>
+        <v>1195.4</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1158.48</v>
+        <v>1159.01</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1135.11</v>
+        <v>1135.68</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1141.57</v>
+        <v>1142.07</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1146.68</v>
+        <v>1147.12</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1131.66</v>
+        <v>1132.07</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1137.45</v>
+        <v>1137.87</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1124.52</v>
+        <v>1124.98</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1126.23</v>
+        <v>1126.66</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1075.05</v>
+        <v>1075.46</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1063.27</v>
+        <v>1063.66</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1081.02</v>
+        <v>1081.45</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1077.56</v>
+        <v>1077.92</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1098.46</v>
+        <v>1098.74</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1073.99</v>
+        <v>1074.24</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1100.56</v>
+        <v>1100.83</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1102.5</v>
+        <v>1102.78</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1099.53</v>
+        <v>1099.73</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1084.93</v>
+        <v>1085.16</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1048.31</v>
+        <v>1048.55</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1038.65</v>
+        <v>1038.89</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1053.24</v>
+        <v>1053.54</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.34</v>
+        <v>1086.67</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1081.17</v>
+        <v>1081.55</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1081.19</v>
+        <v>1081.59</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1038.2</v>
+        <v>1038.71</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1052.66</v>
+        <v>1053.2</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1056.56</v>
+        <v>1057.15</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1085.23</v>
+        <v>1085.77</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1072.45</v>
+        <v>1073.05</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1067.28</v>
+        <v>1068</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1063.33</v>
+        <v>1064.05</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1078.77</v>
+        <v>1079.55</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1076.55</v>
+        <v>1077.3</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1045.24</v>
+        <v>1046.02</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1046.71</v>
+        <v>1047.49</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1045.71</v>
+        <v>1046.49</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1060.13</v>
+        <v>1060.88</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1046.12</v>
+        <v>1046.87</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1048.15</v>
+        <v>1048.82</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1040.67</v>
+        <v>1041.35</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1052.87</v>
+        <v>1053.53</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1044.99</v>
+        <v>1045.66</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1057.51</v>
+        <v>1058.21</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1029.53</v>
+        <v>1030.26</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1067.69</v>
+        <v>1051.97</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11152,7 +11152,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1067.69</v>
+        <v>1051.97</v>
       </c>
     </row>
     <row r="64">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-14.95%</t>
+          <t>-16.25%</t>
         </is>
       </c>
     </row>
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>142.4</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-23 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -732,10 +732,10 @@
         <v>-0.6509999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>19.173</v>
+        <v>19.156</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>30.054</v>
+        <v>30.856</v>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
@@ -746,10 +746,10 @@
         <v>10.127618</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>14.097</v>
+        <v>14.473</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="O3" s="8" t="n">
         <v>1.177</v>
@@ -796,7 +796,7 @@
         <v>11.927</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>12.562</v>
+        <v>12.574</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
@@ -807,10 +807,10 @@
         <v>12.310537</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>46.034</v>
+        <v>46.079</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.682</v>
@@ -975,7 +975,7 @@
         <v>6.186</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8.476000000000001</v>
+        <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.6320925</v>
@@ -984,7 +984,7 @@
         <v>10.057183</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>7.058</v>
+        <v>7.113</v>
       </c>
       <c r="N7" s="7" t="n">
         <v>5.9</v>
@@ -1093,7 +1093,7 @@
         <v>5.898</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>10.878</v>
+        <v>10.94</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>15.99622</v>
@@ -1102,10 +1102,10 @@
         <v>11.396572</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>11.371</v>
+        <v>11.435</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>0.66</v>
@@ -1396,7 +1396,7 @@
         <v>2.408</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>5.928</v>
+        <v>5.976</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
@@ -1407,10 +1407,10 @@
         <v>12.110919</v>
       </c>
       <c r="M14" s="7" t="n">
-        <v>6.721</v>
+        <v>6.776</v>
       </c>
       <c r="N14" s="7" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="O14" s="8" t="n">
         <v>1.082</v>
@@ -1696,7 +1696,7 @@
         <v>-0.154</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.919</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
@@ -3398,7 +3398,7 @@
         <v>109.38</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>19.173</v>
+        <v>19.156</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3409,19 +3409,19 @@
         <v>10.127618</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>14.097</v>
+        <v>14.473</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1.834</v>
+        <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.1205893</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1703084</v>
+        <v>1.1692576</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3464,13 +3464,13 @@
         <v>12.310537</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>46.034</v>
+        <v>46.079</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>2.075</v>
+        <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>18.777428</v>
@@ -3623,13 +3623,13 @@
         <v>10.057183</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>7.058</v>
+        <v>7.113</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>5.9</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>2.071</v>
+        <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>2.3989227</v>
@@ -3729,13 +3729,13 @@
         <v>11.396572</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>11.371</v>
+        <v>11.435</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.718</v>
+        <v>3.739</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>5.8330464</v>
@@ -4004,13 +4004,13 @@
         <v>12.110919</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>6.721</v>
+        <v>6.776</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>2.361</v>
+        <v>2.38</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.7866752</v>
@@ -4266,7 +4266,7 @@
         <v>11.26</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.919</v>
       </c>
       <c r="F19" s="7" t="n">
         <v>18.766666</v>
@@ -4287,7 +4287,7 @@
         <v>3.4360697</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.70394415</v>
+        <v>0.6901145</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4400,7 +4400,7 @@
         <v>0.23902032</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-12.58</v>
+        <v>-12.65</v>
       </c>
       <c r="N21" s="3" t="n">
         <v>-0.8100000000000001</v>
@@ -6283,7 +6283,7 @@
         <v>0.41693002</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>1.98</v>
+        <v>1.94</v>
       </c>
       <c r="P2" s="5" t="n">
         <v>0.4255</v>
@@ -6455,7 +6455,7 @@
         <v>0.68557</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -6569,7 +6569,7 @@
         <v>0.73223996</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.91</v>
+        <v>0.9</v>
       </c>
       <c r="P7" s="5" t="n">
         <v>0.0319</v>
@@ -6625,7 +6625,7 @@
         <v>0.88882005</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>1.81</v>
+        <v>1.79</v>
       </c>
       <c r="P8" s="5" t="n">
         <v>0.32369998</v>
@@ -6713,13 +6713,13 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.926596</v>
+        <v>28.92324</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.29507</v>
+        <v>37.290745</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.99768</v>
+        <v>21.995129</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>0.481</v>
@@ -6795,7 +6795,7 @@
         <v>0.19124001</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>1.63</v>
+        <v>1.59</v>
       </c>
       <c r="P11" s="5" t="n">
         <v>0.2831</v>
@@ -6967,7 +6967,7 @@
         <v>0.46126</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7.19</v>
+        <v>7.05</v>
       </c>
       <c r="P14" s="5" t="n">
         <v>8.8889</v>
@@ -7141,7 +7141,7 @@
         <v>0.64762</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="P17" s="5" t="n">
         <v>0.221</v>
@@ -7313,7 +7313,7 @@
         <v>0.68561995</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>3.81</v>
+        <v>3.8</v>
       </c>
       <c r="P20" s="5" t="n">
         <v>4.5455</v>
@@ -7957,7 +7957,7 @@
         <v>-0.047</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>7.058</v>
+        <v>7.113</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>5.9</v>
@@ -8001,10 +8001,10 @@
         <v>-0.244</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.371</v>
+        <v>11.435</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>9.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L11" s="7" t="n">
         <v>63.5</v>
@@ -8473,10 +8473,10 @@
         <v>-0.328</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>46.034</v>
+        <v>46.079</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>19.7</v>
+        <v>19.8</v>
       </c>
       <c r="L23" s="7" t="n">
         <v>52</v>
@@ -8499,7 +8499,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>19.173</v>
+        <v>19.156</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8519,10 +8519,10 @@
         <v>-0.499</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>14.097</v>
+        <v>14.473</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>9.6</v>
+        <v>9.9</v>
       </c>
       <c r="L24" s="7" t="n">
         <v>48</v>
@@ -8611,7 +8611,7 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.919</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>18.766666</v>
@@ -8675,10 +8675,10 @@
         <v>-0.132</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>6.721</v>
+        <v>6.776</v>
       </c>
       <c r="K29" s="7" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
       <c r="L29" s="7" t="n">
         <v>63.3</v>
@@ -10196,7 +10196,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1267.92</v>
+        <v>1267.98</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1213.06</v>
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1273.82</v>
+        <v>1273.89</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1212.93</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1263.51</v>
+        <v>1263.57</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1258.49</v>
+        <v>1258.56</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1251.13</v>
+        <v>1251.2</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1256.04</v>
+        <v>1256.1</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1256.72</v>
+        <v>1256.79</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1241.94</v>
+        <v>1242</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1194.87</v>
+        <v>1194.92</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1219.59</v>
+        <v>1219.64</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1191.13</v>
+        <v>1191.17</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1186.74</v>
+        <v>1186.79</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1178.93</v>
+        <v>1178.98</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1176.59</v>
+        <v>1176.64</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1195.4</v>
+        <v>1195.46</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1159.01</v>
+        <v>1159.07</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1135.68</v>
+        <v>1135.73</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1142.07</v>
+        <v>1142.13</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1147.12</v>
+        <v>1147.18</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1132.07</v>
+        <v>1132.12</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1137.87</v>
+        <v>1137.93</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1124.98</v>
+        <v>1125.04</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1126.66</v>
+        <v>1126.72</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1075.46</v>
+        <v>1075.5</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1063.66</v>
+        <v>1063.7</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1081.45</v>
+        <v>1081.5</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1077.92</v>
+        <v>1077.98</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1098.74</v>
+        <v>1098.8</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1074.24</v>
+        <v>1074.29</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1100.83</v>
+        <v>1100.89</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1102.78</v>
+        <v>1102.84</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1099.73</v>
+        <v>1099.79</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1085.16</v>
+        <v>1085.22</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1048.55</v>
+        <v>1048.61</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1038.89</v>
+        <v>1038.95</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1053.54</v>
+        <v>1053.61</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.67</v>
+        <v>1086.74</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1081.55</v>
+        <v>1081.62</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1081.59</v>
+        <v>1081.66</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1038.71</v>
+        <v>1038.78</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1053.2</v>
+        <v>1053.26</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1057.15</v>
+        <v>1057.22</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1085.77</v>
+        <v>1085.84</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1073.05</v>
+        <v>1073.12</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1068</v>
+        <v>1068.07</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1064.05</v>
+        <v>1064.12</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1079.55</v>
+        <v>1079.6</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1077.3</v>
+        <v>1077.36</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1046.02</v>
+        <v>1046.08</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1047.49</v>
+        <v>1047.55</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1046.49</v>
+        <v>1046.55</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1060.88</v>
+        <v>1060.94</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1046.87</v>
+        <v>1046.94</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1048.82</v>
+        <v>1048.89</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1041.35</v>
+        <v>1041.42</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1053.53</v>
+        <v>1053.6</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1045.66</v>
+        <v>1045.73</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1058.21</v>
+        <v>1058.29</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1030.26</v>
+        <v>1030.33</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1051.97</v>
+        <v>1052.04</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11152,7 +11152,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1051.97</v>
+        <v>1052.04</v>
       </c>
     </row>
     <row r="64">
@@ -11184,7 +11184,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>140</v>
+        <v>139.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 13:03
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.69</v>
+        <v>107.66</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.015464293</v>
+        <v>-0.015724937</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.657</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.86</v>
+        <v>18.855</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.97113</v>
+        <v>9.968362000000001</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.25</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.030917058</v>
+        <v>-0.02882802</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>21.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.524</v>
+        <v>-0.523</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.546</v>
+        <v>11.571</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>11.917484</v>
+        <v>11.943174</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.428</v>
+        <v>-0.426</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.35</v>
+        <v>-0.348</v>
       </c>
     </row>
     <row r="5">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.95</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>36.96</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>0.027059056</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -913,16 +913,16 @@
         <v>-0.08</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.106</v>
+        <v>10.109</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.618423</v>
+        <v>48.631577</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.769639</v>
+        <v>15.773907</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.81</v>
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.59</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.020136611</v>
+        <v>0.01989257</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.07099999999999999</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.31</v>
+        <v>6.309</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7052305</v>
+        <v>3.704344</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.259701</v>
+        <v>10.257247</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.16</v>
+        <v>86.2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.018199017</v>
+        <v>0.018730785</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1028,19 +1028,19 @@
         <v>80.23999999999999</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.273</v>
+        <v>-0.272</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.005</v>
+        <v>6.008</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>10.94</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.287336</v>
+        <v>16.295841</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.603979</v>
+        <v>11.610039</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.435</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.33</v>
+        <v>58.31</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.43044075</v>
+        <v>0.4046087999999999</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1090,16 +1090,16 @@
         <v>-0.155</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.998</v>
+        <v>5.996</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.847</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>18.695515</v>
+        <v>18.690706</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.751444</v>
+        <v>17.746878</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.413</v>
@@ -1111,7 +1111,7 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.365</v>
+        <v>0.364</v>
       </c>
       <c r="Q9" s="9" t="n">
         <v>-0.055</v>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.18</v>
+        <v>19.16</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.017939538</v>
+        <v>-0.018674841</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1149,16 +1149,16 @@
         <v>-0.405</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.676</v>
+        <v>5.672</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.277775</v>
+        <v>53.23611</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.384747</v>
+        <v>23.366459</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.78</v>
+        <v>10.79</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.9363242000000001</v>
+        <v>0.010299593</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1208,16 +1208,16 @@
         <v>-0.25</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.451</v>
+        <v>5.456</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.666666</v>
+        <v>25.690477</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.427802</v>
+        <v>12.439331</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1229,10 +1229,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.5489999999999999</v>
+        <v>0.551</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06900000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.73</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>-0.09195613</v>
+        <v>21.77</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>0.09195613</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.04099999999999999</v>
+        <v>-0.039</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.058</v>
+        <v>5.068</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>70.09677000000001</v>
+        <v>70.22581</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.03799</v>
+        <v>29.091444</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.9159999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.125</v>
+        <v>0.127</v>
       </c>
     </row>
     <row r="14">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.95</v>
-      </c>
-      <c r="E17" s="9" t="n">
-        <v>-0.3104013</v>
+        <v>98.3</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>0.040709257</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.14</v>
+        <v>-0.137</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.752</v>
+        <v>1.758</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.674</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>18.039597</v>
+        <v>18.103132</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.476871</v>
+        <v>16.534903</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.779</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.023</v>
+        <v>0.027</v>
       </c>
     </row>
     <row r="18">
@@ -1621,7 +1621,7 @@
         <v>4.47</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>-0.048936176</v>
+        <v>-0.04787232399999999</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1633,7 +1633,7 @@
         <v>-0.674</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.15</v>
+        <v>1.151</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.908</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.515151</v>
+        <v>4.5202017</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.528</v>
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.67</v>
+        <v>26.66</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.011760222</v>
+        <v>0.011380851</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,7 +1752,7 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.186</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0.704</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>22.04132</v>
+        <v>22.033056</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.449</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>-0.012</v>
+        <v>-0.013</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>-0.014</v>
+        <v>-0.015</v>
       </c>
     </row>
     <row r="21">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.48</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.69230884</v>
+        <v>-0.30769202</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1882,7 +1882,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.351</v>
+        <v>-0.349</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.175</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.616317</v>
+        <v>8.649687999999999</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.818</v>
@@ -1908,10 +1908,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>-0.295</v>
+        <v>-0.292</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>-0.28</v>
+        <v>-0.278</v>
       </c>
     </row>
     <row r="23">
@@ -2205,10 +2205,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.69</v>
+        <v>107.66</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.015464293</v>
+        <v>-0.015724937</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.507</v>
@@ -2252,28 +2252,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.25</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.030917058</v>
+        <v>-0.02882802</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.35</v>
+        <v>-0.348</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.428</v>
+        <v>-0.426</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>-36.1</v>
+        <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.146</v>
+        <v>-0.144</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.35</v>
+        <v>-0.349</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.524</v>
+        <v>-0.523</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2346,10 +2346,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.95</v>
+        <v>36.96</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0</v>
+        <v>0.027059056</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.013</v>
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.59</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.020136611</v>
+        <v>0.01989257</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.028</v>
@@ -2411,7 +2411,7 @@
         <v>-0.004</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.01</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="K7" s="5" t="n">
         <v>-0.07099999999999999</v>
@@ -2440,10 +2440,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.16</v>
+        <v>86.2</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.018199017</v>
+        <v>0.018730785</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.23</v>
@@ -2458,10 +2458,10 @@
         <v>-0.091</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.147</v>
+        <v>-0.146</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.273</v>
+        <v>-0.272</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>0.66</v>
@@ -2487,16 +2487,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.33</v>
+        <v>58.31</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.43044075</v>
+        <v>0.4046087999999999</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.055</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.365</v>
+        <v>0.364</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>39.1</v>
@@ -2505,7 +2505,7 @@
         <v>-0.05400000000000001</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>-0.155</v>
@@ -2534,10 +2534,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.18</v>
+        <v>19.16</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.017939538</v>
+        <v>-0.018674841</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>-0.178</v>
@@ -2549,7 +2549,7 @@
         <v>-28.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>-0.218</v>
@@ -2581,25 +2581,25 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.78</v>
+        <v>10.79</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.9363242000000001</v>
+        <v>0.010299593</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.5489999999999999</v>
+        <v>0.551</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.07200000000000001</v>
+        <v>0.073</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.04</v>
+        <v>-0.039</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>-0.25</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.73</v>
+        <v>21.77</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.09195613</v>
+        <v>0.09195613</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.125</v>
+        <v>0.127</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.9159999999999999</v>
+        <v>0.92</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.155</v>
+        <v>0.157</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.188</v>
+        <v>0.191</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.04099999999999999</v>
+        <v>-0.039</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2863,28 +2863,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.95</v>
+        <v>98.3</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.3104013</v>
+        <v>0.040709257</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.023</v>
+        <v>0.027</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.223</v>
+        <v>0.227</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.032</v>
+        <v>0.036</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.019</v>
+        <v>0.023</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.14</v>
+        <v>-0.137</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2913,7 +2913,7 @@
         <v>4.47</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.048936176</v>
+        <v>-0.04787232399999999</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>-0.585</v>
@@ -3004,16 +3004,16 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.67</v>
+        <v>26.66</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.011760222</v>
+        <v>0.011380851</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.014</v>
+        <v>-0.015</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.013</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
@@ -3025,7 +3025,7 @@
         <v>-0.008</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.186</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3100,28 +3100,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.48</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.69230884</v>
+        <v>-0.30769202</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.28</v>
+        <v>-0.278</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.295</v>
+        <v>-0.292</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.229</v>
+        <v>-0.226</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.246</v>
+        <v>-0.243</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.351</v>
+        <v>-0.349</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.69</v>
+        <v>107.66</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.86</v>
+        <v>18.855</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.97113</v>
+        <v>9.968362000000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0878227</v>
+        <v>2.087243</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1511908</v>
+        <v>1.1508712</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.25</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.546</v>
+        <v>11.571</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>11.917484</v>
+        <v>11.943174</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.177898</v>
+        <v>18.217085</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.906976</v>
+        <v>1.9110868</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3564,16 +3564,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.95</v>
+        <v>36.96</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.106</v>
+        <v>10.109</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.618423</v>
+        <v>48.631577</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.769639</v>
+        <v>15.773907</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.81</v>
@@ -3585,10 +3585,10 @@
         <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9279263</v>
+        <v>3.9289892</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.57624847</v>
+        <v>0.5764044</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.59</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.31</v>
+        <v>6.309</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7052305</v>
+        <v>3.704344</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.259701</v>
+        <v>10.257247</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4472287</v>
+        <v>2.4466434</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5421335</v>
+        <v>1.5417646</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3670,16 +3670,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.16</v>
+        <v>86.2</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.005</v>
+        <v>6.008</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.287336</v>
+        <v>16.295841</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.603979</v>
+        <v>11.610039</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.435</v>
@@ -3691,10 +3691,10 @@
         <v>3.739</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>5.939202</v>
+        <v>5.9423037</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0523736</v>
+        <v>2.0534453</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.33</v>
+        <v>58.31</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.998</v>
+        <v>5.996</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>18.695515</v>
+        <v>18.690706</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.751444</v>
+        <v>17.746878</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.413</v>
@@ -3744,10 +3744,10 @@
         <v>3.404</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.329788</v>
+        <v>16.325588</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.9818263</v>
+        <v>2.9810596</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3776,16 +3776,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.18</v>
+        <v>19.16</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.676</v>
+        <v>5.672</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.277775</v>
+        <v>53.23611</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.384747</v>
+        <v>23.366459</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.0928216</v>
+        <v>5.088839</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.4003925</v>
+        <v>4.396951</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.78</v>
+        <v>10.79</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.451</v>
+        <v>5.456</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.666666</v>
+        <v>25.690477</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.427802</v>
+        <v>12.439331</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.3183975</v>
+        <v>7.3251863</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.326495</v>
+        <v>2.328653</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.73</v>
+        <v>21.77</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.058</v>
+        <v>5.068</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>70.09677000000001</v>
+        <v>70.22581</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.03799</v>
+        <v>29.091444</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.752206</v>
+        <v>14.779362</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4589944</v>
+        <v>4.4672027</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -4159,16 +4159,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.95</v>
+        <v>98.3</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.752</v>
+        <v>1.758</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>18.039597</v>
+        <v>18.103132</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.476871</v>
+        <v>16.534903</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.779</v>
@@ -4180,10 +4180,10 @@
         <v>3.071</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.246338</v>
+        <v>3.2577717</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.214006</v>
+        <v>3.2253258</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4215,7 +4215,7 @@
         <v>4.47</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.15</v>
+        <v>1.151</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.515151</v>
+        <v>4.5202017</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.528</v>
@@ -4237,10 +4237,10 @@
         <v>1.356</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.5198911</v>
+        <v>1.5215913</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.7175908</v>
+        <v>1.7195121</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4322,7 +4322,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.67</v>
+        <v>26.66</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0.704</v>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>22.04132</v>
+        <v>22.033056</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.449</v>
@@ -4345,10 +4345,10 @@
         <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6592013</v>
+        <v>1.6585791</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1089056</v>
+        <v>1.1084898</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.48</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.175</v>
@@ -4449,7 +4449,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.616317</v>
+        <v>8.649687999999999</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.818</v>
@@ -4461,10 +4461,10 @@
         <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.704809</v>
+        <v>-10.746269</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.5743819</v>
+        <v>0.5766065</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.69</v>
+        <v>107.66</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.975</v>
+        <v>0.976</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.25</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.5589999999999999</v>
+        <v>0.556</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>36.95</v>
+        <v>36.96</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.155</v>
+        <v>0.154</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>83.59</v>
+        <v>83.56999999999999</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6599,7 +6599,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>86.16</v>
+        <v>86.2</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6622,7 +6622,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.573</v>
+        <v>0.5720000000000001</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.68</v>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>58.33</v>
+        <v>58.31</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.257</v>
+        <v>0.258</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>3.89</v>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>19.18</v>
+        <v>19.16</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6725,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.889751</v>
+        <v>28.883062</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.247566</v>
+        <v>37.238945</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.969662</v>
+        <v>21.964575</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.506</v>
+        <v>0.507</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.78</v>
+        <v>10.79</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.612</v>
+        <v>0.61</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.73</v>
+        <v>21.77</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6906,7 +6906,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.141</v>
+        <v>0.139</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>97.95</v>
+        <v>98.3</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7138,7 +7138,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.099</v>
+        <v>0.095</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.53</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.67</v>
+        <v>26.66</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.48</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.064</v>
+        <v>1.058</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.106</v>
+        <v>10.109</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48.618423</v>
+        <v>48.631577</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.31</v>
+        <v>6.309</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7052305</v>
+        <v>3.704344</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7995,10 +7995,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.005</v>
+        <v>6.008</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.287336</v>
+        <v>16.295841</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8039,10 +8039,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.752</v>
+        <v>1.758</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>18.039597</v>
+        <v>18.103132</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.041</v>
@@ -8054,7 +8054,7 @@
         <v>0.19214001</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.023</v>
+        <v>0.027</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>8.779</v>
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5.998</v>
+        <v>5.996</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.695515</v>
+        <v>18.690706</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8190,7 +8190,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.014</v>
+        <v>-0.015</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.449</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.451</v>
+        <v>5.456</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.666666</v>
+        <v>25.690477</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8377,10 +8377,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.676</v>
+        <v>5.672</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.277775</v>
+        <v>53.23611</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.058</v>
+        <v>5.068</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>70.09677000000001</v>
+        <v>70.22581</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.125</v>
+        <v>0.127</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.546</v>
+        <v>11.571</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.35</v>
+        <v>-0.348</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.86</v>
+        <v>18.855</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8561,7 +8561,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.15</v>
+        <v>1.151</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.28</v>
+        <v>-0.278</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.818</v>
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.61</v>
+        <v>1277.59</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1212.93</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.27</v>
+        <v>1267.25</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.13</v>
+        <v>1262.11</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1254.82</v>
+        <v>1254.8</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1259.66</v>
+        <v>1259.64</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.24</v>
+        <v>1260.23</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.52</v>
+        <v>1245.5</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.22</v>
+        <v>1198.21</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1222.89</v>
+        <v>1222.87</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.21</v>
+        <v>1194.2</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1190</v>
+        <v>1189.99</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.27</v>
+        <v>1182.25</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1179.97</v>
+        <v>1179.96</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1198.78</v>
+        <v>1198.77</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.54</v>
+        <v>1162.53</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.17</v>
+        <v>1139.16</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1145.74</v>
+        <v>1145.73</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1150.84</v>
+        <v>1150.82</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1135.92</v>
+        <v>1135.9</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1141.77</v>
+        <v>1141.75</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1128.9</v>
+        <v>1128.87</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1130.69</v>
+        <v>1130.67</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.1</v>
+        <v>1067.09</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.19</v>
+        <v>1085.17</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1081.87</v>
+        <v>1081.85</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1102.76</v>
+        <v>1102.74</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.44</v>
+        <v>1078.41</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105.07</v>
+        <v>1105.04</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1106.92</v>
+        <v>1106.89</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1103.9</v>
+        <v>1103.87</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.47</v>
+        <v>1089.45</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1052.8</v>
+        <v>1052.77</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1043.61</v>
+        <v>1043.57</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.28</v>
+        <v>1058.25</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.47</v>
+        <v>1091.44</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.37</v>
+        <v>1086.35</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1086.48</v>
+        <v>1086.45</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.41</v>
+        <v>1043.39</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1057.85</v>
+        <v>1057.83</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1061.73</v>
+        <v>1061.72</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.33</v>
+        <v>1090.32</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1077.73</v>
+        <v>1077.72</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1083.93</v>
+        <v>1083.94</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1081.57</v>
+        <v>1081.58</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.11</v>
+        <v>1050.13</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1051.66</v>
+        <v>1051.68</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1050.75</v>
+        <v>1050.76</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.14</v>
+        <v>1065.15</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1051.01</v>
+        <v>1051.02</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1052.95</v>
+        <v>1052.97</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1045.55</v>
+        <v>1045.56</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1057.81</v>
+        <v>1057.82</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1049.92</v>
+        <v>1049.93</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1062.51</v>
+        <v>1062.52</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1034.47</v>
+        <v>1034.48</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.25</v>
+        <v>1056.26</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1060.9</v>
+        <v>1061.07</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1060.9</v>
+        <v>1061.07</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.78%</t>
+          <t>-15.76%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 13:06
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.75</v>
+        <v>54.78</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.013888888</v>
+        <v>0.014537034</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.222</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>37.018</v>
+        <v>37.042</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.818</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.297873</v>
+        <v>23.312767</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>14.5707035</v>
+        <v>14.580018</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.77</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.347</v>
+        <v>0.348</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.156</v>
+        <v>-0.155</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.66</v>
+        <v>107.75</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.015724937</v>
+        <v>-0.014902151</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.657</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.855</v>
+        <v>18.87</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.968362000000001</v>
+        <v>9.976694999999999</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -758,7 +758,7 @@
         <v>-0.5629999999999999</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>-0.507</v>
+        <v>-0.506</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.25</v>
+        <v>23.3</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.02882802</v>
+        <v>-0.02673906</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>21.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.523</v>
+        <v>-0.522</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.571</v>
+        <v>11.596</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>11.943174</v>
+        <v>11.9688635</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.426</v>
+        <v>-0.425</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.348</v>
+        <v>-0.347</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.04</v>
+        <v>102.08</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.8998355000000001</v>
+        <v>0.9393895000000001</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,19 +851,19 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.243</v>
+        <v>-0.242</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.641</v>
+        <v>10.645</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.496815</v>
+        <v>32.509552</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.173334</v>
+        <v>17.180065</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.354</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.213</v>
+        <v>0.214</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>-0.166</v>
+        <v>-0.165</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.96</v>
+        <v>36.99</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.027059056</v>
+        <v>0.10825688</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.079</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.109</v>
+        <v>10.117</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.631577</v>
+        <v>48.671055</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.773907</v>
+        <v>15.786711</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.81</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.56999999999999</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.01989257</v>
+        <v>0.019526464</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.07099999999999999</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.309</v>
+        <v>6.307</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.704344</v>
+        <v>3.7030144</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.257247</v>
+        <v>10.253565</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -1019,7 +1019,7 @@
         <v>86.2</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.018730785</v>
+        <v>0.01867164</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1037,10 +1037,10 @@
         <v>10.94</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.295841</v>
+        <v>16.294895</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.610039</v>
+        <v>11.609365</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.435</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.31</v>
+        <v>58.34</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.4046087999999999</v>
+        <v>0.45650196</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,19 +1087,19 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.155</v>
+        <v>-0.154</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.996</v>
+        <v>5.999</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.847</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>18.690706</v>
+        <v>18.700321</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.746878</v>
+        <v>17.756008</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.413</v>
@@ -1111,7 +1111,7 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="4" t="n">
-        <v>0.364</v>
+        <v>0.365</v>
       </c>
       <c r="Q9" s="9" t="n">
         <v>-0.055</v>
@@ -1137,7 +1137,7 @@
         <v>19.16</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.018674841</v>
+        <v>-0.018945255</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1149,16 +1149,16 @@
         <v>-0.405</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.672</v>
+        <v>5.67</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.23611</v>
+        <v>53.22222</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.366459</v>
+        <v>23.360363</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1170,7 +1170,7 @@
         <v>2.002</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.166</v>
+        <v>-0.167</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>-0.178</v>
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.79</v>
+        <v>10.8</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.010299593</v>
+        <v>0.01170412</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1205,19 +1205,19 @@
         <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.25</v>
+        <v>-0.249</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.456</v>
+        <v>5.463</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.690477</v>
+        <v>25.726192</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.439331</v>
+        <v>12.456624</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1229,10 +1229,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.551</v>
+        <v>0.5529999999999999</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.067</v>
       </c>
     </row>
     <row r="12">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.77</v>
+        <v>21.78</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.09195613</v>
+        <v>0.1379342</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.039</v>
+        <v>-0.038</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.068</v>
+        <v>5.07</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>70.22581</v>
+        <v>70.258064</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.091444</v>
+        <v>29.104807</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.92</v>
+        <v>0.9209999999999999</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
     </row>
     <row r="14">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.53</v>
+        <v>5.54</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.010968999</v>
+        <v>0.01188301</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,19 +1451,19 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.455</v>
+        <v>-0.454</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.25</v>
+        <v>2.252</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.021739</v>
+        <v>12.032608</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9508166</v>
+        <v>6.957101</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.582</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.006</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>-0.264</v>
+        <v>-0.263</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.4</v>
+        <v>14.41</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>-0.27700806</v>
+        <v>-0.17312756</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1513,7 +1513,7 @@
         <v>-0.301</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.923</v>
+        <v>1.925</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.411</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.273342</v>
+        <v>8.28196</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.184</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>-0.17</v>
+        <v>-0.169</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.03</v>
+        <v>-0.029</v>
       </c>
     </row>
     <row r="17">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.24</v>
-      </c>
-      <c r="E19" s="9" t="n">
-        <v>-0.17762396</v>
+        <v>11.26</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,19 +1693,19 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.154</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.917</v>
+        <v>0.919</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.733332</v>
+        <v>18.766666</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>12.1378355</v>
+        <v>12.159433</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>-0.011</v>
+        <v>-0.01</v>
       </c>
     </row>
     <row r="20">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.30769202</v>
+        <v>-0.46154168</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1882,7 +1882,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.349</v>
+        <v>-0.35</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.175</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.649687999999999</v>
+        <v>8.636339</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.818</v>
@@ -1908,10 +1908,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>-0.292</v>
+        <v>-0.293</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>-0.278</v>
+        <v>-0.279</v>
       </c>
     </row>
     <row r="23">
@@ -2158,16 +2158,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.75</v>
+        <v>54.78</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.013888888</v>
+        <v>0.014537034</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.155</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.347</v>
+        <v>0.348</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>53.2</v>
@@ -2179,7 +2179,7 @@
         <v>-0.017</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.222</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2205,13 +2205,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.66</v>
+        <v>107.75</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.015724937</v>
+        <v>-0.014902151</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.507</v>
+        <v>-0.506</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>-0.5629999999999999</v>
@@ -2220,10 +2220,10 @@
         <v>-56.8</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.252</v>
+        <v>-0.251</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.532</v>
+        <v>-0.531</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>-0.657</v>
@@ -2252,28 +2252,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.25</v>
+        <v>23.3</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.02882802</v>
+        <v>-0.02673906</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.348</v>
+        <v>-0.347</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.426</v>
+        <v>-0.425</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.144</v>
+        <v>-0.142</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.349</v>
+        <v>-0.348</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.523</v>
+        <v>-0.522</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2299,28 +2299,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.04</v>
+        <v>102.08</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.8998355000000001</v>
+        <v>0.9393895000000001</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.165</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.213</v>
+        <v>0.214</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>34.7</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.07200000000000001</v>
+        <v>-0.07099999999999999</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>-0.107</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.243</v>
+        <v>-0.242</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2346,28 +2346,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.96</v>
+        <v>36.99</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.027059056</v>
+        <v>0.10825688</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>11.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.043</v>
+        <v>0.044</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.051</v>
+        <v>0.052</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.079</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.56999999999999</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.01989257</v>
+        <v>0.019526464</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.028</v>
@@ -2443,7 +2443,7 @@
         <v>86.2</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.018730785</v>
+        <v>0.01867164</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.23</v>
@@ -2487,28 +2487,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.31</v>
+        <v>58.34</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.4046087999999999</v>
+        <v>0.45650196</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.055</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.364</v>
+        <v>0.365</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>39.1</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.05400000000000001</v>
+        <v>-0.053</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.006</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.155</v>
+        <v>-0.154</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2537,13 +2537,13 @@
         <v>19.16</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.018674841</v>
+        <v>-0.018945255</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>-0.178</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.167</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-28.1</v>
@@ -2581,28 +2581,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.79</v>
+        <v>10.8</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.010299593</v>
+        <v>0.01170412</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.067</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.551</v>
+        <v>0.5529999999999999</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.073</v>
+        <v>0.07400000000000001</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.039</v>
+        <v>-0.038</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.25</v>
+        <v>-0.249</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.1</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.77</v>
+        <v>21.78</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.09195613</v>
+        <v>0.1379342</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.92</v>
+        <v>0.9209999999999999</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.157</v>
+        <v>0.158</v>
       </c>
       <c r="J13" s="5" t="n">
         <v>0.191</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.039</v>
+        <v>-0.038</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2769,28 +2769,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.53</v>
+        <v>5.54</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.010968999</v>
+        <v>0.01188301</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.263</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.006</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>8.6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.081</v>
+        <v>-0.08</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.294</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.455</v>
+        <v>-0.454</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2816,25 +2816,25 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.4</v>
+        <v>14.41</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.27700806</v>
+        <v>-0.17312756</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.03</v>
+        <v>-0.029</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.169</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.3</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.114</v>
+        <v>-0.113</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>-0.301</v>
@@ -2957,28 +2957,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.24</v>
+        <v>11.26</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.17762396</v>
+        <v>0</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.01</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.105</v>
+        <v>0.107</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.2</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.005</v>
+        <v>-0.003</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.154</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -3100,28 +3100,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.30769202</v>
+        <v>-0.46154168</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.278</v>
+        <v>-0.279</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.292</v>
+        <v>-0.293</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.226</v>
+        <v>-0.228</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.243</v>
+        <v>-0.244</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.349</v>
+        <v>-0.35</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3348,16 +3348,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.75</v>
+        <v>54.78</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>37.018</v>
+        <v>37.042</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.297873</v>
+        <v>23.312767</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>14.5707035</v>
+        <v>14.580018</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.77</v>
@@ -3369,10 +3369,10 @@
         <v>3.75</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.23854</v>
+        <v>23.253397</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.8438475</v>
+        <v>2.8456655</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.66</v>
+        <v>107.75</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.855</v>
+        <v>18.87</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.968362000000001</v>
+        <v>9.976694999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.087243</v>
+        <v>2.0889878</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1508712</v>
+        <v>1.1518332</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.25</v>
+        <v>23.3</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.571</v>
+        <v>11.596</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>11.943174</v>
+        <v>11.9688635</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.217085</v>
+        <v>18.25627</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.9110868</v>
+        <v>1.9151975</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,16 +3511,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.04</v>
+        <v>102.08</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.641</v>
+        <v>10.645</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.496815</v>
+        <v>32.509552</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.173334</v>
+        <v>17.180065</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.354</v>
@@ -3532,10 +3532,10 @@
         <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-37.96131</v>
+        <v>-37.976192</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4907789</v>
+        <v>1.4913633</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3564,16 +3564,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.96</v>
+        <v>36.99</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.109</v>
+        <v>10.117</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.631577</v>
+        <v>48.671055</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.773907</v>
+        <v>15.786711</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.81</v>
@@ -3585,10 +3585,10 @@
         <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9289892</v>
+        <v>3.9321785</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5764044</v>
+        <v>0.5768723</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.56999999999999</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.309</v>
+        <v>6.307</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.704344</v>
+        <v>3.7030144</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.257247</v>
+        <v>10.253565</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4466434</v>
+        <v>2.445765</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5417646</v>
+        <v>1.5412111</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3676,10 +3676,10 @@
         <v>6.008</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.295841</v>
+        <v>16.294895</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.610039</v>
+        <v>11.609365</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.435</v>
@@ -3691,10 +3691,10 @@
         <v>3.739</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>5.9423037</v>
+        <v>5.941959</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0534453</v>
+        <v>2.0533264</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.31</v>
+        <v>58.34</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.996</v>
+        <v>5.999</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>18.690706</v>
+        <v>18.700321</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.746878</v>
+        <v>17.756008</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.413</v>
@@ -3744,10 +3744,10 @@
         <v>3.404</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.325588</v>
+        <v>16.333986</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.9810596</v>
+        <v>2.982593</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3779,13 +3779,13 @@
         <v>19.16</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.672</v>
+        <v>5.67</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.23611</v>
+        <v>53.22222</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.366459</v>
+        <v>23.360363</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.088839</v>
+        <v>5.087511</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.396951</v>
+        <v>4.395804</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.79</v>
+        <v>10.8</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.456</v>
+        <v>5.463</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.690477</v>
+        <v>25.726192</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.439331</v>
+        <v>12.456624</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.3251863</v>
+        <v>7.33537</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.328653</v>
+        <v>2.3318906</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.77</v>
+        <v>21.78</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.068</v>
+        <v>5.07</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>70.22581</v>
+        <v>70.258064</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.091444</v>
+        <v>29.104807</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.779362</v>
+        <v>14.786151</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4672027</v>
+        <v>4.4692545</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -4051,16 +4051,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.53</v>
+        <v>5.54</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.25</v>
+        <v>2.252</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.021739</v>
+        <v>12.032608</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9508166</v>
+        <v>6.957101</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.582</v>
@@ -4072,10 +4072,10 @@
         <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7329991</v>
+        <v>-1.734566</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43568265</v>
+        <v>0.43607658</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.4</v>
+        <v>14.41</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.923</v>
+        <v>1.925</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.273342</v>
+        <v>8.28196</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.184</v>
@@ -4127,10 +4127,10 @@
         <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.9912576</v>
+        <v>0.9922902</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27626294</v>
+        <v>0.2765507</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4269,16 +4269,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.24</v>
+        <v>11.26</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.917</v>
+        <v>0.919</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.733332</v>
+        <v>18.766666</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>12.1378355</v>
+        <v>12.159433</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4290,10 +4290,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.4299664</v>
+        <v>3.4360697</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.68888867</v>
+        <v>0.6901145</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.175</v>
@@ -4449,7 +4449,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.649687999999999</v>
+        <v>8.636339</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.818</v>
@@ -4461,10 +4461,10 @@
         <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.746269</v>
+        <v>-10.729685</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.5766065</v>
+        <v>0.5757166</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -6257,7 +6257,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>54.75</v>
+        <v>54.78</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.66</v>
+        <v>107.75</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.976</v>
+        <v>0.9740000000000001</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.25</v>
+        <v>23.3</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.556</v>
+        <v>0.5529999999999999</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>102.04</v>
+        <v>102.08</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6452,7 +6452,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.39</v>
+        <v>0.389</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.24</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>36.96</v>
+        <v>36.99</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.154</v>
+        <v>0.153</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>83.56999999999999</v>
+        <v>83.54000000000001</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6566,7 +6566,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.13</v>
+        <v>0.131</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.32</v>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>58.31</v>
+        <v>58.34</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.258</v>
+        <v>0.257</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>3.89</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.79</v>
+        <v>10.8</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.61</v>
+        <v>0.609</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.77</v>
+        <v>21.78</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.53</v>
+        <v>5.54</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7020,7 +7020,7 @@
         <v>6.3</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.677</v>
+        <v>0.674</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.08</v>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.4</v>
+        <v>14.41</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.327</v>
+        <v>0.326</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.24</v>
+        <v>11.26</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7252,7 +7252,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.379</v>
+        <v>0.377</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.68</v>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.058</v>
+        <v>1.061</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7707,10 +7707,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>37.018</v>
+        <v>37.042</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.297873</v>
+        <v>23.312767</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7722,7 +7722,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.156</v>
+        <v>-0.155</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.77</v>
@@ -7797,10 +7797,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.25</v>
+        <v>2.252</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.021739</v>
+        <v>12.032608</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.263</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>10.582</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.109</v>
+        <v>10.117</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48.631577</v>
+        <v>48.671055</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7858,7 +7858,7 @@
         <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>16.81</v>
@@ -7887,10 +7887,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.641</v>
+        <v>10.645</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>32.496815</v>
+        <v>32.509552</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7904,7 +7904,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.165</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>11.354</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.309</v>
+        <v>6.307</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.704344</v>
+        <v>3.7030144</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7998,7 +7998,7 @@
         <v>6.008</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.295841</v>
+        <v>16.294895</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5.996</v>
+        <v>5.999</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.690706</v>
+        <v>18.700321</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.923</v>
+        <v>1.925</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.03</v>
+        <v>-0.029</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.184</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.456</v>
+        <v>5.463</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.690477</v>
+        <v>25.726192</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.06900000000000001</v>
+        <v>-0.067</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8377,10 +8377,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.672</v>
+        <v>5.67</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.23611</v>
+        <v>53.22222</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.068</v>
+        <v>5.07</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>70.22581</v>
+        <v>70.258064</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.127</v>
+        <v>0.128</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.571</v>
+        <v>11.596</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.348</v>
+        <v>-0.347</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.855</v>
+        <v>18.87</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8532,7 +8532,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.507</v>
+        <v>-0.506</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>14.473</v>
@@ -8627,10 +8627,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.917</v>
+        <v>0.919</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.733332</v>
+        <v>18.766666</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8642,7 +8642,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.01</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.278</v>
+        <v>-0.279</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.818</v>
@@ -10212,10 +10212,10 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.59</v>
+        <v>1277.56</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>1212.93</v>
+        <v>1212.94</v>
       </c>
       <c r="D2" s="13" t="n">
         <v>1068.57</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.25</v>
+        <v>1267.23</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.11</v>
+        <v>1262.08</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1254.8</v>
+        <v>1254.78</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1259.64</v>
+        <v>1259.62</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.23</v>
+        <v>1260.2</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.5</v>
+        <v>1245.47</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.21</v>
+        <v>1198.18</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1222.87</v>
+        <v>1222.85</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.2</v>
+        <v>1194.17</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1189.99</v>
+        <v>1189.97</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.25</v>
+        <v>1182.22</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1179.96</v>
+        <v>1179.93</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1198.77</v>
+        <v>1198.74</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.53</v>
+        <v>1162.49</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.16</v>
+        <v>1139.13</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1145.73</v>
+        <v>1145.7</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1150.82</v>
+        <v>1150.79</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1135.9</v>
+        <v>1135.86</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1141.75</v>
+        <v>1141.72</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1128.87</v>
+        <v>1128.84</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1130.67</v>
+        <v>1130.63</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1078.7</v>
+        <v>1078.66</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.09</v>
+        <v>1067.04</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.17</v>
+        <v>1085.12</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1081.85</v>
+        <v>1081.8</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1102.74</v>
+        <v>1102.69</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.41</v>
+        <v>1078.36</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105.04</v>
+        <v>1105</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1106.89</v>
+        <v>1106.85</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1103.87</v>
+        <v>1103.83</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.45</v>
+        <v>1089.4</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1052.77</v>
+        <v>1052.73</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1043.57</v>
+        <v>1043.52</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.25</v>
+        <v>1058.2</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.44</v>
+        <v>1091.38</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.35</v>
+        <v>1086.28</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1086.45</v>
+        <v>1086.39</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.39</v>
+        <v>1043.33</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1057.83</v>
+        <v>1057.78</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1061.72</v>
+        <v>1061.67</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.32</v>
+        <v>1090.26</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1077.72</v>
+        <v>1077.67</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1072.59</v>
+        <v>1072.54</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1068.53</v>
+        <v>1068.49</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1083.94</v>
+        <v>1083.89</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1081.58</v>
+        <v>1081.53</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.13</v>
+        <v>1050.08</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1051.68</v>
+        <v>1051.63</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1050.76</v>
+        <v>1050.72</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.15</v>
+        <v>1065.11</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1051.02</v>
+        <v>1050.98</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1052.97</v>
+        <v>1052.92</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1045.56</v>
+        <v>1045.51</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1057.82</v>
+        <v>1057.77</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1049.93</v>
+        <v>1049.88</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1062.52</v>
+        <v>1062.47</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1034.48</v>
+        <v>1034.43</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.26</v>
+        <v>1056.21</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1061.07</v>
+        <v>1061.72</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1061.07</v>
+        <v>1061.72</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.76%</t>
+          <t>-15.71%</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>140</v>
+        <v>140.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 14:09
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.78</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.014537034</v>
+        <v>0.017222228</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.222</v>
+        <v>-0.22</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>37.042</v>
+        <v>37.14</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.818</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.312767</v>
+        <v>23.37447</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>14.580018</v>
+        <v>14.618607</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.77</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.348</v>
+        <v>0.351</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.155</v>
+        <v>-0.153</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.75</v>
+        <v>107.92</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.014902151</v>
+        <v>-0.013347954</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.657</v>
+        <v>-0.6559999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.87</v>
+        <v>18.9</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.976694999999999</v>
+        <v>9.992435</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -755,7 +755,7 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="Q3" s="9" t="n">
         <v>-0.506</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.3</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.02673906</v>
+        <v>-0.021307719</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>21.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.522</v>
+        <v>-0.52</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.596</v>
+        <v>11.66</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>11.9688635</v>
+        <v>12.035657</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.425</v>
+        <v>-0.422</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.347</v>
+        <v>-0.343</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.08</v>
+        <v>102.95</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.9393895000000001</v>
+        <v>0.017996635</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,19 +851,19 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.242</v>
+        <v>-0.236</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.645</v>
+        <v>10.736</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.509552</v>
+        <v>32.78662</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.180065</v>
+        <v>17.326487</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.354</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.214</v>
+        <v>0.224</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>-0.165</v>
+        <v>-0.158</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.99</v>
+        <v>37.23</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.10825688</v>
+        <v>0.75777745</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.079</v>
+        <v>-0.073</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.117</v>
+        <v>10.183</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.671055</v>
+        <v>48.986843</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.786711</v>
+        <v>15.889138</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.81</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.141</v>
+        <v>0.148</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.014</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.54000000000001</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.019526464</v>
+        <v>0.024286036</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,19 +969,19 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.067</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.307</v>
+        <v>6.336</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7030144</v>
+        <v>3.7203016</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.253565</v>
+        <v>10.301433</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -993,21 +993,21 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.219</v>
+        <v>0.224</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1016,57 +1016,57 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.2</v>
+        <v>58.56</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.01867164</v>
+        <v>0.82644546</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>118.46</v>
+        <v>68.98999999999999</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>80.23999999999999</v>
+        <v>35.09</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.272</v>
+        <v>-0.151</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.008</v>
+        <v>6.022</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.94</v>
+        <v>6.847</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.294895</v>
+        <v>18.769232</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.609365</v>
+        <v>17.82144</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>11.435</v>
+        <v>8.413</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>7.3</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="P8" s="9" t="n">
-        <v>-0.239</v>
+        <v>1.453</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0.37</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.23</v>
+        <v>-0.051</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1075,46 +1075,46 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.34</v>
+        <v>85.86</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.45650196</v>
+        <v>0.014712776</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>68.98999999999999</v>
+        <v>118.46</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>35.09</v>
+        <v>80.23999999999999</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.275</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.999</v>
+        <v>5.984</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6.847</v>
+        <v>10.94</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>18.700321</v>
+        <v>16.23157</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.756008</v>
+        <v>11.564247</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>8.413</v>
+        <v>11.435</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>7.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>1.453</v>
-      </c>
-      <c r="P9" s="4" t="n">
-        <v>0.365</v>
+        <v>0.66</v>
+      </c>
+      <c r="P9" s="9" t="n">
+        <v>-0.242</v>
       </c>
       <c r="Q9" s="9" t="n">
-        <v>-0.055</v>
+        <v>-0.233</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.16</v>
+        <v>19.33</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.018945255</v>
+        <v>-0.010240694</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1146,19 +1146,19 @@
         <v>15.725</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.4</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.67</v>
+        <v>5.721</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.22222</v>
+        <v>53.694443</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.360363</v>
+        <v>23.56763</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1170,10 +1170,10 @@
         <v>2.002</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.167</v>
+        <v>-0.159</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.178</v>
+        <v>-0.171</v>
       </c>
     </row>
     <row r="11">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.01170412</v>
+        <v>0.020599186</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1205,19 +1205,19 @@
         <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.249</v>
+        <v>-0.242</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.463</v>
+        <v>5.511</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.726192</v>
+        <v>25.952381</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.456624</v>
+        <v>12.566145</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1229,10 +1229,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.5529999999999999</v>
+        <v>0.5660000000000001</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.067</v>
+        <v>-0.059</v>
       </c>
     </row>
     <row r="12">
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.36</v>
+        <v>26.41</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.30257156</v>
+        <v>-0.09455226</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>31.58</v>
@@ -1264,10 +1264,10 @@
         <v>17.86</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.165</v>
+        <v>-0.164</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.38</v>
+        <v>5.392</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>30.298</v>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>28.497297</v>
+        <v>28.556757</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>8.669</v>
@@ -1290,10 +1290,10 @@
         <v>1.977</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>-0.063</v>
+        <v>-0.061</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>0.119</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.78</v>
+        <v>22.04</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.1379342</v>
+        <v>0.013333375</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.038</v>
+        <v>-0.027</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.07</v>
+        <v>5.131</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>70.258064</v>
+        <v>71.09678</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.104807</v>
+        <v>29.452248</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.9209999999999999</v>
+        <v>0.9440000000000001</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.128</v>
+        <v>0.141</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.96</v>
+        <v>13</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>-0.6896563</v>
+        <v>-0.3831432200000001</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.302</v>
+        <v>-0.3</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.391</v>
+        <v>2.399</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.976</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>12.027395</v>
+        <v>12.064517</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.776</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="9" t="n">
-        <v>-0.036</v>
+        <v>-0.033</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>-0.138</v>
+        <v>-0.135</v>
       </c>
     </row>
     <row r="15">
@@ -1442,7 +1442,7 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.01188301</v>
+        <v>0.013711205</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1454,16 +1454,16 @@
         <v>-0.454</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.252</v>
+        <v>2.256</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.032608</v>
+        <v>12.054348</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.957101</v>
+        <v>6.969671</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.582</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.006</v>
+        <v>-0.004</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>-0.263</v>
+        <v>-0.262</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.41</v>
-      </c>
-      <c r="E16" s="9" t="n">
-        <v>-0.17312756</v>
+        <v>14.54</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.6578966000000002</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,10 +1510,10 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.301</v>
+        <v>-0.295</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.925</v>
+        <v>1.941</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.411</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.28196</v>
+        <v>8.350904</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.184</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>-0.169</v>
+        <v>-0.162</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.029</v>
+        <v>-0.021</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.3</v>
+        <v>98.72</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.040709257</v>
+        <v>0.4681448</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.137</v>
+        <v>-0.133</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.758</v>
+        <v>1.766</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.674</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>18.103132</v>
+        <v>18.18048</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.534903</v>
+        <v>16.60555</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.779</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.227</v>
+        <v>0.232</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.027</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="18">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.47</v>
+        <v>4.51</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>-0.04787232399999999</v>
+        <v>-0.039361691</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1630,10 +1630,10 @@
         <v>4.46</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>-0.674</v>
+        <v>-0.672</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.151</v>
+        <v>1.161</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.908</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.5202017</v>
+        <v>4.560606</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.528</v>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="9" t="n">
-        <v>-0.595</v>
+        <v>-0.591</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>-0.585</v>
+        <v>-0.581</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.26</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>0</v>
+        <v>11.29</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>0.26642746</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,19 +1693,19 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.152</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.919</v>
+        <v>0.921</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.766666</v>
+        <v>18.816666</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>12.159433</v>
+        <v>12.19183</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0.107</v>
+        <v>0.11</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>-0.01</v>
+        <v>-0.006999999999999999</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.66</v>
+        <v>26.72</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.011380851</v>
+        <v>0.013657007</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,10 +1752,10 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.186</v>
+        <v>-0.184</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.704</v>
+        <v>0.705</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>1.153</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>22.033056</v>
+        <v>22.082644</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.449</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>-0.013</v>
+        <v>-0.011</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>-0.015</v>
+        <v>-0.012</v>
       </c>
     </row>
     <row r="21">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.47</v>
+        <v>6.46</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.46154168</v>
+        <v>-0.5388737300000001</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1882,7 +1882,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.35</v>
+        <v>-0.351</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.175</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.636339</v>
+        <v>8.629664999999999</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.818</v>
@@ -1934,7 +1934,7 @@
         <v>2.27</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>-0.021551704</v>
+        <v>-0.02150854</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>-5.5365853</v>
+        <v>-5.5368295</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>12.539</v>
@@ -2158,28 +2158,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.78</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.014537034</v>
+        <v>0.017222228</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.155</v>
+        <v>-0.153</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.348</v>
+        <v>0.351</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>53.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.034</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.014</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.222</v>
+        <v>-0.22</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2205,28 +2205,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.75</v>
+        <v>107.92</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.014902151</v>
+        <v>-0.013347954</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.506</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-56.8</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.251</v>
+        <v>-0.25</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>-0.531</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.657</v>
+        <v>-0.6559999999999999</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2252,28 +2252,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.3</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.02673906</v>
+        <v>-0.021307719</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.347</v>
+        <v>-0.343</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.425</v>
+        <v>-0.422</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.142</v>
+        <v>-0.137</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.348</v>
+        <v>-0.344</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.522</v>
+        <v>-0.52</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2299,28 +2299,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.08</v>
+        <v>102.95</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.9393895000000001</v>
+        <v>0.017996635</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.165</v>
+        <v>-0.158</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.214</v>
+        <v>0.224</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>34.7</v>
+        <v>34.8</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.063</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.107</v>
+        <v>-0.1</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.242</v>
+        <v>-0.236</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2346,28 +2346,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.99</v>
+        <v>37.23</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.10825688</v>
+        <v>0.75777745</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.014</v>
+        <v>0.02</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.141</v>
+        <v>0.148</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>11.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.044</v>
+        <v>0.05</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.052</v>
+        <v>0.059</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.079</v>
+        <v>-0.073</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2393,28 +2393,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.54000000000001</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.019526464</v>
+        <v>0.024286036</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.219</v>
+        <v>0.224</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.5</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.004</v>
+        <v>0</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.014</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.07099999999999999</v>
+        <v>-0.067</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2426,12 +2426,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2440,45 +2440,45 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.2</v>
+        <v>58.56</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.01867164</v>
+        <v>0.82644546</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.23</v>
+        <v>-0.051</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.239</v>
+        <v>0.37</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>-3.2</v>
+        <v>39.1</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.091</v>
+        <v>-0.05</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.146</v>
+        <v>-0.002</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.272</v>
+        <v>-0.151</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>0.66</v>
+        <v>1.453</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>1091240</v>
+        <v>941430</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -2487,34 +2487,34 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.34</v>
+        <v>85.86</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.45650196</v>
+        <v>0.014712776</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.055</v>
+        <v>-0.233</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.365</v>
+        <v>-0.242</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>39.1</v>
+        <v>-3.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.053</v>
+        <v>-0.094</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.15</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.275</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>1.453</v>
+        <v>0.66</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>941430</v>
+        <v>1091240</v>
       </c>
     </row>
     <row r="10">
@@ -2534,28 +2534,28 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.16</v>
+        <v>19.33</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.018945255</v>
+        <v>-0.010240694</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-0.178</v>
+        <v>-0.171</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.167</v>
+        <v>-0.159</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-28.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.043</v>
+        <v>0.052</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-0.218</v>
+        <v>-0.211</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.4</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>2.002</v>
@@ -2581,28 +2581,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.01170412</v>
+        <v>0.020599186</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.059</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.5529999999999999</v>
+        <v>0.5660000000000001</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.07400000000000001</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.038</v>
+        <v>-0.029</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.249</v>
+        <v>-0.242</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.1</v>
@@ -2628,28 +2628,28 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.36</v>
+        <v>26.41</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.30257156</v>
+        <v>-0.09455226</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.119</v>
+        <v>0.121</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.063</v>
+        <v>-0.061</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>-22.7</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.124</v>
+        <v>0.126</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.165</v>
+        <v>-0.164</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>1.977</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.78</v>
+        <v>22.04</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.1379342</v>
+        <v>0.013333375</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.128</v>
+        <v>0.141</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.9209999999999999</v>
+        <v>0.9440000000000001</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.158</v>
+        <v>0.172</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.191</v>
+        <v>0.205</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.038</v>
+        <v>-0.027</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2722,28 +2722,28 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.96</v>
+        <v>13</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.6896563</v>
+        <v>-0.3831432200000001</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.138</v>
+        <v>-0.135</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.036</v>
+        <v>-0.033</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>13.4</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.057</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.161</v>
+        <v>-0.159</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.302</v>
+        <v>-0.3</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2772,13 +2772,13 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.01188301</v>
+        <v>0.013711205</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.263</v>
+        <v>-0.262</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.004</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>8.6</v>
@@ -2816,28 +2816,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.41</v>
+        <v>14.54</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.17312756</v>
+        <v>0.6578966000000002</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.029</v>
+        <v>-0.021</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.162</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.3</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.046</v>
+        <v>0.055</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.113</v>
+        <v>-0.105</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.301</v>
+        <v>-0.295</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2863,28 +2863,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.3</v>
+        <v>98.72</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.040709257</v>
+        <v>0.4681448</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.027</v>
+        <v>0.031</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.227</v>
+        <v>0.232</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.036</v>
+        <v>0.04</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.023</v>
+        <v>0.027</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.137</v>
+        <v>-0.133</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2910,28 +2910,28 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.47</v>
+        <v>4.51</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.04787232399999999</v>
+        <v>-0.039361691</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.585</v>
+        <v>-0.581</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.595</v>
+        <v>-0.591</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-32.1</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.379</v>
+        <v>-0.374</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5589999999999999</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.674</v>
+        <v>-0.672</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>1.993</v>
@@ -2957,28 +2957,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.26</v>
+        <v>11.29</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0</v>
+        <v>0.26642746</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.01</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.107</v>
+        <v>0.11</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.2</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.003</v>
+        <v>-0</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.152</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -3004,28 +3004,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.66</v>
+        <v>26.72</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.011380851</v>
+        <v>0.013657007</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.015</v>
+        <v>-0.012</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-0.013</v>
+        <v>-0.011</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.046</v>
+        <v>-0.044</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.008</v>
+        <v>-0.006</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.186</v>
+        <v>-0.184</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3100,10 +3100,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.47</v>
+        <v>6.46</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.46154168</v>
+        <v>-0.5388737300000001</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-0.279</v>
@@ -3115,13 +3115,13 @@
         <v>4.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.228</v>
+        <v>-0.229</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.244</v>
+        <v>-0.246</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.35</v>
+        <v>-0.351</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3150,7 +3150,7 @@
         <v>2.27</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.021551704</v>
+        <v>-0.02150854</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-0.092</v>
@@ -3348,16 +3348,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.78</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>37.042</v>
+        <v>37.14</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.312767</v>
+        <v>23.37447</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>14.580018</v>
+        <v>14.618607</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.77</v>
@@ -3369,10 +3369,10 @@
         <v>3.75</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.253397</v>
+        <v>23.314941</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.8456655</v>
+        <v>2.853197</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.75</v>
+        <v>107.92</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.87</v>
+        <v>18.9</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.976694999999999</v>
+        <v>9.992435</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0889878</v>
+        <v>2.0922837</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1518332</v>
+        <v>1.1536504</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.3</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.596</v>
+        <v>11.66</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>11.9688635</v>
+        <v>12.035657</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.25627</v>
+        <v>18.35815</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.9151975</v>
+        <v>1.9258853</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,16 +3511,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.08</v>
+        <v>102.95</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.645</v>
+        <v>10.736</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.509552</v>
+        <v>32.78662</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.180065</v>
+        <v>17.326487</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.354</v>
@@ -3532,10 +3532,10 @@
         <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-37.976192</v>
+        <v>-38.29985</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4913633</v>
+        <v>1.5040737</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3564,16 +3564,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.99</v>
+        <v>37.23</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.117</v>
+        <v>10.183</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.671055</v>
+        <v>48.986843</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.786711</v>
+        <v>15.889138</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.81</v>
@@ -3585,10 +3585,10 @@
         <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9321785</v>
+        <v>3.9576912</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5768723</v>
+        <v>0.58061516</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.54000000000001</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.307</v>
+        <v>6.336</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7030144</v>
+        <v>3.7203016</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.253565</v>
+        <v>10.301433</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.445765</v>
+        <v>2.457183</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5412111</v>
+        <v>1.5484061</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3656,12 +3656,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -3670,51 +3670,51 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>86.2</v>
+        <v>58.56</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.008</v>
+        <v>6.022</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.294895</v>
+        <v>18.769232</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.609365</v>
+        <v>17.82144</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>11.435</v>
+        <v>8.413</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>7.3</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.739</v>
+        <v>3.404</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>5.941959</v>
+        <v>16.394176</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0533264</v>
+        <v>2.9935842</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>5.29</v>
+        <v>3.12</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>7.42504</v>
+        <v>3.28593</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>14.507</v>
+        <v>3.572</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -3723,40 +3723,40 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>58.34</v>
+        <v>85.86</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.999</v>
+        <v>5.984</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>18.700321</v>
+        <v>16.23157</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.756008</v>
+        <v>11.564247</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>8.413</v>
+        <v>11.435</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7.3</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.404</v>
+        <v>3.739</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.333986</v>
+        <v>5.9188666</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.982593</v>
+        <v>2.0453465</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>3.12</v>
+        <v>5.29</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>3.28593</v>
+        <v>7.42504</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>3.572</v>
+        <v>14.507</v>
       </c>
     </row>
     <row r="10">
@@ -3776,16 +3776,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.16</v>
+        <v>19.33</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.67</v>
+        <v>5.721</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.22222</v>
+        <v>53.694443</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.360363</v>
+        <v>23.56763</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.087511</v>
+        <v>5.132651</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.395804</v>
+        <v>4.4348063</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.463</v>
+        <v>5.511</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.726192</v>
+        <v>25.952381</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.456624</v>
+        <v>12.566145</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.33537</v>
+        <v>7.3998637</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.3318906</v>
+        <v>2.352393</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3882,10 +3882,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.36</v>
+        <v>26.41</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.38</v>
+        <v>5.392</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>28.497297</v>
+        <v>28.556757</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>8.669</v>
@@ -3905,10 +3905,10 @@
         <v>2.638</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.5243163</v>
+        <v>1.5274968</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>0.46842116</v>
+        <v>0.46939853</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>-2.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.78</v>
+        <v>22.04</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.07</v>
+        <v>5.131</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>70.258064</v>
+        <v>71.09678</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.104807</v>
+        <v>29.452248</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.786151</v>
+        <v>14.962662</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4692545</v>
+        <v>4.522607</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3996,10 +3996,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.96</v>
+        <v>13</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.391</v>
+        <v>2.399</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>12.027395</v>
+        <v>12.064517</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.776</v>
@@ -4019,10 +4019,10 @@
         <v>2.38</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7674568</v>
+        <v>2.7759984</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.9524057</v>
+        <v>0.95534515</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4054,13 +4054,13 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.252</v>
+        <v>2.256</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.032608</v>
+        <v>12.054348</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.957101</v>
+        <v>6.969671</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.582</v>
@@ -4072,10 +4072,10 @@
         <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.734566</v>
+        <v>-1.7376999</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43607658</v>
+        <v>0.43686444</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.41</v>
+        <v>14.54</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.925</v>
+        <v>1.941</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.28196</v>
+        <v>8.350904</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.184</v>
@@ -4127,10 +4127,10 @@
         <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.9922902</v>
+        <v>1.0005506</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.2765507</v>
+        <v>0.2788529</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4159,16 +4159,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.3</v>
+        <v>98.72</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.758</v>
+        <v>1.766</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>18.103132</v>
+        <v>18.18048</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.534903</v>
+        <v>16.60555</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.779</v>
@@ -4180,10 +4180,10 @@
         <v>3.071</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2577717</v>
+        <v>3.2716908</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.2253258</v>
+        <v>3.2391062</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4212,10 +4212,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.47</v>
+        <v>4.51</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.151</v>
+        <v>1.161</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.5202017</v>
+        <v>4.560606</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.528</v>
@@ -4237,10 +4237,10 @@
         <v>1.356</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.5215913</v>
+        <v>1.5351921</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.7195121</v>
+        <v>1.7348821</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4269,16 +4269,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.26</v>
+        <v>11.29</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.919</v>
+        <v>0.921</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.766666</v>
+        <v>18.816666</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>12.159433</v>
+        <v>12.19183</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4290,10 +4290,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.4360697</v>
+        <v>3.4452243</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6901145</v>
+        <v>0.6919532</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4322,10 +4322,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.66</v>
+        <v>26.72</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.704</v>
+        <v>0.705</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>22.033056</v>
+        <v>22.082644</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.449</v>
@@ -4345,10 +4345,10 @@
         <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6585791</v>
+        <v>1.6623118</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1084898</v>
+        <v>1.1109846</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.47</v>
+        <v>6.46</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.175</v>
@@ -4449,7 +4449,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.636339</v>
+        <v>8.629664999999999</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.818</v>
@@ -4461,10 +4461,10 @@
         <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.729685</v>
+        <v>-10.721394</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.5757166</v>
+        <v>0.5752718</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5.5365853</v>
+        <v>-5.5368295</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>12.539</v>
@@ -4516,10 +4516,10 @@
         <v>1.911</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>32.42857</v>
+        <v>32.43</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.27163392</v>
+        <v>0.27164587</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>-1.12</v>
@@ -5086,12 +5086,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -5100,57 +5100,57 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>2.926</v>
+        <v>2.011</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.067</v>
+        <v>0.032</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.33583</v>
+        <v>0.6747</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.18802</v>
+        <v>0.31768</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.1309</v>
+        <v>0.0935</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>0.32698002</v>
+        <v>0.4046</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.35709</v>
+        <v>1.113</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>0.06236</v>
+        <v>0.09383000399999999</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.957</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>0.082</v>
+        <v>0.193</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>5.197</v>
+        <v>3.475</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>0.201</v>
+        <v>0.142</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>492.233</v>
+        <v>1045.932</v>
       </c>
       <c r="Q8" s="7" t="n">
-        <v>0.604</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -5159,46 +5159,46 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>2.011</v>
+        <v>2.926</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.032</v>
+        <v>0.067</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.6747</v>
+        <v>0.33583</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.31768</v>
+        <v>0.18802</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.0935</v>
+        <v>0.1309</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>0.4046</v>
+        <v>0.32698002</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>1.113</v>
+        <v>0.35709</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>0.09383000399999999</v>
+        <v>0.06236</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.957</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>0.193</v>
+        <v>0.082</v>
       </c>
       <c r="N9" s="6" t="n">
-        <v>3.475</v>
+        <v>5.197</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>0.142</v>
+        <v>0.201</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>1045.932</v>
+        <v>492.233</v>
       </c>
       <c r="Q9" s="7" t="n">
-        <v>0.79</v>
+        <v>0.604</v>
       </c>
     </row>
     <row r="10">
@@ -6257,7 +6257,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>54.78</v>
+        <v>54.93</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6280,7 +6280,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.276</v>
+        <v>0.272</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>1.8</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.75</v>
+        <v>107.92</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.9740000000000001</v>
+        <v>0.971</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.3</v>
+        <v>23.43</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.5529999999999999</v>
+        <v>0.544</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>102.08</v>
+        <v>102.95</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6452,7 +6452,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.389</v>
+        <v>0.3779999999999999</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.24</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>36.99</v>
+        <v>37.23</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.153</v>
+        <v>0.146</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>83.54000000000001</v>
+        <v>83.93000000000001</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6566,7 +6566,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.131</v>
+        <v>0.126</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.32</v>
@@ -6590,113 +6590,113 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>86.2</v>
+        <v>58.56</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>strong_buy</t>
+          <t>buy</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>1.25</v>
+        <v>1.5625</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>135.5</v>
+        <v>72.9375</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>152</v>
+        <v>80</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>110</v>
+        <v>59</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.5720000000000001</v>
+        <v>0.246</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>2.68</v>
+        <v>3.89</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>0.044499997</v>
+        <v>0.0762</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>0.06136</v>
+        <v>0.07914</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>0.81711</v>
+        <v>0.88882005</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>0.52</v>
+        <v>1.79</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>0.0828</v>
+        <v>0.32369998</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>58.34</v>
+        <v>85.86</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>buy</t>
+          <t>strong_buy</t>
         </is>
       </c>
       <c r="E9" s="7" t="n">
-        <v>1.6</v>
+        <v>1.25</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>73.33333</v>
+        <v>135.5</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>80</v>
+        <v>152</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>59</v>
+        <v>110</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.257</v>
+        <v>0.578</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>3.89</v>
+        <v>2.68</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.0762</v>
+        <v>0.044499997</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>0.07914</v>
+        <v>0.06136</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.88882005</v>
+        <v>0.81711</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>1.79</v>
+        <v>0.52</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>0.32369998</v>
+        <v>0.0828</v>
       </c>
     </row>
     <row r="10">
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>19.16</v>
+        <v>19.33</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6725,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.883062</v>
+        <v>28.919893</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.238945</v>
+        <v>37.286427</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.964575</v>
+        <v>21.992582</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.507</v>
+        <v>0.496</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.609</v>
+        <v>0.594</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6825,7 +6825,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>26.36</v>
+        <v>26.41</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.212</v>
+        <v>0.21</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>3.8</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.78</v>
+        <v>22.04</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6906,7 +6906,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.139</v>
+        <v>0.125</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -6941,7 +6941,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.96</v>
+        <v>13</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6964,7 +6964,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.395</v>
+        <v>0.391</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.42</v>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.41</v>
+        <v>14.54</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.326</v>
+        <v>0.314</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>98.3</v>
+        <v>98.72</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7138,7 +7138,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.095</v>
+        <v>0.091</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.53</v>
@@ -7171,7 +7171,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4.47</v>
+        <v>4.51</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -7194,7 +7194,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1.632</v>
+        <v>1.609</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>1.77</v>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.26</v>
+        <v>11.29</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7252,7 +7252,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.377</v>
+        <v>0.373</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.68</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.66</v>
+        <v>26.72</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.144</v>
+        <v>0.141</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>2.5</v>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.47</v>
+        <v>6.46</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.061</v>
+        <v>1.064</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7707,10 +7707,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>37.042</v>
+        <v>37.14</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.312767</v>
+        <v>23.37447</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7722,7 +7722,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.155</v>
+        <v>-0.153</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.77</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.38</v>
+        <v>5.392</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7768,7 +7768,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.119</v>
+        <v>0.121</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.669</v>
@@ -7797,10 +7797,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.252</v>
+        <v>2.256</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.032608</v>
+        <v>12.054348</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.263</v>
+        <v>-0.262</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>10.582</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.117</v>
+        <v>10.183</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48.671055</v>
+        <v>48.986843</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7858,7 +7858,7 @@
         <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.014</v>
+        <v>0.02</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>16.81</v>
@@ -7887,10 +7887,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.645</v>
+        <v>10.736</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>32.509552</v>
+        <v>32.78662</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7904,7 +7904,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.165</v>
+        <v>-0.158</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>11.354</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.307</v>
+        <v>6.336</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7030144</v>
+        <v>3.7203016</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7966,7 +7966,7 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.024</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>7.113</v>
@@ -7975,18 +7975,18 @@
         <v>5.9</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>71.40000000000001</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Monarch Casino &amp; Resort</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -7995,42 +7995,42 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.008</v>
+        <v>1.766</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.294895</v>
+        <v>18.18048</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.067</v>
+        <v>0.041</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.32698002</v>
+        <v>0.34986</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.35709</v>
+        <v>0.19214001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-0.23</v>
+        <v>0.031</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.435</v>
+        <v>8.779</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>9.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>63.5</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MCRI</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Monarch Casino &amp; Resort</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -8039,31 +8039,31 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.758</v>
+        <v>5.984</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>18.103132</v>
+        <v>16.23157</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.041</v>
+        <v>0.067</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.34986</v>
+        <v>0.32698002</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.19214001</v>
+        <v>0.35709</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.027</v>
+        <v>-0.233</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.779</v>
+        <v>11.435</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>62.7</v>
+        <v>61.1</v>
       </c>
     </row>
     <row r="13">
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5.999</v>
+        <v>6.022</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.700321</v>
+        <v>18.769232</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8098,7 +8098,7 @@
         <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.055</v>
+        <v>-0.051</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.413</v>
@@ -8107,7 +8107,7 @@
         <v>7.3</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>57.1</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="14">
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.925</v>
+        <v>1.941</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.029</v>
+        <v>-0.021</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.184</v>
@@ -8153,7 +8153,7 @@
         <v>10.9</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>48.6</v>
+        <v>51.4</v>
       </c>
     </row>
     <row r="15">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.704</v>
+        <v>0.705</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8190,7 +8190,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.015</v>
+        <v>-0.012</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.449</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.463</v>
+        <v>5.511</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.726192</v>
+        <v>25.952381</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.059</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8377,10 +8377,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.67</v>
+        <v>5.721</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.22222</v>
+        <v>53.694443</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8392,7 +8392,7 @@
         <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.178</v>
+        <v>-0.171</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>10.962</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.07</v>
+        <v>5.131</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>70.258064</v>
+        <v>71.09678</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.128</v>
+        <v>0.141</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.596</v>
+        <v>11.66</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.347</v>
+        <v>-0.343</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.87</v>
+        <v>18.9</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8561,7 +8561,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.151</v>
+        <v>1.161</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.585</v>
+        <v>-0.581</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>-7.528</v>
@@ -8627,10 +8627,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.919</v>
+        <v>0.921</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.766666</v>
+        <v>18.816666</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8642,7 +8642,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.01</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.391</v>
+        <v>2.399</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8688,7 +8688,7 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.138</v>
+        <v>-0.135</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>6.776</v>
@@ -9696,55 +9696,55 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Churchill Downs</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0.06136</v>
+        <v>0.07914</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.81711</v>
+        <v>0.88882005</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2.68</v>
+        <v>3.89</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.044499997</v>
+        <v>0.0762</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>2574942</v>
+        <v>3025746</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>CHDN</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Churchill Downs</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.07914</v>
+        <v>0.06136</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.88882005</v>
+        <v>0.81711</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>3.89</v>
+        <v>2.68</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.0762</v>
+        <v>0.044499997</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>3025746</v>
+        <v>2574942</v>
       </c>
     </row>
     <row r="10">
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.56</v>
+        <v>1277.79</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1212.94</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.23</v>
+        <v>1267.48</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.08</v>
+        <v>1262.34</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1254.78</v>
+        <v>1255.02</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1259.62</v>
+        <v>1259.86</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.2</v>
+        <v>1260.45</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.47</v>
+        <v>1245.7</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.18</v>
+        <v>1198.38</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1222.85</v>
+        <v>1223.06</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.17</v>
+        <v>1194.42</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1189.97</v>
+        <v>1190.2</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.22</v>
+        <v>1182.44</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1179.93</v>
+        <v>1180.15</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1198.74</v>
+        <v>1198.99</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.49</v>
+        <v>1162.74</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.13</v>
+        <v>1139.36</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1145.7</v>
+        <v>1145.92</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1150.79</v>
+        <v>1151.01</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1135.86</v>
+        <v>1136.05</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1141.72</v>
+        <v>1141.91</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1128.84</v>
+        <v>1129.05</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1130.63</v>
+        <v>1130.83</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1078.66</v>
+        <v>1078.96</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.04</v>
+        <v>1067.31</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.12</v>
+        <v>1085.38</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1081.8</v>
+        <v>1082.04</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1102.69</v>
+        <v>1102.95</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.36</v>
+        <v>1078.59</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105</v>
+        <v>1105.28</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1106.85</v>
+        <v>1107.13</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1103.83</v>
+        <v>1104.09</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.4</v>
+        <v>1089.64</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1052.73</v>
+        <v>1052.93</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1043.52</v>
+        <v>1043.77</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.2</v>
+        <v>1058.49</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.38</v>
+        <v>1091.71</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.28</v>
+        <v>1086.62</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1086.39</v>
+        <v>1086.73</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.33</v>
+        <v>1043.65</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1057.78</v>
+        <v>1058.14</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1061.67</v>
+        <v>1062.04</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.26</v>
+        <v>1090.68</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1077.67</v>
+        <v>1078.08</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1072.54</v>
+        <v>1072.95</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1068.49</v>
+        <v>1068.88</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1083.89</v>
+        <v>1084.33</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1081.53</v>
+        <v>1081.99</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.08</v>
+        <v>1050.54</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1051.63</v>
+        <v>1052.09</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1050.72</v>
+        <v>1051.18</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.11</v>
+        <v>1065.55</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1050.98</v>
+        <v>1051.44</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1052.92</v>
+        <v>1053.36</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1045.51</v>
+        <v>1045.94</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1057.77</v>
+        <v>1058.22</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1049.88</v>
+        <v>1050.33</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1062.47</v>
+        <v>1062.95</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1034.43</v>
+        <v>1034.89</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.21</v>
+        <v>1056.7</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1061.72</v>
+        <v>1067.31</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1061.72</v>
+        <v>1067.31</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.71%</t>
+          <t>-15.28%</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>140.1</v>
+        <v>140.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 14:15
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.93</v>
+        <v>54.89</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.017222228</v>
+        <v>0.01648147</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.22</v>
+        <v>-0.221</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>37.14</v>
+        <v>37.113</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.818</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.37447</v>
+        <v>23.357447</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>14.618607</v>
+        <v>14.607962</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.77</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.153</v>
+        <v>-0.154</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.92</v>
+        <v>107.67</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.013347954</v>
+        <v>-0.015633563</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.6559999999999999</v>
+        <v>-0.657</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.9</v>
+        <v>18.856</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.992435</v>
+        <v>9.969288000000001</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -755,10 +755,10 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>-0.506</v>
+        <v>-0.507</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.4</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.021307719</v>
+        <v>-0.022352197</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -793,7 +793,7 @@
         <v>-0.52</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.66</v>
+        <v>11.648</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>12.035657</v>
+        <v>12.022812</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.422</v>
+        <v>-0.423</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.343</v>
+        <v>-0.344</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.95</v>
+        <v>102.89</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.017996635</v>
+        <v>0.017403364</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -854,16 +854,16 @@
         <v>-0.236</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.736</v>
+        <v>10.73</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.78662</v>
+        <v>32.767513</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.326487</v>
+        <v>17.31639</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.354</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.224</v>
+        <v>0.223</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>-0.158</v>
+        <v>-0.159</v>
       </c>
     </row>
     <row r="6">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.93000000000001</v>
+        <v>83.92</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.024286036</v>
+        <v>0.024102983</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.067</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.336</v>
+        <v>6.335</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7203016</v>
+        <v>3.7196367</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.301433</v>
+        <v>10.299592</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.56</v>
+        <v>58.63</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.82644546</v>
+        <v>0.9450702</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1028,19 +1028,19 @@
         <v>35.09</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.151</v>
+        <v>-0.15</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.022</v>
+        <v>6.029</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>6.847</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>18.769232</v>
+        <v>18.791315</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>17.82144</v>
+        <v>17.842407</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>8.413</v>
@@ -1052,10 +1052,10 @@
         <v>1.453</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0.37</v>
+        <v>0.3720000000000001</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.051</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="9">
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.86</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.014712776</v>
+        <v>0.014358264</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>118.46</v>
@@ -1090,16 +1090,16 @@
         <v>-0.275</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.984</v>
+        <v>5.982</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>10.94</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.23157</v>
+        <v>16.225899</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>11.564247</v>
+        <v>11.560207</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>11.435</v>
@@ -1137,7 +1137,7 @@
         <v>19.33</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.010240694</v>
+        <v>-0.010245773</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1155,10 +1155,10 @@
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.694443</v>
+        <v>53.694168</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.56763</v>
+        <v>23.56751</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.9</v>
+        <v>10.89</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.020599186</v>
+        <v>0.0201311</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1205,19 +1205,19 @@
         <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.242</v>
+        <v>-0.243</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.511</v>
+        <v>5.509</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.952381</v>
+        <v>25.940477</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.566145</v>
+        <v>12.560381</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1232,7 +1232,7 @@
         <v>0.5660000000000001</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.059</v>
+        <v>-0.06</v>
       </c>
     </row>
     <row r="12">
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.41</v>
+        <v>26.33</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.09455226</v>
+        <v>-0.4160386</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>31.58</v>
@@ -1264,10 +1264,10 @@
         <v>17.86</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.164</v>
+        <v>-0.166</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.392</v>
+        <v>5.374</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>30.298</v>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>28.556757</v>
+        <v>28.464865</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>8.669</v>
@@ -1290,10 +1290,10 @@
         <v>1.977</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>-0.061</v>
+        <v>-0.064</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>0.121</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.04</v>
+        <v>22.11</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.013333375</v>
+        <v>0.016551752</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.024</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.131</v>
+        <v>5.147</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>71.09678</v>
+        <v>71.32258</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.452248</v>
+        <v>29.54579</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.9440000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.141</v>
+        <v>0.145</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13</v>
+        <v>13.01</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>-0.3831432200000001</v>
+        <v>-0.3065131</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.3</v>
+        <v>-0.299</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.399</v>
+        <v>2.401</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.976</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>12.064517</v>
+        <v>12.073797</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.776</v>
@@ -1442,7 +1442,7 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.013711205</v>
+        <v>0.012797107</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1454,16 +1454,16 @@
         <v>-0.454</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.256</v>
+        <v>2.254</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.043478</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.969671</v>
+        <v>6.9633856</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.582</v>
@@ -1475,7 +1475,7 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.004</v>
+        <v>-0.005</v>
       </c>
       <c r="Q15" s="9" t="n">
         <v>-0.262</v>
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.54</v>
+        <v>14.53</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.6578966000000002</v>
+        <v>0.58864295</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1513,7 +1513,7 @@
         <v>-0.295</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.941</v>
+        <v>1.94</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.411</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.350904</v>
+        <v>8.345159000000001</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.184</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>-0.162</v>
+        <v>-0.163</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.021</v>
+        <v>-0.022</v>
       </c>
     </row>
     <row r="17">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.72</v>
+        <v>26.75</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.013657007</v>
+        <v>0.014795121</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,10 +1752,10 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.184</v>
+        <v>-0.183</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>1.153</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>22.082644</v>
+        <v>22.107437</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.449</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
+        <v>-0.009000000000000001</v>
+      </c>
+      <c r="Q20" s="9" t="n">
         <v>-0.011</v>
-      </c>
-      <c r="Q20" s="9" t="n">
-        <v>-0.012</v>
       </c>
     </row>
     <row r="21">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.5388737300000001</v>
+        <v>-0.7692337</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1882,7 +1882,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.351</v>
+        <v>-0.352</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.175</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.629664999999999</v>
+        <v>8.609643</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.818</v>
@@ -1908,10 +1908,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>-0.293</v>
+        <v>-0.295</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>-0.279</v>
+        <v>-0.281</v>
       </c>
     </row>
     <row r="23">
@@ -1931,10 +1931,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>-0.02150854</v>
+        <v>-0.012919884</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1943,10 +1943,10 @@
         <v>2.02</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.537</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.082</v>
+        <v>0.083</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0.578</v>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>-5.5368295</v>
+        <v>-5.585366</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>12.539</v>
@@ -1969,10 +1969,10 @@
         <v>1.327</v>
       </c>
       <c r="P23" s="9" t="n">
-        <v>-0.492</v>
+        <v>-0.488</v>
       </c>
       <c r="Q23" s="9" t="n">
-        <v>-0.092</v>
+        <v>-0.08400000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -2158,28 +2158,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.93</v>
+        <v>54.89</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.017222228</v>
+        <v>0.01648147</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.153</v>
+        <v>-0.154</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.351</v>
+        <v>0.35</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>53.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.034</v>
+        <v>-0.035</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.014</v>
+        <v>-0.015</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.22</v>
+        <v>-0.221</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2205,28 +2205,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.92</v>
+        <v>107.67</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.013347954</v>
+        <v>-0.015633563</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.506</v>
+        <v>-0.507</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-56.8</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.25</v>
+        <v>-0.252</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.531</v>
+        <v>-0.532</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.6559999999999999</v>
+        <v>-0.657</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2252,25 +2252,25 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.4</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.021307719</v>
+        <v>-0.022352197</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.343</v>
+        <v>-0.344</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.422</v>
+        <v>-0.423</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.137</v>
+        <v>-0.138</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.344</v>
+        <v>-0.345</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>-0.52</v>
@@ -2299,22 +2299,22 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.95</v>
+        <v>102.89</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.017996635</v>
+        <v>0.017403364</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.158</v>
+        <v>-0.159</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.224</v>
+        <v>0.223</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>34.8</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.063</v>
+        <v>-0.064</v>
       </c>
       <c r="J5" s="5" t="n">
         <v>-0.1</v>
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.93000000000001</v>
+        <v>83.92</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.024286036</v>
+        <v>0.024102983</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.024</v>
@@ -2440,28 +2440,28 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.56</v>
+        <v>58.63</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.82644546</v>
+        <v>0.9450702</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.051</v>
+        <v>-0.05</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.37</v>
+        <v>0.3720000000000001</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>39.1</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.049</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.002</v>
+        <v>-0.001</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.151</v>
+        <v>-0.15</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>1.453</v>
@@ -2487,10 +2487,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.86</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.014712776</v>
+        <v>0.014358264</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.233</v>
@@ -2502,7 +2502,7 @@
         <v>-3.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>-0.15</v>
@@ -2537,7 +2537,7 @@
         <v>19.33</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.010240694</v>
+        <v>-0.010245773</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>-0.171</v>
@@ -2581,13 +2581,13 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.9</v>
+        <v>10.89</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.020599186</v>
+        <v>0.0201311</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.059</v>
+        <v>-0.06</v>
       </c>
       <c r="G11" s="5" t="n">
         <v>0.5660000000000001</v>
@@ -2596,13 +2596,13 @@
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.083</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.029</v>
+        <v>-0.03</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.242</v>
+        <v>-0.243</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.1</v>
@@ -2628,28 +2628,28 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.41</v>
+        <v>26.33</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.09455226</v>
+        <v>-0.4160386</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.121</v>
+        <v>0.118</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.064</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>-22.7</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.126</v>
+        <v>0.123</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.068</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.164</v>
+        <v>-0.166</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>1.977</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.04</v>
+        <v>22.11</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.013333375</v>
+        <v>0.016551752</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.141</v>
+        <v>0.145</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.9440000000000001</v>
+        <v>0.95</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.172</v>
+        <v>0.175</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.205</v>
+        <v>0.209</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.024</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2722,10 +2722,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13</v>
+        <v>13.01</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.3831432200000001</v>
+        <v>-0.3065131</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>-0.135</v>
@@ -2737,13 +2737,13 @@
         <v>13.4</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.057</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.159</v>
+        <v>-0.158</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.3</v>
+        <v>-0.299</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2772,13 +2772,13 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.013711205</v>
+        <v>0.012797107</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.262</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.004</v>
+        <v>-0.005</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>8.6</v>
@@ -2816,16 +2816,16 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.54</v>
+        <v>14.53</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.6578966000000002</v>
+        <v>0.58864295</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.021</v>
+        <v>-0.022</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.162</v>
+        <v>-0.163</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.3</v>
@@ -2834,7 +2834,7 @@
         <v>0.055</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.105</v>
+        <v>-0.106</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>-0.295</v>
@@ -3004,28 +3004,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.72</v>
+        <v>26.75</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.013657007</v>
+        <v>0.014795121</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.011</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.044</v>
+        <v>-0.043</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.005</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.184</v>
+        <v>-0.183</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3100,28 +3100,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.5388737300000001</v>
+        <v>-0.7692337</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.279</v>
+        <v>-0.281</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.293</v>
+        <v>-0.295</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.229</v>
+        <v>-0.23</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.246</v>
+        <v>-0.247</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.351</v>
+        <v>-0.352</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3147,28 +3147,28 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.02150854</v>
+        <v>-0.012919884</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-0.492</v>
+        <v>-0.488</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>-53</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.052</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.257</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.537</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>1.327</v>
@@ -3348,16 +3348,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.93</v>
+        <v>54.89</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>37.14</v>
+        <v>37.113</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.37447</v>
+        <v>23.357447</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>14.618607</v>
+        <v>14.607962</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.77</v>
@@ -3369,10 +3369,10 @@
         <v>3.75</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.314941</v>
+        <v>23.297962</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.853197</v>
+        <v>2.8511193</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.92</v>
+        <v>107.67</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.9</v>
+        <v>18.856</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.992435</v>
+        <v>9.969288000000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0922837</v>
+        <v>2.087437</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1536504</v>
+        <v>1.1509781</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.4</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.66</v>
+        <v>11.648</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12.035657</v>
+        <v>12.022812</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.35815</v>
+        <v>18.338558</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.9258853</v>
+        <v>1.9238299</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,16 +3511,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.95</v>
+        <v>102.89</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.736</v>
+        <v>10.73</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.78662</v>
+        <v>32.767513</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.326487</v>
+        <v>17.31639</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.354</v>
@@ -3532,10 +3532,10 @@
         <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-38.29985</v>
+        <v>-38.27753</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.5040737</v>
+        <v>1.5031972</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.93000000000001</v>
+        <v>83.92</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.336</v>
+        <v>6.335</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7203016</v>
+        <v>3.7196367</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.301433</v>
+        <v>10.299592</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.457183</v>
+        <v>2.4567437</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5484061</v>
+        <v>1.5481296</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3670,16 +3670,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.56</v>
+        <v>58.63</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.022</v>
+        <v>6.029</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>18.769232</v>
+        <v>18.791315</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>17.82144</v>
+        <v>17.842407</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>8.413</v>
@@ -3691,10 +3691,10 @@
         <v>3.404</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.394176</v>
+        <v>16.413465</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.9935842</v>
+        <v>2.9971058</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>3.12</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.86</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.984</v>
+        <v>5.982</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.23157</v>
+        <v>16.225899</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>11.564247</v>
+        <v>11.560207</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>11.435</v>
@@ -3744,10 +3744,10 @@
         <v>3.739</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>5.9188666</v>
+        <v>5.9167986</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.0453465</v>
+        <v>2.0446317</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>5.29</v>
@@ -3782,10 +3782,10 @@
         <v>5.721</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.694443</v>
+        <v>53.694168</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.56763</v>
+        <v>23.56751</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.132651</v>
+        <v>5.1326246</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.4348063</v>
+        <v>4.4347835</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.9</v>
+        <v>10.89</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.511</v>
+        <v>5.509</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.952381</v>
+        <v>25.940477</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.566145</v>
+        <v>12.560381</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.3998637</v>
+        <v>7.39647</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.352393</v>
+        <v>2.351314</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3882,10 +3882,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.41</v>
+        <v>26.33</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.392</v>
+        <v>5.374</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>28.556757</v>
+        <v>28.464865</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>8.669</v>
@@ -3905,10 +3905,10 @@
         <v>2.638</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.5274968</v>
+        <v>1.5225815</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>0.46939853</v>
+        <v>0.46788803</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>-2.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.04</v>
+        <v>22.11</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.131</v>
+        <v>5.147</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>71.09678</v>
+        <v>71.32258</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.452248</v>
+        <v>29.54579</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.962662</v>
+        <v>15.010183</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.522607</v>
+        <v>4.5369706</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3996,10 +3996,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13</v>
+        <v>13.01</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.399</v>
+        <v>2.401</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>12.064517</v>
+        <v>12.073797</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.776</v>
@@ -4019,10 +4019,10 @@
         <v>2.38</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7759984</v>
+        <v>2.7781336</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.95534515</v>
+        <v>0.95608014</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4054,13 +4054,13 @@
         <v>5.54</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.256</v>
+        <v>2.254</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.043478</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.969671</v>
+        <v>6.9633856</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.582</v>
@@ -4072,10 +4072,10 @@
         <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7376999</v>
+        <v>-1.7361329</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43686444</v>
+        <v>0.4364705</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.54</v>
+        <v>14.53</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.941</v>
+        <v>1.94</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.350904</v>
+        <v>8.345159000000001</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.184</v>
@@ -4127,10 +4127,10 @@
         <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>1.0005506</v>
+        <v>0.99986225</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.2788529</v>
+        <v>0.27866104</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4322,10 +4322,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.72</v>
+        <v>26.75</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>22.082644</v>
+        <v>22.107437</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.449</v>
@@ -4345,10 +4345,10 @@
         <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6623118</v>
+        <v>1.6641783</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1109846</v>
+        <v>1.1122319</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.175</v>
@@ -4449,7 +4449,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.629664999999999</v>
+        <v>8.609643</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.818</v>
@@ -4461,10 +4461,10 @@
         <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.721394</v>
+        <v>-10.696517</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.5752718</v>
+        <v>0.573937</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -4493,10 +4493,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.082</v>
+        <v>0.083</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5.5368295</v>
+        <v>-5.585366</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>12.539</v>
@@ -4516,10 +4516,10 @@
         <v>1.911</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>32.43</v>
+        <v>32.714287</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.27164587</v>
+        <v>0.27402714</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>-1.12</v>
@@ -6257,7 +6257,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>54.93</v>
+        <v>54.89</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6280,7 +6280,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.272</v>
+        <v>0.273</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>1.8</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.92</v>
+        <v>107.67</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.971</v>
+        <v>0.976</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.4</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.544</v>
+        <v>0.546</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>102.95</v>
+        <v>102.89</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>83.93000000000001</v>
+        <v>83.92</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6599,7 +6599,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>58.56</v>
+        <v>58.63</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6622,7 +6622,7 @@
         <v>59</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.246</v>
+        <v>0.244</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>3.89</v>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>85.86</v>
+        <v>85.83</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.578</v>
+        <v>0.579</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>2.68</v>
@@ -6725,13 +6725,13 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.919893</v>
+        <v>28.926596</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.286427</v>
+        <v>37.29507</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.992582</v>
+        <v>21.99768</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>0.496</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.9</v>
+        <v>10.89</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.594</v>
+        <v>0.596</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6825,7 +6825,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>26.41</v>
+        <v>26.33</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.21</v>
+        <v>0.214</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>3.8</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>22.04</v>
+        <v>22.11</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6906,7 +6906,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.125</v>
+        <v>0.122</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -6941,7 +6941,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>13</v>
+        <v>13.01</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6964,7 +6964,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.391</v>
+        <v>0.39</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.42</v>
@@ -7011,16 +7011,16 @@
         <v>13</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>9.27308</v>
+        <v>9.24231</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>12.3</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>6.3</v>
+        <v>6</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.674</v>
+        <v>0.6679999999999999</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.08</v>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.54</v>
+        <v>14.53</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.314</v>
+        <v>0.315</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.72</v>
+        <v>26.75</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.141</v>
+        <v>0.14</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>2.5</v>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.46</v>
+        <v>6.45</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.064</v>
+        <v>1.067</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -7482,7 +7482,7 @@
         <v>2.5</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0.4320000000000001</v>
+        <v>0.419</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>5.72</v>
@@ -7707,10 +7707,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>37.14</v>
+        <v>37.113</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.37447</v>
+        <v>23.357447</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7722,7 +7722,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.153</v>
+        <v>-0.154</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.77</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.392</v>
+        <v>5.374</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7768,7 +7768,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.121</v>
+        <v>0.118</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.669</v>
@@ -7797,10 +7797,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.256</v>
+        <v>2.254</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.043478</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7887,10 +7887,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.736</v>
+        <v>10.73</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>32.78662</v>
+        <v>32.767513</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7904,7 +7904,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.158</v>
+        <v>-0.159</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>11.354</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.336</v>
+        <v>6.335</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7203016</v>
+        <v>3.7196367</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -8039,10 +8039,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.984</v>
+        <v>5.982</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>16.23157</v>
+        <v>16.225899</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.067</v>
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>6.022</v>
+        <v>6.029</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.769232</v>
+        <v>18.791315</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8098,7 +8098,7 @@
         <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.051</v>
+        <v>-0.05</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.413</v>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.941</v>
+        <v>1.94</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.021</v>
+        <v>-0.022</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.184</v>
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8190,7 +8190,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.011</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.449</v>
@@ -8269,7 +8269,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.082</v>
+        <v>0.083</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -8286,7 +8286,7 @@
         <v>-1.8681101</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.08400000000000001</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>12.539</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.511</v>
+        <v>5.509</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.952381</v>
+        <v>25.940477</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.059</v>
+        <v>-0.06</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8380,7 +8380,7 @@
         <v>5.721</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.694443</v>
+        <v>53.694168</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.131</v>
+        <v>5.147</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>71.09678</v>
+        <v>71.32258</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.141</v>
+        <v>0.145</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.66</v>
+        <v>11.648</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.343</v>
+        <v>-0.344</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.9</v>
+        <v>18.856</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8532,7 +8532,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.506</v>
+        <v>-0.507</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>14.473</v>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.399</v>
+        <v>2.401</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.279</v>
+        <v>-0.281</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.818</v>
@@ -10212,10 +10212,10 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.79</v>
+        <v>1277.97</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>1212.94</v>
+        <v>1212.93</v>
       </c>
       <c r="D2" s="13" t="n">
         <v>1068.57</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.48</v>
+        <v>1267.67</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.34</v>
+        <v>1262.54</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1255.02</v>
+        <v>1255.21</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1259.86</v>
+        <v>1260.04</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.45</v>
+        <v>1260.63</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.7</v>
+        <v>1245.88</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.38</v>
+        <v>1198.55</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1223.06</v>
+        <v>1223.23</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.42</v>
+        <v>1194.6</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1190.2</v>
+        <v>1190.38</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.44</v>
+        <v>1182.62</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1180.15</v>
+        <v>1180.34</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1198.99</v>
+        <v>1199.18</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.74</v>
+        <v>1162.94</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.36</v>
+        <v>1139.56</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1145.92</v>
+        <v>1146.12</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1151.01</v>
+        <v>1151.19</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1136.05</v>
+        <v>1136.24</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1141.91</v>
+        <v>1142.09</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1129.05</v>
+        <v>1129.25</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1130.83</v>
+        <v>1131.02</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1078.96</v>
+        <v>1079.17</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.31</v>
+        <v>1067.53</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.38</v>
+        <v>1085.61</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1082.04</v>
+        <v>1082.26</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1102.95</v>
+        <v>1103.18</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.59</v>
+        <v>1078.82</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105.28</v>
+        <v>1105.51</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1107.13</v>
+        <v>1107.37</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1104.09</v>
+        <v>1104.32</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.64</v>
+        <v>1089.88</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1052.93</v>
+        <v>1053.15</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1043.77</v>
+        <v>1044.01</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.49</v>
+        <v>1058.74</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.71</v>
+        <v>1091.97</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.62</v>
+        <v>1086.89</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1086.73</v>
+        <v>1087.01</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.65</v>
+        <v>1043.92</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1058.14</v>
+        <v>1058.42</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1062.04</v>
+        <v>1062.32</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.68</v>
+        <v>1090.96</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1078.08</v>
+        <v>1078.37</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1072.95</v>
+        <v>1073.24</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1068.88</v>
+        <v>1069.16</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1084.33</v>
+        <v>1084.62</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1081.99</v>
+        <v>1082.28</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.54</v>
+        <v>1050.82</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1052.09</v>
+        <v>1052.38</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1051.18</v>
+        <v>1051.46</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.55</v>
+        <v>1065.83</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1051.44</v>
+        <v>1051.72</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1053.36</v>
+        <v>1053.63</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1045.94</v>
+        <v>1046.21</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1058.22</v>
+        <v>1058.5</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1050.33</v>
+        <v>1050.6</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1062.95</v>
+        <v>1063.24</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1034.89</v>
+        <v>1035.18</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.7</v>
+        <v>1056.99</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1067.31</v>
+        <v>1067.69</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1067.31</v>
+        <v>1067.69</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.28%</t>
+          <t>-15.27%</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>140.7</v>
+        <v>140.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 14:29
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.67</v>
+        <v>107.54</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.015633563</v>
+        <v>-0.016821902</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.657</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.856</v>
+        <v>18.834</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.969288000000001</v>
+        <v>9.957250999999999</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -755,7 +755,7 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="9" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="Q3" s="9" t="n">
         <v>-0.507</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.4</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.022352197</v>
+        <v>-0.021307719</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -793,7 +793,7 @@
         <v>-0.52</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.648</v>
+        <v>11.66</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>12.022812</v>
+        <v>12.035657</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.423</v>
+        <v>-0.422</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.344</v>
+        <v>-0.343</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.89</v>
+        <v>102.97</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.017403364</v>
+        <v>0.018243858</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -854,16 +854,16 @@
         <v>-0.236</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.73</v>
+        <v>10.739</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.767513</v>
+        <v>32.794586</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.31639</v>
+        <v>17.330694</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.354</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="4" t="n">
-        <v>0.223</v>
+        <v>0.224</v>
       </c>
       <c r="Q5" s="9" t="n">
-        <v>-0.159</v>
+        <v>-0.158</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.23</v>
+        <v>37.09</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.75777745</v>
+        <v>0.39242342</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.073</v>
+        <v>-0.076</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.183</v>
+        <v>10.146</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.986843</v>
+        <v>48.80921</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.889138</v>
+        <v>15.831523</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.81</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.148</v>
+        <v>0.144</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.92</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.024102983</v>
+        <v>0.028313396</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,19 +969,19 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.063</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.335</v>
+        <v>6.361</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7196367</v>
+        <v>3.7349293</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.299592</v>
+        <v>10.341937</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -993,10 +993,10 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.224</v>
+        <v>0.229</v>
       </c>
       <c r="Q7" s="9" t="n">
-        <v>-0.024</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="8">
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.63</v>
+        <v>58.53</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.9450702</v>
+        <v>0.78339875</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1028,19 +1028,19 @@
         <v>35.09</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.152</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.029</v>
+        <v>6.019</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>6.847</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>18.791315</v>
+        <v>18.761219</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>17.842407</v>
+        <v>17.813831</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>8.413</v>
@@ -1052,10 +1052,10 @@
         <v>1.453</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0.3720000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="Q8" s="9" t="n">
-        <v>-0.05</v>
+        <v>-0.052</v>
       </c>
     </row>
     <row r="9">
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.83</v>
+        <v>85.92</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.014358264</v>
+        <v>0.015303688</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>118.46</v>
@@ -1090,16 +1090,16 @@
         <v>-0.275</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.982</v>
+        <v>5.988</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>10.94</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.225899</v>
+        <v>16.24102</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>11.560207</v>
+        <v>11.570982</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>11.435</v>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.33</v>
+        <v>19.37</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.010245773</v>
+        <v>-0.8192515999999999</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1146,19 +1146,19 @@
         <v>15.725</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.4</v>
+        <v>-0.399</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.721</v>
+        <v>5.733</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.694168</v>
+        <v>53.805557</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.56751</v>
+        <v>23.616402</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1170,10 +1170,10 @@
         <v>2.002</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.159</v>
+        <v>-0.157</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.171</v>
+        <v>-0.169</v>
       </c>
     </row>
     <row r="11">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.89</v>
+        <v>10.83</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.0201311</v>
+        <v>0.014044908</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1205,19 +1205,19 @@
         <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.243</v>
+        <v>-0.247</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.509</v>
+        <v>5.476</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.940477</v>
+        <v>25.785715</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.560381</v>
+        <v>12.485445</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1229,10 +1229,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.5660000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.06</v>
+        <v>-0.065</v>
       </c>
     </row>
     <row r="12">
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.33</v>
+        <v>26.34</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.4160386</v>
+        <v>-0.39713106</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>31.58</v>
@@ -1267,7 +1267,7 @@
         <v>-0.166</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.374</v>
+        <v>5.375</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>30.298</v>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>28.464865</v>
+        <v>28.470268</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>8.669</v>
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.11</v>
+        <v>22.02</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.016551752</v>
+        <v>0.012413814</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.028</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.147</v>
+        <v>5.126</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>71.32258</v>
+        <v>71.03225999999999</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.54579</v>
+        <v>29.425522</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.95</v>
+        <v>0.9420000000000001</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.145</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="14">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.55</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.012797107</v>
+        <v>0.014625303</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,19 +1451,19 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.453</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.254</v>
+        <v>2.258</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.043478</v>
+        <v>12.065218</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9633856</v>
+        <v>6.9759555</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.582</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.005</v>
+        <v>-0.004</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>-0.262</v>
+        <v>-0.261</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.53</v>
+        <v>14.49</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.58864295</v>
+        <v>0.3462617</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,10 +1510,10 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.295</v>
+        <v>-0.297</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.94</v>
+        <v>1.935</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.411</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.345159000000001</v>
+        <v>8.325049999999999</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.184</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="9" t="n">
-        <v>-0.163</v>
+        <v>-0.165</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.022</v>
+        <v>-0.024</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.72</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.4681448</v>
+        <v>0.23406851</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.133</v>
+        <v>-0.135</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.766</v>
+        <v>1.762</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.674</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>18.18048</v>
+        <v>18.138123</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.60555</v>
+        <v>16.566862</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.779</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.232</v>
+        <v>0.229</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.031</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="18">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.51</v>
+        <v>4.54</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>-0.039361691</v>
+        <v>-0.035143015</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1630,10 +1630,10 @@
         <v>4.46</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>-0.672</v>
+        <v>-0.669</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.161</v>
+        <v>1.167</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.908</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.560606</v>
+        <v>4.5808077</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.528</v>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="9" t="n">
-        <v>-0.591</v>
+        <v>-0.589</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>-0.581</v>
+        <v>-0.579</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.27</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.26642746</v>
+        <v>0.08881198</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,19 +1693,19 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.152</v>
+        <v>-0.153</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.921</v>
+        <v>0.919</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.816666</v>
+        <v>18.783333</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>12.19183</v>
+        <v>12.170233</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0.11</v>
+        <v>0.108</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.009000000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.75</v>
+        <v>26.71</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.014795121</v>
+        <v>0.013467357</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,10 +1752,10 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.183</v>
+        <v>-0.184</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.706</v>
+        <v>0.705</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>1.153</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>22.107437</v>
+        <v>22.078512</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.449</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.011</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>-0.011</v>
+        <v>-0.013</v>
       </c>
     </row>
     <row r="21">
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.83</v>
+        <v>11.76</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>-0.023121367</v>
+        <v>-0.02931458</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,10 +1813,10 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.43</v>
+        <v>-0.433</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.582</v>
+        <v>0.578</v>
       </c>
       <c r="J21" s="6" t="inlineStr">
         <is>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-14.6049385</v>
+        <v>-14.512345</v>
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
@@ -1847,10 +1847,10 @@
         </is>
       </c>
       <c r="P21" s="9" t="n">
-        <v>-0.326</v>
+        <v>-0.33</v>
       </c>
       <c r="Q21" s="9" t="n">
-        <v>-0.289</v>
+        <v>-0.294</v>
       </c>
     </row>
     <row r="22">
@@ -1931,10 +1931,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>-0.012919884</v>
+        <v>-0.023706822</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1943,10 +1943,10 @@
         <v>2.02</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>-0.537</v>
+        <v>-0.541</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.083</v>
+        <v>0.082</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0.578</v>
@@ -1957,7 +1957,7 @@
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>-5.585366</v>
+        <v>-5.5243907</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>12.539</v>
@@ -1969,10 +1969,10 @@
         <v>1.327</v>
       </c>
       <c r="P23" s="9" t="n">
-        <v>-0.488</v>
+        <v>-0.493</v>
       </c>
       <c r="Q23" s="9" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.094</v>
       </c>
     </row>
     <row r="24">
@@ -2205,22 +2205,22 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.67</v>
+        <v>107.54</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.015633563</v>
+        <v>-0.016821902</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.507</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-56.8</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.252</v>
+        <v>-0.253</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>-0.532</v>
@@ -2252,25 +2252,25 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.4</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.022352197</v>
+        <v>-0.021307719</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.344</v>
+        <v>-0.343</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.423</v>
+        <v>-0.422</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.138</v>
+        <v>-0.137</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.345</v>
+        <v>-0.344</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>-0.52</v>
@@ -2299,25 +2299,25 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.89</v>
+        <v>102.97</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.017403364</v>
+        <v>0.018243858</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.159</v>
+        <v>-0.158</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.223</v>
+        <v>0.224</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>34.8</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.064</v>
+        <v>-0.063</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.1</v>
+        <v>-0.099</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>-0.236</v>
@@ -2346,28 +2346,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.23</v>
+        <v>37.09</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.75777745</v>
+        <v>0.39242342</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.148</v>
+        <v>0.144</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>11.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.05</v>
+        <v>0.046</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.059</v>
+        <v>0.055</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.073</v>
+        <v>-0.076</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2393,28 +2393,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.92</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.024102983</v>
+        <v>0.028313396</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.02</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.224</v>
+        <v>0.229</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.5</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.014</v>
+        <v>0.018</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.063</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2440,28 +2440,28 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.63</v>
+        <v>58.53</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.9450702</v>
+        <v>0.78339875</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.052</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.3720000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>39.1</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.049</v>
+        <v>-0.05</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.001</v>
+        <v>-0.003</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.152</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>1.453</v>
@@ -2487,10 +2487,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.83</v>
+        <v>85.92</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.014358264</v>
+        <v>0.015303688</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.233</v>
@@ -2502,10 +2502,10 @@
         <v>-3.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.095</v>
+        <v>-0.094</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.149</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>-0.275</v>
@@ -2534,28 +2534,28 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.33</v>
+        <v>19.37</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.010245773</v>
+        <v>-0.8192515999999999</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-0.171</v>
+        <v>-0.169</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.159</v>
+        <v>-0.157</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-28.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.052</v>
+        <v>0.05400000000000001</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-0.211</v>
+        <v>-0.21</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-0.4</v>
+        <v>-0.399</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>2.002</v>
@@ -2581,28 +2581,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.89</v>
+        <v>10.83</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.0201311</v>
+        <v>0.014044908</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.065</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.5660000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.083</v>
+        <v>0.077</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.03</v>
+        <v>-0.036</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.243</v>
+        <v>-0.247</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.1</v>
@@ -2628,10 +2628,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.33</v>
+        <v>26.34</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.4160386</v>
+        <v>-0.39713106</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.118</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.11</v>
+        <v>22.02</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.016551752</v>
+        <v>0.012413814</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.145</v>
+        <v>0.14</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.95</v>
+        <v>0.9420000000000001</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.175</v>
+        <v>0.171</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.209</v>
+        <v>0.204</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.028</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2769,28 +2769,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.55</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.012797107</v>
+        <v>0.014625303</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.261</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.005</v>
+        <v>-0.004</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>8.6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.078</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.294</v>
+        <v>-0.293</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.453</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2816,28 +2816,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.53</v>
+        <v>14.49</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.58864295</v>
+        <v>0.3462617</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.022</v>
+        <v>-0.024</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.163</v>
+        <v>-0.165</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.3</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.055</v>
+        <v>0.052</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.106</v>
+        <v>-0.108</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.295</v>
+        <v>-0.297</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2863,28 +2863,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.72</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.4681448</v>
+        <v>0.23406851</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.031</v>
+        <v>0.029</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.232</v>
+        <v>0.229</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.04</v>
+        <v>0.038</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.027</v>
+        <v>0.025</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.133</v>
+        <v>-0.135</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2910,28 +2910,28 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.51</v>
+        <v>4.54</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.039361691</v>
+        <v>-0.035143015</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.581</v>
+        <v>-0.579</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.591</v>
+        <v>-0.589</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-32.1</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.374</v>
+        <v>-0.37</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.5589999999999999</v>
+        <v>-0.556</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.672</v>
+        <v>-0.669</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>1.993</v>
@@ -2957,28 +2957,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.27</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.26642746</v>
+        <v>0.08881198</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.11</v>
+        <v>0.108</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.2</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0</v>
+        <v>-0.002</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.152</v>
+        <v>-0.153</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -3004,28 +3004,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.75</v>
+        <v>26.71</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.014795121</v>
+        <v>0.013467357</v>
       </c>
       <c r="F20" s="5" t="n">
+        <v>-0.013</v>
+      </c>
+      <c r="G20" s="5" t="n">
         <v>-0.011</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>-0.009000000000000001</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.043</v>
+        <v>-0.044</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.005</v>
+        <v>-0.006</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.183</v>
+        <v>-0.184</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3051,28 +3051,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.83</v>
+        <v>11.76</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.023121367</v>
+        <v>-0.02931458</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.289</v>
+        <v>-0.294</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.326</v>
+        <v>-0.33</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>37.9</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.19</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.11</v>
+        <v>-0.115</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.43</v>
+        <v>-0.433</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3147,28 +3147,28 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.012919884</v>
+        <v>-0.023706822</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.094</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-0.488</v>
+        <v>-0.493</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>-53</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.052</v>
+        <v>-0.06</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.257</v>
+        <v>-0.264</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>-0.537</v>
+        <v>-0.541</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>1.327</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.67</v>
+        <v>107.54</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.856</v>
+        <v>18.834</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.969288000000001</v>
+        <v>9.957250999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.087437</v>
+        <v>2.0849166</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1509781</v>
+        <v>1.1495883</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.4</v>
+        <v>23.43</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.648</v>
+        <v>11.66</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12.022812</v>
+        <v>12.035657</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.338558</v>
+        <v>18.35815</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.9238299</v>
+        <v>1.9258853</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,16 +3511,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.89</v>
+        <v>102.97</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.73</v>
+        <v>10.739</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.767513</v>
+        <v>32.794586</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.31639</v>
+        <v>17.330694</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.354</v>
@@ -3532,10 +3532,10 @@
         <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-38.27753</v>
+        <v>-38.30915</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.5031972</v>
+        <v>1.504439</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3564,16 +3564,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.23</v>
+        <v>37.09</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.183</v>
+        <v>10.146</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.986843</v>
+        <v>48.80921</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.889138</v>
+        <v>15.831523</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.81</v>
@@ -3585,10 +3585,10 @@
         <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9576912</v>
+        <v>3.9433403</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.58061516</v>
+        <v>0.57850975</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>83.92</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.335</v>
+        <v>6.361</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7196367</v>
+        <v>3.7349293</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.299592</v>
+        <v>10.341937</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4567437</v>
+        <v>2.4668443</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5481296</v>
+        <v>1.5544944</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3670,16 +3670,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.63</v>
+        <v>58.53</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.029</v>
+        <v>6.019</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>18.791315</v>
+        <v>18.761219</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>17.842407</v>
+        <v>17.813831</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>8.413</v>
@@ -3691,10 +3691,10 @@
         <v>3.404</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.413465</v>
+        <v>16.387178</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.9971058</v>
+        <v>2.9923058</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>3.12</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.83</v>
+        <v>85.92</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.982</v>
+        <v>5.988</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.225899</v>
+        <v>16.24102</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>11.560207</v>
+        <v>11.570982</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>11.435</v>
@@ -3744,10 +3744,10 @@
         <v>3.739</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>5.9167986</v>
+        <v>5.922313</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.0446317</v>
+        <v>2.0465376</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>5.29</v>
@@ -3776,16 +3776,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.33</v>
+        <v>19.37</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.721</v>
+        <v>5.733</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.694168</v>
+        <v>53.805557</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.56751</v>
+        <v>23.616402</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.1326246</v>
+        <v>5.143272</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.4347835</v>
+        <v>4.4439836</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.89</v>
+        <v>10.83</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.509</v>
+        <v>5.476</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.940477</v>
+        <v>25.785715</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.560381</v>
+        <v>12.485445</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.39647</v>
+        <v>7.3523417</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.351314</v>
+        <v>2.3372858</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3882,10 +3882,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.33</v>
+        <v>26.34</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.374</v>
+        <v>5.375</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>28.464865</v>
+        <v>28.470268</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>8.669</v>
@@ -3905,10 +3905,10 @@
         <v>2.638</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.5225815</v>
+        <v>1.5228705</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>0.46788803</v>
+        <v>0.46797687</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>-2.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.11</v>
+        <v>22.02</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.147</v>
+        <v>5.126</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>71.32258</v>
+        <v>71.03225999999999</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.54579</v>
+        <v>29.425522</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>15.010183</v>
+        <v>14.949083</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.5369706</v>
+        <v>4.5185027</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -4051,16 +4051,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.55</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.254</v>
+        <v>2.258</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.043478</v>
+        <v>12.065218</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9633856</v>
+        <v>6.9759555</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.582</v>
@@ -4072,10 +4072,10 @@
         <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7361329</v>
+        <v>-1.7392668</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.4364705</v>
+        <v>0.4372584</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.53</v>
+        <v>14.49</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.94</v>
+        <v>1.935</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.345159000000001</v>
+        <v>8.325049999999999</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.184</v>
@@ -4127,10 +4127,10 @@
         <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.99986225</v>
+        <v>0.997453</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27866104</v>
+        <v>0.27798957</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4159,16 +4159,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.72</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.766</v>
+        <v>1.762</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>18.18048</v>
+        <v>18.138123</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.60555</v>
+        <v>16.566862</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.779</v>
@@ -4180,10 +4180,10 @@
         <v>3.071</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2716908</v>
+        <v>3.2640684</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.2391062</v>
+        <v>3.2315598</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4212,10 +4212,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.51</v>
+        <v>4.54</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.161</v>
+        <v>1.167</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.560606</v>
+        <v>4.5808077</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.528</v>
@@ -4237,10 +4237,10 @@
         <v>1.356</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.5351921</v>
+        <v>1.5419924</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.7348821</v>
+        <v>1.7425671</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4269,16 +4269,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.27</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.921</v>
+        <v>0.919</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.816666</v>
+        <v>18.783333</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>12.19183</v>
+        <v>12.170233</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4290,10 +4290,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.4452243</v>
+        <v>3.4391212</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6919532</v>
+        <v>0.6907274</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4322,10 +4322,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.75</v>
+        <v>26.71</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.706</v>
+        <v>0.705</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>22.107437</v>
+        <v>22.078512</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.449</v>
@@ -4345,10 +4345,10 @@
         <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6641783</v>
+        <v>1.6620008</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1122319</v>
+        <v>1.1107767</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4377,10 +4377,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.83</v>
+        <v>11.76</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.582</v>
+        <v>0.578</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4388,7 +4388,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-14.6049385</v>
+        <v>-14.512345</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
@@ -4406,10 +4406,10 @@
         </is>
       </c>
       <c r="K21" s="7" t="n">
-        <v>1.1144607</v>
+        <v>1.1073952</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.21891479</v>
+        <v>0.21752691</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-12.65</v>
@@ -4493,10 +4493,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.083</v>
+        <v>0.082</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -4504,7 +4504,7 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5.585366</v>
+        <v>-5.5243907</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>12.539</v>
@@ -4516,10 +4516,10 @@
         <v>1.911</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>32.714287</v>
+        <v>32.357143</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.27402714</v>
+        <v>0.2710356</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>-1.12</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.67</v>
+        <v>107.54</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.976</v>
+        <v>0.978</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.4</v>
+        <v>23.43</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.546</v>
+        <v>0.544</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>102.89</v>
+        <v>102.97</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6452,7 +6452,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.3779999999999999</v>
+        <v>0.377</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.24</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.23</v>
+        <v>37.09</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.146</v>
+        <v>0.15</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>83.92</v>
+        <v>84.26000000000001</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6566,7 +6566,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>0.126</v>
+        <v>0.121</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.32</v>
@@ -6599,7 +6599,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>58.63</v>
+        <v>58.53</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6622,7 +6622,7 @@
         <v>59</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.244</v>
+        <v>0.246</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>3.89</v>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>85.83</v>
+        <v>85.92</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.579</v>
+        <v>0.5770000000000001</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>2.68</v>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>19.33</v>
+        <v>19.37</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6725,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.926596</v>
+        <v>28.919893</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.29507</v>
+        <v>37.286427</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.99768</v>
+        <v>21.992582</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.496</v>
+        <v>0.493</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.89</v>
+        <v>10.83</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.596</v>
+        <v>0.604</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6825,7 +6825,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>26.33</v>
+        <v>26.34</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.214</v>
+        <v>0.213</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>3.8</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>22.11</v>
+        <v>22.02</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6906,7 +6906,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.122</v>
+        <v>0.126</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.55</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7020,7 +7020,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.6679999999999999</v>
+        <v>0.665</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.08</v>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.53</v>
+        <v>14.49</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.315</v>
+        <v>0.319</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>98.72</v>
+        <v>98.48999999999999</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7138,7 +7138,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.091</v>
+        <v>0.09300000000000001</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.53</v>
@@ -7171,7 +7171,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4.51</v>
+        <v>4.54</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -7194,7 +7194,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1.609</v>
+        <v>1.591</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>1.77</v>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.29</v>
+        <v>11.27</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7252,7 +7252,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.373</v>
+        <v>0.375</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.68</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.75</v>
+        <v>26.71</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.14</v>
+        <v>0.142</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>2.5</v>
@@ -7343,7 +7343,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>11.83</v>
+        <v>11.76</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7366,7 +7366,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>0.324</v>
+        <v>0.332</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>9.16</v>
@@ -7459,7 +7459,7 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2.29</v>
+        <v>2.27</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -7482,7 +7482,7 @@
         <v>2.5</v>
       </c>
       <c r="J23" s="4" t="n">
-        <v>0.419</v>
+        <v>0.4320000000000001</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>5.72</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.374</v>
+        <v>5.375</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7797,10 +7797,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.254</v>
+        <v>2.258</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.043478</v>
+        <v>12.065218</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.261</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>10.582</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.183</v>
+        <v>10.146</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48.986843</v>
+        <v>48.80921</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7858,7 +7858,7 @@
         <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>16.81</v>
@@ -7887,10 +7887,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.73</v>
+        <v>10.739</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>32.767513</v>
+        <v>32.794586</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7904,7 +7904,7 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.159</v>
+        <v>-0.158</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>11.354</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.335</v>
+        <v>6.361</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7196367</v>
+        <v>3.7349293</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7966,7 +7966,7 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.02</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>7.113</v>
@@ -7975,7 +7975,7 @@
         <v>5.9</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>69</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -7995,10 +7995,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.766</v>
+        <v>1.762</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>18.18048</v>
+        <v>18.138123</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.041</v>
@@ -8010,7 +8010,7 @@
         <v>0.19214001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.031</v>
+        <v>0.029</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>8.779</v>
@@ -8039,10 +8039,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.982</v>
+        <v>5.988</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>16.225899</v>
+        <v>16.24102</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.067</v>
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>6.029</v>
+        <v>6.019</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.791315</v>
+        <v>18.761219</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8098,7 +8098,7 @@
         <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.052</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.413</v>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.94</v>
+        <v>1.935</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.022</v>
+        <v>-0.024</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.184</v>
@@ -8153,7 +8153,7 @@
         <v>10.9</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>51.4</v>
+        <v>48.6</v>
       </c>
     </row>
     <row r="15">
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.706</v>
+        <v>0.705</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8190,7 +8190,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.013</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.449</v>
@@ -8219,7 +8219,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.582</v>
+        <v>0.578</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8236,7 +8236,7 @@
         <v>-0.5564</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.289</v>
+        <v>-0.294</v>
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
@@ -8269,7 +8269,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.083</v>
+        <v>0.082</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -8286,7 +8286,7 @@
         <v>-1.8681101</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-0.08400000000000001</v>
+        <v>-0.094</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>12.539</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.509</v>
+        <v>5.476</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.940477</v>
+        <v>25.785715</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.065</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8377,10 +8377,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.721</v>
+        <v>5.733</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.694168</v>
+        <v>53.805557</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8392,7 +8392,7 @@
         <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.171</v>
+        <v>-0.169</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>10.962</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.147</v>
+        <v>5.126</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>71.32258</v>
+        <v>71.03225999999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.145</v>
+        <v>0.14</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.648</v>
+        <v>11.66</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.344</v>
+        <v>-0.343</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.856</v>
+        <v>18.834</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8561,7 +8561,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.161</v>
+        <v>1.167</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.581</v>
+        <v>-0.579</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>-7.528</v>
@@ -8627,10 +8627,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.921</v>
+        <v>0.919</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.816666</v>
+        <v>18.783333</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8642,7 +8642,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.006999999999999999</v>
+        <v>-0.009000000000000001</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.97</v>
+        <v>1277.85</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1212.93</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.67</v>
+        <v>1267.54</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.54</v>
+        <v>1262.41</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1255.21</v>
+        <v>1255.09</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1260.04</v>
+        <v>1259.93</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.63</v>
+        <v>1260.51</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.88</v>
+        <v>1245.77</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.55</v>
+        <v>1198.47</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1223.23</v>
+        <v>1223.15</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.6</v>
+        <v>1194.5</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1190.38</v>
+        <v>1190.29</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.62</v>
+        <v>1182.54</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1180.34</v>
+        <v>1180.26</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1199.18</v>
+        <v>1199.1</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.94</v>
+        <v>1162.85</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.56</v>
+        <v>1139.47</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1146.12</v>
+        <v>1146.03</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1151.19</v>
+        <v>1151.11</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1136.24</v>
+        <v>1136.16</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1142.09</v>
+        <v>1142.02</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1129.25</v>
+        <v>1129.17</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1131.02</v>
+        <v>1130.96</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1079.17</v>
+        <v>1079.06</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.53</v>
+        <v>1067.42</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.61</v>
+        <v>1085.51</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1082.26</v>
+        <v>1082.17</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1103.18</v>
+        <v>1103.09</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.82</v>
+        <v>1078.72</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105.51</v>
+        <v>1105.39</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1107.37</v>
+        <v>1107.24</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1104.32</v>
+        <v>1104.22</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.88</v>
+        <v>1089.79</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1053.15</v>
+        <v>1053.07</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1044.01</v>
+        <v>1043.91</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.74</v>
+        <v>1058.63</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.97</v>
+        <v>1091.84</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.89</v>
+        <v>1086.76</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1087.01</v>
+        <v>1086.86</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.92</v>
+        <v>1043.78</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1058.42</v>
+        <v>1058.26</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1062.32</v>
+        <v>1062.14</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.96</v>
+        <v>1090.76</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1078.37</v>
+        <v>1078.18</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1073.24</v>
+        <v>1073.05</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1069.16</v>
+        <v>1068.95</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1084.62</v>
+        <v>1084.39</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1082.28</v>
+        <v>1082.05</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.82</v>
+        <v>1050.6</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1052.38</v>
+        <v>1052.16</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1051.46</v>
+        <v>1051.25</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.83</v>
+        <v>1065.61</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1051.72</v>
+        <v>1051.5</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1053.63</v>
+        <v>1053.43</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1046.21</v>
+        <v>1046.01</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1058.5</v>
+        <v>1058.29</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1050.6</v>
+        <v>1050.4</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1063.24</v>
+        <v>1063.03</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1035.18</v>
+        <v>1034.97</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.99</v>
+        <v>1056.76</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1067.69</v>
+        <v>1066.28</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1067.69</v>
+        <v>1066.28</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.27%</t>
+          <t>-15.37%</t>
         </is>
       </c>
     </row>
@@ -11200,7 +11200,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>140.6</v>
+        <v>140.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 14:33
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.89</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.01648147</v>
+        <v>0.017222228</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.221</v>
+        <v>-0.22</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>37.113</v>
+        <v>37.14</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.818</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.357447</v>
+        <v>23.37447</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>14.607962</v>
+        <v>14.618607</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.77</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="4" t="n">
-        <v>0.35</v>
+        <v>0.351</v>
       </c>
       <c r="Q2" s="9" t="n">
-        <v>-0.154</v>
+        <v>-0.153</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.54</v>
+        <v>107.47</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>-0.016821902</v>
+        <v>-0.017451072</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.657</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.834</v>
+        <v>18.822</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>30.856</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.957250999999999</v>
+        <v>9.95088</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>14.473</v>
@@ -758,7 +758,7 @@
         <v>-0.5639999999999999</v>
       </c>
       <c r="Q3" s="9" t="n">
-        <v>-0.507</v>
+        <v>-0.508</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.36</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>-0.021307719</v>
+        <v>-0.02402335</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>21.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.52</v>
+        <v>-0.521</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>11.66</v>
+        <v>11.628</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>12.574</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>12.035657</v>
+        <v>12.002261</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>46.079</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="9" t="n">
-        <v>-0.422</v>
+        <v>-0.423</v>
       </c>
       <c r="Q4" s="9" t="n">
-        <v>-0.343</v>
+        <v>-0.345</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.97</v>
+        <v>102.96</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.018243858</v>
+        <v>0.01809554</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -854,16 +854,16 @@
         <v>-0.236</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.739</v>
+        <v>10.737</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.864</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.794586</v>
+        <v>32.789806</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>17.330694</v>
+        <v>17.328169</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.354</v>
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.09</v>
+        <v>37.15</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>0.39242342</v>
+        <v>0.5412741</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.076</v>
+        <v>-0.075</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.146</v>
+        <v>10.161</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.58</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>48.80921</v>
+        <v>48.88158</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.831523</v>
+        <v>15.854997</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.81</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="4" t="n">
-        <v>0.144</v>
+        <v>0.146</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.26000000000001</v>
+        <v>84.28</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>0.028313396</v>
+        <v>0.028618515</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.063</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.361</v>
+        <v>6.363</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.542999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7349293</v>
+        <v>3.7360375</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.341937</v>
+        <v>10.345005</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.113</v>
@@ -993,7 +993,7 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="4" t="n">
-        <v>0.229</v>
+        <v>0.23</v>
       </c>
       <c r="Q7" s="9" t="n">
         <v>-0.02</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.53</v>
+        <v>58.52</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>0.78339875</v>
+        <v>0.75757337</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1031,16 +1031,16 @@
         <v>-0.152</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.019</v>
+        <v>6.017</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>6.847</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>18.761219</v>
+        <v>18.75641</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>17.813831</v>
+        <v>17.809267</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>8.413</v>
@@ -1052,7 +1052,7 @@
         <v>1.453</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>0.37</v>
+        <v>0.369</v>
       </c>
       <c r="Q8" s="9" t="n">
         <v>-0.052</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.92</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.015303688</v>
+        <v>0.014240063</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>118.46</v>
@@ -1090,16 +1090,16 @@
         <v>-0.275</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.988</v>
+        <v>5.982</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>10.94</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.24102</v>
+        <v>16.224007</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>11.570982</v>
+        <v>11.55886</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>11.435</v>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.37</v>
+        <v>19.34</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>-0.8192515999999999</v>
+        <v>-0.9728650000000001</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>32.22</v>
@@ -1146,19 +1146,19 @@
         <v>15.725</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.399</v>
+        <v>-0.4</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.733</v>
+        <v>5.724</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>5.563</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>53.805557</v>
+        <v>53.72222</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>23.616402</v>
+        <v>23.579823</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>10.962</v>
@@ -1170,10 +1170,10 @@
         <v>2.002</v>
       </c>
       <c r="P10" s="9" t="n">
-        <v>-0.157</v>
+        <v>-0.159</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>-0.169</v>
+        <v>-0.171</v>
       </c>
     </row>
     <row r="11">
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.83</v>
+        <v>10.85</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.014044908</v>
+        <v>0.015449435</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1205,19 +1205,19 @@
         <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.247</v>
+        <v>-0.245</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.476</v>
+        <v>5.484</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.993</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.785715</v>
+        <v>25.82143</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.485445</v>
+        <v>12.502738</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.175</v>
@@ -1229,10 +1229,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>0.556</v>
+        <v>0.5589999999999999</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>-0.065</v>
+        <v>-0.064</v>
       </c>
     </row>
     <row r="12">
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.34</v>
+        <v>26.36</v>
       </c>
       <c r="E12" s="9" t="n">
-        <v>-0.39713106</v>
+        <v>-0.283664</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>31.58</v>
@@ -1264,10 +1264,10 @@
         <v>17.86</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.165</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.375</v>
+        <v>5.381</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>30.298</v>
@@ -1278,7 +1278,7 @@
         </is>
       </c>
       <c r="L12" s="7" t="n">
-        <v>28.470268</v>
+        <v>28.502703</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>8.669</v>
@@ -1290,10 +1290,10 @@
         <v>1.977</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>-0.064</v>
+        <v>-0.063</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>0.118</v>
+        <v>0.119</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.02</v>
+        <v>21.96</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.012413814</v>
+        <v>0.96551305</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.03</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.126</v>
+        <v>5.112</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>71.03225999999999</v>
+        <v>70.83871000000001</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.425522</v>
+        <v>29.34534</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="4" t="n">
-        <v>0.9420000000000001</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="Q13" s="4" t="n">
-        <v>0.14</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.01</v>
+        <v>13.02</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>-0.3065131</v>
+        <v>-0.26819807</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1393,7 +1393,7 @@
         <v>-0.299</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.401</v>
+        <v>2.402</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.976</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>12.073797</v>
+        <v>12.078438</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.776</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="9" t="n">
-        <v>-0.033</v>
+        <v>-0.032</v>
       </c>
       <c r="Q14" s="9" t="n">
-        <v>-0.135</v>
+        <v>-0.134</v>
       </c>
     </row>
     <row r="15">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.55</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.014625303</v>
+        <v>0.016468464</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,19 +1451,19 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.453</v>
+        <v>-0.452</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.258</v>
+        <v>2.262</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.762</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.065218</v>
+        <v>12.086956</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9759555</v>
+        <v>6.9885244</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.582</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>-0.004</v>
+        <v>-0.002</v>
       </c>
       <c r="Q15" s="9" t="n">
-        <v>-0.261</v>
+        <v>-0.26</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.49</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.3462617</v>
+        <v>0.3116349</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1513,7 +1513,7 @@
         <v>-0.297</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.935</v>
+        <v>1.934</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.411</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.325049999999999</v>
+        <v>8.322177999999999</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.184</v>
@@ -1539,7 +1539,7 @@
         <v>-0.165</v>
       </c>
       <c r="Q16" s="9" t="n">
-        <v>-0.024</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.48999999999999</v>
+        <v>98.41</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.23406851</v>
+        <v>0.15265776</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.135</v>
+        <v>-0.136</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.762</v>
+        <v>1.76</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.674</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>18.138123</v>
+        <v>18.12339</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.566862</v>
+        <v>16.553406</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.779</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="4" t="n">
-        <v>0.229</v>
+        <v>0.228</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="18">
@@ -1621,7 +1621,7 @@
         <v>4.54</v>
       </c>
       <c r="E18" s="9" t="n">
-        <v>-0.035143015</v>
+        <v>-0.032978668</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1633,7 +1633,7 @@
         <v>-0.669</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.167</v>
+        <v>1.169</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.908</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.5808077</v>
+        <v>4.590909</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.528</v>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="9" t="n">
-        <v>-0.589</v>
+        <v>-0.588</v>
       </c>
       <c r="Q18" s="9" t="n">
-        <v>-0.579</v>
+        <v>-0.578</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.27</v>
+        <v>11.28</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>0.08881198</v>
+        <v>0.17761548</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1696,16 +1696,16 @@
         <v>-0.153</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.919</v>
+        <v>0.92</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.783333</v>
+        <v>18.8</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>12.170233</v>
+        <v>12.181031</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="4" t="n">
-        <v>0.108</v>
+        <v>0.109</v>
       </c>
       <c r="Q19" s="9" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.008</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.71</v>
+        <v>26.74</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.013467357</v>
+        <v>0.014415749</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,10 +1752,10 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.184</v>
+        <v>-0.183</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>1.153</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>22.078512</v>
+        <v>22.099173</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.449</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>-0.011</v>
+        <v>-0.01</v>
       </c>
       <c r="Q20" s="9" t="n">
-        <v>-0.013</v>
+        <v>-0.012</v>
       </c>
     </row>
     <row r="21">
@@ -1870,10 +1870,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.45</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.7692337</v>
+        <v>-0.46154168</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1882,7 +1882,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.352</v>
+        <v>-0.35</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.175</v>
@@ -1896,7 +1896,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>8.609643</v>
+        <v>8.636339</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.818</v>
@@ -1908,10 +1908,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="9" t="n">
-        <v>-0.295</v>
+        <v>-0.293</v>
       </c>
       <c r="Q22" s="9" t="n">
-        <v>-0.281</v>
+        <v>-0.279</v>
       </c>
     </row>
     <row r="23">
@@ -2158,28 +2158,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.89</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.01648147</v>
+        <v>0.017222228</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.153</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.35</v>
+        <v>0.351</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>53.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.035</v>
+        <v>-0.034</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.015</v>
+        <v>-0.014</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.221</v>
+        <v>-0.22</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2205,13 +2205,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.54</v>
+        <v>107.47</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.016821902</v>
+        <v>-0.017451072</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.507</v>
+        <v>-0.508</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>-0.5639999999999999</v>
@@ -2223,7 +2223,7 @@
         <v>-0.253</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.532</v>
+        <v>-0.5329999999999999</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>-0.657</v>
@@ -2252,28 +2252,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.36</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.021307719</v>
+        <v>-0.02402335</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.343</v>
+        <v>-0.345</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.422</v>
+        <v>-0.423</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-36</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.137</v>
+        <v>-0.14</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.344</v>
+        <v>-0.346</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.52</v>
+        <v>-0.521</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2299,10 +2299,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.97</v>
+        <v>102.96</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.018243858</v>
+        <v>0.01809554</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.158</v>
@@ -2346,28 +2346,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.09</v>
+        <v>37.15</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.39242342</v>
+        <v>0.5412741</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.144</v>
+        <v>0.146</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>11.9</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.046</v>
+        <v>0.048</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.055</v>
+        <v>0.05599999999999999</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.076</v>
+        <v>-0.075</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2393,16 +2393,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.26000000000001</v>
+        <v>84.28</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.028313396</v>
+        <v>0.028618515</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.02</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.229</v>
+        <v>0.23</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.5</v>
@@ -2440,16 +2440,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.53</v>
+        <v>58.52</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.78339875</v>
+        <v>0.75757337</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.052</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.37</v>
+        <v>0.369</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>39.1</v>
@@ -2487,10 +2487,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.92</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.015303688</v>
+        <v>0.014240063</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.233</v>
@@ -2502,10 +2502,10 @@
         <v>-3.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.15</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>-0.275</v>
@@ -2534,28 +2534,28 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.37</v>
+        <v>19.34</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.8192515999999999</v>
+        <v>-0.9728650000000001</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.171</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.157</v>
+        <v>-0.159</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-28.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.05400000000000001</v>
+        <v>0.052</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-0.21</v>
+        <v>-0.211</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-0.399</v>
+        <v>-0.4</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>2.002</v>
@@ -2581,28 +2581,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.83</v>
+        <v>10.85</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.014044908</v>
+        <v>0.015449435</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.064</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.556</v>
+        <v>0.5589999999999999</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>27.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.077</v>
+        <v>0.079</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.036</v>
+        <v>-0.034</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.247</v>
+        <v>-0.245</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.1</v>
@@ -2628,28 +2628,28 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.34</v>
+        <v>26.36</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.39713106</v>
+        <v>-0.283664</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.118</v>
+        <v>0.119</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.064</v>
+        <v>-0.063</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>-22.7</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.123</v>
+        <v>0.124</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.165</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>1.977</v>
@@ -2675,28 +2675,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.02</v>
+        <v>21.96</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.012413814</v>
+        <v>0.96551305</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.14</v>
+        <v>0.137</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.9420000000000001</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>51.2</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.171</v>
+        <v>0.167</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.204</v>
+        <v>0.201</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.028</v>
+        <v>-0.03</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2722,25 +2722,25 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.01</v>
+        <v>13.02</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.3065131</v>
+        <v>-0.26819807</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.135</v>
+        <v>-0.134</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.033</v>
+        <v>-0.032</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>13.4</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.055</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.158</v>
+        <v>-0.157</v>
       </c>
       <c r="K14" s="5" t="n">
         <v>-0.299</v>
@@ -2769,28 +2769,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.55</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.014625303</v>
+        <v>0.016468464</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.261</v>
+        <v>-0.26</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>-0.004</v>
+        <v>-0.002</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>8.6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.078</v>
+        <v>-0.076</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.293</v>
+        <v>-0.292</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.453</v>
+        <v>-0.452</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2816,13 +2816,13 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.49</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.3462617</v>
+        <v>0.3116349</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.025</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>-0.165</v>
@@ -2831,10 +2831,10 @@
         <v>-19.3</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.052</v>
+        <v>0.051</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.108</v>
+        <v>-0.109</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>-0.297</v>
@@ -2863,28 +2863,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.48999999999999</v>
+        <v>98.41</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.23406851</v>
+        <v>0.15265776</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.229</v>
+        <v>0.228</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.038</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.135</v>
+        <v>-0.136</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2913,13 +2913,13 @@
         <v>4.54</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.035143015</v>
+        <v>-0.032978668</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.579</v>
+        <v>-0.578</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.589</v>
+        <v>-0.588</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-32.1</v>
@@ -2957,25 +2957,25 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.27</v>
+        <v>11.28</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.08881198</v>
+        <v>0.17761548</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.108</v>
+        <v>0.109</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.2</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.002</v>
+        <v>-0.001</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.006</v>
+        <v>0.006999999999999999</v>
       </c>
       <c r="K19" s="5" t="n">
         <v>-0.153</v>
@@ -3004,28 +3004,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.71</v>
+        <v>26.74</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.013467357</v>
+        <v>0.014415749</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.013</v>
+        <v>-0.012</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.01</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.3</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.044</v>
+        <v>-0.043</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.006</v>
+        <v>-0.005</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.184</v>
+        <v>-0.183</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3100,28 +3100,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.45</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.7692337</v>
+        <v>-0.46154168</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.281</v>
+        <v>-0.279</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.295</v>
+        <v>-0.293</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.23</v>
+        <v>-0.228</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.247</v>
+        <v>-0.244</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.352</v>
+        <v>-0.35</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3348,16 +3348,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>54.89</v>
+        <v>54.93</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>37.113</v>
+        <v>37.14</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.357447</v>
+        <v>23.37447</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>14.607962</v>
+        <v>14.618607</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.77</v>
@@ -3369,10 +3369,10 @@
         <v>3.75</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.297962</v>
+        <v>23.314941</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.8511193</v>
+        <v>2.853197</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3401,10 +3401,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>107.54</v>
+        <v>107.47</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.834</v>
+        <v>18.822</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3412,7 +3412,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.957250999999999</v>
+        <v>9.95088</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>14.473</v>
@@ -3424,10 +3424,10 @@
         <v>1.883</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0849166</v>
+        <v>2.0835826</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1495883</v>
+        <v>1.148853</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3456,10 +3456,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.36</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>11.66</v>
+        <v>11.628</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3467,7 +3467,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>12.035657</v>
+        <v>12.002261</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>46.079</v>
@@ -3479,10 +3479,10 @@
         <v>2.077</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>18.35815</v>
+        <v>18.30721</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.9258853</v>
+        <v>1.9205415</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,16 +3511,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>102.97</v>
+        <v>102.96</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.739</v>
+        <v>10.737</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.794586</v>
+        <v>32.789806</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>17.330694</v>
+        <v>17.328169</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.354</v>
@@ -3532,10 +3532,10 @@
         <v>2.783</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-38.30915</v>
+        <v>-38.30357</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.504439</v>
+        <v>1.5042199</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3564,16 +3564,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.09</v>
+        <v>37.15</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.146</v>
+        <v>10.161</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>48.80921</v>
+        <v>48.88158</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.831523</v>
+        <v>15.854997</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.81</v>
@@ -3585,10 +3585,10 @@
         <v>2.257</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9433403</v>
+        <v>3.949187</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.57850975</v>
+        <v>0.5793675</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3617,16 +3617,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>84.26000000000001</v>
+        <v>84.28</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.361</v>
+        <v>6.363</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7349293</v>
+        <v>3.7360375</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.341937</v>
+        <v>10.345005</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.113</v>
@@ -3638,10 +3638,10 @@
         <v>2.088</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4668443</v>
+        <v>2.4675763</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5544944</v>
+        <v>1.5549556</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3670,16 +3670,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>58.53</v>
+        <v>58.52</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.019</v>
+        <v>6.017</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>18.761219</v>
+        <v>18.75641</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>17.813831</v>
+        <v>17.809267</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>8.413</v>
@@ -3691,10 +3691,10 @@
         <v>3.404</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.387178</v>
+        <v>16.382978</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.9923058</v>
+        <v>2.991539</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>3.12</v>
@@ -3723,16 +3723,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>85.92</v>
+        <v>85.83</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.988</v>
+        <v>5.982</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.24102</v>
+        <v>16.224007</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>11.570982</v>
+        <v>11.55886</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>11.435</v>
@@ -3744,10 +3744,10 @@
         <v>3.739</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>5.922313</v>
+        <v>5.916109</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.0465376</v>
+        <v>2.0443935</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>5.29</v>
@@ -3776,16 +3776,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>19.37</v>
+        <v>19.34</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.733</v>
+        <v>5.724</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>53.805557</v>
+        <v>53.72222</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>23.616402</v>
+        <v>23.579823</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>10.962</v>
@@ -3797,10 +3797,10 @@
         <v>4.312</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>5.143272</v>
+        <v>5.1353064</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>4.4439836</v>
+        <v>4.437101</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>0.36</v>
@@ -3829,16 +3829,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.83</v>
+        <v>10.85</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.476</v>
+        <v>5.484</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.785715</v>
+        <v>25.82143</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.485445</v>
+        <v>12.502738</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.175</v>
@@ -3850,10 +3850,10 @@
         <v>2.131</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.3523417</v>
+        <v>7.3625255</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.3372858</v>
+        <v>2.3405232</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3882,10 +3882,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>26.34</v>
+        <v>26.36</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.375</v>
+        <v>5.381</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>28.470268</v>
+        <v>28.502703</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>8.669</v>
@@ -3905,10 +3905,10 @@
         <v>2.638</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>1.5228705</v>
+        <v>1.5246054</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>0.46797687</v>
+        <v>0.46851</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>-2.42</v>
@@ -3937,16 +3937,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>22.02</v>
+        <v>21.96</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.126</v>
+        <v>5.112</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>71.03225999999999</v>
+        <v>70.83871000000001</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.425522</v>
+        <v>29.34534</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3964,10 +3964,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.949083</v>
+        <v>14.908349</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.5185027</v>
+        <v>4.5061903</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3996,10 +3996,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>13.01</v>
+        <v>13.02</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.401</v>
+        <v>2.402</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4007,7 +4007,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>12.073797</v>
+        <v>12.078438</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.776</v>
@@ -4019,10 +4019,10 @@
         <v>2.38</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7781336</v>
+        <v>2.7792013</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.95608014</v>
+        <v>0.9564476</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4051,16 +4051,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.55</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.258</v>
+        <v>2.262</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.065218</v>
+        <v>12.086956</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9759555</v>
+        <v>6.9885244</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.582</v>
@@ -4072,10 +4072,10 @@
         <v>2.472</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7392668</v>
+        <v>-1.7424005</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.4372584</v>
+        <v>0.43804622</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4104,10 +4104,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.49</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.935</v>
+        <v>1.934</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.325049999999999</v>
+        <v>8.322177999999999</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.184</v>
@@ -4127,10 +4127,10 @@
         <v>1.783</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.997453</v>
+        <v>0.99710876</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27798957</v>
+        <v>0.27789366</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4159,16 +4159,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>98.48999999999999</v>
+        <v>98.41</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.762</v>
+        <v>1.76</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>18.138123</v>
+        <v>18.12339</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.566862</v>
+        <v>16.553406</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.779</v>
@@ -4180,10 +4180,10 @@
         <v>3.071</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2640684</v>
+        <v>3.2614172</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.2315598</v>
+        <v>3.228935</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4215,7 +4215,7 @@
         <v>4.54</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.167</v>
+        <v>1.169</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4223,7 +4223,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.5808077</v>
+        <v>4.590909</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.528</v>
@@ -4237,10 +4237,10 @@
         <v>1.356</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.5419924</v>
+        <v>1.5453928</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.7425671</v>
+        <v>1.7464095</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4269,16 +4269,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.27</v>
+        <v>11.28</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.919</v>
+        <v>0.92</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.783333</v>
+        <v>18.8</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>12.170233</v>
+        <v>12.181031</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4290,10 +4290,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.4391212</v>
+        <v>3.4421728</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6907274</v>
+        <v>0.69134027</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4322,10 +4322,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.71</v>
+        <v>26.74</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4333,7 +4333,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>22.078512</v>
+        <v>22.099173</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.449</v>
@@ -4345,10 +4345,10 @@
         <v>1.816</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6620008</v>
+        <v>1.6635561</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.1107767</v>
+        <v>1.1118162</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.45</v>
+        <v>6.47</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.175</v>
@@ -4449,7 +4449,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>8.609643</v>
+        <v>8.636339</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.818</v>
@@ -4461,10 +4461,10 @@
         <v>1.666</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-10.696517</v>
+        <v>-10.729685</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.573937</v>
+        <v>0.5757166</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -6257,7 +6257,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>54.89</v>
+        <v>54.93</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6280,7 +6280,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.273</v>
+        <v>0.272</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>1.8</v>
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>107.54</v>
+        <v>107.47</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6336,7 +6336,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.978</v>
+        <v>0.98</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>1.72</v>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.43</v>
+        <v>23.36</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6394,7 +6394,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.544</v>
+        <v>0.5489999999999999</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>1.74</v>
@@ -6429,7 +6429,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>102.97</v>
+        <v>102.96</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6452,7 +6452,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>0.377</v>
+        <v>0.3779999999999999</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.24</v>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.09</v>
+        <v>37.15</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>0.15</v>
+        <v>0.148</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.2</v>
@@ -6543,7 +6543,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>84.26000000000001</v>
+        <v>84.28</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6599,7 +6599,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>58.53</v>
+        <v>58.52</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6655,7 +6655,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>85.92</v>
+        <v>85.83</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6678,7 +6678,7 @@
         <v>110</v>
       </c>
       <c r="J9" s="4" t="n">
-        <v>0.5770000000000001</v>
+        <v>0.579</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>2.68</v>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>19.37</v>
+        <v>19.34</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6725,16 +6725,16 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.919893</v>
+        <v>28.913189</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.286427</v>
+        <v>37.277786</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>21.992582</v>
+        <v>21.987484</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>0.493</v>
+        <v>0.495</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>4.19</v>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.83</v>
+        <v>10.85</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>0.604</v>
+        <v>0.601</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.92</v>
@@ -6825,7 +6825,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>26.34</v>
+        <v>26.36</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>0.213</v>
+        <v>0.212</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>3.8</v>
@@ -6883,7 +6883,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>22.02</v>
+        <v>21.96</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6906,7 +6906,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.126</v>
+        <v>0.129</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.71</v>
@@ -6941,7 +6941,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>13.01</v>
+        <v>13.02</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6964,7 +6964,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>0.39</v>
+        <v>0.389</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.42</v>
@@ -6997,7 +6997,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.55</v>
+        <v>5.56</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7020,7 +7020,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.665</v>
+        <v>0.662</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.08</v>
@@ -7055,7 +7055,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.49</v>
+        <v>14.48</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7078,7 +7078,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.319</v>
+        <v>0.32</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.18</v>
@@ -7113,7 +7113,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>98.48999999999999</v>
+        <v>98.41</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7138,7 +7138,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.09300000000000001</v>
+        <v>0.094</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.53</v>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.27</v>
+        <v>11.28</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7252,7 +7252,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.375</v>
+        <v>0.374</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.68</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.71</v>
+        <v>26.74</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7310,7 +7310,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="4" t="n">
-        <v>0.142</v>
+        <v>0.141</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>2.5</v>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.45</v>
+        <v>6.47</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="4" t="n">
-        <v>1.067</v>
+        <v>1.061</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>13.9</v>
@@ -7707,10 +7707,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>37.113</v>
+        <v>37.14</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.357447</v>
+        <v>23.37447</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7722,7 +7722,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.154</v>
+        <v>-0.153</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.77</v>
@@ -7751,7 +7751,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.375</v>
+        <v>5.381</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7768,7 +7768,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.118</v>
+        <v>0.119</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.669</v>
@@ -7797,10 +7797,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.258</v>
+        <v>2.262</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.065218</v>
+        <v>12.086956</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.261</v>
+        <v>-0.26</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>10.582</v>
@@ -7843,10 +7843,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10.146</v>
+        <v>10.161</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>48.80921</v>
+        <v>48.88158</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7858,7 +7858,7 @@
         <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>16.81</v>
@@ -7887,10 +7887,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.739</v>
+        <v>10.737</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>32.794586</v>
+        <v>32.789806</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7951,10 +7951,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.361</v>
+        <v>6.363</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7349293</v>
+        <v>3.7360375</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7995,10 +7995,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.762</v>
+        <v>1.76</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>18.138123</v>
+        <v>18.12339</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.041</v>
@@ -8010,7 +8010,7 @@
         <v>0.19214001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>8.779</v>
@@ -8039,10 +8039,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.988</v>
+        <v>5.982</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>16.24102</v>
+        <v>16.224007</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.067</v>
@@ -8083,10 +8083,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>6.019</v>
+        <v>6.017</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.761219</v>
+        <v>18.75641</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.032</v>
@@ -8127,7 +8127,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.935</v>
+        <v>1.934</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8144,7 +8144,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.025</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.184</v>
@@ -8173,7 +8173,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.705</v>
+        <v>0.706</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8190,7 +8190,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.013</v>
+        <v>-0.012</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.449</v>
@@ -8333,10 +8333,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.476</v>
+        <v>5.484</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.785715</v>
+        <v>25.82143</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8348,7 +8348,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.064</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.175</v>
@@ -8377,10 +8377,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.733</v>
+        <v>5.724</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>53.805557</v>
+        <v>53.72222</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8392,7 +8392,7 @@
         <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.171</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>10.962</v>
@@ -8421,10 +8421,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.126</v>
+        <v>5.112</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>71.03225999999999</v>
+        <v>70.83871000000001</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8436,7 +8436,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.14</v>
+        <v>0.137</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8469,7 +8469,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>11.66</v>
+        <v>11.628</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.343</v>
+        <v>-0.345</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>46.079</v>
@@ -8515,7 +8515,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.834</v>
+        <v>18.822</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8532,7 +8532,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.507</v>
+        <v>-0.508</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>14.473</v>
@@ -8561,7 +8561,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.167</v>
+        <v>1.169</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8578,7 +8578,7 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.579</v>
+        <v>-0.578</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>-7.528</v>
@@ -8627,10 +8627,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.919</v>
+        <v>0.92</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.783333</v>
+        <v>18.8</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8642,7 +8642,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.009000000000000001</v>
+        <v>-0.008</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -8671,7 +8671,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.401</v>
+        <v>2.402</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8688,7 +8688,7 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.135</v>
+        <v>-0.134</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>6.776</v>
@@ -8736,7 +8736,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.281</v>
+        <v>-0.279</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.818</v>
@@ -10212,7 +10212,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1277.85</v>
+        <v>1278.02</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1212.93</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1267.54</v>
+        <v>1267.7</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1208.61</v>
@@ -10244,7 +10244,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1262.41</v>
+        <v>1262.56</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1207.14</v>
@@ -10260,7 +10260,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1255.09</v>
+        <v>1255.24</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1198.19</v>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1259.93</v>
+        <v>1260.08</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1200.39</v>
@@ -10292,7 +10292,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1260.51</v>
+        <v>1260.65</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1208.38</v>
@@ -10308,7 +10308,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1245.77</v>
+        <v>1245.91</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1215.57</v>
@@ -10324,7 +10324,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1198.47</v>
+        <v>1198.6</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1211.65</v>
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1223.15</v>
+        <v>1223.27</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1211.53</v>
@@ -10356,7 +10356,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1194.5</v>
+        <v>1194.61</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1219.54</v>
@@ -10372,7 +10372,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1190.29</v>
+        <v>1190.42</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1221.46</v>
@@ -10388,7 +10388,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1182.54</v>
+        <v>1182.67</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1219.01</v>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1180.26</v>
+        <v>1180.39</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1213.02</v>
@@ -10420,7 +10420,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1199.1</v>
+        <v>1199.22</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1216.33</v>
@@ -10436,7 +10436,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1162.85</v>
+        <v>1162.98</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.31</v>
@@ -10452,7 +10452,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1139.47</v>
+        <v>1139.6</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1190.57</v>
@@ -10468,7 +10468,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1146.03</v>
+        <v>1146.17</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1204.31</v>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1151.11</v>
+        <v>1151.26</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1210.6</v>
@@ -10500,7 +10500,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1136.16</v>
+        <v>1136.33</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1211.04</v>
@@ -10516,7 +10516,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1142.02</v>
+        <v>1142.19</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1217.19</v>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1129.17</v>
+        <v>1129.34</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1222.04</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1130.96</v>
+        <v>1131.13</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1221.91</v>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1079.06</v>
+        <v>1079.18</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1219.49</v>
@@ -10580,7 +10580,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1067.42</v>
+        <v>1067.55</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1215.85</v>
@@ -10596,7 +10596,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1085.51</v>
+        <v>1085.65</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1221.9</v>
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1082.17</v>
+        <v>1082.34</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1211.56</v>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1103.09</v>
+        <v>1103.26</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1205.7</v>
@@ -10644,7 +10644,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1078.72</v>
+        <v>1078.9</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1190.64</v>
@@ -10660,7 +10660,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1105.39</v>
+        <v>1105.57</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1213.48</v>
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1107.24</v>
+        <v>1107.42</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1219.33</v>
@@ -10692,7 +10692,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1104.22</v>
+        <v>1104.39</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1216.12</v>
@@ -10708,7 +10708,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1089.79</v>
+        <v>1089.97</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1215.83</v>
@@ -10724,7 +10724,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1053.07</v>
+        <v>1053.25</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1197.05</v>
@@ -10740,7 +10740,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1043.91</v>
+        <v>1044.12</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1197.89</v>
@@ -10756,7 +10756,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1058.63</v>
+        <v>1058.84</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1199.83</v>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1091.84</v>
+        <v>1092.05</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1205.87</v>
@@ -10788,7 +10788,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1086.76</v>
+        <v>1086.96</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1202.69</v>
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1086.86</v>
+        <v>1087.07</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1211.39</v>
@@ -10820,7 +10820,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1043.78</v>
+        <v>1043.97</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1199.02</v>
@@ -10836,7 +10836,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1058.26</v>
+        <v>1058.45</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1207.73</v>
@@ -10852,7 +10852,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1062.14</v>
+        <v>1062.33</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.93</v>
@@ -10868,7 +10868,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1090.76</v>
+        <v>1090.96</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1211.16</v>
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1078.18</v>
+        <v>1078.38</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1205.34</v>
@@ -10900,7 +10900,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1073.05</v>
+        <v>1073.24</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1206.03</v>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1068.95</v>
+        <v>1069.14</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1195.4</v>
@@ -10932,7 +10932,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1084.39</v>
+        <v>1084.58</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1203.83</v>
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1082.05</v>
+        <v>1082.23</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1197.12</v>
@@ -10964,7 +10964,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1050.6</v>
+        <v>1050.76</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1181.43</v>
@@ -10980,7 +10980,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1052.16</v>
+        <v>1052.33</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1191.78</v>
@@ -10996,7 +10996,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1051.25</v>
+        <v>1051.41</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1189.86</v>
@@ -11012,7 +11012,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1065.61</v>
+        <v>1065.78</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1188.37</v>
@@ -11028,7 +11028,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1051.5</v>
+        <v>1051.67</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1170.33</v>
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1053.43</v>
+        <v>1053.6</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1163.7</v>
@@ -11060,7 +11060,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1046.01</v>
+        <v>1046.18</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1175.54</v>
@@ -11076,7 +11076,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1058.29</v>
+        <v>1058.46</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1178.64</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1050.4</v>
+        <v>1050.57</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1162.19</v>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1063.03</v>
+        <v>1063.19</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1159.33</v>
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1034.97</v>
+        <v>1035.14</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1142.71</v>
@@ -11140,7 +11140,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1056.76</v>
+        <v>1056.93</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1154.7</v>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1066.28</v>
+        <v>1066.6</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11168,7 +11168,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1066.28</v>
+        <v>1066.6</v>
       </c>
     </row>
     <row r="64">
@@ -11179,7 +11179,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-15.37%</t>
+          <t>-15.35%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-24 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6569,10 +6569,10 @@
         <v>0.118</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.32</v>
+        <v>3.91</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0.0583</v>
+        <v>0.065</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>0.309</v>
@@ -6581,7 +6581,7 @@
         <v>0.73225</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
       <c r="P7" s="5" t="n">
         <v>0.0319</v>
@@ -6681,10 +6681,10 @@
         <v>0.575</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>2.68</v>
+        <v>2.17</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>0.044499997</v>
+        <v>0.0368</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>0.06136</v>
@@ -6693,7 +6693,7 @@
         <v>0.81711</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="P9" s="5" t="n">
         <v>0.0828</v>
@@ -6725,13 +6725,13 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>29.015823</v>
+        <v>29.005722</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.347034</v>
+        <v>37.33403</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>23.055845</v>
+        <v>23.04782</v>
       </c>
       <c r="J10" s="4" t="n">
         <v>0.503</v>
@@ -6807,7 +6807,7 @@
         <v>0.19124001</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>1.59</v>
+        <v>1.55</v>
       </c>
       <c r="P11" s="5" t="n">
         <v>0.2831</v>
@@ -6967,10 +6967,10 @@
         <v>0.389</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.42</v>
+        <v>2.58</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>0.0226</v>
+        <v>0.024600001</v>
       </c>
       <c r="M14" s="5" t="n">
         <v>0.48116</v>
@@ -6979,7 +6979,7 @@
         <v>0.46126</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7.05</v>
+        <v>7.07</v>
       </c>
       <c r="P14" s="5" t="n">
         <v>8.8889</v>
@@ -7325,7 +7325,7 @@
         <v>0.68561995</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>3.8</v>
+        <v>3.76</v>
       </c>
       <c r="P20" s="5" t="n">
         <v>4.5455</v>
@@ -9684,13 +9684,13 @@
         <v>0.73225</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>3.32</v>
+        <v>3.91</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0583</v>
+        <v>0.065</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>3367790</v>
+        <v>3749544</v>
       </c>
     </row>
     <row r="8">
@@ -9738,13 +9738,13 @@
         <v>0.81711</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2.68</v>
+        <v>2.17</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.044499997</v>
+        <v>0.0368</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>2574942</v>
+        <v>2415829</v>
       </c>
     </row>
     <row r="10">
@@ -9873,13 +9873,13 @@
         <v>0.46126</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>2.42</v>
+        <v>2.58</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.0226</v>
+        <v>0.024600001</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>4092356</v>
+        <v>4452753</v>
       </c>
     </row>
     <row r="15">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-25 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6713,13 +6713,13 @@
         <v>21</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>28.905075</v>
+        <v>28.918455</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>37.204487</v>
+        <v>37.221706</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>22.967846</v>
+        <v>22.978477</v>
       </c>
       <c r="J10" s="9" t="n">
         <v>0.5620000000000001</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 14:43
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.49</v>
+        <v>52.47</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.031013412</v>
+        <v>-0.03147495</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -673,16 +673,16 @@
         <v>-0.255</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.49</v>
+        <v>35.473</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.336172</v>
+        <v>22.325533</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.969246</v>
+        <v>13.962593</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.19</v>
+        <v>103.27</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>-0.20309389</v>
+        <v>-0.12573005</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.6709999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.053</v>
+        <v>18.067</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.693781</v>
+        <v>9.701295</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.2</v>
+        <v>21.23</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.010037355</v>
+        <v>-0.8636763</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -793,7 +793,7 @@
         <v>-0.5649999999999999</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.555</v>
+        <v>10.57</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>11.322</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.895031</v>
+        <v>10.910445</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.491</v>
@@ -816,7 +816,7 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>-0.4370000000000001</v>
+        <v>-0.436</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>-0.405</v>
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.36</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.024781642</v>
+        <v>-0.0244381</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -854,16 +854,16 @@
         <v>-0.262</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.362</v>
+        <v>10.366</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.942</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.644903</v>
+        <v>31.65605</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.723131</v>
+        <v>16.729021</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.398</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>-0.188</v>
+        <v>-0.187</v>
       </c>
     </row>
     <row r="6">
@@ -901,7 +901,7 @@
         <v>37.51</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.04000904</v>
+        <v>0.053338602</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -913,16 +913,16 @@
         <v>-0.066</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.258</v>
+        <v>10.259</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.348686</v>
+        <v>49.355263</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.006504</v>
+        <v>16.008636</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.97</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.022321742</v>
+        <v>-0.022858517</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.078</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.264</v>
+        <v>6.261</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.67797</v>
+        <v>3.6759753</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.184217</v>
+        <v>10.178695</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -993,7 +993,7 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.225</v>
+        <v>0.224</v>
       </c>
       <c r="Q7" s="4" t="n">
         <v>-0.035</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.73999999999999</v>
+        <v>87.72</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.6192671</v>
+        <v>0.5963352</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1031,16 +1031,16 @@
         <v>-0.259</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.115</v>
+        <v>6.114</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>11.12</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.586012</v>
+        <v>16.582232</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.8167715</v>
+        <v>11.814078</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.623</v>
@@ -1052,7 +1052,7 @@
         <v>0.66</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>-0.223</v>
+        <v>-0.224</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>-0.216</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.98</v>
+        <v>55.96</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.04714895</v>
+        <v>-0.047489376</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1090,16 +1090,16 @@
         <v>-0.189</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.756</v>
+        <v>5.754</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.886</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.942308</v>
+        <v>17.935898</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.036274</v>
+        <v>17.030186</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.461</v>
@@ -1114,7 +1114,7 @@
         <v>0.325</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.09300000000000001</v>
+        <v>-0.094</v>
       </c>
     </row>
     <row r="10">
@@ -1137,7 +1137,7 @@
         <v>26.8</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-0.09322998</v>
+        <v>-0.055926137</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1149,7 +1149,7 @@
         <v>-0.151</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.469</v>
+        <v>5.471</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>30.375</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>26.115984</v>
+        <v>26.12573</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -1175,7 +1175,7 @@
         <v>-0.029</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.137</v>
+        <v>0.138</v>
       </c>
     </row>
     <row r="11">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
+        <v>10.55</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.18975766</v>
+        <v>0.09487883</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1210,16 +1210,16 @@
         <v>-0.266</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.34</v>
+        <v>5.334</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.922</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.142859</v>
+        <v>25.11905</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.174174</v>
+        <v>12.162645</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.031</v>
@@ -1231,7 +1231,7 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.555</v>
+        <v>0.5539999999999999</v>
       </c>
       <c r="Q11" s="4" t="n">
         <v>-0.08900000000000001</v>
@@ -1257,7 +1257,7 @@
         <v>17.82</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.037006993</v>
+        <v>-0.037277176</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>32.22</v>
@@ -1269,16 +1269,16 @@
         <v>-0.447</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.275</v>
+        <v>5.274</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>5.256</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>49.51389</v>
+        <v>49.499996</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>21.632576</v>
+        <v>21.626507</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>10.358</v>
@@ -1442,7 +1442,7 @@
         <v>5.5</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.3649631400000001</v>
+        <v>0.4562061</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1454,16 +1454,16 @@
         <v>-0.458</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.237</v>
+        <v>2.239</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.774</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>11.956522</v>
+        <v>11.967391</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.913109</v>
+        <v>6.9193935</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.592</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>-0.268</v>
+        <v>-0.267</v>
       </c>
     </row>
     <row r="16">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.07</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.017317997</v>
+        <v>-0.016429877</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,7 +1693,7 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.168</v>
       </c>
       <c r="I19" s="6" t="n">
         <v>0.903</v>
@@ -1702,10 +1702,10 @@
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.441666</v>
+        <v>18.458332</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>11.948856</v>
+        <v>11.959656</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>0.083</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>-0.027</v>
+        <v>-0.026</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.38</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-0.03789401</v>
+        <v>-0.113674805</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,7 +1752,7 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.194</v>
+        <v>-0.195</v>
       </c>
       <c r="I20" s="6" t="n">
         <v>0.696</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.801651</v>
+        <v>21.785124</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.455</v>
@@ -1781,7 +1781,7 @@
         <v>0.003</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
     </row>
     <row r="21">
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.52</v>
+        <v>11.42</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.033976488</v>
+        <v>-0.041946306</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,10 +1813,10 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.445</v>
+        <v>-0.449</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>7.795</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-14.21605</v>
+        <v>-14.098765</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>22.644</v>
@@ -1841,10 +1841,10 @@
         </is>
       </c>
       <c r="P21" s="4" t="n">
-        <v>-0.174</v>
+        <v>-0.181</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>-0.308</v>
+        <v>-0.314</v>
       </c>
     </row>
     <row r="22">
@@ -2152,10 +2152,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.49</v>
+        <v>52.47</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.031013412</v>
+        <v>-0.03147495</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>-0.191</v>
@@ -2199,10 +2199,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.19</v>
+        <v>103.27</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.20309389</v>
+        <v>-0.12573005</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.527</v>
@@ -2214,7 +2214,7 @@
         <v>-59.4</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.283</v>
+        <v>-0.282</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>-0.551</v>
@@ -2246,22 +2246,22 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.2</v>
+        <v>21.23</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.010037355</v>
+        <v>-0.8636763</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.405</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.4370000000000001</v>
+        <v>-0.436</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-37.5</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.219</v>
+        <v>-0.218</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>-0.406</v>
@@ -2293,16 +2293,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.36</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.024781642</v>
+        <v>-0.0244381</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.187</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>33.4</v>
@@ -2343,7 +2343,7 @@
         <v>37.51</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.04000904</v>
+        <v>0.053338602</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.028</v>
@@ -2387,22 +2387,22 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.97</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.022321742</v>
+        <v>-0.022858517</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.035</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.225</v>
+        <v>0.224</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.1</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.012</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0.002</v>
@@ -2434,22 +2434,22 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.73999999999999</v>
+        <v>87.72</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.6192671</v>
+        <v>0.5963352</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.216</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.224</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>-3.2</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.07400000000000001</v>
+        <v>-0.075</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>-0.131</v>
@@ -2481,13 +2481,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.98</v>
+        <v>55.96</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.04714895</v>
+        <v>-0.047489376</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.09300000000000001</v>
+        <v>-0.094</v>
       </c>
       <c r="G9" s="5" t="n">
         <v>0.325</v>
@@ -2499,7 +2499,7 @@
         <v>-0.092</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.046</v>
+        <v>-0.047</v>
       </c>
       <c r="K9" s="5" t="n">
         <v>-0.189</v>
@@ -2531,10 +2531,10 @@
         <v>26.8</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.09322998</v>
+        <v>-0.055926137</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.137</v>
+        <v>0.138</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>-0.029</v>
@@ -2575,25 +2575,25 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
+        <v>10.55</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.18975766</v>
+        <v>0.09487883</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>-0.08900000000000001</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.555</v>
+        <v>0.5539999999999999</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>26</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.051</v>
+        <v>0.05</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.061</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>-0.266</v>
@@ -2625,7 +2625,7 @@
         <v>17.82</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.037006993</v>
+        <v>-0.037277176</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>-0.236</v>
@@ -2766,13 +2766,13 @@
         <v>5.5</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.3649631400000001</v>
+        <v>0.4562061</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.268</v>
+        <v>-0.267</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.022</v>
+        <v>0.023</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>6.2</v>
@@ -2951,28 +2951,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.07</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.017317997</v>
+        <v>-0.016429877</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.026</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.083</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.6</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.021</v>
+        <v>-0.02</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.011</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.168</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -2998,13 +2998,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.38</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.03789401</v>
+        <v>-0.113674805</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>0.003</v>
@@ -3013,13 +3013,13 @@
         <v>5.4</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.057</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>-0.019</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.194</v>
+        <v>-0.195</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3045,28 +3045,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.52</v>
+        <v>11.42</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.033976488</v>
+        <v>-0.041946306</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.308</v>
+        <v>-0.314</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.174</v>
+        <v>-0.181</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>38.9</v>
+        <v>38.8</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.207</v>
+        <v>-0.214</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.133</v>
+        <v>-0.141</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.445</v>
+        <v>-0.449</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.49</v>
+        <v>52.47</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.49</v>
+        <v>35.473</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.336172</v>
+        <v>22.325533</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.969246</v>
+        <v>13.962593</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.279287</v>
+        <v>22.268677</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.7264578</v>
+        <v>2.7251592</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.19</v>
+        <v>103.27</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.053</v>
+        <v>18.067</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.693781</v>
+        <v>9.701295</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0005815</v>
+        <v>2.0021324</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1019554</v>
+        <v>1.1028097</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.2</v>
+        <v>21.23</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.555</v>
+        <v>10.57</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.895031</v>
+        <v>10.910445</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.491</v>
@@ -3473,10 +3473,10 @@
         <v>1.87</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.618338</v>
+        <v>16.64185</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7433681</v>
+        <v>1.7458347</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,16 +3505,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.36</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.362</v>
+        <v>10.366</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.644903</v>
+        <v>31.65605</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.723131</v>
+        <v>16.729021</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.398</v>
@@ -3526,10 +3526,10 @@
         <v>2.794</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.966145</v>
+        <v>-36.979168</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4516978</v>
+        <v>1.4522092</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3561,13 +3561,13 @@
         <v>37.51</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.258</v>
+        <v>10.259</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.348686</v>
+        <v>49.355263</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.006504</v>
+        <v>16.008636</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.986925</v>
+        <v>3.987456</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.58490384</v>
+        <v>0.5849818</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.97</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.264</v>
+        <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.67797</v>
+        <v>3.6759753</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.184217</v>
+        <v>10.178695</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4292238</v>
+        <v>2.4279063</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5307875</v>
+        <v>1.5299574</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,16 +3664,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.73999999999999</v>
+        <v>87.72</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.115</v>
+        <v>6.114</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.586012</v>
+        <v>16.582232</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.8167715</v>
+        <v>11.814078</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.623</v>
@@ -3685,10 +3685,10 @@
         <v>3.801</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6.048115</v>
+        <v>6.0467362</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.09001</v>
+        <v>2.0895336</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.98</v>
+        <v>55.96</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.756</v>
+        <v>5.754</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.942308</v>
+        <v>17.935898</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.036274</v>
+        <v>17.030186</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.461</v>
@@ -3738,10 +3738,10 @@
         <v>3.423</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.671892</v>
+        <v>15.666293</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.8616943</v>
+        <v>2.860672</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3773,7 +3773,7 @@
         <v>26.8</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.469</v>
+        <v>5.471</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>26.115984</v>
+        <v>26.12573</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -3793,10 +3793,10 @@
         <v>2.645</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.5494709</v>
+        <v>1.5500492</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.47615117</v>
+        <v>0.47632885</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>-2.42</v>
@@ -3825,16 +3825,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
+        <v>10.55</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.34</v>
+        <v>5.334</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.142859</v>
+        <v>25.11905</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.174174</v>
+        <v>12.162645</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.031</v>
@@ -3846,10 +3846,10 @@
         <v>2.101</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.1690426</v>
+        <v>7.162254</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.2790158</v>
+        <v>2.2768576</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3881,13 +3881,13 @@
         <v>17.82</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.275</v>
+        <v>5.274</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>49.51389</v>
+        <v>49.499996</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>21.632576</v>
+        <v>21.626507</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>10.358</v>
@@ -3899,7 +3899,7 @@
         <v>4.075</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.711227</v>
+        <v>4.709905</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>4.0895205</v>
@@ -4048,13 +4048,13 @@
         <v>5.5</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.237</v>
+        <v>2.239</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>11.956522</v>
+        <v>11.967391</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.913109</v>
+        <v>6.9193935</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.592</v>
@@ -4066,10 +4066,10 @@
         <v>2.474</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7235976</v>
+        <v>-1.7251645</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43331912</v>
+        <v>0.43371302</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4263,16 +4263,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.07</v>
       </c>
       <c r="E19" s="6" t="n">
         <v>0.903</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.441666</v>
+        <v>18.458332</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>11.948856</v>
+        <v>11.959656</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4284,10 +4284,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.3765638</v>
+        <v>3.3796155</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6781631</v>
+        <v>0.67877597</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.38</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0.696</v>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.801651</v>
+        <v>21.785124</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.455</v>
@@ -4339,10 +4339,10 @@
         <v>1.818</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6411597</v>
+        <v>1.6399155</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.0968477</v>
+        <v>1.0960162</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4371,10 +4371,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.52</v>
+        <v>11.42</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-14.21605</v>
+        <v>-14.098765</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>22.644</v>
@@ -4394,10 +4394,10 @@
         <v>2.934</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.56176215</v>
+        <v>0.55712754</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.2130857</v>
+        <v>0.21132772</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-12.45</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.49</v>
+        <v>52.47</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.331</v>
+        <v>0.332</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.19</v>
+        <v>103.27</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.01</v>
+        <v>1.009</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>21.2</v>
+        <v>21.23</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.706</v>
+        <v>0.7040000000000001</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>99.36</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.97</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87.73999999999999</v>
+        <v>87.72</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.544</v>
+        <v>0.545</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.17</v>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55.98</v>
+        <v>55.96</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.56</v>
+        <v>10.55</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.645</v>
+        <v>0.647</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.72</v>
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.815092</v>
+        <v>28.81177</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.088665</v>
+        <v>37.08439</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.896345</v>
+        <v>22.893705</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.617</v>
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.07</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>0.401</v>
+        <v>0.4</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>2.55</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.38</v>
+        <v>26.36</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7300,7 +7300,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0.156</v>
+        <v>0.157</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>4.41</v>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>11.52</v>
+        <v>11.42</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7356,7 +7356,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.36</v>
+        <v>0.3720000000000001</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>8.01</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.49</v>
+        <v>35.473</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.336172</v>
+        <v>22.325533</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.469</v>
+        <v>5.471</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7758,7 +7758,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.137</v>
+        <v>0.138</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.691000000000001</v>
@@ -7787,10 +7787,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10.362</v>
+        <v>10.366</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.644903</v>
+        <v>31.65605</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.187</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.398</v>
@@ -7833,10 +7833,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.237</v>
+        <v>2.239</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11.956522</v>
+        <v>11.967391</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7850,7 +7850,7 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-0.268</v>
+        <v>-0.267</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>10.592</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.258</v>
+        <v>10.259</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.348686</v>
+        <v>49.355263</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7941,10 +7941,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.264</v>
+        <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.67797</v>
+        <v>3.6759753</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.115</v>
+        <v>6.114</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.586012</v>
+        <v>16.582232</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8029,10 +8029,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.756</v>
+        <v>5.754</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.942308</v>
+        <v>17.935898</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.032</v>
@@ -8044,7 +8044,7 @@
         <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.09300000000000001</v>
+        <v>-0.094</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>8.461</v>
@@ -8180,7 +8180,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.455</v>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>-0.5564</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.308</v>
+        <v>-0.314</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>22.644</v>
@@ -8319,10 +8319,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.34</v>
+        <v>5.334</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.142859</v>
+        <v>25.11905</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8411,10 +8411,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.275</v>
+        <v>5.274</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>49.51389</v>
+        <v>49.499996</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.201</v>
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.555</v>
+        <v>10.57</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.053</v>
+        <v>18.067</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8616,7 +8616,7 @@
         <v>0.903</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.441666</v>
+        <v>18.458332</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8628,7 +8628,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.026</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1294.3</v>
+        <v>1294.16</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1218.79</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1286.75</v>
+        <v>1286.61</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1209.76</v>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1291.58</v>
+        <v>1291.45</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1211.98</v>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1292.47</v>
+        <v>1292.34</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1220.05</v>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1277.41</v>
+        <v>1277.28</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1227.31</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1228.74</v>
+        <v>1228.62</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1223.35</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1254.15</v>
+        <v>1254.03</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1223.23</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1224.86</v>
+        <v>1224.75</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1231.32</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1220.54</v>
+        <v>1220.43</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1233.25</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1212.6</v>
+        <v>1212.48</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1230.78</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1210.23</v>
+        <v>1210.11</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1224.74</v>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1229.68</v>
+        <v>1229.57</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1228.07</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1192.58</v>
+        <v>1192.46</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1227.04</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1168.44</v>
+        <v>1168.32</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1202.06</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1175.05</v>
+        <v>1174.92</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.94</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1180.25</v>
+        <v>1180.12</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1222.29</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1164.92</v>
+        <v>1164.78</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1222.73</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1170.76</v>
+        <v>1170.62</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1228.94</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1157.44</v>
+        <v>1157.29</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1233.84</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1159.06</v>
+        <v>1158.92</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1233.71</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1106.46</v>
+        <v>1106.34</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1231.26</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1094.61</v>
+        <v>1094.49</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1227.59</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1112.91</v>
+        <v>1112.78</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1233.69</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1109.31</v>
+        <v>1109.17</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1223.26</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1130.92</v>
+        <v>1130.78</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1217.34</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1105.79</v>
+        <v>1105.65</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1202.13</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1133.12</v>
+        <v>1132.97</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1225.2</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1135.04</v>
+        <v>1134.91</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1231.1</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1131.89</v>
+        <v>1131.75</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1227.86</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1116.94</v>
+        <v>1116.8</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1227.57</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1079.22</v>
+        <v>1079.08</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1208.61</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1069.65</v>
+        <v>1069.48</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1209.46</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1084.77</v>
+        <v>1084.6</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1211.41</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1119.15</v>
+        <v>1118.98</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1217.51</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1114.05</v>
+        <v>1113.88</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1214.3</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1114.21</v>
+        <v>1114.03</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1223.09</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1070.18</v>
+        <v>1070.01</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1210.6</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1085.06</v>
+        <v>1084.89</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1219.4</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1089.21</v>
+        <v>1089.04</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1229.68</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1118.8</v>
+        <v>1118.64</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1222.85</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1105.87</v>
+        <v>1105.69</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1216.98</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1100.6</v>
+        <v>1100.43</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.67</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1096.67</v>
+        <v>1096.5</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1206.94</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1112.41</v>
+        <v>1112.24</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1215.46</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1110.13</v>
+        <v>1109.96</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1208.68</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1077.88</v>
+        <v>1077.73</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1192.84</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1079.36</v>
+        <v>1079.2</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.29</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1078.33</v>
+        <v>1078.17</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1201.35</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1093.51</v>
+        <v>1093.35</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1199.85</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1078.92</v>
+        <v>1078.76</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1181.63</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1080.83</v>
+        <v>1080.68</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1174.94</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1073.18</v>
+        <v>1073.02</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1186.89</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1085.74</v>
+        <v>1085.58</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1190.02</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1077.62</v>
+        <v>1077.47</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1173.41</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1090.51</v>
+        <v>1090.35</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1170.52</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1061.69</v>
+        <v>1061.53</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1153.74</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1084.18</v>
+        <v>1084.02</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1165.85</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1095.28</v>
+        <v>1095.11</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1161.94</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1081.07</v>
+        <v>1080.9</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1168.42</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1060</v>
+        <v>1060.02</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1060</v>
+        <v>1060.02</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-17.93%</t>
+          <t>-17.92%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 14:50
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.47</v>
+        <v>52.36</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.03147495</v>
+        <v>-0.033413284</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.255</v>
+        <v>-0.257</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.473</v>
+        <v>35.402</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.325533</v>
+        <v>22.280851</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.962593</v>
+        <v>13.9346485</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.329</v>
+        <v>0.326</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>-0.191</v>
+        <v>-0.193</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.27</v>
+        <v>103.32</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>-0.12573005</v>
+        <v>-0.07735625</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.6709999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.067</v>
+        <v>18.076</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.701295</v>
+        <v>9.705992999999999</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.23</v>
+        <v>21.22</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.8636763</v>
+        <v>-0.9337104000000001</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -793,7 +793,7 @@
         <v>-0.5649999999999999</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.57</v>
+        <v>10.563</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>11.322</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.910445</v>
+        <v>10.902738</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.491</v>
@@ -816,7 +816,7 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>-0.436</v>
+        <v>-0.4370000000000001</v>
       </c>
       <c r="Q4" s="4" t="n">
         <v>-0.405</v>
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.0244381</v>
+        <v>-0.025321443</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,19 +851,19 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.263</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.366</v>
+        <v>10.356</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.942</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.65605</v>
+        <v>31.627386</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.729021</v>
+        <v>16.713875</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.398</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.169</v>
+        <v>0.168</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>-0.187</v>
+        <v>-0.188</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.51</v>
+        <v>37.56</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.053338602</v>
+        <v>0.18671563</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.066</v>
+        <v>-0.065</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.259</v>
+        <v>10.273</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.355263</v>
+        <v>49.421055</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.008636</v>
+        <v>16.029978</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.022858517</v>
+        <v>-0.022151582</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,19 +969,19 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.078</v>
+        <v>-0.077</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.261</v>
+        <v>6.265</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6786346</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.178695</v>
+        <v>10.186058</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -993,7 +993,7 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.224</v>
+        <v>0.225</v>
       </c>
       <c r="Q7" s="4" t="n">
         <v>-0.035</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.72</v>
+        <v>87.8</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.5963352</v>
+        <v>0.68521065</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1031,16 +1031,16 @@
         <v>-0.259</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.114</v>
+        <v>6.119</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>11.12</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.582232</v>
+        <v>16.596882</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.814078</v>
+        <v>11.824516</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.623</v>
@@ -1052,7 +1052,7 @@
         <v>0.66</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>-0.224</v>
+        <v>-0.223</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>-0.216</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.96</v>
+        <v>55.9</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.047489376</v>
+        <v>-0.04851061299999999</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,19 +1087,19 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.19</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.754</v>
+        <v>5.748</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.886</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.935898</v>
+        <v>17.916668</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.030186</v>
+        <v>17.011927</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.461</v>
@@ -1111,10 +1111,10 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.325</v>
+        <v>0.323</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.8</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>-0.055926137</v>
+        <v>26.87</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0.1864323</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1146,10 +1146,10 @@
         <v>17.86</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-0.151</v>
+        <v>-0.149</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.471</v>
+        <v>5.484</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>30.375</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>26.12573</v>
+        <v>26.189085</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -1172,10 +1172,10 @@
         <v>1.977</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>-0.029</v>
+        <v>-0.026</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
     </row>
     <row r="11">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="E11" s="9" t="n">
-        <v>0.09487883</v>
+        <v>0.23718803</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>14.38</v>
@@ -1210,16 +1210,16 @@
         <v>-0.266</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.334</v>
+        <v>5.342</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>4.922</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.11905</v>
+        <v>25.154762</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.162645</v>
+        <v>12.179937</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.031</v>
@@ -1231,10 +1231,10 @@
         <v>1.1</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.5539999999999999</v>
+        <v>0.556</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>-0.08900000000000001</v>
+        <v>-0.08800000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.82</v>
+        <v>17.93</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.037277176</v>
+        <v>-0.031064332</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>32.22</v>
@@ -1266,19 +1266,19 @@
         <v>15.725</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.447</v>
+        <v>-0.444</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.274</v>
+        <v>5.308</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>5.256</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>49.499996</v>
+        <v>49.819443</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>21.626507</v>
+        <v>21.766071</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>10.358</v>
@@ -1290,10 +1290,10 @@
         <v>2.002</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>-0.236</v>
+        <v>-0.231</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.62</v>
+        <v>21.68</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.013686097</v>
+        <v>-0.010948895</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.045</v>
+        <v>-0.043</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.033</v>
+        <v>5.047</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.741936</v>
+        <v>69.935486</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>28.979681</v>
+        <v>29.060104</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.982</v>
+        <v>0.987</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.12</v>
+        <v>0.123</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.86</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.61823744</v>
+        <v>-0.5795967</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1393,7 +1393,7 @@
         <v>-0.307</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.373</v>
+        <v>2.374</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.956</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>11.934591</v>
+        <v>11.939231</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.753</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>-0.038</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>-0.145</v>
+        <v>-0.144</v>
       </c>
     </row>
     <row r="15">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.4562061</v>
+        <v>0.6386833</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,19 +1451,19 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.458</v>
+        <v>-0.457</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.239</v>
+        <v>2.243</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.774</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>11.967391</v>
+        <v>11.98913</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9193935</v>
+        <v>6.9319625</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.592</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.023</v>
+        <v>0.025</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>-0.267</v>
+        <v>-0.266</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.01057297</v>
+        <v>-0.010917765</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1513,7 +1513,7 @@
         <v>-0.296</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.937</v>
+        <v>1.936</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.438</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.381824999999999</v>
+        <v>8.378935999999999</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.223</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-0.164</v>
+        <v>-0.165</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.023</v>
+        <v>-0.024</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.54000000000001</v>
+        <v>97.36</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.019402838</v>
+        <v>-0.021162193</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.143</v>
+        <v>-0.145</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.745</v>
+        <v>1.741</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.696</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>17.96317</v>
+        <v>17.930939</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.407064</v>
+        <v>16.377628</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.218</v>
+        <v>0.215</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>0.019</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="18">
@@ -1618,10 +1618,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-0.0391304</v>
+        <v>-0.04130436000000001</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1630,10 +1630,10 @@
         <v>4.4</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>-0.6779999999999999</v>
+        <v>-0.679</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.137</v>
+        <v>1.134</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.883</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.4646463</v>
+        <v>4.454545</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.324</v>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>-0.584</v>
+        <v>-0.585</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>-0.59</v>
+        <v>-0.591</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.07</v>
+        <v>11.06</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.016429877</v>
+        <v>-0.017761972</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,19 +1693,19 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.168</v>
+        <v>-0.169</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.903</v>
+        <v>0.902</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.458332</v>
+        <v>18.433332</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>11.959656</v>
+        <v>11.943459</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>-0.026</v>
+        <v>-0.027</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.35</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-0.113674805</v>
+        <v>-0.15156882</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.785124</v>
+        <v>21.77686</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.455</v>
@@ -1778,7 +1778,7 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="Q20" s="4" t="n">
         <v>-0.026</v>
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.42</v>
+        <v>11.38</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.041946306</v>
+        <v>-0.044882536</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,10 +1813,10 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.449</v>
+        <v>-0.451</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>7.795</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-14.098765</v>
+        <v>-14.055555</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>22.644</v>
@@ -1841,10 +1841,10 @@
         </is>
       </c>
       <c r="P21" s="4" t="n">
-        <v>-0.181</v>
+        <v>-0.183</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>-0.314</v>
+        <v>-0.316</v>
       </c>
     </row>
     <row r="22">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.83</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.020149288</v>
+        <v>0.025373147</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,10 +1876,10 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.314</v>
+        <v>-0.31</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.185</v>
+        <v>0.186</v>
       </c>
       <c r="J22" s="6" t="n">
         <v>0.512</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>9.123552</v>
+        <v>9.170271</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.891</v>
@@ -1902,10 +1902,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>-0.238</v>
+        <v>-0.234</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>-0.238</v>
+        <v>-0.234</v>
       </c>
     </row>
     <row r="23">
@@ -2152,28 +2152,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.47</v>
+        <v>52.36</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.03147495</v>
+        <v>-0.033413284</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.191</v>
+        <v>-0.193</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.329</v>
+        <v>0.326</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>52.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.077</v>
+        <v>-0.079</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.058</v>
+        <v>-0.06</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.255</v>
+        <v>-0.257</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2199,10 +2199,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.27</v>
+        <v>103.32</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.12573005</v>
+        <v>-0.07735625</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.527</v>
@@ -2246,22 +2246,22 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.23</v>
+        <v>21.22</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.8636763</v>
+        <v>-0.9337104000000001</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.405</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.436</v>
+        <v>-0.4370000000000001</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-37.5</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.218</v>
+        <v>-0.219</v>
       </c>
       <c r="J4" s="5" t="n">
         <v>-0.406</v>
@@ -2293,16 +2293,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.0244381</v>
+        <v>-0.025321443</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.187</v>
+        <v>-0.188</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.169</v>
+        <v>0.168</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>33.4</v>
@@ -2314,7 +2314,7 @@
         <v>-0.131</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.263</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2340,28 +2340,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.51</v>
+        <v>37.56</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.053338602</v>
+        <v>0.18671563</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>12</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.058</v>
+        <v>0.06</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.067</v>
+        <v>0.068</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.066</v>
+        <v>-0.065</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,28 +2387,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.022858517</v>
+        <v>-0.022151582</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.035</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.224</v>
+        <v>0.225</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.1</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.011</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0.002</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.078</v>
+        <v>-0.077</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2434,25 +2434,25 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.72</v>
+        <v>87.8</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.5963352</v>
+        <v>0.68521065</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.216</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.224</v>
+        <v>-0.223</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>-3.2</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.075</v>
+        <v>-0.07400000000000001</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.131</v>
+        <v>-0.13</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>-0.259</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.96</v>
+        <v>55.9</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.047489376</v>
+        <v>-0.04851061299999999</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.325</v>
+        <v>0.323</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>38.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.09300000000000001</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.047</v>
+        <v>-0.048</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.19</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2528,28 +2528,28 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.8</v>
+        <v>26.87</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.055926137</v>
+        <v>0.1864323</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.029</v>
+        <v>-0.026</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-21.9</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.143</v>
+        <v>0.146</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08900000000000001</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-0.151</v>
+        <v>-0.149</v>
       </c>
       <c r="L10" s="8" t="n">
         <v>1.977</v>
@@ -2575,25 +2575,25 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.09487883</v>
+        <v>0.23718803</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.08900000000000001</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.5539999999999999</v>
+        <v>0.556</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>26</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.05</v>
+        <v>0.051</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.06</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>-0.266</v>
@@ -2622,28 +2622,28 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.82</v>
+        <v>17.93</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.037277176</v>
+        <v>-0.031064332</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-0.236</v>
+        <v>-0.231</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.205</v>
+        <v>-0.2</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>-29.6</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.03</v>
+        <v>-0.024</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.273</v>
+        <v>-0.269</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.447</v>
+        <v>-0.444</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>2.002</v>
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.62</v>
+        <v>21.68</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.013686097</v>
+        <v>-0.010948895</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.12</v>
+        <v>0.123</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.982</v>
+        <v>0.987</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>50.7</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.149</v>
+        <v>0.153</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.182</v>
+        <v>0.186</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.045</v>
+        <v>-0.043</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2716,25 +2716,25 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.86</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.61823744</v>
+        <v>-0.5795967</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.145</v>
+        <v>-0.144</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.038</v>
+        <v>-0.03700000000000001</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>12.6</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.066</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.168</v>
+        <v>-0.167</v>
       </c>
       <c r="K14" s="5" t="n">
         <v>-0.307</v>
@@ -2763,28 +2763,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.4562061</v>
+        <v>0.6386833</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.267</v>
+        <v>-0.266</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.023</v>
+        <v>0.025</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>6.2</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.08599999999999999</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.3</v>
+        <v>-0.298</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.458</v>
+        <v>-0.457</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2810,22 +2810,22 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.01057297</v>
+        <v>-0.010917765</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.023</v>
+        <v>-0.024</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.164</v>
+        <v>-0.165</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>-19.3</v>
+        <v>-19.4</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.053</v>
+        <v>0.052</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>-0.107</v>
@@ -2857,28 +2857,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.54000000000001</v>
+        <v>97.36</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.019402838</v>
+        <v>-0.021162193</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.019</v>
+        <v>0.017</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.218</v>
+        <v>0.215</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>20.3</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.028</v>
+        <v>0.026</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.015</v>
+        <v>0.013</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.143</v>
+        <v>-0.145</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2904,28 +2904,28 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.0391304</v>
+        <v>-0.04130436000000001</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.59</v>
+        <v>-0.591</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.584</v>
+        <v>-0.585</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-34.5</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.386</v>
+        <v>-0.388</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.5670000000000001</v>
+        <v>-0.5679999999999999</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.6779999999999999</v>
+        <v>-0.679</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>1.993</v>
@@ -2951,28 +2951,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.07</v>
+        <v>11.06</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.016429877</v>
+        <v>-0.017761972</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>-1.6</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.02</v>
+        <v>-0.021</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.012</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.168</v>
+        <v>-0.169</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -2998,16 +2998,16 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.35</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.113674805</v>
+        <v>-0.15156882</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>-0.026</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.4</v>
@@ -3016,7 +3016,7 @@
         <v>-0.057</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.019</v>
+        <v>-0.02</v>
       </c>
       <c r="K20" s="5" t="n">
         <v>-0.195</v>
@@ -3045,28 +3045,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.42</v>
+        <v>11.38</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.041946306</v>
+        <v>-0.044882536</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.314</v>
+        <v>-0.316</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.181</v>
+        <v>-0.183</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>38.8</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.214</v>
+        <v>-0.216</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.141</v>
+        <v>-0.144</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.449</v>
+        <v>-0.451</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.83</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.020149288</v>
+        <v>0.025373147</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.238</v>
+        <v>-0.234</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.238</v>
+        <v>-0.234</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>3.9</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.18</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.202</v>
+        <v>-0.198</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.314</v>
+        <v>-0.31</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.47</v>
+        <v>52.36</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.473</v>
+        <v>35.402</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.325533</v>
+        <v>22.280851</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.962593</v>
+        <v>13.9346485</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.268677</v>
+        <v>22.22411</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.7251592</v>
+        <v>2.719705</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.27</v>
+        <v>103.32</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.067</v>
+        <v>18.076</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.701295</v>
+        <v>9.705992999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0021324</v>
+        <v>2.0031018</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1028097</v>
+        <v>1.1033436</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.23</v>
+        <v>21.22</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.57</v>
+        <v>10.563</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.910445</v>
+        <v>10.902738</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.491</v>
@@ -3473,10 +3473,10 @@
         <v>1.87</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.64185</v>
+        <v>16.630093</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7458347</v>
+        <v>1.7446012</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,16 +3505,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.366</v>
+        <v>10.356</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.65605</v>
+        <v>31.627386</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.729021</v>
+        <v>16.713875</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.398</v>
@@ -3526,10 +3526,10 @@
         <v>2.794</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.979168</v>
+        <v>-36.945683</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4522092</v>
+        <v>1.4508944</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,16 +3558,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.51</v>
+        <v>37.56</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.259</v>
+        <v>10.273</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.355263</v>
+        <v>49.421055</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.008636</v>
+        <v>16.029978</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.987456</v>
+        <v>3.9927716</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5849818</v>
+        <v>0.5857616</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.261</v>
+        <v>6.265</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6786346</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.178695</v>
+        <v>10.186058</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4279063</v>
+        <v>2.429663</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5299574</v>
+        <v>1.5310643</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,16 +3664,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.72</v>
+        <v>87.8</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.114</v>
+        <v>6.119</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.582232</v>
+        <v>16.596882</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.814078</v>
+        <v>11.824516</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.623</v>
@@ -3685,10 +3685,10 @@
         <v>3.801</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6.0467362</v>
+        <v>6.0520782</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0895336</v>
+        <v>2.0913796</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.96</v>
+        <v>55.9</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.754</v>
+        <v>5.748</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.935898</v>
+        <v>17.916668</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.030186</v>
+        <v>17.011927</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.461</v>
@@ -3738,10 +3738,10 @@
         <v>3.423</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.666293</v>
+        <v>15.649496</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.860672</v>
+        <v>2.857605</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3770,10 +3770,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.8</v>
+        <v>26.87</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.471</v>
+        <v>5.484</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>26.12573</v>
+        <v>26.189085</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -3793,10 +3793,10 @@
         <v>2.645</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.5500492</v>
+        <v>1.553808</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.47632885</v>
+        <v>0.4774839</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>-2.42</v>
@@ -3825,16 +3825,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.334</v>
+        <v>5.342</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.11905</v>
+        <v>25.154762</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.162645</v>
+        <v>12.179937</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.031</v>
@@ -3846,10 +3846,10 @@
         <v>2.101</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.162254</v>
+        <v>7.1724367</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.2768576</v>
+        <v>2.2800946</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.42</v>
@@ -3878,16 +3878,16 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.82</v>
+        <v>17.93</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.274</v>
+        <v>5.308</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>49.499996</v>
+        <v>49.819443</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>21.626507</v>
+        <v>21.766071</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>10.358</v>
@@ -3899,10 +3899,10 @@
         <v>4.075</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.709905</v>
+        <v>4.7403</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>4.0895205</v>
+        <v>4.114757</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0.36</v>
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.62</v>
+        <v>21.68</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.033</v>
+        <v>5.047</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.741936</v>
+        <v>69.935486</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>28.979681</v>
+        <v>29.060104</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.677529</v>
+        <v>14.718262</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.436423</v>
+        <v>4.4487348</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.86</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.373</v>
+        <v>2.374</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11.934591</v>
+        <v>11.939231</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.753</v>
@@ -4013,10 +4013,10 @@
         <v>2.372</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7461028</v>
+        <v>2.7471704</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.94505686</v>
+        <v>0.94542426</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4045,16 +4045,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.239</v>
+        <v>2.243</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>11.967391</v>
+        <v>11.98913</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9193935</v>
+        <v>6.9319625</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.592</v>
@@ -4066,10 +4066,10 @@
         <v>2.474</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7251645</v>
+        <v>-1.7282983</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43371302</v>
+        <v>0.43450087</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.937</v>
+        <v>1.936</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.381824999999999</v>
+        <v>8.378935999999999</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.223</v>
@@ -4121,10 +4121,10 @@
         <v>1.787</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.99848557</v>
+        <v>0.99814135</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27827737</v>
+        <v>0.27818143</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,16 +4153,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.54000000000001</v>
+        <v>97.36</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.745</v>
+        <v>1.741</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>17.96317</v>
+        <v>17.930939</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.407064</v>
+        <v>16.377628</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -4174,10 +4174,10 @@
         <v>3.111</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2325845</v>
+        <v>3.2267847</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.2003894</v>
+        <v>3.194647</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.137</v>
+        <v>1.134</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.4646463</v>
+        <v>4.454545</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.324</v>
@@ -4231,10 +4231,10 @@
         <v>1.319</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.5028902</v>
+        <v>1.4994899</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.6983784</v>
+        <v>1.694536</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4263,16 +4263,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.07</v>
+        <v>11.06</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.903</v>
+        <v>0.902</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.458332</v>
+        <v>18.433332</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>11.959656</v>
+        <v>11.943459</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4284,10 +4284,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.3796155</v>
+        <v>3.3750384</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.67877597</v>
+        <v>0.6778567</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.35</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0.696</v>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.785124</v>
+        <v>21.77686</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.455</v>
@@ -4339,10 +4339,10 @@
         <v>1.818</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6399155</v>
+        <v>1.6392933</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.0960162</v>
+        <v>1.0956004</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4371,10 +4371,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.42</v>
+        <v>11.38</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-14.098765</v>
+        <v>-14.055555</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>22.644</v>
@@ -4394,10 +4394,10 @@
         <v>2.934</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.55712754</v>
+        <v>0.5554201</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.21132772</v>
+        <v>0.21068002</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-12.45</v>
@@ -4426,10 +4426,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.83</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.185</v>
+        <v>0.186</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.123552</v>
+        <v>9.170271</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.891</v>
@@ -4449,10 +4449,10 @@
         <v>1.684</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-11.334992</v>
+        <v>-11.393035</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.60819525</v>
+        <v>0.61130965</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.47</v>
+        <v>52.36</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.332</v>
+        <v>0.334</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.27</v>
+        <v>103.32</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.009</v>
+        <v>1.008</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>21.23</v>
+        <v>21.22</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.7040000000000001</v>
+        <v>0.705</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>99.40000000000001</v>
+        <v>99.31</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.427</v>
+        <v>0.428</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.38</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.51</v>
+        <v>37.56</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.137</v>
+        <v>0.136</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.98999999999999</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6554,7 +6554,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.139</v>
+        <v>0.138</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.91</v>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87.72</v>
+        <v>87.8</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.545</v>
+        <v>0.5429999999999999</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.17</v>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55.96</v>
+        <v>55.9</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.303</v>
+        <v>0.305</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>4.01</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>26.8</v>
+        <v>26.87</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6722,7 +6722,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.192</v>
+        <v>0.189</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>3.37</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.55</v>
+        <v>10.56</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>16</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.647</v>
+        <v>0.645</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.72</v>
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>17.82</v>
+        <v>17.93</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.81177</v>
+        <v>28.805126</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.08439</v>
+        <v>37.07584</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.893705</v>
+        <v>22.888426</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.617</v>
+        <v>0.607</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.62</v>
+        <v>21.68</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6894,7 +6894,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.152</v>
+        <v>0.149</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.89</v>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.86</v>
+        <v>12.87</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6952,7 +6952,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.406</v>
+        <v>0.405</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.58</v>
@@ -6985,7 +6985,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.5</v>
+        <v>5.51</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0.68</v>
+        <v>0.677</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.37</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.5</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7066,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.317</v>
+        <v>0.318</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.3</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>97.54000000000001</v>
+        <v>97.36</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7126,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.104</v>
+        <v>0.106</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.64</v>
@@ -7159,7 +7159,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4.42</v>
+        <v>4.41</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -7182,7 +7182,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>1.662</v>
+        <v>1.668</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>2.41</v>
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.07</v>
+        <v>11.06</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>0.4</v>
+        <v>0.401</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>2.55</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.35</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>11.42</v>
+        <v>11.38</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7356,7 +7356,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.3720000000000001</v>
+        <v>0.377</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>8.01</v>
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.83</v>
+        <v>6.87</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7414,7 +7414,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.9520000000000001</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>9.81</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.473</v>
+        <v>35.402</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.325533</v>
+        <v>22.280851</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7712,7 +7712,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.191</v>
+        <v>-0.193</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.795</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.471</v>
+        <v>5.484</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7758,7 +7758,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.138</v>
+        <v>0.14</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.691000000000001</v>
@@ -7787,10 +7787,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10.366</v>
+        <v>10.356</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.65605</v>
+        <v>31.627386</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.187</v>
+        <v>-0.188</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.398</v>
@@ -7833,10 +7833,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.239</v>
+        <v>2.243</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11.967391</v>
+        <v>11.98913</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7850,7 +7850,7 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-0.267</v>
+        <v>-0.266</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>10.592</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.259</v>
+        <v>10.273</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.355263</v>
+        <v>49.421055</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7894,7 +7894,7 @@
         <v>0.1489</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>16.869</v>
@@ -7941,10 +7941,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.261</v>
+        <v>6.265</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6786346</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.114</v>
+        <v>6.119</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.582232</v>
+        <v>16.596882</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8029,10 +8029,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.754</v>
+        <v>5.748</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.935898</v>
+        <v>17.916668</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.032</v>
@@ -8044,7 +8044,7 @@
         <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.095</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>8.461</v>
@@ -8073,10 +8073,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.745</v>
+        <v>1.741</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.96317</v>
+        <v>17.930939</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.041</v>
@@ -8088,7 +8088,7 @@
         <v>0.19214001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.019</v>
+        <v>0.017</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.893000000000001</v>
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.937</v>
+        <v>1.936</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8134,7 +8134,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.023</v>
+        <v>-0.024</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.223</v>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>-0.5564</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.314</v>
+        <v>-0.316</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>22.644</v>
@@ -8319,10 +8319,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.334</v>
+        <v>5.342</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.11905</v>
+        <v>25.154762</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8334,7 +8334,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.08900000000000001</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.031</v>
@@ -8363,10 +8363,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.033</v>
+        <v>5.047</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>69.741936</v>
+        <v>69.935486</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.888</v>
@@ -8378,7 +8378,7 @@
         <v>0.29505</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.12</v>
+        <v>0.123</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -8411,10 +8411,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.274</v>
+        <v>5.308</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>49.499996</v>
+        <v>49.819443</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.201</v>
@@ -8426,7 +8426,7 @@
         <v>0.10515001</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.236</v>
+        <v>-0.231</v>
       </c>
       <c r="J22" s="7" t="n">
         <v>10.358</v>
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.57</v>
+        <v>10.563</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.067</v>
+        <v>18.076</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8547,7 +8547,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.137</v>
+        <v>1.134</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8564,7 +8564,7 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.59</v>
+        <v>-0.591</v>
       </c>
       <c r="J25" s="7" t="n">
         <v>-7.324</v>
@@ -8613,10 +8613,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.903</v>
+        <v>0.902</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.458332</v>
+        <v>18.433332</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8628,7 +8628,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -8657,7 +8657,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.373</v>
+        <v>2.374</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8674,7 +8674,7 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.145</v>
+        <v>-0.144</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>6.753</v>
@@ -8703,7 +8703,7 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.185</v>
+        <v>0.186</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
@@ -8722,7 +8722,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.238</v>
+        <v>-0.234</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.891</v>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1294.16</v>
+        <v>1293.93</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1218.79</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1286.61</v>
+        <v>1286.37</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1209.76</v>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1291.45</v>
+        <v>1291.19</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1211.98</v>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1292.34</v>
+        <v>1292.1</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1220.05</v>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1277.28</v>
+        <v>1277.03</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1227.31</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1228.62</v>
+        <v>1228.37</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1223.35</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1254.03</v>
+        <v>1253.79</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1223.23</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1224.75</v>
+        <v>1224.54</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1231.32</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1220.43</v>
+        <v>1220.2</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1233.25</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1212.48</v>
+        <v>1212.24</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1230.78</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1210.11</v>
+        <v>1209.87</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1224.74</v>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1229.57</v>
+        <v>1229.33</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1228.07</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1192.46</v>
+        <v>1192.22</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1227.04</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1168.32</v>
+        <v>1168.07</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1202.06</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1174.92</v>
+        <v>1174.65</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.94</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1180.12</v>
+        <v>1179.84</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1222.29</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1164.78</v>
+        <v>1164.5</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1222.73</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1170.62</v>
+        <v>1170.32</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1228.94</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1157.29</v>
+        <v>1157</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1233.84</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1158.92</v>
+        <v>1158.6</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1233.71</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1106.34</v>
+        <v>1106.15</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1231.26</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1094.49</v>
+        <v>1094.29</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1227.59</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1112.78</v>
+        <v>1112.55</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1233.69</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1109.17</v>
+        <v>1108.9</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1223.26</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1130.78</v>
+        <v>1130.52</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1217.34</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1105.65</v>
+        <v>1105.38</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1202.13</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1132.97</v>
+        <v>1132.7</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1225.2</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1134.91</v>
+        <v>1134.64</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1231.1</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1131.75</v>
+        <v>1131.48</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1227.86</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1116.8</v>
+        <v>1116.5</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1227.57</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1079.08</v>
+        <v>1078.77</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1208.61</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1069.48</v>
+        <v>1069.17</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1209.46</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1084.6</v>
+        <v>1084.3</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1211.41</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1118.98</v>
+        <v>1118.69</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1217.51</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1113.88</v>
+        <v>1113.61</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1214.3</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1114.03</v>
+        <v>1113.78</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1223.09</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1070.01</v>
+        <v>1069.77</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1210.6</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1084.89</v>
+        <v>1084.67</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1219.4</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1089.04</v>
+        <v>1088.84</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1229.68</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1118.64</v>
+        <v>1118.45</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1222.85</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1105.69</v>
+        <v>1105.49</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1216.98</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1100.43</v>
+        <v>1100.25</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.67</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1096.5</v>
+        <v>1096.31</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1206.94</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1112.24</v>
+        <v>1112.07</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1215.46</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1109.96</v>
+        <v>1109.81</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1208.68</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1077.73</v>
+        <v>1077.58</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1192.84</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1079.2</v>
+        <v>1079.05</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.29</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1078.17</v>
+        <v>1078.01</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1201.35</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1093.35</v>
+        <v>1093.19</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1199.85</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1078.76</v>
+        <v>1078.63</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1181.63</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1080.68</v>
+        <v>1080.54</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1174.94</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1073.02</v>
+        <v>1072.87</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1186.89</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1085.58</v>
+        <v>1085.43</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1190.02</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1077.47</v>
+        <v>1077.32</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1173.41</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1090.35</v>
+        <v>1090.23</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1170.52</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1061.53</v>
+        <v>1061.41</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1153.74</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1084.02</v>
+        <v>1083.9</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1165.85</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1095.11</v>
+        <v>1094.98</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1161.94</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1080.9</v>
+        <v>1080.77</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1168.42</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1060.02</v>
+        <v>1059.88</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1060.02</v>
+        <v>1059.88</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-17.92%</t>
+          <t>-17.91%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 14:54
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.36</v>
+        <v>52.29</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.033413284</v>
+        <v>-0.034705508</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.257</v>
+        <v>-0.258</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.402</v>
+        <v>35.355</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.280851</v>
+        <v>22.251064</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.9346485</v>
+        <v>13.916019</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.326</v>
+        <v>0.324</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>-0.193</v>
+        <v>-0.194</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.32</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>-0.07735625</v>
+        <v>103.47</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0.08703708</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.6709999999999999</v>
+        <v>-0.67</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.076</v>
+        <v>18.106</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.705992999999999</v>
+        <v>9.721962</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -755,10 +755,10 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>-0.527</v>
+        <v>-0.526</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.22</v>
+        <v>21.21</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.9337104000000001</v>
+        <v>-0.95704913</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -793,7 +793,7 @@
         <v>-0.5649999999999999</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.563</v>
+        <v>10.56</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>11.322</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.902738</v>
+        <v>10.900169</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.491</v>
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.31</v>
+        <v>99.19</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.025321443</v>
+        <v>-0.02645009</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,19 +851,19 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.263</v>
+        <v>-0.264</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.356</v>
+        <v>10.344</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.942</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.627386</v>
+        <v>31.590763</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.713875</v>
+        <v>16.69452</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.398</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.168</v>
+        <v>0.166</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>-0.188</v>
+        <v>-0.189</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.56</v>
+        <v>37.52</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.18671563</v>
+        <v>0.08001808000000001</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.066</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.273</v>
+        <v>10.262</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.421055</v>
+        <v>49.368423</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.029978</v>
+        <v>16.012905</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.169</v>
+        <v>0.168</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.98999999999999</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.022151582</v>
+        <v>-0.022799637</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,19 +969,19 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.077</v>
+        <v>-0.078</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.265</v>
+        <v>6.261</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6786346</v>
+        <v>3.6761968</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.186058</v>
+        <v>10.179308</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -993,7 +993,7 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.225</v>
+        <v>0.224</v>
       </c>
       <c r="Q7" s="4" t="n">
         <v>-0.035</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.8</v>
+        <v>87.51000000000001</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.68521065</v>
+        <v>0.35551056</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1028,19 +1028,19 @@
         <v>80.23999999999999</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>-0.259</v>
+        <v>-0.261</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.119</v>
+        <v>6.099</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>11.12</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.596882</v>
+        <v>16.542534</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.824516</v>
+        <v>11.785796</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.623</v>
@@ -1052,10 +1052,10 @@
         <v>0.66</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>-0.223</v>
+        <v>-0.226</v>
       </c>
       <c r="Q8" s="4" t="n">
-        <v>-0.216</v>
+        <v>-0.218</v>
       </c>
     </row>
     <row r="9">
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.9</v>
+        <v>55.73</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.04851061299999999</v>
+        <v>-0.051489387</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,19 +1087,19 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.19</v>
+        <v>-0.192</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.748</v>
+        <v>5.73</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.886</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.916668</v>
+        <v>17.860577</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.011927</v>
+        <v>16.95867</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.461</v>
@@ -1111,10 +1111,10 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.323</v>
+        <v>0.319</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.095</v>
+        <v>-0.09699999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.87</v>
+        <v>26.86</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.1864323</v>
+        <v>0.14914584</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1149,7 +1149,7 @@
         <v>-0.149</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.484</v>
+        <v>5.482</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>30.375</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>26.189085</v>
+        <v>26.179337</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -1172,7 +1172,7 @@
         <v>1.977</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>-0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>0.14</v>
@@ -1181,12 +1181,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1195,57 +1195,57 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
-      </c>
-      <c r="E11" s="9" t="n">
-        <v>0.23718803</v>
+        <v>17.93</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>-0.03133441</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>14.38</v>
+        <v>32.22</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>5.59</v>
+        <v>15.725</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.266</v>
+        <v>-0.444</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.342</v>
+        <v>5.306</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>4.922</v>
+        <v>5.256</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>25.154762</v>
+        <v>49.805553</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>12.179937</v>
+        <v>21.760006</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>10.031</v>
+        <v>10.358</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="P11" s="9" t="n">
-        <v>0.556</v>
+        <v>2.002</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>-0.201</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>-0.08800000000000001</v>
+        <v>-0.231</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1254,46 +1254,46 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.93</v>
+        <v>10.49</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.031064332</v>
+        <v>-0.4743851</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>32.22</v>
+        <v>14.38</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>15.725</v>
+        <v>5.59</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.444</v>
+        <v>-0.271</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.308</v>
+        <v>5.304</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>5.256</v>
+        <v>4.922</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>49.819443</v>
+        <v>24.97619</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>21.766071</v>
+        <v>12.093473</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>10.358</v>
+        <v>10.031</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>2.002</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>-0.2</v>
+        <v>1.1</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>0.545</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>-0.231</v>
+        <v>-0.095</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.68</v>
+        <v>21.52</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.010948895</v>
+        <v>-0.018248158</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.043</v>
+        <v>-0.05</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.047</v>
+        <v>5.01</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.935486</v>
+        <v>69.41936</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>29.060104</v>
+        <v>28.84564</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.987</v>
+        <v>0.973</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.123</v>
+        <v>0.114</v>
       </c>
     </row>
     <row r="14">
@@ -1442,7 +1442,7 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.6386833</v>
+        <v>0.5474491</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1454,16 +1454,16 @@
         <v>-0.457</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.243</v>
+        <v>2.241</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.774</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>11.98913</v>
+        <v>11.978261</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9319625</v>
+        <v>6.9256783</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.592</v>
@@ -1475,7 +1475,7 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>-0.266</v>
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.5</v>
+        <v>14.51</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.010917765</v>
+        <v>-0.010231898</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1513,7 +1513,7 @@
         <v>-0.296</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.936</v>
+        <v>1.938</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.438</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.378935999999999</v>
+        <v>8.384714000000001</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.223</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-0.165</v>
+        <v>-0.164</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.024</v>
+        <v>-0.023</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.36</v>
+        <v>97</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.021162193</v>
+        <v>-0.02483162</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.145</v>
+        <v>-0.148</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.741</v>
+        <v>1.735</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.696</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>17.930939</v>
+        <v>17.86372</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.377628</v>
+        <v>16.31623</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.215</v>
+        <v>0.211</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>0.017</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="18">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.35</v>
+        <v>26.37</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-0.15156882</v>
+        <v>-0.075780794</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.77686</v>
+        <v>21.793388</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.455</v>
@@ -1778,10 +1778,10 @@
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>-0.026</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="21">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.87</v>
+        <v>6.88</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.025373147</v>
+        <v>0.026865718</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,7 +1876,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.31</v>
+        <v>-0.309</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.186</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>9.170271</v>
+        <v>9.183619500000001</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.891</v>
@@ -1902,10 +1902,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>-0.234</v>
+        <v>-0.233</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>-0.234</v>
+        <v>-0.233</v>
       </c>
     </row>
     <row r="23">
@@ -2152,28 +2152,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.36</v>
+        <v>52.29</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.033413284</v>
+        <v>-0.034705508</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.193</v>
+        <v>-0.194</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.326</v>
+        <v>0.324</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>52.2</v>
+        <v>52.1</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.079</v>
+        <v>-0.081</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.061</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.257</v>
+        <v>-0.258</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2199,28 +2199,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.32</v>
+        <v>103.47</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.07735625</v>
+        <v>0.08703708</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.527</v>
+        <v>-0.526</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-59.4</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.282</v>
+        <v>-0.281</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.551</v>
+        <v>-0.55</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.6709999999999999</v>
+        <v>-0.67</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.22</v>
+        <v>21.21</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.9337104000000001</v>
+        <v>-0.95704913</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.405</v>
@@ -2293,28 +2293,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.31</v>
+        <v>99.19</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.025321443</v>
+        <v>-0.02645009</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.189</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.168</v>
+        <v>0.166</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>33.4</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.096</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.131</v>
+        <v>-0.132</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.263</v>
+        <v>-0.264</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2340,28 +2340,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.56</v>
+        <v>37.52</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.18671563</v>
+        <v>0.08001808000000001</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.169</v>
+        <v>0.168</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>12</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.06</v>
+        <v>0.059</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.068</v>
+        <v>0.067</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.066</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,28 +2387,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.98999999999999</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.022151582</v>
+        <v>-0.022799637</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.035</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.225</v>
+        <v>0.224</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>20.1</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.011</v>
+        <v>-0.012</v>
       </c>
       <c r="J7" s="5" t="n">
         <v>0.002</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.077</v>
+        <v>-0.078</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2434,28 +2434,28 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.8</v>
+        <v>87.51000000000001</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.68521065</v>
+        <v>0.35551056</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>-0.216</v>
+        <v>-0.218</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.223</v>
+        <v>-0.226</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>-3.2</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.07400000000000001</v>
+        <v>-0.077</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.13</v>
+        <v>-0.133</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>-0.259</v>
+        <v>-0.261</v>
       </c>
       <c r="L8" s="8" t="n">
         <v>0.66</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.9</v>
+        <v>55.73</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.04851061299999999</v>
+        <v>-0.051489387</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.095</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.323</v>
+        <v>0.319</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>38.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.09300000000000001</v>
+        <v>-0.096</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.048</v>
+        <v>-0.051</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.19</v>
+        <v>-0.192</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2528,16 +2528,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.87</v>
+        <v>26.86</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.1864323</v>
+        <v>0.14914584</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.14</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.027</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-21.9</v>
@@ -2561,12 +2561,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2575,45 +2575,45 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
+        <v>17.93</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.23718803</v>
+        <v>-0.03133441</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.08800000000000001</v>
+        <v>-0.231</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.556</v>
+        <v>-0.201</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>26</v>
+        <v>-29.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.051</v>
+        <v>-0.024</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.269</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.266</v>
+        <v>-0.444</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>1.1</v>
+        <v>2.002</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>1926430</v>
+        <v>2485880</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2622,34 +2622,34 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.93</v>
+        <v>10.49</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.031064332</v>
+        <v>-0.4743851</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-0.231</v>
+        <v>-0.095</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.2</v>
+        <v>0.545</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>-29.6</v>
+        <v>26</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.024</v>
+        <v>0.044</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.269</v>
+        <v>-0.066</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.444</v>
+        <v>-0.271</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>2.002</v>
+        <v>1.1</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>2485880</v>
+        <v>1926430</v>
       </c>
     </row>
     <row r="13">
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.68</v>
+        <v>21.52</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.010948895</v>
+        <v>-0.018248158</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.123</v>
+        <v>0.114</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.987</v>
+        <v>0.973</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>50.7</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.153</v>
+        <v>0.144</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.186</v>
+        <v>0.177</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.043</v>
+        <v>-0.05</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2766,13 +2766,13 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.6386833</v>
+        <v>0.5474491</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.266</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>6.2</v>
@@ -2810,22 +2810,22 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.5</v>
+        <v>14.51</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.010917765</v>
+        <v>-0.010231898</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.023</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.165</v>
+        <v>-0.164</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>-19.4</v>
+        <v>-19.3</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.052</v>
+        <v>0.053</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>-0.107</v>
@@ -2857,28 +2857,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.36</v>
+        <v>97</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.021162193</v>
+        <v>-0.02483162</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.017</v>
+        <v>0.013</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.215</v>
+        <v>0.211</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.026</v>
+        <v>0.022</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.013</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.145</v>
+        <v>-0.148</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2998,25 +2998,25 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.35</v>
+        <v>26.37</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.15156882</v>
+        <v>-0.075780794</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.025</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.4</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.057</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.02</v>
+        <v>-0.019</v>
       </c>
       <c r="K20" s="5" t="n">
         <v>-0.195</v>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.87</v>
+        <v>6.88</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.025373147</v>
+        <v>0.026865718</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.233</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.233</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>3.9</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.18</v>
+        <v>-0.179</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.198</v>
+        <v>-0.197</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.31</v>
+        <v>-0.309</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.36</v>
+        <v>52.29</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.402</v>
+        <v>35.355</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.280851</v>
+        <v>22.251064</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.9346485</v>
+        <v>13.916019</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.22411</v>
+        <v>22.194399</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.719705</v>
+        <v>2.716069</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.32</v>
+        <v>103.47</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.076</v>
+        <v>18.106</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.705992999999999</v>
+        <v>9.721962</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0031018</v>
+        <v>2.0063977</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1033436</v>
+        <v>1.1048921</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.22</v>
+        <v>21.21</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.563</v>
+        <v>10.56</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.902738</v>
+        <v>10.900169</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.491</v>
@@ -3473,10 +3473,10 @@
         <v>1.87</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.630093</v>
+        <v>16.626175</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7446012</v>
+        <v>1.7441903</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,16 +3505,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.31</v>
+        <v>99.19</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.356</v>
+        <v>10.344</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.627386</v>
+        <v>31.590763</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.713875</v>
+        <v>16.69452</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.398</v>
@@ -3526,10 +3526,10 @@
         <v>2.794</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.945683</v>
+        <v>-36.9029</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4508944</v>
+        <v>1.4492141</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,16 +3558,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.56</v>
+        <v>37.52</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.273</v>
+        <v>10.262</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.421055</v>
+        <v>49.368423</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.029978</v>
+        <v>16.012905</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9927716</v>
+        <v>3.9885194</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5857616</v>
+        <v>0.5851378</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.98999999999999</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.265</v>
+        <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6786346</v>
+        <v>3.6761968</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.186058</v>
+        <v>10.179308</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.429663</v>
+        <v>2.4280527</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5310643</v>
+        <v>1.5300496</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,16 +3664,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.8</v>
+        <v>87.51000000000001</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.119</v>
+        <v>6.099</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.596882</v>
+        <v>16.542534</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.824516</v>
+        <v>11.785796</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.623</v>
@@ -3685,10 +3685,10 @@
         <v>3.801</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6.0520782</v>
+        <v>6.0322604</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0913796</v>
+        <v>2.084531</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.9</v>
+        <v>55.73</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.748</v>
+        <v>5.73</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.916668</v>
+        <v>17.860577</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.011927</v>
+        <v>16.95867</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.461</v>
@@ -3738,10 +3738,10 @@
         <v>3.423</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.649496</v>
+        <v>15.600503</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.857605</v>
+        <v>2.8486588</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3770,10 +3770,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.87</v>
+        <v>26.86</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.484</v>
+        <v>5.482</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>26.189085</v>
+        <v>26.179337</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -3793,10 +3793,10 @@
         <v>2.645</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.553808</v>
+        <v>1.5532297</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.4774839</v>
+        <v>0.47730622</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>-2.42</v>
@@ -3811,12 +3811,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3825,51 +3825,51 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10.56</v>
+        <v>17.93</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.342</v>
+        <v>5.306</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>25.154762</v>
+        <v>49.805553</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>12.179937</v>
+        <v>21.760006</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>10.031</v>
+        <v>10.358</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2.101</v>
+        <v>4.075</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>7.1724367</v>
+        <v>4.738979</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>2.2800946</v>
+        <v>4.11361</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.86741</v>
+        <v>0.8239888</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>1.473</v>
+        <v>3.7835155</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3878,40 +3878,40 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>17.93</v>
+        <v>10.49</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.308</v>
+        <v>5.304</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>49.819443</v>
+        <v>24.97619</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>21.766071</v>
+        <v>12.093473</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10.358</v>
+        <v>10.031</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>4.075</v>
+        <v>2.101</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.7403</v>
+        <v>7.1215205</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>4.114757</v>
+        <v>2.2639084</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.8239888</v>
+        <v>0.86741</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>3.7835155</v>
+        <v>1.473</v>
       </c>
     </row>
     <row r="13">
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.68</v>
+        <v>21.52</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.047</v>
+        <v>5.01</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.935486</v>
+        <v>69.41936</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>29.060104</v>
+        <v>28.84564</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.718262</v>
+        <v>14.60964</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4487348</v>
+        <v>4.4159026</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -4048,13 +4048,13 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.243</v>
+        <v>2.241</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>11.98913</v>
+        <v>11.978261</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9319625</v>
+        <v>6.9256783</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.592</v>
@@ -4066,10 +4066,10 @@
         <v>2.474</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7282983</v>
+        <v>-1.7267315</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43450087</v>
+        <v>0.434107</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.5</v>
+        <v>14.51</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.936</v>
+        <v>1.938</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.378935999999999</v>
+        <v>8.384714000000001</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.223</v>
@@ -4121,10 +4121,10 @@
         <v>1.787</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.99814135</v>
+        <v>0.9988297</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27818143</v>
+        <v>0.27837327</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,16 +4153,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.36</v>
+        <v>97</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.741</v>
+        <v>1.735</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>17.930939</v>
+        <v>17.86372</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.377628</v>
+        <v>16.31623</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -4174,10 +4174,10 @@
         <v>3.111</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2267847</v>
+        <v>3.214688</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.194647</v>
+        <v>3.182671</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.35</v>
+        <v>26.37</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0.696</v>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.77686</v>
+        <v>21.793388</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.455</v>
@@ -4339,10 +4339,10 @@
         <v>1.818</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6392933</v>
+        <v>1.6405376</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.0956004</v>
+        <v>1.096432</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.87</v>
+        <v>6.88</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.186</v>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.170271</v>
+        <v>9.183619500000001</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.891</v>
@@ -4449,10 +4449,10 @@
         <v>1.684</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-11.393035</v>
+        <v>-11.409619</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.61130965</v>
+        <v>0.6121995</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -5251,12 +5251,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -5265,59 +5265,57 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>2.343</v>
+        <v>1.29</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.178</v>
+        <v>0.201</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.51058</v>
+        <v>0.26816</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.23518999</v>
+        <v>0.15614</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.09804</v>
+        <v>0.07777000000000001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.20945999</v>
+        <v>0.39339</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.32813</v>
+        <v>0.10515001</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0.23642</v>
+        <v>0.04121</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="M11" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.507</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.341</v>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>0.478</v>
+        <v>0.365</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>9.69</v>
+        <v>6.424</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>1.75</v>
+        <v>1.167</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -5326,46 +5324,48 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.29</v>
+        <v>2.343</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.201</v>
+        <v>0.178</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.26816</v>
+        <v>0.51058</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.15614</v>
+        <v>0.23518999</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.07777000000000001</v>
+        <v>0.09804</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.39339</v>
+        <v>0.20945999</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.10515001</v>
+        <v>0.32813</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0.04121</v>
+        <v>0.23642</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.507</v>
-      </c>
-      <c r="M12" s="6" t="n">
-        <v>0.341</v>
+        <v>0.491</v>
+      </c>
+      <c r="M12" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0.063</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>0.365</v>
+        <v>0.478</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>6.424</v>
+        <v>9.69</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>1.167</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="13">
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.36</v>
+        <v>52.29</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.334</v>
+        <v>0.336</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.32</v>
+        <v>103.47</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.008</v>
+        <v>1.005</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>21.22</v>
+        <v>21.21</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>99.31</v>
+        <v>99.19</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.428</v>
+        <v>0.43</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.38</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.56</v>
+        <v>37.52</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.136</v>
+        <v>0.137</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.98999999999999</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6554,7 +6554,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.138</v>
+        <v>0.139</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.91</v>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87.8</v>
+        <v>87.51000000000001</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.5429999999999999</v>
+        <v>0.5479999999999999</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.17</v>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55.9</v>
+        <v>55.73</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.305</v>
+        <v>0.309</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>4.01</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>26.87</v>
+        <v>26.86</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6722,7 +6722,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.189</v>
+        <v>0.19</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>3.37</v>
@@ -6748,16 +6748,16 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>10.56</v>
+        <v>17.93</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6765,55 +6765,57 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1.25</v>
+        <v>1.33333</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>17.375</v>
+        <v>28.808449</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>20</v>
+        <v>37.080116</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>16</v>
+        <v>22.891066</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.645</v>
+        <v>0.607</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4.72</v>
+        <v>4.54</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0.095</v>
+        <v>0.1046</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.01337</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>0.19124001</v>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>1.61</v>
+        <v>0.91643</v>
+      </c>
+      <c r="O11" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="P11" s="5" t="n">
-        <v>0.2831</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>17.93</v>
+        <v>10.49</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6821,42 +6823,40 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1.33333</v>
+        <v>1.25</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.805126</v>
+        <v>17.375</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.07584</v>
+        <v>20</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.888426</v>
+        <v>16</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.607</v>
+        <v>0.6559999999999999</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.54</v>
+        <v>4.72</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.095</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.68889</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.91643</v>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.19124001</v>
+      </c>
+      <c r="O12" s="5" t="n">
+        <v>1.61</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>0</v>
+        <v>0.2831</v>
       </c>
     </row>
     <row r="13">
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.68</v>
+        <v>21.52</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6894,7 +6894,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.149</v>
+        <v>0.157</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.89</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.5</v>
+        <v>14.51</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7066,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.318</v>
+        <v>0.317</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.3</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>97.36</v>
+        <v>97</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7126,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.106</v>
+        <v>0.11</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.64</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.35</v>
+        <v>26.37</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.87</v>
+        <v>6.88</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7414,7 +7414,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>9.81</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.402</v>
+        <v>35.355</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.280851</v>
+        <v>22.251064</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7712,7 +7712,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.193</v>
+        <v>-0.194</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.795</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.484</v>
+        <v>5.482</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7787,10 +7787,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10.356</v>
+        <v>10.344</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.627386</v>
+        <v>31.590763</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.189</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.398</v>
@@ -7833,10 +7833,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.243</v>
+        <v>2.241</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11.98913</v>
+        <v>11.978261</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.273</v>
+        <v>10.262</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.421055</v>
+        <v>49.368423</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7894,7 +7894,7 @@
         <v>0.1489</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>16.869</v>
@@ -7941,10 +7941,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.265</v>
+        <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6786346</v>
+        <v>3.6761968</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.119</v>
+        <v>6.099</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.596882</v>
+        <v>16.542534</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8000,7 +8000,7 @@
         <v>0.35709</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-0.216</v>
+        <v>-0.218</v>
       </c>
       <c r="J11" s="7" t="n">
         <v>11.623</v>
@@ -8029,10 +8029,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.748</v>
+        <v>5.73</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.916668</v>
+        <v>17.860577</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.032</v>
@@ -8044,7 +8044,7 @@
         <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.095</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="J12" s="7" t="n">
         <v>8.461</v>
@@ -8073,10 +8073,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.741</v>
+        <v>1.735</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.930939</v>
+        <v>17.86372</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.041</v>
@@ -8088,7 +8088,7 @@
         <v>0.19214001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.017</v>
+        <v>0.013</v>
       </c>
       <c r="J13" s="7" t="n">
         <v>8.893000000000001</v>
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.936</v>
+        <v>1.938</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8134,7 +8134,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.023</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.223</v>
@@ -8180,7 +8180,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.025</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.455</v>
@@ -8319,10 +8319,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.342</v>
+        <v>5.304</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>25.154762</v>
+        <v>24.97619</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8334,7 +8334,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.08800000000000001</v>
+        <v>-0.095</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.031</v>
@@ -8343,18 +8343,18 @@
         <v>7.8</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>70</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Rush Street Interactive</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -8363,46 +8363,42 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.047</v>
+        <v>5.306</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>69.935486</v>
+        <v>49.805553</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.888</v>
+        <v>0.201</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0.11229999</v>
+        <v>0.39339</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0.29505</v>
+        <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="J21" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>-0.231</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>10.358</v>
+      </c>
+      <c r="K21" s="7" t="n">
+        <v>9</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>56.7</v>
+        <v>58.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Rush Street Interactive</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -8411,31 +8407,35 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.308</v>
+        <v>5.01</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>49.819443</v>
+        <v>69.41936</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.201</v>
+        <v>0.888</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0.39339</v>
+        <v>0.11229999</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.10515001</v>
+        <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.231</v>
-      </c>
-      <c r="J22" s="7" t="n">
-        <v>10.358</v>
-      </c>
-      <c r="K22" s="7" t="n">
-        <v>9</v>
+        <v>0.114</v>
+      </c>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>55</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="23">
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.563</v>
+        <v>10.56</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.076</v>
+        <v>18.106</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8518,7 +8518,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.527</v>
+        <v>-0.526</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>13.981</v>
@@ -8722,7 +8722,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.233</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.891</v>
@@ -9763,55 +9763,55 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.01337</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.19124001</v>
+        <v>0.91643</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4.72</v>
+        <v>4.54</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.095</v>
+        <v>0.1046</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>14945381</v>
+        <v>10753999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.68889</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.91643</v>
+        <v>0.19124001</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4.54</v>
+        <v>4.72</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.095</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>10753999</v>
+        <v>14945381</v>
       </c>
     </row>
     <row r="13">
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1293.93</v>
+        <v>1293.49</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1218.79</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1286.37</v>
+        <v>1285.94</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1209.76</v>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1291.19</v>
+        <v>1290.78</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1211.98</v>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1292.1</v>
+        <v>1291.68</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1220.05</v>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1277.03</v>
+        <v>1276.62</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1227.31</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1228.37</v>
+        <v>1228</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1223.35</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1253.79</v>
+        <v>1253.41</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1223.23</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1224.54</v>
+        <v>1224.16</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1231.32</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1220.2</v>
+        <v>1219.82</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1233.25</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1212.24</v>
+        <v>1211.87</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1230.78</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1209.87</v>
+        <v>1209.49</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1224.74</v>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1229.33</v>
+        <v>1228.93</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1228.07</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1192.22</v>
+        <v>1191.81</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1227.04</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1168.07</v>
+        <v>1167.67</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1202.06</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1174.65</v>
+        <v>1174.24</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.94</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1179.84</v>
+        <v>1179.45</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1222.29</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1164.5</v>
+        <v>1164.11</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1222.73</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1170.32</v>
+        <v>1169.93</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1228.94</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1157</v>
+        <v>1156.59</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1233.84</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1158.6</v>
+        <v>1158.2</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1233.71</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1106.15</v>
+        <v>1105.73</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1231.26</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1094.29</v>
+        <v>1093.88</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1227.59</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1112.55</v>
+        <v>1112.12</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1233.69</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1108.9</v>
+        <v>1108.49</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1223.26</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1130.52</v>
+        <v>1130.1</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1217.34</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1105.38</v>
+        <v>1104.97</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1202.13</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1132.7</v>
+        <v>1132.26</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1225.2</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1134.64</v>
+        <v>1134.21</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1231.1</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1131.48</v>
+        <v>1131.06</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1227.86</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1116.5</v>
+        <v>1116.08</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1227.57</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1078.77</v>
+        <v>1078.37</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1208.61</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1069.17</v>
+        <v>1068.72</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1209.46</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1084.3</v>
+        <v>1083.81</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1211.41</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1118.69</v>
+        <v>1118.18</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1217.51</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1113.61</v>
+        <v>1113.09</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1214.3</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1113.78</v>
+        <v>1113.24</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1223.09</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1069.77</v>
+        <v>1069.23</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1210.6</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1084.67</v>
+        <v>1084.1</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1219.4</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1088.84</v>
+        <v>1088.25</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1229.68</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1118.45</v>
+        <v>1117.87</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1222.85</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1105.49</v>
+        <v>1104.89</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1216.98</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1100.25</v>
+        <v>1099.63</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.67</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1096.31</v>
+        <v>1095.7</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1206.94</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1112.07</v>
+        <v>1111.45</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1215.46</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1109.81</v>
+        <v>1109.2</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1208.68</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1077.58</v>
+        <v>1076.99</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1192.84</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1079.05</v>
+        <v>1078.45</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.29</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1078.01</v>
+        <v>1077.4</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1201.35</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1093.19</v>
+        <v>1092.58</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1199.85</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1078.63</v>
+        <v>1078.02</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1181.63</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1080.54</v>
+        <v>1079.94</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1174.94</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1072.87</v>
+        <v>1072.28</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1186.89</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1085.43</v>
+        <v>1084.83</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1190.02</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1077.32</v>
+        <v>1076.72</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1173.41</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1090.23</v>
+        <v>1089.61</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1170.52</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1061.41</v>
+        <v>1060.8</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1153.74</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1083.9</v>
+        <v>1083.27</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1165.85</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1094.98</v>
+        <v>1094.33</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1161.94</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1080.77</v>
+        <v>1080.12</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1168.42</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1059.88</v>
+        <v>1057.39</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1059.88</v>
+        <v>1057.39</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-17.91%</t>
+          <t>-18.08%</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>135.8</v>
+        <v>135.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 14:56
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.29</v>
+        <v>52.28</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.034705508</v>
+        <v>-0.03489015</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -673,16 +673,16 @@
         <v>-0.258</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.355</v>
+        <v>35.348</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.251064</v>
+        <v>22.246809</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.916019</v>
+        <v>13.913358</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.47</v>
+        <v>103.75</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>0.08703708</v>
+        <v>0.3384898</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.67</v>
+        <v>-0.669</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.106</v>
+        <v>18.151</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.721962</v>
+        <v>9.746387500000001</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -755,10 +755,10 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5610000000000001</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>-0.526</v>
+        <v>-0.525</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.21</v>
+        <v>21.32</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.95704913</v>
+        <v>-0.49019393</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>20.89</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.5649999999999999</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.56</v>
+        <v>10.61</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>11.322</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.900169</v>
+        <v>10.95155</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.491</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>-0.4370000000000001</v>
+        <v>-0.434</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>-0.405</v>
+        <v>-0.402</v>
       </c>
     </row>
     <row r="5">
@@ -842,7 +842,7 @@
         <v>99.19</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.02645009</v>
+        <v>-0.026499135</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -860,10 +860,10 @@
         <v>19.942</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.590763</v>
+        <v>31.589172</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.69452</v>
+        <v>16.69368</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.398</v>
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.52</v>
+        <v>37.55</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.08001808000000001</v>
+        <v>0.17337589</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.066</v>
+        <v>-0.065</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.262</v>
+        <v>10.272</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.368423</v>
+        <v>49.414474</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.012905</v>
+        <v>16.027843</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.94</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.022799637</v>
+        <v>-0.022858517</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -978,10 +978,10 @@
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6761968</v>
+        <v>3.6759753</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.179308</v>
+        <v>10.178695</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.51000000000001</v>
+        <v>87.55</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.35551056</v>
+        <v>0.40138316</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1031,16 +1031,16 @@
         <v>-0.261</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.099</v>
+        <v>6.102</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>11.12</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.542534</v>
+        <v>16.550095</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.785796</v>
+        <v>11.791183</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.623</v>
@@ -1052,7 +1052,7 @@
         <v>0.66</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>-0.226</v>
+        <v>-0.225</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>-0.218</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.73</v>
+        <v>55.94</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.051489387</v>
+        <v>-0.04782981</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,19 +1087,19 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.192</v>
+        <v>-0.189</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.73</v>
+        <v>5.752</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.886</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.860577</v>
+        <v>17.929487</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>16.95867</v>
+        <v>17.0241</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.461</v>
@@ -1111,10 +1111,10 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.319</v>
+        <v>0.324</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.09699999999999999</v>
+        <v>-0.094</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.86</v>
+        <v>26.88</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.14914584</v>
+        <v>0.22371165</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1149,7 +1149,7 @@
         <v>-0.149</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.482</v>
+        <v>5.486</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>30.375</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>26.179337</v>
+        <v>26.19883</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -1172,10 +1172,10 @@
         <v>1.977</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>-0.027</v>
+        <v>-0.026</v>
       </c>
       <c r="Q10" s="9" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
     </row>
     <row r="11">
@@ -1195,10 +1195,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-0.03133441</v>
+        <v>-0.028363025</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>32.22</v>
@@ -1207,19 +1207,19 @@
         <v>15.725</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.444</v>
+        <v>-0.442</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.306</v>
+        <v>5.323</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>5.256</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>49.805553</v>
+        <v>49.958332</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>21.760006</v>
+        <v>21.826754</v>
       </c>
       <c r="M11" s="7" t="n">
         <v>10.358</v>
@@ -1231,10 +1231,10 @@
         <v>2.002</v>
       </c>
       <c r="P11" s="4" t="n">
-        <v>-0.201</v>
+        <v>-0.198</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>-0.231</v>
+        <v>-0.229</v>
       </c>
     </row>
     <row r="12">
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.49</v>
+        <v>10.48</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.4743851</v>
+        <v>-0.52182454</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>14.38</v>
@@ -1269,16 +1269,16 @@
         <v>-0.271</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.304</v>
+        <v>5.302</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>4.922</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>24.97619</v>
+        <v>24.964285</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>12.093473</v>
+        <v>12.087708</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>10.031</v>
@@ -1290,7 +1290,7 @@
         <v>1.1</v>
       </c>
       <c r="P12" s="9" t="n">
-        <v>0.545</v>
+        <v>0.544</v>
       </c>
       <c r="Q12" s="4" t="n">
         <v>-0.095</v>
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.52</v>
+        <v>21.55</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.018248158</v>
+        <v>-0.016651449</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.049</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.01</v>
+        <v>5.018</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.41936</v>
+        <v>69.53225999999999</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>28.84564</v>
+        <v>28.892553</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.973</v>
+        <v>0.976</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.114</v>
+        <v>0.116</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.5795967</v>
+        <v>-0.50231516</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.307</v>
+        <v>-0.306</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.374</v>
+        <v>2.376</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.956</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>11.939231</v>
+        <v>11.948512</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.753</v>
@@ -1416,7 +1416,7 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.036</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>-0.144</v>
@@ -1442,7 +1442,7 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.5474491</v>
+        <v>0.6386833</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1454,16 +1454,16 @@
         <v>-0.457</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.241</v>
+        <v>2.243</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.774</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>11.978261</v>
+        <v>11.98913</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9256783</v>
+        <v>6.9319625</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.592</v>
@@ -1475,7 +1475,7 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="Q15" s="4" t="n">
         <v>-0.266</v>
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.010231898</v>
+        <v>-0.011937257</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,10 +1510,10 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.297</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.938</v>
+        <v>1.934</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.438</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.384714000000001</v>
+        <v>8.370267999999999</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.223</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-0.164</v>
+        <v>-0.166</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.023</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97</v>
+        <v>97.31</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.02483162</v>
+        <v>-0.021765366</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,19 +1571,19 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.148</v>
+        <v>-0.146</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.735</v>
+        <v>1.74</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.696</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>17.86372</v>
+        <v>17.91989</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.31623</v>
+        <v>16.367535</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.211</v>
+        <v>0.215</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="18">
@@ -1621,7 +1621,7 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-0.04130436000000001</v>
+        <v>-0.04239124</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1633,7 +1633,7 @@
         <v>-0.679</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.134</v>
+        <v>1.133</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.883</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.454545</v>
+        <v>4.4494953</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.324</v>
@@ -1658,7 +1658,7 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>-0.585</v>
+        <v>-0.586</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>-0.591</v>
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-0.075780794</v>
+        <v>-0.113674805</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.793388</v>
+        <v>21.785124</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.455</v>
@@ -1781,7 +1781,7 @@
         <v>0.003</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
     </row>
     <row r="21">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.88</v>
+        <v>6.89</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.026865718</v>
+        <v>0.028358219</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,7 +1876,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.309</v>
+        <v>-0.308</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.186</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>9.183619500000001</v>
+        <v>9.196967000000001</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.891</v>
@@ -1902,10 +1902,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>-0.233</v>
+        <v>-0.232</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>-0.233</v>
+        <v>-0.232</v>
       </c>
     </row>
     <row r="23">
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-0.0130869</v>
+        <v>-0.87466025</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1937,7 +1937,7 @@
         <v>2.02</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.539</v>
       </c>
       <c r="I23" s="6" t="n">
         <v>0.082</v>
@@ -1951,7 +1951,7 @@
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>-5.5363417</v>
+        <v>-5.5609756</v>
       </c>
       <c r="M23" s="7" t="n">
         <v>12.524</v>
@@ -1963,10 +1963,10 @@
         <v>1.327</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>-0.457</v>
+        <v>-0.455</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>-0.092</v>
+        <v>-0.08800000000000001</v>
       </c>
     </row>
     <row r="24">
@@ -2152,10 +2152,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.29</v>
+        <v>52.28</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.034705508</v>
+        <v>-0.03489015</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>-0.194</v>
@@ -2170,7 +2170,7 @@
         <v>-0.081</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.062</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>-0.258</v>
@@ -2199,28 +2199,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.47</v>
+        <v>103.75</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.08703708</v>
+        <v>0.3384898</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.526</v>
+        <v>-0.525</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5610000000000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-59.4</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.281</v>
+        <v>-0.279</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.55</v>
+        <v>-0.5489999999999999</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.67</v>
+        <v>-0.669</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2246,28 +2246,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.21</v>
+        <v>21.32</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.95704913</v>
+        <v>-0.49019393</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.402</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.4370000000000001</v>
+        <v>-0.434</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-37.5</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.219</v>
+        <v>-0.215</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.406</v>
+        <v>-0.403</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.5649999999999999</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2296,7 +2296,7 @@
         <v>99.19</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.02645009</v>
+        <v>-0.026499135</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.189</v>
@@ -2340,16 +2340,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.52</v>
+        <v>37.55</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.08001808000000001</v>
+        <v>0.17337589</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.168</v>
+        <v>0.169</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>12</v>
@@ -2358,10 +2358,10 @@
         <v>0.059</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.067</v>
+        <v>0.068</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.066</v>
+        <v>-0.065</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,10 +2387,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.94</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.022799637</v>
+        <v>-0.022858517</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>-0.035</v>
@@ -2434,16 +2434,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.51000000000001</v>
+        <v>87.55</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.35551056</v>
+        <v>0.40138316</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.218</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.226</v>
+        <v>-0.225</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>-3.2</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.73</v>
+        <v>55.94</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.051489387</v>
+        <v>-0.04782981</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.09699999999999999</v>
+        <v>-0.094</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.319</v>
+        <v>0.324</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>38.2</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.096</v>
+        <v>-0.092</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.051</v>
+        <v>-0.047</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.192</v>
+        <v>-0.189</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2528,16 +2528,16 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.86</v>
+        <v>26.88</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.14914584</v>
+        <v>0.22371165</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.026</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-21.9</v>
@@ -2546,7 +2546,7 @@
         <v>0.146</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.08900000000000001</v>
+        <v>0.09</v>
       </c>
       <c r="K10" s="5" t="n">
         <v>-0.149</v>
@@ -2575,28 +2575,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>-0.03133441</v>
+        <v>-0.028363025</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.231</v>
+        <v>-0.229</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>-0.201</v>
+        <v>-0.198</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>-29.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-0.024</v>
+        <v>-0.022</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.269</v>
+        <v>-0.267</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.444</v>
+        <v>-0.442</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>2.002</v>
@@ -2622,25 +2622,25 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.49</v>
+        <v>10.48</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.4743851</v>
+        <v>-0.52182454</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>-0.095</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.545</v>
+        <v>0.544</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.044</v>
+        <v>0.043</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.066</v>
+        <v>-0.067</v>
       </c>
       <c r="K12" s="5" t="n">
         <v>-0.271</v>
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.52</v>
+        <v>21.55</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.018248158</v>
+        <v>-0.016651449</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.114</v>
+        <v>0.116</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.973</v>
+        <v>0.976</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>50.7</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.144</v>
+        <v>0.146</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.177</v>
+        <v>0.179</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.049</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2716,16 +2716,16 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.5795967</v>
+        <v>-0.50231516</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>-0.144</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.03700000000000001</v>
+        <v>-0.036</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>12.6</v>
@@ -2734,10 +2734,10 @@
         <v>-0.066</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.167</v>
+        <v>-0.166</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.307</v>
+        <v>-0.306</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2766,13 +2766,13 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.5474491</v>
+        <v>0.6386833</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.266</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.024</v>
+        <v>0.025</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>6.2</v>
@@ -2810,28 +2810,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.010231898</v>
+        <v>-0.011937257</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.023</v>
+        <v>-0.025</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.164</v>
+        <v>-0.166</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>-19.3</v>
+        <v>-19.4</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.053</v>
+        <v>0.051</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.107</v>
+        <v>-0.109</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.297</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2857,28 +2857,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97</v>
+        <v>97.31</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.02483162</v>
+        <v>-0.021765366</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.013</v>
+        <v>0.016</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.211</v>
+        <v>0.215</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>20.2</v>
+        <v>20.3</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.022</v>
+        <v>0.026</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.012</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.148</v>
+        <v>-0.146</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2907,13 +2907,13 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.04130436000000001</v>
+        <v>-0.04239124</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>-0.591</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.585</v>
+        <v>-0.586</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-34.5</v>
@@ -2998,13 +2998,13 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.075780794</v>
+        <v>-0.113674805</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>0.003</v>
@@ -3013,7 +3013,7 @@
         <v>5.4</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.057</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>-0.019</v>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.88</v>
+        <v>6.89</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.026865718</v>
+        <v>0.028358219</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.232</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.232</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>3.9</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.179</v>
+        <v>-0.177</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.197</v>
+        <v>-0.195</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.309</v>
+        <v>-0.308</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3141,28 +3141,28 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.0130869</v>
+        <v>-0.87466025</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-0.457</v>
+        <v>-0.455</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>-52.6</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.05599999999999999</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.26</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.539</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>1.327</v>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.29</v>
+        <v>52.28</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.355</v>
+        <v>35.348</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.251064</v>
+        <v>22.246809</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.916019</v>
+        <v>13.913358</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.194399</v>
+        <v>22.190153</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.716069</v>
+        <v>2.7155495</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.47</v>
+        <v>103.75</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.106</v>
+        <v>18.151</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.721962</v>
+        <v>9.746387500000001</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0063977</v>
+        <v>2.0114384</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1048921</v>
+        <v>1.1079355</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.21</v>
+        <v>21.32</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.56</v>
+        <v>10.61</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.900169</v>
+        <v>10.95155</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.491</v>
@@ -3473,10 +3473,10 @@
         <v>1.87</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.626175</v>
+        <v>16.704546</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7441903</v>
+        <v>1.7524118</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3511,10 +3511,10 @@
         <v>10.344</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.590763</v>
+        <v>31.589172</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.69452</v>
+        <v>16.69368</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.398</v>
@@ -3526,10 +3526,10 @@
         <v>2.794</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.9029</v>
+        <v>-36.901043</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4492141</v>
+        <v>1.4491411</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,16 +3558,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.52</v>
+        <v>37.55</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.262</v>
+        <v>10.272</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.368423</v>
+        <v>49.414474</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.012905</v>
+        <v>16.027843</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9885194</v>
+        <v>3.99224</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5851378</v>
+        <v>0.5856836399999999</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.94</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6761968</v>
+        <v>3.6759753</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.179308</v>
+        <v>10.178695</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4280527</v>
+        <v>2.4279063</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5300496</v>
+        <v>1.5299574</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,16 +3664,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.51000000000001</v>
+        <v>87.55</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.099</v>
+        <v>6.102</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.542534</v>
+        <v>16.550095</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.785796</v>
+        <v>11.791183</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.623</v>
@@ -3685,10 +3685,10 @@
         <v>3.801</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6.0322604</v>
+        <v>6.035018</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.084531</v>
+        <v>2.085484</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.73</v>
+        <v>55.94</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.73</v>
+        <v>5.752</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.860577</v>
+        <v>17.929487</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>16.95867</v>
+        <v>17.0241</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.461</v>
@@ -3738,10 +3738,10 @@
         <v>3.423</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.600503</v>
+        <v>15.660694</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.8486588</v>
+        <v>2.8596494</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3770,10 +3770,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.86</v>
+        <v>26.88</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.482</v>
+        <v>5.486</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>26.179337</v>
+        <v>26.19883</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -3793,10 +3793,10 @@
         <v>2.645</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.5532297</v>
+        <v>1.5543861</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.47730622</v>
+        <v>0.47766158</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>-2.42</v>
@@ -3825,16 +3825,16 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.306</v>
+        <v>5.323</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>49.805553</v>
+        <v>49.958332</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>21.760006</v>
+        <v>21.826754</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>10.358</v>
@@ -3846,10 +3846,10 @@
         <v>4.075</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4.738979</v>
+        <v>4.7535157</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>4.11361</v>
+        <v>4.1262283</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>0.36</v>
@@ -3878,16 +3878,16 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.49</v>
+        <v>10.48</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.304</v>
+        <v>5.302</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>24.97619</v>
+        <v>24.964285</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>12.093473</v>
+        <v>12.087708</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>10.031</v>
@@ -3899,10 +3899,10 @@
         <v>2.101</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.1215205</v>
+        <v>7.118126</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>2.2639084</v>
+        <v>2.2628293</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0.42</v>
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.52</v>
+        <v>21.55</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.01</v>
+        <v>5.018</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.41936</v>
+        <v>69.53225999999999</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>28.84564</v>
+        <v>28.892553</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.60964</v>
+        <v>14.633401</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4159026</v>
+        <v>4.4230847</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.374</v>
+        <v>2.376</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11.939231</v>
+        <v>11.948512</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.753</v>
@@ -4013,10 +4013,10 @@
         <v>2.372</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7471704</v>
+        <v>2.749306</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.94542426</v>
+        <v>0.94615924</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4048,13 +4048,13 @@
         <v>5.51</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.241</v>
+        <v>2.243</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>11.978261</v>
+        <v>11.98913</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9256783</v>
+        <v>6.9319625</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.592</v>
@@ -4066,10 +4066,10 @@
         <v>2.474</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7267315</v>
+        <v>-1.7282983</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.434107</v>
+        <v>0.43450087</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.48</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.938</v>
+        <v>1.934</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.384714000000001</v>
+        <v>8.370267999999999</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.223</v>
@@ -4121,10 +4121,10 @@
         <v>1.787</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.9988297</v>
+        <v>0.99710876</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27837327</v>
+        <v>0.27789366</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,16 +4153,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97</v>
+        <v>97.31</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.735</v>
+        <v>1.74</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>17.86372</v>
+        <v>17.91989</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.31623</v>
+        <v>16.367535</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -4174,10 +4174,10 @@
         <v>3.111</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.214688</v>
+        <v>3.2247963</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.182671</v>
+        <v>3.1926787</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4209,7 +4209,7 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.134</v>
+        <v>1.133</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.454545</v>
+        <v>4.4494953</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.324</v>
@@ -4231,10 +4231,10 @@
         <v>1.319</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.4994899</v>
+        <v>1.49779</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.694536</v>
+        <v>1.6926149</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4316,7 +4316,7 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.36</v>
       </c>
       <c r="E20" s="6" t="n">
         <v>0.696</v>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.793388</v>
+        <v>21.785124</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.455</v>
@@ -4339,10 +4339,10 @@
         <v>1.818</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6405376</v>
+        <v>1.6399155</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.096432</v>
+        <v>1.0960162</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.88</v>
+        <v>6.89</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.186</v>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.183619500000001</v>
+        <v>9.196967000000001</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.891</v>
@@ -4449,10 +4449,10 @@
         <v>1.684</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-11.409619</v>
+        <v>-11.426203</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.6121995</v>
+        <v>0.61308926</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -4481,7 +4481,7 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="E23" s="6" t="n">
         <v>0.082</v>
@@ -4492,7 +4492,7 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5.5363417</v>
+        <v>-5.5609756</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>12.524</v>
@@ -4504,10 +4504,10 @@
         <v>1.909</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>32.427143</v>
+        <v>32.571426</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.27162194</v>
+        <v>0.27283052</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>-1.12</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.29</v>
+        <v>52.28</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.336</v>
+        <v>0.337</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.47</v>
+        <v>103.75</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.005</v>
+        <v>0.9990000000000001</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>21.21</v>
+        <v>21.32</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.705</v>
+        <v>0.6970000000000001</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.52</v>
+        <v>37.55</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.137</v>
+        <v>0.136</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.94</v>
+        <v>82.93000000000001</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87.51000000000001</v>
+        <v>87.55</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55.73</v>
+        <v>55.94</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.309</v>
+        <v>0.304</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>4.01</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>26.86</v>
+        <v>26.88</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6722,7 +6722,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.19</v>
+        <v>0.189</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>3.37</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>17.93</v>
+        <v>17.98</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>22.891066</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.607</v>
+        <v>0.602</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>4.54</v>
@@ -6815,7 +6815,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>10.49</v>
+        <v>10.48</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6838,7 +6838,7 @@
         <v>16</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.6559999999999999</v>
+        <v>0.6579999999999999</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.72</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.52</v>
+        <v>21.55</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6894,7 +6894,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.157</v>
+        <v>0.156</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.89</v>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6952,7 +6952,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.405</v>
+        <v>0.404</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.58</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.51</v>
+        <v>14.48</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7066,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.317</v>
+        <v>0.32</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.3</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>97</v>
+        <v>97.31</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7126,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.11</v>
+        <v>0.106</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.64</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.36</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.88</v>
+        <v>6.89</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7414,7 +7414,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>9.81</v>
@@ -7449,7 +7449,7 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2.27</v>
+        <v>2.28</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -7472,7 +7472,7 @@
         <v>2.5</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>0.4320000000000001</v>
+        <v>0.425</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>5.74</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.355</v>
+        <v>35.348</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.251064</v>
+        <v>22.246809</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.482</v>
+        <v>5.486</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7758,7 +7758,7 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.14</v>
+        <v>0.141</v>
       </c>
       <c r="J4" s="7" t="n">
         <v>8.691000000000001</v>
@@ -7790,7 +7790,7 @@
         <v>10.344</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.590763</v>
+        <v>31.589172</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7833,10 +7833,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.241</v>
+        <v>2.243</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11.978261</v>
+        <v>11.98913</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.262</v>
+        <v>10.272</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.368423</v>
+        <v>49.414474</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7894,7 +7894,7 @@
         <v>0.1489</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.028</v>
+        <v>0.029</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>16.869</v>
@@ -7944,7 +7944,7 @@
         <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6761968</v>
+        <v>3.6759753</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.099</v>
+        <v>6.102</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.542534</v>
+        <v>16.550095</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8015,12 +8015,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Monarch Casino &amp; Resort</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -8029,42 +8029,42 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.73</v>
+        <v>1.74</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.860577</v>
+        <v>17.91989</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.032</v>
+        <v>0.041</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.4046</v>
+        <v>0.34986</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>1.113</v>
+        <v>0.19214001</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.09699999999999999</v>
+        <v>0.016</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.461</v>
+        <v>8.893000000000001</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>60.3</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MCRI</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Monarch Casino &amp; Resort</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -8073,31 +8073,31 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.735</v>
+        <v>5.752</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.86372</v>
+        <v>17.929487</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.041</v>
+        <v>0.032</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.34986</v>
+        <v>0.4046</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.19214001</v>
+        <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.013</v>
+        <v>-0.094</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.893000000000001</v>
+        <v>8.461</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>57.1</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="14">
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.938</v>
+        <v>1.934</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8134,7 +8134,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.023</v>
+        <v>-0.025</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.223</v>
@@ -8180,7 +8180,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.026</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.455</v>
@@ -8272,7 +8272,7 @@
         <v>-1.8681101</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.08800000000000001</v>
       </c>
       <c r="J17" s="7" t="n">
         <v>12.524</v>
@@ -8319,10 +8319,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.304</v>
+        <v>5.302</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>24.97619</v>
+        <v>24.964285</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8363,10 +8363,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.306</v>
+        <v>5.323</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>49.805553</v>
+        <v>49.958332</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.201</v>
@@ -8378,7 +8378,7 @@
         <v>0.10515001</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.231</v>
+        <v>-0.229</v>
       </c>
       <c r="J21" s="7" t="n">
         <v>10.358</v>
@@ -8407,10 +8407,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.01</v>
+        <v>5.018</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>69.41936</v>
+        <v>69.53225999999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.888</v>
@@ -8422,7 +8422,7 @@
         <v>0.29505</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.114</v>
+        <v>0.116</v>
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.56</v>
+        <v>10.61</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.405</v>
+        <v>-0.402</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>41.491</v>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.106</v>
+        <v>18.151</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8518,7 +8518,7 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.526</v>
+        <v>-0.525</v>
       </c>
       <c r="J24" s="7" t="n">
         <v>13.981</v>
@@ -8547,7 +8547,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.134</v>
+        <v>1.133</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.374</v>
+        <v>2.376</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8722,7 +8722,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.232</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.891</v>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1293.49</v>
+        <v>1293.21</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1218.79</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1285.94</v>
+        <v>1285.65</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1209.76</v>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1290.78</v>
+        <v>1290.51</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1211.98</v>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1291.68</v>
+        <v>1291.41</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1220.05</v>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1276.62</v>
+        <v>1276.35</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1227.31</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1228</v>
+        <v>1227.75</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1223.35</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1253.41</v>
+        <v>1253.18</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1223.23</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1224.16</v>
+        <v>1223.94</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1231.32</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1219.82</v>
+        <v>1219.58</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1233.25</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1211.87</v>
+        <v>1211.63</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1230.78</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1209.49</v>
+        <v>1209.25</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1224.74</v>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1228.93</v>
+        <v>1228.69</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1228.07</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1191.81</v>
+        <v>1191.55</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1227.04</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1167.67</v>
+        <v>1167.42</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1202.06</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1174.24</v>
+        <v>1173.97</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1215.94</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1179.45</v>
+        <v>1179.17</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1222.29</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1164.11</v>
+        <v>1163.81</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1222.73</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1169.93</v>
+        <v>1169.64</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1228.94</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1156.59</v>
+        <v>1156.3</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1233.84</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1158.2</v>
+        <v>1157.9</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1233.71</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1105.73</v>
+        <v>1105.51</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1231.26</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1093.88</v>
+        <v>1093.64</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1227.59</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1112.12</v>
+        <v>1111.87</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1233.69</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1108.49</v>
+        <v>1108.21</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1223.26</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1130.1</v>
+        <v>1129.81</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1217.34</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1104.97</v>
+        <v>1104.67</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1202.13</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1132.26</v>
+        <v>1131.97</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1225.2</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1134.21</v>
+        <v>1133.93</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1231.1</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1131.06</v>
+        <v>1130.77</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1227.86</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1116.08</v>
+        <v>1115.79</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1227.57</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1078.37</v>
+        <v>1078.07</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1208.61</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1068.72</v>
+        <v>1068.38</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1209.46</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1083.81</v>
+        <v>1083.47</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1211.41</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1118.18</v>
+        <v>1117.83</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1217.51</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1113.09</v>
+        <v>1112.74</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1214.3</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1113.24</v>
+        <v>1112.88</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1223.09</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1069.23</v>
+        <v>1068.89</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1210.6</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1084.1</v>
+        <v>1083.77</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1219.4</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1088.25</v>
+        <v>1087.92</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1229.68</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1117.87</v>
+        <v>1117.53</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1222.85</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1104.89</v>
+        <v>1104.53</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1216.98</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1099.63</v>
+        <v>1099.29</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1217.67</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1095.7</v>
+        <v>1095.37</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1206.94</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1111.45</v>
+        <v>1111.11</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1215.46</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1109.2</v>
+        <v>1108.88</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1208.68</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1076.99</v>
+        <v>1076.68</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1192.84</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1078.45</v>
+        <v>1078.14</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1203.29</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1077.4</v>
+        <v>1077.08</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1201.35</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1092.58</v>
+        <v>1092.27</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1199.85</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1078.02</v>
+        <v>1077.72</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1181.63</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1079.94</v>
+        <v>1079.64</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1174.94</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1072.28</v>
+        <v>1071.97</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1186.89</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1084.83</v>
+        <v>1084.52</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1190.02</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1076.72</v>
+        <v>1076.41</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1173.41</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1089.61</v>
+        <v>1089.3</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1170.52</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1060.8</v>
+        <v>1060.5</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1153.74</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1083.27</v>
+        <v>1082.96</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1165.85</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1094.33</v>
+        <v>1094</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1161.94</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1080.12</v>
+        <v>1079.78</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1168.42</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1057.39</v>
+        <v>1057.51</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1057.39</v>
+        <v>1057.51</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-18.08%</t>
+          <t>-18.05%</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>135.7</v>
+        <v>135.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:07
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.28</v>
+        <v>52.41</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.03489015</v>
+        <v>-0.0325826</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -670,19 +670,19 @@
         <v>30.18</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>-0.258</v>
+        <v>-0.256</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.348</v>
+        <v>35.433</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.246809</v>
+        <v>22.300001</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.913358</v>
+        <v>13.946625</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -694,10 +694,10 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.324</v>
+        <v>0.327</v>
       </c>
       <c r="Q2" s="4" t="n">
-        <v>-0.194</v>
+        <v>-0.192</v>
       </c>
     </row>
     <row r="3">
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.75</v>
+        <v>103.63</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>0.3384898</v>
+        <v>0.22243302</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -729,10 +729,10 @@
         <v>99.95999999999999</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.669</v>
+        <v>-0.67</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.151</v>
+        <v>18.13</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.746387500000001</v>
+        <v>9.735113999999999</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -755,7 +755,7 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="Q3" s="4" t="n">
         <v>-0.525</v>
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.32</v>
+        <v>21.27</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.49019393</v>
+        <v>-0.70027834</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,10 +790,10 @@
         <v>20.89</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.61</v>
+        <v>10.588</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>11.322</v>
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.95155</v>
+        <v>10.928429</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.491</v>
@@ -816,10 +816,10 @@
         <v>1.682</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>-0.434</v>
+        <v>-0.426</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>-0.402</v>
+        <v>-0.404</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.19</v>
+        <v>99.47</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.026499135</v>
+        <v>-0.023751085</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,19 +851,19 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.262</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.344</v>
+        <v>10.373</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>19.942</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.589172</v>
+        <v>31.678343</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.69368</v>
+        <v>16.740803</v>
       </c>
       <c r="M5" s="7" t="n">
         <v>11.398</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.166</v>
+        <v>0.165</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>-0.189</v>
+        <v>-0.187</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.55</v>
+        <v>37.58</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.17337589</v>
+        <v>0.24006441</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,19 +910,19 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.064</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.272</v>
+        <v>10.278</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.414474</v>
+        <v>49.447372</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.027843</v>
+        <v>16.038513</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -934,10 +934,10 @@
         <v>1.396</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.169</v>
+        <v>0.189</v>
       </c>
       <c r="Q6" s="9" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.92</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.022858517</v>
+        <v>-0.02297637</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.078</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.261</v>
+        <v>6.26</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6755319</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.178695</v>
+        <v>10.177466</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -993,10 +993,10 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.224</v>
+        <v>0.235</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>-0.035</v>
+        <v>-0.036</v>
       </c>
     </row>
     <row r="8">
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.55</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.40138316</v>
+        <v>0.4243151000000001</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1031,16 +1031,16 @@
         <v>-0.261</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>6.102</v>
+        <v>6.103</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>11.12</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.550095</v>
+        <v>16.553875</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.791183</v>
+        <v>11.793877</v>
       </c>
       <c r="M8" s="7" t="n">
         <v>11.623</v>
@@ -1052,7 +1052,7 @@
         <v>0.66</v>
       </c>
       <c r="P8" s="4" t="n">
-        <v>-0.225</v>
+        <v>-0.218</v>
       </c>
       <c r="Q8" s="4" t="n">
         <v>-0.218</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.94</v>
+        <v>55.74</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.04782981</v>
+        <v>-0.051234016</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,19 +1087,19 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.192</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.752</v>
+        <v>5.732</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>6.886</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.929487</v>
+        <v>17.865385</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>17.0241</v>
+        <v>16.963236</v>
       </c>
       <c r="M9" s="7" t="n">
         <v>8.461</v>
@@ -1111,10 +1111,10 @@
         <v>1.453</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.324</v>
+        <v>0.325</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.094</v>
+        <v>-0.09699999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.88</v>
+        <v>26.89</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.22371165</v>
+        <v>0.26099813</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1149,7 +1149,7 @@
         <v>-0.149</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>5.486</v>
+        <v>5.488</v>
       </c>
       <c r="J10" s="6" t="n">
         <v>30.375</v>
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="L10" s="7" t="n">
-        <v>26.19883</v>
+        <v>26.208576</v>
       </c>
       <c r="M10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -1172,7 +1172,7 @@
         <v>1.977</v>
       </c>
       <c r="P10" s="4" t="n">
-        <v>-0.026</v>
+        <v>-0.004</v>
       </c>
       <c r="Q10" s="9" t="n">
         <v>0.141</v>
@@ -1181,12 +1181,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1195,57 +1195,57 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.98</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>-0.028363025</v>
+        <v>10.54</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>32.22</v>
+        <v>14.38</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>15.725</v>
+        <v>5.59</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.442</v>
+        <v>-0.267</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.323</v>
+        <v>5.329</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>5.256</v>
+        <v>4.922</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>49.958332</v>
+        <v>25.09524</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>21.826754</v>
+        <v>12.151116</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>10.358</v>
+        <v>10.031</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>2.002</v>
-      </c>
-      <c r="P11" s="4" t="n">
-        <v>-0.198</v>
+        <v>1.1</v>
+      </c>
+      <c r="P11" s="9" t="n">
+        <v>0.578</v>
       </c>
       <c r="Q11" s="4" t="n">
-        <v>-0.229</v>
+        <v>-0.09</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1254,46 +1254,46 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.48</v>
+        <v>18</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.52182454</v>
+        <v>-0.027552686</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>14.38</v>
+        <v>32.22</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>5.59</v>
+        <v>15.725</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.271</v>
+        <v>-0.441</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>5.302</v>
+        <v>5.327</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>4.922</v>
+        <v>5.256</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>24.964285</v>
+        <v>49.999996</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>12.087708</v>
+        <v>21.844957</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>10.031</v>
+        <v>10.358</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="P12" s="9" t="n">
-        <v>0.544</v>
+        <v>2.002</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>-0.2</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>-0.095</v>
+        <v>-0.228</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.55</v>
+        <v>21.46</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.016651449</v>
+        <v>-0.020985446</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.049</v>
+        <v>-0.053</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>5.018</v>
+        <v>4.996</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.53225999999999</v>
+        <v>69.22580000000001</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>28.892553</v>
+        <v>28.765213</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.976</v>
+        <v>0.953</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.116</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="14">
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.50231516</v>
+        <v>-0.5409559</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.306</v>
+        <v>-0.307</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.376</v>
+        <v>2.375</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.956</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>11.948512</v>
+        <v>11.9438715</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.753</v>
@@ -1416,7 +1416,7 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>-0.036</v>
+        <v>-0.008</v>
       </c>
       <c r="Q14" s="4" t="n">
         <v>-0.144</v>
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.6386833</v>
+        <v>0.9124123000000001</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,19 +1451,19 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.457</v>
+        <v>-0.455</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.243</v>
+        <v>2.25</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>12.774</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>11.98913</v>
+        <v>12.021739</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.9319625</v>
+        <v>6.9508166</v>
       </c>
       <c r="M15" s="7" t="n">
         <v>10.592</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>-0.266</v>
+        <v>-0.264</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.48</v>
+        <v>14.57</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.011937257</v>
+        <v>-0.61391646</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,10 +1510,10 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.297</v>
+        <v>-0.293</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.934</v>
+        <v>1.946</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>12.438</v>
@@ -1524,7 +1524,7 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.370267999999999</v>
+        <v>8.419385999999999</v>
       </c>
       <c r="M16" s="7" t="n">
         <v>17.223</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-0.166</v>
+        <v>-0.149</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.025</v>
+        <v>-0.019</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.31</v>
+        <v>97.22</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.021765366</v>
+        <v>-0.022619884</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1574,16 +1574,16 @@
         <v>-0.146</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.74</v>
+        <v>1.739</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>1.696</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>17.91989</v>
+        <v>17.904236</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>16.367535</v>
+        <v>16.353237</v>
       </c>
       <c r="M17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.215</v>
+        <v>0.223</v>
       </c>
       <c r="Q17" s="9" t="n">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="18">
@@ -1621,19 +1621,19 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-0.04239124</v>
+        <v>-0.04130436000000001</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>4.4</v>
+        <v>4.395</v>
       </c>
       <c r="H18" s="5" t="n">
         <v>-0.679</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.133</v>
+        <v>1.134</v>
       </c>
       <c r="J18" s="6" t="n">
         <v>0.883</v>
@@ -1644,7 +1644,7 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.4494953</v>
+        <v>4.454545</v>
       </c>
       <c r="M18" s="7" t="n">
         <v>-7.324</v>
@@ -1658,7 +1658,7 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>-0.586</v>
+        <v>-0.593</v>
       </c>
       <c r="Q18" s="4" t="n">
         <v>-0.591</v>
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.017761972</v>
+        <v>-0.015090996</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,19 +1693,19 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.167</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.902</v>
+        <v>0.905</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.242</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>18.433332</v>
+        <v>18.483334</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>11.943459</v>
+        <v>11.975854</v>
       </c>
       <c r="M19" s="7" t="n">
         <v>6.569</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>0.08199999999999999</v>
+        <v>0.083</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>-0.027</v>
+        <v>-0.025</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
-      </c>
-      <c r="E20" s="4" t="n">
-        <v>-0.113674805</v>
+        <v>26.42</v>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>0.11368203</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,10 +1752,10 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.195</v>
+        <v>-0.193</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.696</v>
+        <v>0.697</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>1.154</v>
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.785124</v>
+        <v>21.83471</v>
       </c>
       <c r="M20" s="7" t="n">
         <v>9.455</v>
@@ -1777,11 +1777,11 @@
       <c r="O20" s="8" t="n">
         <v>1.412</v>
       </c>
-      <c r="P20" s="9" t="n">
-        <v>0.003</v>
+      <c r="P20" s="4" t="n">
+        <v>-0.005</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>-0.026</v>
+        <v>-0.023</v>
       </c>
     </row>
     <row r="21">
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.38</v>
+        <v>11.31</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.044882536</v>
+        <v>-0.05117447</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,10 +1813,10 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.451</v>
+        <v>-0.455</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>7.795</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-14.055555</v>
+        <v>-13.962963</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>22.644</v>
@@ -1841,10 +1841,10 @@
         </is>
       </c>
       <c r="P21" s="4" t="n">
-        <v>-0.183</v>
+        <v>-0.105</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>-0.316</v>
+        <v>-0.32</v>
       </c>
     </row>
     <row r="22">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.89</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.028358219</v>
+        <v>0.025373147</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,7 +1876,7 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.308</v>
+        <v>-0.31</v>
       </c>
       <c r="I22" s="6" t="n">
         <v>0.186</v>
@@ -1890,7 +1890,7 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>9.196967000000001</v>
+        <v>9.170271</v>
       </c>
       <c r="M22" s="7" t="n">
         <v>6.891</v>
@@ -1902,10 +1902,10 @@
         <v>1.206</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>-0.232</v>
+        <v>-0.225</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>-0.232</v>
+        <v>-0.234</v>
       </c>
     </row>
     <row r="23">
@@ -1928,7 +1928,7 @@
         <v>2.28</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-0.87466025</v>
+        <v>-0.8695644</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1963,7 +1963,7 @@
         <v>1.327</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>-0.455</v>
+        <v>-0.461</v>
       </c>
       <c r="Q23" s="4" t="n">
         <v>-0.08800000000000001</v>
@@ -2152,28 +2152,28 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.28</v>
+        <v>52.41</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.03489015</v>
+        <v>-0.0325826</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>-0.194</v>
+        <v>-0.192</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.324</v>
+        <v>0.327</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.081</v>
+        <v>-0.078</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.062</v>
+        <v>-0.059</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>-0.258</v>
+        <v>-0.256</v>
       </c>
       <c r="L2" s="8" t="n">
         <v>0.888</v>
@@ -2199,28 +2199,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.75</v>
+        <v>103.63</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.3384898</v>
+        <v>0.22243302</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.525</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5610000000000001</v>
+        <v>-0.5629999999999999</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>-59.4</v>
+        <v>-60</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.279</v>
+        <v>-0.28</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>-0.5489999999999999</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.669</v>
+        <v>-0.67</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2246,28 +2246,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.32</v>
+        <v>21.27</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.49019393</v>
+        <v>-0.70027834</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.402</v>
+        <v>-0.404</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.434</v>
+        <v>-0.426</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>-37.5</v>
+        <v>-37.8</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.215</v>
+        <v>-0.217</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.403</v>
+        <v>-0.405</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2293,28 +2293,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.19</v>
+        <v>99.47</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.026499135</v>
+        <v>-0.023751085</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.187</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.166</v>
+        <v>0.165</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>33.4</v>
+        <v>33.2</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.09699999999999999</v>
+        <v>-0.095</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.132</v>
+        <v>-0.13</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.264</v>
+        <v>-0.262</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2340,28 +2340,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.55</v>
+        <v>37.58</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.17337589</v>
+        <v>0.24006441</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.169</v>
+        <v>0.189</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>12</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.059</v>
+        <v>0.06</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.068</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.064</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,19 +2387,19 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.92</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.022858517</v>
+        <v>-0.02297637</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.035</v>
+        <v>-0.036</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.224</v>
+        <v>0.235</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>20.1</v>
+        <v>19.9</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>-0.012</v>
@@ -2434,22 +2434,22 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.55</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.40138316</v>
+        <v>0.4243151000000001</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.218</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>-0.225</v>
+        <v>-0.218</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>-3.2</v>
+        <v>-2.9</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.077</v>
+        <v>-0.076</v>
       </c>
       <c r="J8" s="5" t="n">
         <v>-0.133</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.94</v>
+        <v>55.74</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.04782981</v>
+        <v>-0.051234016</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.094</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.324</v>
+        <v>0.325</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>38.2</v>
+        <v>38.1</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.092</v>
+        <v>-0.096</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.047</v>
+        <v>-0.051</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.192</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2528,22 +2528,22 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.88</v>
+        <v>26.89</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.22371165</v>
+        <v>0.26099813</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.141</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.004</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>-21.9</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.146</v>
+        <v>0.147</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.09</v>
@@ -2561,12 +2561,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -2575,45 +2575,45 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.98</v>
+        <v>10.54</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>-0.028363025</v>
+        <v>0</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>-0.229</v>
+        <v>-0.09</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>-0.198</v>
+        <v>0.578</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>-29.6</v>
+        <v>25.4</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>-0.022</v>
+        <v>0.049</v>
       </c>
       <c r="J11" s="5" t="n">
+        <v>-0.061</v>
+      </c>
+      <c r="K11" s="5" t="n">
         <v>-0.267</v>
       </c>
-      <c r="K11" s="5" t="n">
-        <v>-0.442</v>
-      </c>
       <c r="L11" s="8" t="n">
-        <v>2.002</v>
+        <v>1.1</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>2485880</v>
+        <v>1926430</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -2622,34 +2622,34 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.48</v>
+        <v>18</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.52182454</v>
+        <v>-0.027552686</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-0.095</v>
+        <v>-0.228</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.544</v>
+        <v>-0.2</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>25.9</v>
+        <v>-30.1</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.043</v>
+        <v>-0.021</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.067</v>
+        <v>-0.266</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.271</v>
+        <v>-0.441</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>1.1</v>
+        <v>2.002</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1926430</v>
+        <v>2485880</v>
       </c>
     </row>
     <row r="13">
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.55</v>
+        <v>21.46</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.016651449</v>
+        <v>-0.020985446</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.116</v>
+        <v>0.111</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.976</v>
+        <v>0.953</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>50.7</v>
+        <v>50.3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.146</v>
+        <v>0.141</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.179</v>
+        <v>0.174</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.049</v>
+        <v>-0.053</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2716,16 +2716,16 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.50231516</v>
+        <v>-0.5409559</v>
       </c>
       <c r="F14" s="5" t="n">
         <v>-0.144</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.036</v>
+        <v>-0.008</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>12.6</v>
@@ -2734,10 +2734,10 @@
         <v>-0.066</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.167</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.306</v>
+        <v>-0.307</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2763,28 +2763,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.6386833</v>
+        <v>0.9124123000000001</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.266</v>
+        <v>-0.264</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.025</v>
+        <v>0.024</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>6.2</v>
+        <v>5.6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.08500000000000001</v>
+        <v>-0.081</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.298</v>
+        <v>-0.296</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.457</v>
+        <v>-0.455</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2810,28 +2810,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.48</v>
+        <v>14.57</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.011937257</v>
+        <v>-0.61391646</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.019</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.166</v>
+        <v>-0.149</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.4</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.051</v>
+        <v>0.057</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.109</v>
+        <v>-0.103</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.297</v>
+        <v>-0.293</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2857,25 +2857,25 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.31</v>
+        <v>97.22</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.021765366</v>
+        <v>-0.022619884</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.215</v>
+        <v>0.223</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.026</v>
+        <v>0.025</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>-0.146</v>
@@ -2907,16 +2907,16 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.04239124</v>
+        <v>-0.04130436000000001</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>-0.591</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.586</v>
+        <v>-0.593</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-34.5</v>
+        <v>-34.8</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>-0.388</v>
@@ -2951,28 +2951,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.017761972</v>
+        <v>-0.015090996</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.025</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.08199999999999999</v>
+        <v>0.083</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>-1.6</v>
+        <v>-1.8</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.021</v>
+        <v>-0.018</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.01</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.169</v>
+        <v>-0.167</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -2998,28 +2998,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.42</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.113674805</v>
+        <v>0.11368203</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.023</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0.003</v>
+        <v>-0.005</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>5.4</v>
+        <v>5.5</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.057</v>
+        <v>-0.055</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.019</v>
+        <v>-0.017</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.195</v>
+        <v>-0.193</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3045,28 +3045,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.38</v>
+        <v>11.31</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.044882536</v>
+        <v>-0.05117447</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.316</v>
+        <v>-0.32</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.183</v>
+        <v>-0.105</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>38.8</v>
+        <v>39.4</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.216</v>
+        <v>-0.221</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.144</v>
+        <v>-0.149</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.451</v>
+        <v>-0.455</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.89</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.028358219</v>
+        <v>0.025373147</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.232</v>
+        <v>-0.234</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.232</v>
+        <v>-0.225</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>3.9</v>
+        <v>4.2</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.177</v>
+        <v>-0.18</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.195</v>
+        <v>-0.198</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.308</v>
+        <v>-0.31</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3144,16 +3144,16 @@
         <v>2.28</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.87466025</v>
+        <v>-0.8695644</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-0.08800000000000001</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-0.455</v>
+        <v>-0.461</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>-52.6</v>
+        <v>-52.4</v>
       </c>
       <c r="I23" s="5" t="n">
         <v>-0.05599999999999999</v>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.28</v>
+        <v>52.41</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.348</v>
+        <v>35.433</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.246809</v>
+        <v>22.300001</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.913358</v>
+        <v>13.946625</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.190153</v>
+        <v>22.243208</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.7155495</v>
+        <v>2.7220423</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.75</v>
+        <v>103.63</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.151</v>
+        <v>18.13</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.746387500000001</v>
+        <v>9.735113999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.0114384</v>
+        <v>2.009112</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1079355</v>
+        <v>1.106654</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>21.32</v>
+        <v>21.27</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.61</v>
+        <v>10.588</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.95155</v>
+        <v>10.928429</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.491</v>
@@ -3473,10 +3473,10 @@
         <v>1.87</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.704546</v>
+        <v>16.66928</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7524118</v>
+        <v>1.7487122</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,16 +3505,16 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>99.19</v>
+        <v>99.47</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.344</v>
+        <v>10.373</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.589172</v>
+        <v>31.678343</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.69368</v>
+        <v>16.740803</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>11.398</v>
@@ -3526,10 +3526,10 @@
         <v>2.794</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.901043</v>
+        <v>-37.00521</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4491411</v>
+        <v>1.4532318</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,16 +3558,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.55</v>
+        <v>37.58</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.272</v>
+        <v>10.278</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.414474</v>
+        <v>49.447372</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.027843</v>
+        <v>16.038513</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.99224</v>
+        <v>3.9948978</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5856836399999999</v>
+        <v>0.5860735</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.92</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.261</v>
+        <v>6.26</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6755319</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.178695</v>
+        <v>10.177466</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4279063</v>
+        <v>2.4276135</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5299574</v>
+        <v>1.5297729</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,16 +3664,16 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>87.55</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>6.102</v>
+        <v>6.103</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.550095</v>
+        <v>16.553875</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.791183</v>
+        <v>11.793877</v>
       </c>
       <c r="H8" s="7" t="n">
         <v>11.623</v>
@@ -3685,10 +3685,10 @@
         <v>3.801</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6.035018</v>
+        <v>6.036396</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.085484</v>
+        <v>2.0859604</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,16 +3717,16 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>55.94</v>
+        <v>55.74</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.752</v>
+        <v>5.732</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.929487</v>
+        <v>17.865385</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>17.0241</v>
+        <v>16.963236</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>8.461</v>
@@ -3738,10 +3738,10 @@
         <v>3.423</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>15.660694</v>
+        <v>15.604704</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.8596494</v>
+        <v>2.8494256</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3770,10 +3770,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>26.88</v>
+        <v>26.89</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>5.486</v>
+        <v>5.488</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
@@ -3781,7 +3781,7 @@
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>26.19883</v>
+        <v>26.208576</v>
       </c>
       <c r="H10" s="7" t="n">
         <v>8.691000000000001</v>
@@ -3793,10 +3793,10 @@
         <v>2.645</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>1.5543861</v>
+        <v>1.5549644</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>0.47766158</v>
+        <v>0.47783932</v>
       </c>
       <c r="M10" s="3" t="n">
         <v>-2.42</v>
@@ -3811,12 +3811,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3825,51 +3825,51 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>17.98</v>
+        <v>10.54</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.323</v>
+        <v>5.329</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>49.958332</v>
+        <v>25.09524</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>21.826754</v>
+        <v>12.151116</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>10.358</v>
+        <v>10.031</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>9</v>
+        <v>7.8</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>4.075</v>
+        <v>2.101</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4.7535157</v>
+        <v>7.1554646</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>4.1262283</v>
+        <v>2.2746992</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>0.36</v>
+        <v>0.42</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>0.8239888</v>
+        <v>0.86741</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>3.7835155</v>
+        <v>1.473</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3878,40 +3878,40 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>10.48</v>
+        <v>18</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>5.302</v>
+        <v>5.327</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>24.964285</v>
+        <v>49.999996</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>12.087708</v>
+        <v>21.844957</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10.031</v>
+        <v>10.358</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>7.8</v>
+        <v>9</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>2.101</v>
+        <v>4.075</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.118126</v>
+        <v>4.75748</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>2.2628293</v>
+        <v>4.1296697</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.42</v>
+        <v>0.36</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.86741</v>
+        <v>0.8239888</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>1.473</v>
+        <v>3.7835155</v>
       </c>
     </row>
     <row r="13">
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.55</v>
+        <v>21.46</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>5.018</v>
+        <v>4.996</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.53225999999999</v>
+        <v>69.22580000000001</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>28.892553</v>
+        <v>28.765213</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.633401</v>
+        <v>14.568906</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.4230847</v>
+        <v>4.40359</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.376</v>
+        <v>2.375</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11.948512</v>
+        <v>11.9438715</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.753</v>
@@ -4013,10 +4013,10 @@
         <v>2.372</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.749306</v>
+        <v>2.7482383</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.94615924</v>
+        <v>0.9457917</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4045,16 +4045,16 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.243</v>
+        <v>2.25</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>11.98913</v>
+        <v>12.021739</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.9319625</v>
+        <v>6.9508166</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>10.592</v>
@@ -4066,10 +4066,10 @@
         <v>2.474</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7282983</v>
+        <v>-1.7329991</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43450087</v>
+        <v>0.43568265</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>14.48</v>
+        <v>14.57</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.934</v>
+        <v>1.946</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,7 +4109,7 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.370267999999999</v>
+        <v>8.419385999999999</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>17.223</v>
@@ -4121,10 +4121,10 @@
         <v>1.787</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.99710876</v>
+        <v>1.00296</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.27789366</v>
+        <v>0.27952436</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,16 +4153,16 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>97.31</v>
+        <v>97.22</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.74</v>
+        <v>1.739</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>17.91989</v>
+        <v>17.904236</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>16.367535</v>
+        <v>16.353237</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>8.893000000000001</v>
@@ -4174,10 +4174,10 @@
         <v>3.111</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.2247963</v>
+        <v>3.2219791</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.1926787</v>
+        <v>3.1898897</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4209,7 +4209,7 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.133</v>
+        <v>1.134</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4217,7 +4217,7 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.4494953</v>
+        <v>4.454545</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-7.324</v>
@@ -4231,10 +4231,10 @@
         <v>1.319</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.49779</v>
+        <v>1.4994899</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.6926149</v>
+        <v>1.694536</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4263,16 +4263,16 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.902</v>
+        <v>0.905</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>18.433332</v>
+        <v>18.483334</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>11.943459</v>
+        <v>11.975854</v>
       </c>
       <c r="H19" s="7" t="n">
         <v>6.569</v>
@@ -4284,10 +4284,10 @@
         <v>0.9330000000000001</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.3750384</v>
+        <v>3.384193</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6778567</v>
+        <v>0.67969537</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4316,10 +4316,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.42</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.696</v>
+        <v>0.697</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4327,7 +4327,7 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.785124</v>
+        <v>21.83471</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>9.455</v>
@@ -4339,10 +4339,10 @@
         <v>1.818</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6399155</v>
+        <v>1.6436481</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.0960162</v>
+        <v>1.0985109</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4371,10 +4371,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>11.38</v>
+        <v>11.31</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-14.055555</v>
+        <v>-13.962963</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>22.644</v>
@@ -4394,10 +4394,10 @@
         <v>2.934</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.5554201</v>
+        <v>0.5517612</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.21068002</v>
+        <v>0.20929217</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-12.45</v>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.89</v>
+        <v>6.87</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0.186</v>
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.196967000000001</v>
+        <v>9.170271</v>
       </c>
       <c r="H22" s="7" t="n">
         <v>6.891</v>
@@ -4449,10 +4449,10 @@
         <v>1.684</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-11.426203</v>
+        <v>-11.393035</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.61308926</v>
+        <v>0.61130965</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -5251,12 +5251,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -5265,57 +5265,59 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>1.29</v>
+        <v>2.343</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.201</v>
+        <v>0.178</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.26816</v>
+        <v>0.51058</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.15614</v>
+        <v>0.23518999</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.07777000000000001</v>
+        <v>0.09804</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.39339</v>
+        <v>0.20945999</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.10515001</v>
+        <v>0.32813</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>0.04121</v>
+        <v>0.23642</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.507</v>
-      </c>
-      <c r="M11" s="6" t="n">
-        <v>0.341</v>
+        <v>0.491</v>
+      </c>
+      <c r="M11" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="N11" s="6" t="n">
-        <v>0.063</v>
+        <v>0.07199999999999999</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>0.365</v>
+        <v>0.478</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>6.424</v>
+        <v>9.69</v>
       </c>
       <c r="Q11" s="7" t="n">
-        <v>1.167</v>
+        <v>1.75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -5324,48 +5326,46 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>2.343</v>
+        <v>1.29</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.178</v>
+        <v>0.201</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.51058</v>
+        <v>0.26816</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.23518999</v>
+        <v>0.15614</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.09804</v>
+        <v>0.07777000000000001</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.20945999</v>
+        <v>0.39339</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.32813</v>
+        <v>0.10515001</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>0.23642</v>
+        <v>0.04121</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.491</v>
-      </c>
-      <c r="M12" s="6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.507</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0.341</v>
       </c>
       <c r="N12" s="6" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.063</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>0.478</v>
+        <v>0.365</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>9.69</v>
+        <v>6.424</v>
       </c>
       <c r="Q12" s="7" t="n">
-        <v>1.75</v>
+        <v>1.167</v>
       </c>
     </row>
     <row r="13">
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.28</v>
+        <v>52.41</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6268,7 +6268,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.337</v>
+        <v>0.333</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.75</v>
+        <v>103.63</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>0.9990000000000001</v>
+        <v>1.002</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>21.32</v>
+        <v>21.27</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6382,7 +6382,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.6970000000000001</v>
+        <v>0.701</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6417,7 +6417,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>99.19</v>
+        <v>99.47</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6440,7 +6440,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.43</v>
+        <v>0.426</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.38</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.55</v>
+        <v>37.58</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.136</v>
+        <v>0.135</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.93000000000001</v>
+        <v>82.92</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>87.55</v>
+        <v>87.56999999999999</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6610,7 +6610,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.5479999999999999</v>
+        <v>0.547</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.17</v>
@@ -6643,7 +6643,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>55.94</v>
+        <v>55.74</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6666,7 +6666,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.304</v>
+        <v>0.309</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>4.01</v>
@@ -6699,7 +6699,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>26.88</v>
+        <v>26.89</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -6722,7 +6722,7 @@
         <v>22</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.189</v>
+        <v>0.188</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>3.37</v>
@@ -6748,16 +6748,16 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>17.98</v>
+        <v>10.54</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6765,57 +6765,55 @@
         </is>
       </c>
       <c r="E11" s="7" t="n">
-        <v>1.33333</v>
+        <v>1.25</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>28.808449</v>
+        <v>17.375</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>37.080116</v>
+        <v>20</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>22.891066</v>
+        <v>16</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.602</v>
+        <v>0.648</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>4.54</v>
+        <v>4.72</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.095</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.68889</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>0.91643</v>
-      </c>
-      <c r="O11" s="5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>0.19124001</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>1.61</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>0</v>
+        <v>0.2831</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>10.48</v>
+        <v>18</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6823,40 +6821,42 @@
         </is>
       </c>
       <c r="E12" s="7" t="n">
-        <v>1.25</v>
+        <v>1.33333</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>17.375</v>
+        <v>28.801807</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>20</v>
+        <v>37.071568</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>16</v>
+        <v>22.88579</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.6579999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.72</v>
+        <v>4.54</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>0.095</v>
+        <v>0.1046</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.01337</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.19124001</v>
-      </c>
-      <c r="O12" s="5" t="n">
-        <v>1.61</v>
+        <v>0.91643</v>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="P12" s="5" t="n">
-        <v>0.2831</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.55</v>
+        <v>21.46</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6894,7 +6894,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.156</v>
+        <v>0.161</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.89</v>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.88</v>
+        <v>12.87</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6952,7 +6952,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.404</v>
+        <v>0.405</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.58</v>
@@ -6985,7 +6985,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.51</v>
+        <v>5.53</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7008,7 +7008,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0.677</v>
+        <v>0.6709999999999999</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.37</v>
@@ -7043,7 +7043,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>14.48</v>
+        <v>14.57</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7066,7 +7066,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.32</v>
+        <v>0.312</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.3</v>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>97.31</v>
+        <v>97.22</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7126,7 +7126,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.106</v>
+        <v>0.107</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.64</v>
@@ -7217,7 +7217,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>11.06</v>
+        <v>11.09</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>0.401</v>
+        <v>0.398</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>2.55</v>
@@ -7275,7 +7275,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.36</v>
+        <v>26.42</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7300,7 +7300,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0.157</v>
+        <v>0.154</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>4.41</v>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>11.38</v>
+        <v>11.31</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7356,7 +7356,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.377</v>
+        <v>0.385</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>8.01</v>
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.89</v>
+        <v>6.87</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7414,7 +7414,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>9.81</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.348</v>
+        <v>35.433</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.246809</v>
+        <v>22.300001</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7712,7 +7712,7 @@
         <v>0.73263</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.194</v>
+        <v>-0.192</v>
       </c>
       <c r="J3" s="7" t="n">
         <v>10.795</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.486</v>
+        <v>5.488</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7787,10 +7787,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>10.344</v>
+        <v>10.373</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.589172</v>
+        <v>31.678343</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7804,7 +7804,7 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.189</v>
+        <v>-0.187</v>
       </c>
       <c r="J5" s="7" t="n">
         <v>11.398</v>
@@ -7833,10 +7833,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2.243</v>
+        <v>2.25</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>11.98913</v>
+        <v>12.021739</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7850,7 +7850,7 @@
         </is>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-0.266</v>
+        <v>-0.264</v>
       </c>
       <c r="J6" s="7" t="n">
         <v>10.592</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.272</v>
+        <v>10.278</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.414474</v>
+        <v>49.447372</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7894,7 +7894,7 @@
         <v>0.1489</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>0.029</v>
+        <v>0.03</v>
       </c>
       <c r="J7" s="7" t="n">
         <v>16.869</v>
@@ -7941,10 +7941,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.261</v>
+        <v>6.26</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6759753</v>
+        <v>3.6755319</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7956,7 +7956,7 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.035</v>
+        <v>-0.036</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>7.297</v>
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>6.102</v>
+        <v>6.103</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.550095</v>
+        <v>16.553875</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8015,12 +8015,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MCRI</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Monarch Casino &amp; Resort</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -8029,42 +8029,42 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.74</v>
+        <v>5.732</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.91989</v>
+        <v>17.865385</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.041</v>
+        <v>0.032</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.34986</v>
+        <v>0.4046</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.19214001</v>
+        <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.016</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.893000000000001</v>
+        <v>8.461</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>62.7</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Monarch Casino &amp; Resort</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -8073,31 +8073,31 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5.752</v>
+        <v>1.739</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.929487</v>
+        <v>17.904236</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.032</v>
+        <v>0.041</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.4046</v>
+        <v>0.34986</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>1.113</v>
+        <v>0.19214001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.094</v>
+        <v>0.015</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.461</v>
+        <v>8.893000000000001</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>54.8</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="14">
@@ -8117,7 +8117,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.934</v>
+        <v>1.946</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8134,7 +8134,7 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.019</v>
       </c>
       <c r="J14" s="7" t="n">
         <v>17.223</v>
@@ -8163,7 +8163,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.696</v>
+        <v>0.697</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8180,7 +8180,7 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.023</v>
       </c>
       <c r="J15" s="7" t="n">
         <v>9.455</v>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.556</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8226,7 +8226,7 @@
         <v>-0.5564</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.316</v>
+        <v>-0.32</v>
       </c>
       <c r="J16" s="7" t="n">
         <v>22.644</v>
@@ -8319,10 +8319,10 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>5.302</v>
+        <v>5.329</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>24.964285</v>
+        <v>25.09524</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0.178</v>
@@ -8334,7 +8334,7 @@
         <v>0.32813</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.095</v>
+        <v>-0.09</v>
       </c>
       <c r="J20" s="7" t="n">
         <v>10.031</v>
@@ -8343,18 +8343,18 @@
         <v>7.8</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>66.7</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Rush Street Interactive</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -8363,42 +8363,46 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>5.323</v>
+        <v>4.996</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>49.958332</v>
+        <v>69.22580000000001</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.201</v>
+        <v>0.888</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>0.39339</v>
+        <v>0.11229999</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0.10515001</v>
+        <v>0.29505</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.229</v>
-      </c>
-      <c r="J21" s="7" t="n">
-        <v>10.358</v>
-      </c>
-      <c r="K21" s="7" t="n">
-        <v>9</v>
+        <v>0.111</v>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>58.3</v>
+        <v>56.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Rush Street Interactive</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -8407,35 +8411,31 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>5.018</v>
+        <v>5.327</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>69.53225999999999</v>
+        <v>49.999996</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.888</v>
+        <v>0.201</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0.11229999</v>
+        <v>0.39339</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.29505</v>
+        <v>0.10515001</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>-0.228</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>10.358</v>
+      </c>
+      <c r="K22" s="7" t="n">
+        <v>9</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>56.7</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23">
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.61</v>
+        <v>10.588</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8472,7 +8472,7 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.402</v>
+        <v>-0.404</v>
       </c>
       <c r="J23" s="7" t="n">
         <v>41.491</v>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.151</v>
+        <v>18.13</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8547,7 +8547,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.133</v>
+        <v>1.134</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8613,10 +8613,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.902</v>
+        <v>0.905</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>18.433332</v>
+        <v>18.483334</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8628,7 +8628,7 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.025</v>
       </c>
       <c r="J28" s="7" t="n">
         <v>6.569</v>
@@ -8657,7 +8657,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.376</v>
+        <v>2.375</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8722,7 +8722,7 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.232</v>
+        <v>-0.234</v>
       </c>
       <c r="J30" s="7" t="n">
         <v>6.891</v>
@@ -9763,55 +9763,55 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>SRAD</t>
+          <t>SGHC</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Sportradar Group</t>
+          <t>Super Group</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.68889</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.91643</v>
+        <v>0.19124001</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>4.54</v>
+        <v>4.72</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.095</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>10753999</v>
+        <v>14945381</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SGHC</t>
+          <t>SRAD</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Super Group</t>
+          <t>Sportradar Group</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.68889</v>
+        <v>0.01337</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.19124001</v>
+        <v>0.91643</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>4.72</v>
+        <v>4.54</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.095</v>
+        <v>0.1046</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>14945381</v>
+        <v>10753999</v>
       </c>
     </row>
     <row r="13">
@@ -10198,13 +10198,13 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1293.21</v>
+        <v>1298.6</v>
       </c>
       <c r="C2" s="13" t="n">
-        <v>1218.79</v>
+        <v>1222.04</v>
       </c>
       <c r="D2" s="13" t="n">
-        <v>1070.24</v>
+        <v>1078.46</v>
       </c>
     </row>
     <row r="3">
@@ -10214,13 +10214,13 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1285.65</v>
+        <v>1291.07</v>
       </c>
       <c r="C3" s="13" t="n">
-        <v>1209.76</v>
+        <v>1212.98</v>
       </c>
       <c r="D3" s="13" t="n">
-        <v>1072.87</v>
+        <v>1081.11</v>
       </c>
     </row>
     <row r="4">
@@ -10230,13 +10230,13 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1290.51</v>
+        <v>1295.92</v>
       </c>
       <c r="C4" s="13" t="n">
-        <v>1211.98</v>
+        <v>1215.21</v>
       </c>
       <c r="D4" s="13" t="n">
-        <v>1073.92</v>
+        <v>1082.16</v>
       </c>
     </row>
     <row r="5">
@@ -10246,13 +10246,13 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1291.41</v>
+        <v>1296.87</v>
       </c>
       <c r="C5" s="13" t="n">
-        <v>1220.05</v>
+        <v>1223.3</v>
       </c>
       <c r="D5" s="13" t="n">
-        <v>1071.82</v>
+        <v>1080.05</v>
       </c>
     </row>
     <row r="6">
@@ -10262,13 +10262,13 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1276.35</v>
+        <v>1281.75</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>1227.31</v>
+        <v>1230.58</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>1065.26</v>
+        <v>1073.44</v>
       </c>
     </row>
     <row r="7">
@@ -10278,13 +10278,13 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1227.75</v>
+        <v>1232.89</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>1223.35</v>
+        <v>1226.61</v>
       </c>
       <c r="D7" s="13" t="n">
-        <v>1045.83</v>
+        <v>1053.86</v>
       </c>
     </row>
     <row r="8">
@@ -10294,13 +10294,13 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1253.18</v>
+        <v>1258.46</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>1223.23</v>
+        <v>1226.48</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>1063.16</v>
+        <v>1071.32</v>
       </c>
     </row>
     <row r="9">
@@ -10310,13 +10310,13 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1223.94</v>
+        <v>1229.1</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>1231.32</v>
+        <v>1234.6</v>
       </c>
       <c r="D9" s="13" t="n">
-        <v>1055.54</v>
+        <v>1063.65</v>
       </c>
     </row>
     <row r="10">
@@ -10326,13 +10326,13 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1219.58</v>
+        <v>1224.8</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>1233.25</v>
+        <v>1236.53</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>1051.34</v>
+        <v>1059.42</v>
       </c>
     </row>
     <row r="11">
@@ -10342,13 +10342,13 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1211.63</v>
+        <v>1216.78</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>1230.78</v>
+        <v>1234.06</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>1039</v>
+        <v>1046.98</v>
       </c>
     </row>
     <row r="12">
@@ -10358,13 +10358,13 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1209.25</v>
+        <v>1214.38</v>
       </c>
       <c r="C12" s="13" t="n">
-        <v>1224.74</v>
+        <v>1228</v>
       </c>
       <c r="D12" s="13" t="n">
-        <v>1041.63</v>
+        <v>1049.63</v>
       </c>
     </row>
     <row r="13">
@@ -10374,13 +10374,13 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1228.69</v>
+        <v>1233.93</v>
       </c>
       <c r="C13" s="13" t="n">
-        <v>1228.07</v>
+        <v>1231.34</v>
       </c>
       <c r="D13" s="13" t="n">
-        <v>1053.18</v>
+        <v>1061.27</v>
       </c>
     </row>
     <row r="14">
@@ -10390,13 +10390,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1191.55</v>
+        <v>1196.68</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>1227.04</v>
+        <v>1230.31</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>1032.7</v>
+        <v>1040.63</v>
       </c>
     </row>
     <row r="15">
@@ -10406,13 +10406,13 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1167.42</v>
+        <v>1172.37</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>1202.06</v>
+        <v>1205.26</v>
       </c>
       <c r="D15" s="13" t="n">
-        <v>1015.9</v>
+        <v>1023.7</v>
       </c>
     </row>
     <row r="16">
@@ -10422,13 +10422,13 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1173.97</v>
+        <v>1178.98</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>1215.94</v>
+        <v>1219.17</v>
       </c>
       <c r="D16" s="13" t="n">
-        <v>1017.74</v>
+        <v>1025.56</v>
       </c>
     </row>
     <row r="17">
@@ -10438,13 +10438,13 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1179.17</v>
+        <v>1184.29</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>1222.29</v>
+        <v>1225.54</v>
       </c>
       <c r="D17" s="13" t="n">
-        <v>1025.88</v>
+        <v>1033.76</v>
       </c>
     </row>
     <row r="18">
@@ -10454,13 +10454,13 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1163.81</v>
+        <v>1168.86</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>1222.73</v>
+        <v>1225.99</v>
       </c>
       <c r="D18" s="13" t="n">
-        <v>1018.79</v>
+        <v>1026.61</v>
       </c>
     </row>
     <row r="19">
@@ -10470,13 +10470,13 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1169.64</v>
+        <v>1174.69</v>
       </c>
       <c r="C19" s="13" t="n">
-        <v>1228.94</v>
+        <v>1232.21</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>1024.57</v>
+        <v>1032.43</v>
       </c>
     </row>
     <row r="20">
@@ -10486,13 +10486,13 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1156.3</v>
+        <v>1161.28</v>
       </c>
       <c r="C20" s="13" t="n">
-        <v>1233.84</v>
+        <v>1237.12</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>1020.89</v>
+        <v>1028.73</v>
       </c>
     </row>
     <row r="21">
@@ -10502,13 +10502,13 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1157.9</v>
+        <v>1162.85</v>
       </c>
       <c r="C21" s="13" t="n">
-        <v>1233.71</v>
+        <v>1237</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>1013.02</v>
+        <v>1020.8</v>
       </c>
     </row>
     <row r="22">
@@ -10518,13 +10518,13 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1105.51</v>
+        <v>1110.37</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>1231.26</v>
+        <v>1234.54</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>996.48</v>
+        <v>1004.13</v>
       </c>
     </row>
     <row r="23">
@@ -10534,13 +10534,13 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1093.64</v>
+        <v>1098.4</v>
       </c>
       <c r="C23" s="13" t="n">
-        <v>1227.59</v>
+        <v>1230.86</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>974.95</v>
+        <v>982.4400000000001</v>
       </c>
     </row>
     <row r="24">
@@ -10550,13 +10550,13 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1111.87</v>
+        <v>1116.61</v>
       </c>
       <c r="C24" s="13" t="n">
-        <v>1233.69</v>
+        <v>1236.98</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>984.4</v>
+        <v>991.96</v>
       </c>
     </row>
     <row r="25">
@@ -10566,13 +10566,13 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1108.21</v>
+        <v>1112.97</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>1223.26</v>
+        <v>1226.52</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>973.38</v>
+        <v>980.85</v>
       </c>
     </row>
     <row r="26">
@@ -10582,13 +10582,13 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1129.81</v>
+        <v>1134.74</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>1217.34</v>
+        <v>1220.58</v>
       </c>
       <c r="D26" s="13" t="n">
-        <v>994.9</v>
+        <v>1002.54</v>
       </c>
     </row>
     <row r="27">
@@ -10598,13 +10598,13 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1104.67</v>
+        <v>1109.48</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>1202.13</v>
+        <v>1205.33</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>975.48</v>
+        <v>982.97</v>
       </c>
     </row>
     <row r="28">
@@ -10614,13 +10614,13 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1131.97</v>
+        <v>1136.9</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>1225.2</v>
+        <v>1228.46</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>993.85</v>
+        <v>1001.48</v>
       </c>
     </row>
     <row r="29">
@@ -10630,13 +10630,13 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1133.93</v>
+        <v>1138.86</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>1231.1</v>
+        <v>1234.38</v>
       </c>
       <c r="D29" s="13" t="n">
-        <v>1001.2</v>
+        <v>1008.89</v>
       </c>
     </row>
     <row r="30">
@@ -10646,13 +10646,13 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1130.77</v>
+        <v>1135.73</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>1227.86</v>
+        <v>1231.13</v>
       </c>
       <c r="D30" s="13" t="n">
-        <v>1003.04</v>
+        <v>1010.74</v>
       </c>
     </row>
     <row r="31">
@@ -10662,13 +10662,13 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1115.79</v>
+        <v>1120.62</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>1227.57</v>
+        <v>1230.84</v>
       </c>
       <c r="D31" s="13" t="n">
-        <v>995.4299999999999</v>
+        <v>1003.07</v>
       </c>
     </row>
     <row r="32">
@@ -10678,13 +10678,13 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1078.07</v>
+        <v>1082.75</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>1208.61</v>
+        <v>1211.83</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>960.78</v>
+        <v>968.15</v>
       </c>
     </row>
     <row r="33">
@@ -10694,13 +10694,13 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1068.38</v>
+        <v>1073</v>
       </c>
       <c r="C33" s="13" t="n">
-        <v>1209.46</v>
+        <v>1212.68</v>
       </c>
       <c r="D33" s="13" t="n">
-        <v>948.4400000000001</v>
+        <v>955.72</v>
       </c>
     </row>
     <row r="34">
@@ -10710,13 +10710,13 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1083.47</v>
+        <v>1088.18</v>
       </c>
       <c r="C34" s="13" t="n">
-        <v>1211.41</v>
+        <v>1214.64</v>
       </c>
       <c r="D34" s="13" t="n">
-        <v>950.28</v>
+        <v>957.5700000000001</v>
       </c>
     </row>
     <row r="35">
@@ -10726,13 +10726,13 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1117.83</v>
+        <v>1122.75</v>
       </c>
       <c r="C35" s="13" t="n">
-        <v>1217.51</v>
+        <v>1220.76</v>
       </c>
       <c r="D35" s="13" t="n">
-        <v>976</v>
+        <v>983.5</v>
       </c>
     </row>
     <row r="36">
@@ -10742,13 +10742,13 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1112.74</v>
+        <v>1117.62</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>1214.3</v>
+        <v>1217.54</v>
       </c>
       <c r="D36" s="13" t="n">
-        <v>971.28</v>
+        <v>978.74</v>
       </c>
     </row>
     <row r="37">
@@ -10758,13 +10758,13 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1112.88</v>
+        <v>1117.81</v>
       </c>
       <c r="C37" s="13" t="n">
-        <v>1223.09</v>
+        <v>1226.34</v>
       </c>
       <c r="D37" s="13" t="n">
-        <v>968.92</v>
+        <v>976.36</v>
       </c>
     </row>
     <row r="38">
@@ -10774,13 +10774,13 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1068.89</v>
+        <v>1073.63</v>
       </c>
       <c r="C38" s="13" t="n">
-        <v>1210.6</v>
+        <v>1213.82</v>
       </c>
       <c r="D38" s="13" t="n">
-        <v>947.13</v>
+        <v>954.4</v>
       </c>
     </row>
     <row r="39">
@@ -10790,13 +10790,13 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1083.77</v>
+        <v>1088.64</v>
       </c>
       <c r="C39" s="13" t="n">
-        <v>1219.4</v>
+        <v>1222.64</v>
       </c>
       <c r="D39" s="13" t="n">
-        <v>955.26</v>
+        <v>962.6</v>
       </c>
     </row>
     <row r="40">
@@ -10806,13 +10806,13 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1087.92</v>
+        <v>1092.87</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>1229.68</v>
+        <v>1232.96</v>
       </c>
       <c r="D40" s="13" t="n">
-        <v>956.58</v>
+        <v>963.92</v>
       </c>
     </row>
     <row r="41">
@@ -10822,13 +10822,13 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1117.53</v>
+        <v>1122.72</v>
       </c>
       <c r="C41" s="13" t="n">
-        <v>1222.85</v>
+        <v>1226.11</v>
       </c>
       <c r="D41" s="13" t="n">
-        <v>958.9400000000001</v>
+        <v>966.3</v>
       </c>
     </row>
     <row r="42">
@@ -10838,13 +10838,13 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1104.53</v>
+        <v>1109.74</v>
       </c>
       <c r="C42" s="13" t="n">
-        <v>1216.98</v>
+        <v>1220.22</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>963.14</v>
+        <v>970.54</v>
       </c>
     </row>
     <row r="43">
@@ -10854,13 +10854,13 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1099.29</v>
+        <v>1104.43</v>
       </c>
       <c r="C43" s="13" t="n">
-        <v>1217.67</v>
+        <v>1220.92</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>954.48</v>
+        <v>961.8099999999999</v>
       </c>
     </row>
     <row r="44">
@@ -10870,13 +10870,13 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1095.37</v>
+        <v>1100.52</v>
       </c>
       <c r="C44" s="13" t="n">
-        <v>1206.94</v>
+        <v>1210.16</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>947.91</v>
+        <v>955.1900000000001</v>
       </c>
     </row>
     <row r="45">
@@ -10886,13 +10886,13 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1111.11</v>
+        <v>1116.42</v>
       </c>
       <c r="C45" s="13" t="n">
-        <v>1215.46</v>
+        <v>1218.69</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>953.6900000000001</v>
+        <v>961.01</v>
       </c>
     </row>
     <row r="46">
@@ -10902,13 +10902,13 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1108.88</v>
+        <v>1114.17</v>
       </c>
       <c r="C46" s="13" t="n">
-        <v>1208.68</v>
+        <v>1211.9</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>947.65</v>
+        <v>954.9299999999999</v>
       </c>
     </row>
     <row r="47">
@@ -10918,13 +10918,13 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1076.68</v>
+        <v>1081.76</v>
       </c>
       <c r="C47" s="13" t="n">
-        <v>1192.84</v>
+        <v>1196.01</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>937.9400000000001</v>
+        <v>945.14</v>
       </c>
     </row>
     <row r="48">
@@ -10934,13 +10934,13 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1078.14</v>
+        <v>1083.22</v>
       </c>
       <c r="C48" s="13" t="n">
-        <v>1203.29</v>
+        <v>1206.49</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>940.04</v>
+        <v>947.26</v>
       </c>
     </row>
     <row r="49">
@@ -10950,13 +10950,13 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1077.08</v>
+        <v>1082.14</v>
       </c>
       <c r="C49" s="13" t="n">
-        <v>1201.35</v>
+        <v>1204.55</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>938.2</v>
+        <v>945.41</v>
       </c>
     </row>
     <row r="50">
@@ -10966,13 +10966,13 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1092.27</v>
+        <v>1097.52</v>
       </c>
       <c r="C50" s="13" t="n">
-        <v>1199.85</v>
+        <v>1203.04</v>
       </c>
       <c r="D50" s="13" t="n">
-        <v>942.66</v>
+        <v>949.9</v>
       </c>
     </row>
     <row r="51">
@@ -10982,13 +10982,13 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1077.72</v>
+        <v>1082.93</v>
       </c>
       <c r="C51" s="13" t="n">
-        <v>1181.63</v>
+        <v>1184.77</v>
       </c>
       <c r="D51" s="13" t="n">
-        <v>931.38</v>
+        <v>938.53</v>
       </c>
     </row>
     <row r="52">
@@ -10998,13 +10998,13 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1079.64</v>
+        <v>1084.86</v>
       </c>
       <c r="C52" s="13" t="n">
-        <v>1174.94</v>
+        <v>1178.07</v>
       </c>
       <c r="D52" s="13" t="n">
-        <v>929.28</v>
+        <v>936.41</v>
       </c>
     </row>
     <row r="53">
@@ -11014,13 +11014,13 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1071.97</v>
+        <v>1077.08</v>
       </c>
       <c r="C53" s="13" t="n">
-        <v>1186.89</v>
+        <v>1190.06</v>
       </c>
       <c r="D53" s="13" t="n">
-        <v>926.39</v>
+        <v>933.5</v>
       </c>
     </row>
     <row r="54">
@@ -11030,13 +11030,13 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1084.52</v>
+        <v>1089.68</v>
       </c>
       <c r="C54" s="13" t="n">
-        <v>1190.02</v>
+        <v>1193.19</v>
       </c>
       <c r="D54" s="13" t="n">
-        <v>925.6</v>
+        <v>932.71</v>
       </c>
     </row>
     <row r="55">
@@ -11046,13 +11046,13 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1076.41</v>
+        <v>1081.55</v>
       </c>
       <c r="C55" s="13" t="n">
-        <v>1173.41</v>
+        <v>1176.54</v>
       </c>
       <c r="D55" s="13" t="n">
-        <v>915.36</v>
+        <v>922.39</v>
       </c>
     </row>
     <row r="56">
@@ -11062,13 +11062,13 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1089.3</v>
+        <v>1094.46</v>
       </c>
       <c r="C56" s="13" t="n">
-        <v>1170.52</v>
+        <v>1173.64</v>
       </c>
       <c r="D56" s="13" t="n">
-        <v>922.45</v>
+        <v>929.53</v>
       </c>
     </row>
     <row r="57">
@@ -11078,13 +11078,13 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1060.5</v>
+        <v>1065.48</v>
       </c>
       <c r="C57" s="13" t="n">
-        <v>1153.74</v>
+        <v>1156.81</v>
       </c>
       <c r="D57" s="13" t="n">
-        <v>894.63</v>
+        <v>901.5</v>
       </c>
     </row>
     <row r="58">
@@ -11094,13 +11094,13 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1082.96</v>
+        <v>1088.02</v>
       </c>
       <c r="C58" s="13" t="n">
-        <v>1165.85</v>
+        <v>1168.96</v>
       </c>
       <c r="D58" s="13" t="n">
-        <v>932.4299999999999</v>
+        <v>939.59</v>
       </c>
     </row>
     <row r="59">
@@ -11110,13 +11110,13 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1094</v>
+        <v>1099.07</v>
       </c>
       <c r="C59" s="13" t="n">
-        <v>1161.94</v>
+        <v>1165.03</v>
       </c>
       <c r="D59" s="13" t="n">
-        <v>922.45</v>
+        <v>929.53</v>
       </c>
     </row>
     <row r="60">
@@ -11126,13 +11126,13 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1079.78</v>
+        <v>1084.82</v>
       </c>
       <c r="C60" s="13" t="n">
-        <v>1168.42</v>
+        <v>1171.53</v>
       </c>
       <c r="D60" s="13" t="n">
-        <v>916.41</v>
+        <v>923.45</v>
       </c>
     </row>
     <row r="61">
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1057.51</v>
+        <v>1063.67</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1057.51</v>
+        <v>1063.67</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-18.05%</t>
+          <t>-17.92%</t>
         </is>
       </c>
     </row>
@@ -11186,7 +11186,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>135.8</v>
+        <v>135.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:11
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.801807</v>
+        <v>28.798489</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.071568</v>
+        <v>37.067295</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.88579</v>
+        <v>22.883152</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.6</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:19
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.41</v>
+        <v>52.4</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.0325826</v>
+        <v>-0.0326749</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -673,16 +673,16 @@
         <v>-0.256</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>35.433</v>
+        <v>35.429</v>
       </c>
       <c r="J2" s="6" t="n">
         <v>48.933</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.300001</v>
+        <v>22.297874</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.946625</v>
+        <v>13.945294</v>
       </c>
       <c r="M2" s="7" t="n">
         <v>10.795</v>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.63</v>
+        <v>103.57</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>0.22243302</v>
+        <v>0.164408</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
@@ -732,7 +732,7 @@
         <v>-0.67</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.13</v>
+        <v>18.12</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.807</v>
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.735113999999999</v>
+        <v>9.729478</v>
       </c>
       <c r="M3" s="7" t="n">
         <v>13.981</v>
@@ -755,7 +755,7 @@
         <v>1.177</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="Q3" s="4" t="n">
         <v>-0.525</v>
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.58</v>
+        <v>37.57</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>0.24006441</v>
+        <v>0.213385</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -913,16 +913,16 @@
         <v>-0.064</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10.278</v>
+        <v>10.276</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>39.718</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>49.447372</v>
+        <v>49.43421</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>16.038513</v>
+        <v>16.034245</v>
       </c>
       <c r="M6" s="7" t="n">
         <v>16.869</v>
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.92</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>-0.02297637</v>
+        <v>-0.022740667</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -972,16 +972,16 @@
         <v>-0.078</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.26</v>
+        <v>6.261</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>8.763999999999999</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6755319</v>
+        <v>3.6764185</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>10.177466</v>
+        <v>10.179922</v>
       </c>
       <c r="M7" s="7" t="n">
         <v>7.297</v>
@@ -996,7 +996,7 @@
         <v>0.235</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>-0.036</v>
+        <v>-0.035</v>
       </c>
     </row>
     <row r="8">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.46</v>
+        <v>21.45</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.020985446</v>
+        <v>-0.0214416</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1328,7 +1328,7 @@
         <v>-0.053</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4.996</v>
+        <v>4.993</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.22580000000001</v>
+        <v>69.19355</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>28.765213</v>
+        <v>28.751812</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,7 +1355,7 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.953</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="Q13" s="9" t="n">
         <v>0.111</v>
@@ -1378,10 +1378,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.5409559</v>
+        <v>-0.463674</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
@@ -1390,10 +1390,10 @@
         <v>12.53</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.307</v>
+        <v>-0.306</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.375</v>
+        <v>2.377</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>5.956</v>
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>11.9438715</v>
+        <v>11.953153</v>
       </c>
       <c r="M14" s="7" t="n">
         <v>6.753</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>-0.008</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>-0.144</v>
+        <v>-0.143</v>
       </c>
     </row>
     <row r="15">
@@ -1621,7 +1621,7 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-0.04130436000000001</v>
+        <v>-0.0413044</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
@@ -1684,7 +1684,7 @@
         <v>11.09</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-0.015090996</v>
+        <v>-0.0150977</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1804,7 +1804,7 @@
         <v>11.31</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.05117447</v>
+        <v>-0.0511745</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -2152,10 +2152,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.41</v>
+        <v>52.4</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.0325826</v>
+        <v>-0.0326749</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>-0.192</v>
@@ -2167,7 +2167,7 @@
         <v>52.2</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.078</v>
+        <v>-0.079</v>
       </c>
       <c r="J2" s="5" t="n">
         <v>-0.059</v>
@@ -2199,16 +2199,16 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.63</v>
+        <v>103.57</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.22243302</v>
+        <v>0.164408</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>-0.525</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5629999999999999</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-60</v>
@@ -2217,7 +2217,7 @@
         <v>-0.28</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.5489999999999999</v>
+        <v>-0.55</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>-0.67</v>
@@ -2340,10 +2340,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.58</v>
+        <v>37.57</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.24006441</v>
+        <v>0.213385</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.03</v>
@@ -2358,7 +2358,7 @@
         <v>0.06</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.06900000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>-0.064</v>
@@ -2387,13 +2387,13 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.92</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0.02297637</v>
+        <v>-0.022740667</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.036</v>
+        <v>-0.035</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0.235</v>
@@ -2669,25 +2669,25 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.46</v>
+        <v>21.45</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.020985446</v>
+        <v>-0.0214416</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.111</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.953</v>
+        <v>0.9520000000000001</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>50.3</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.141</v>
+        <v>0.14</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.174</v>
+        <v>0.173</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>-0.053</v>
@@ -2716,16 +2716,16 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.5409559</v>
+        <v>-0.463674</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.144</v>
+        <v>-0.143</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.008</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>12.6</v>
@@ -2734,10 +2734,10 @@
         <v>-0.066</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.167</v>
+        <v>-0.166</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.307</v>
+        <v>-0.306</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2907,7 +2907,7 @@
         <v>4.41</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.04130436000000001</v>
+        <v>-0.0413044</v>
       </c>
       <c r="F18" s="5" t="n">
         <v>-0.591</v>
@@ -2954,7 +2954,7 @@
         <v>11.09</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.015090996</v>
+        <v>-0.0150977</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>-0.025</v>
@@ -3048,7 +3048,7 @@
         <v>11.31</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.05117447</v>
+        <v>-0.0511745</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>-0.32</v>
@@ -3342,16 +3342,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>52.41</v>
+        <v>52.4</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>35.433</v>
+        <v>35.429</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.300001</v>
+        <v>22.297874</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.946625</v>
+        <v>13.945294</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>10.795</v>
@@ -3363,10 +3363,10 @@
         <v>3.759</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.243208</v>
+        <v>22.241087</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.7220423</v>
+        <v>2.7217827</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>103.63</v>
+        <v>103.57</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.13</v>
+        <v>18.12</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,7 +3406,7 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.735113999999999</v>
+        <v>9.729478</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>13.981</v>
@@ -3418,10 +3418,10 @@
         <v>1.819</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>2.009112</v>
+        <v>2.0079486</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.106654</v>
+        <v>1.1060134</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3558,16 +3558,16 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>37.58</v>
+        <v>37.57</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>10.278</v>
+        <v>10.276</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>49.447372</v>
+        <v>49.43421</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>16.038513</v>
+        <v>16.034245</v>
       </c>
       <c r="H6" s="7" t="n">
         <v>16.869</v>
@@ -3579,10 +3579,10 @@
         <v>2.265</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.9948978</v>
+        <v>3.9938345</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5860735</v>
+        <v>0.58591753</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,16 +3611,16 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>82.92</v>
+        <v>82.94</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.26</v>
+        <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6755319</v>
+        <v>3.6764185</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>10.177466</v>
+        <v>10.179922</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>7.297</v>
@@ -3632,10 +3632,10 @@
         <v>2.142</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.4276135</v>
+        <v>2.428199</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.5297729</v>
+        <v>1.530142</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>21.46</v>
+        <v>21.45</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>4.996</v>
+        <v>4.993</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.22580000000001</v>
+        <v>69.19355</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>28.765213</v>
+        <v>28.751812</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>14.568906</v>
+        <v>14.562119</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.40359</v>
+        <v>4.401539</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.375</v>
+        <v>2.377</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,7 +4001,7 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11.9438715</v>
+        <v>11.953153</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>6.753</v>
@@ -4013,10 +4013,10 @@
         <v>2.372</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.7482383</v>
+        <v>2.7503736</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.9457917</v>
+        <v>0.9465267000000001</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>52.41</v>
+        <v>52.4</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6301,7 +6301,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>103.63</v>
+        <v>103.57</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6324,7 +6324,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.002</v>
+        <v>1.003</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6473,7 +6473,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>37.58</v>
+        <v>37.57</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.135</v>
+        <v>0.136</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6531,7 +6531,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>82.92</v>
+        <v>82.94</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.798489</v>
+        <v>28.868347</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.067295</v>
+        <v>37.15721</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.883152</v>
+        <v>22.938662</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.6</v>
+        <v>0.604</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>21.46</v>
+        <v>21.45</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6929,7 +6929,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.87</v>
+        <v>12.88</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6952,7 +6952,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.405</v>
+        <v>0.404</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.58</v>
@@ -7697,10 +7697,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>35.433</v>
+        <v>35.429</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.300001</v>
+        <v>22.297874</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.278</v>
+        <v>10.276</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.447372</v>
+        <v>49.43421</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.06</v>
@@ -7941,10 +7941,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.26</v>
+        <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6755319</v>
+        <v>3.6764185</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7956,7 +7956,7 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.036</v>
+        <v>-0.035</v>
       </c>
       <c r="J10" s="7" t="n">
         <v>7.297</v>
@@ -8363,10 +8363,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>4.996</v>
+        <v>4.993</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>69.22580000000001</v>
+        <v>69.19355</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.888</v>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.13</v>
+        <v>18.12</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8657,7 +8657,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.375</v>
+        <v>2.377</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8674,7 +8674,7 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.144</v>
+        <v>-0.143</v>
       </c>
       <c r="J29" s="7" t="n">
         <v>6.753</v>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1298.6</v>
+        <v>1298.61</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1222.04</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1291.07</v>
+        <v>1291.08</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1212.98</v>
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1295.92</v>
+        <v>1295.94</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1215.21</v>
@@ -10246,7 +10246,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1296.87</v>
+        <v>1296.89</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1223.3</v>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1281.75</v>
+        <v>1281.77</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1230.58</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1232.89</v>
+        <v>1232.9</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1226.61</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1258.46</v>
+        <v>1258.47</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1226.48</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1229.1</v>
+        <v>1229.11</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1234.6</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1224.8</v>
+        <v>1224.81</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1236.53</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1216.78</v>
+        <v>1216.79</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1234.06</v>
@@ -10358,7 +10358,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1214.38</v>
+        <v>1214.4</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1228</v>
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1233.93</v>
+        <v>1233.95</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1231.34</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1196.68</v>
+        <v>1196.7</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1230.31</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1172.37</v>
+        <v>1172.38</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1205.26</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1178.98</v>
+        <v>1179</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1219.17</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1184.29</v>
+        <v>1184.3</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1225.54</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1168.86</v>
+        <v>1168.88</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1225.99</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1174.69</v>
+        <v>1174.71</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1232.21</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1161.28</v>
+        <v>1161.3</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1237.12</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1162.85</v>
+        <v>1162.87</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1237</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1110.37</v>
+        <v>1110.39</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1234.54</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1098.4</v>
+        <v>1098.42</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1230.86</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1116.61</v>
+        <v>1116.63</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1236.98</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1112.97</v>
+        <v>1112.99</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1226.52</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1134.74</v>
+        <v>1134.76</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1220.58</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1109.48</v>
+        <v>1109.5</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1205.33</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1136.9</v>
+        <v>1136.92</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1228.46</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1138.86</v>
+        <v>1138.88</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1234.38</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1135.73</v>
+        <v>1135.75</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1231.13</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1120.62</v>
+        <v>1120.64</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1230.84</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1082.75</v>
+        <v>1082.78</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1211.83</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1073</v>
+        <v>1073.03</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1212.68</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1088.18</v>
+        <v>1088.21</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1214.64</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1122.75</v>
+        <v>1122.77</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1220.76</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1117.62</v>
+        <v>1117.65</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1217.54</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1117.81</v>
+        <v>1117.84</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1226.34</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1073.63</v>
+        <v>1073.66</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1213.82</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1088.64</v>
+        <v>1088.67</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1222.64</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1092.87</v>
+        <v>1092.9</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1232.96</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1122.72</v>
+        <v>1122.74</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1226.11</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1109.74</v>
+        <v>1109.77</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1220.22</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1104.43</v>
+        <v>1104.46</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1220.92</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1100.52</v>
+        <v>1100.55</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1210.16</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1116.42</v>
+        <v>1116.45</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1218.69</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1114.17</v>
+        <v>1114.2</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1211.9</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1081.76</v>
+        <v>1081.79</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1196.01</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1083.22</v>
+        <v>1083.25</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1206.49</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1082.14</v>
+        <v>1082.17</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1204.55</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1097.52</v>
+        <v>1097.55</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1203.04</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1082.93</v>
+        <v>1082.95</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1184.77</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1084.86</v>
+        <v>1084.88</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1178.07</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1077.08</v>
+        <v>1077.11</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1190.06</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1089.68</v>
+        <v>1089.71</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1193.19</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1081.55</v>
+        <v>1081.57</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1176.54</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1094.46</v>
+        <v>1094.48</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1173.64</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1065.48</v>
+        <v>1065.51</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1156.81</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1088.02</v>
+        <v>1088.04</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1168.96</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1099.07</v>
+        <v>1099.1</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1165.03</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1084.82</v>
+        <v>1084.84</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1171.53</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1063.67</v>
+        <v>1063.63</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1063.67</v>
+        <v>1063.63</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-17.92%</t>
+          <t>-17.93%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:47
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.831713</v>
+        <v>28.828388</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.110058</v>
+        <v>37.105778</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.909552</v>
+        <v>22.90691</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.602</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 15:50
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.828388</v>
+        <v>28.825064</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.105778</v>
+        <v>37.1015</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.90691</v>
+        <v>22.904268</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.602</v>
+        <v>0.601</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 19:38
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -676,19 +676,19 @@
         <v>35.429</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>48.933</v>
+        <v>47.743</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>22.297874</v>
+        <v>23.083702</v>
       </c>
       <c r="L2" s="7" t="n">
         <v>13.945294</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>10.795</v>
+        <v>10.532</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="O2" s="8" t="n">
         <v>0.888</v>
@@ -732,10 +732,10 @@
         <v>-0.67</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>18.12</v>
+        <v>18.117</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>29.807</v>
+        <v>29.837</v>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
@@ -746,7 +746,7 @@
         <v>9.729478</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>13.981</v>
+        <v>13.995</v>
       </c>
       <c r="N3" s="7" t="n">
         <v>9.6</v>
@@ -781,7 +781,7 @@
         <v>21.27</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.70027834</v>
+        <v>-0.700278</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -796,7 +796,7 @@
         <v>10.588</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>11.322</v>
+        <v>11.248</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
@@ -807,10 +807,10 @@
         <v>10.928429</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>41.491</v>
+        <v>41.22</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.682</v>
@@ -842,7 +842,7 @@
         <v>99.47</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.023751085</v>
+        <v>-0.0237511</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -857,19 +857,19 @@
         <v>10.373</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>19.942</v>
+        <v>19.694</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>31.678343</v>
+        <v>32.50654</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>16.740803</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>11.398</v>
+        <v>11.256</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>1.034</v>
@@ -916,7 +916,7 @@
         <v>10.276</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>39.718</v>
+        <v>39.739</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>49.43421</v>
@@ -925,7 +925,7 @@
         <v>16.034245</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>16.869</v>
+        <v>16.877</v>
       </c>
       <c r="N6" s="7" t="n">
         <v>11.7</v>
@@ -975,19 +975,19 @@
         <v>6.261</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8.763999999999999</v>
+        <v>8.618</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.6764185</v>
+        <v>3.7614515</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>10.179922</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>7.297</v>
+        <v>7.176</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>1.22</v>
@@ -1019,7 +1019,7 @@
         <v>87.56999999999999</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.4243151000000001</v>
+        <v>0.424315</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1034,16 +1034,16 @@
         <v>6.103</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11.12</v>
+        <v>11.147</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.553875</v>
+        <v>16.460526</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>11.793877</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>11.623</v>
+        <v>11.652</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>9.800000000000001</v>
@@ -1078,7 +1078,7 @@
         <v>55.74</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.051234016</v>
+        <v>-0.051234</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1093,19 +1093,19 @@
         <v>5.732</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6.886</v>
+        <v>6.711</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>17.865385</v>
+        <v>18.831081</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>16.963236</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>8.461</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>1.453</v>
@@ -1137,7 +1137,7 @@
         <v>26.89</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>0.26099813</v>
+        <v>0.260998</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1152,7 +1152,7 @@
         <v>5.488</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>30.375</v>
+        <v>30.39</v>
       </c>
       <c r="K10" s="7" t="inlineStr">
         <is>
@@ -1163,7 +1163,7 @@
         <v>26.208576</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>8.691000000000001</v>
+        <v>8.695</v>
       </c>
       <c r="N10" s="7" t="n">
         <v>7.3</v>
@@ -1257,7 +1257,7 @@
         <v>18</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.027552686</v>
+        <v>-0.0275527</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>32.22</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>69.19355</v>
+        <v>71.5</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>28.751812</v>
@@ -1396,7 +1396,7 @@
         <v>2.377</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>5.956</v>
+        <v>5.945</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
@@ -1407,7 +1407,7 @@
         <v>11.953153</v>
       </c>
       <c r="M14" s="7" t="n">
-        <v>6.753</v>
+        <v>6.74</v>
       </c>
       <c r="N14" s="7" t="n">
         <v>5.8</v>
@@ -1442,7 +1442,7 @@
         <v>5.53</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.9124123000000001</v>
+        <v>0.9124120000000001</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1457,7 +1457,7 @@
         <v>2.25</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12.774</v>
+        <v>12.833</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>12.021739</v>
@@ -1466,10 +1466,10 @@
         <v>6.9508166</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>10.592</v>
+        <v>10.64</v>
       </c>
       <c r="N15" s="7" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="O15" s="8" t="n">
         <v>0.603</v>
@@ -1501,7 +1501,7 @@
         <v>14.57</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.61391646</v>
+        <v>-0.613916</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1562,7 +1562,7 @@
         <v>97.22</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.022619884</v>
+        <v>-0.0226199</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1577,7 +1577,7 @@
         <v>1.739</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.696</v>
+        <v>1.656</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>17.904236</v>
@@ -1586,10 +1586,10 @@
         <v>16.353237</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>8.893000000000001</v>
+        <v>8.682</v>
       </c>
       <c r="N17" s="7" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>1.376</v>
@@ -1636,7 +1636,7 @@
         <v>1.134</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0.883</v>
+        <v>0.836</v>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
@@ -1647,7 +1647,7 @@
         <v>4.454545</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>-7.324</v>
+        <v>-6.936</v>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
@@ -1743,7 +1743,7 @@
         <v>26.42</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>0.11368203</v>
+        <v>0.113682</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1758,7 +1758,7 @@
         <v>0.697</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.154</v>
+        <v>1.155</v>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
@@ -1769,7 +1769,7 @@
         <v>21.83471</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>9.455</v>
+        <v>9.462</v>
       </c>
       <c r="N20" s="7" t="n">
         <v>7.2</v>
@@ -1867,7 +1867,7 @@
         <v>6.87</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.025373147</v>
+        <v>0.0253731</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1928,7 +1928,7 @@
         <v>2.28</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-0.8695644</v>
+        <v>-0.869564</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1943,7 +1943,7 @@
         <v>0.082</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.577</v>
+        <v>0.576</v>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
         <v>-5.5609756</v>
       </c>
       <c r="M23" s="7" t="n">
-        <v>12.524</v>
+        <v>12.508</v>
       </c>
       <c r="N23" s="7" t="n">
         <v>9</v>
@@ -2249,7 +2249,7 @@
         <v>21.27</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.70027834</v>
+        <v>-0.700278</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.404</v>
@@ -2296,7 +2296,7 @@
         <v>99.47</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.023751085</v>
+        <v>-0.0237511</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.187</v>
@@ -2437,7 +2437,7 @@
         <v>87.56999999999999</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.4243151000000001</v>
+        <v>0.424315</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.218</v>
@@ -2484,7 +2484,7 @@
         <v>55.74</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.051234016</v>
+        <v>-0.051234</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.09699999999999999</v>
@@ -2531,7 +2531,7 @@
         <v>26.89</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.26099813</v>
+        <v>0.260998</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.141</v>
@@ -2625,7 +2625,7 @@
         <v>18</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.027552686</v>
+        <v>-0.0275527</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>-0.228</v>
@@ -2766,7 +2766,7 @@
         <v>5.53</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.9124123000000001</v>
+        <v>0.9124120000000001</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.264</v>
@@ -2813,7 +2813,7 @@
         <v>14.57</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.61391646</v>
+        <v>-0.613916</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-0.019</v>
@@ -2860,7 +2860,7 @@
         <v>97.22</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.022619884</v>
+        <v>-0.0226199</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>0.015</v>
@@ -3001,7 +3001,7 @@
         <v>26.42</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.11368203</v>
+        <v>0.113682</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>-0.023</v>
@@ -3097,7 +3097,7 @@
         <v>6.87</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.025373147</v>
+        <v>0.0253731</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-0.234</v>
@@ -3144,7 +3144,7 @@
         <v>2.28</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.8695644</v>
+        <v>-0.869564</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-0.08800000000000001</v>
@@ -3348,19 +3348,19 @@
         <v>35.429</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>22.297874</v>
+        <v>23.083702</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>13.945294</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>10.795</v>
+        <v>10.532</v>
       </c>
       <c r="I2" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>3.759</v>
+        <v>3.668</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>22.241087</v>
@@ -3369,7 +3369,7 @@
         <v>2.7217827</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>2.35</v>
+        <v>2.27</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>3.75754</v>
@@ -3398,7 +3398,7 @@
         <v>103.57</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>18.12</v>
+        <v>18.117</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3409,19 +3409,19 @@
         <v>9.729478</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>13.981</v>
+        <v>13.995</v>
       </c>
       <c r="I3" s="7" t="n">
         <v>9.6</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1.819</v>
+        <v>1.821</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.0079486</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.1060134</v>
+        <v>1.1058283</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3464,13 +3464,13 @@
         <v>10.928429</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>41.491</v>
+        <v>41.22</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1.87</v>
+        <v>1.858</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>16.66928</v>
@@ -3511,28 +3511,28 @@
         <v>10.373</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>31.678343</v>
+        <v>32.50654</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>16.740803</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>11.398</v>
+        <v>11.256</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2.794</v>
+        <v>2.759</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>-37.00521</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4532318</v>
+        <v>1.4532319</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>3.14</v>
+        <v>3.06</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>5.94177</v>
@@ -3570,13 +3570,13 @@
         <v>16.034245</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>16.869</v>
+        <v>16.877</v>
       </c>
       <c r="I6" s="7" t="n">
         <v>11.7</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>2.265</v>
+        <v>2.266</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>3.9938345</v>
@@ -3617,19 +3617,19 @@
         <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.6764185</v>
+        <v>3.7614515</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>10.179922</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>7.297</v>
+        <v>7.176</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>2.142</v>
+        <v>2.106</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>2.428199</v>
@@ -3638,7 +3638,7 @@
         <v>1.530142</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>22.56</v>
+        <v>22.05</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>8.147410000000001</v>
@@ -3670,19 +3670,19 @@
         <v>6.103</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.553875</v>
+        <v>16.460526</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>11.793877</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>11.623</v>
+        <v>11.652</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.801</v>
+        <v>3.81</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>6.036396</v>
@@ -3691,7 +3691,7 @@
         <v>2.0859604</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>5.29</v>
+        <v>5.32</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>7.42504</v>
@@ -3723,19 +3723,19 @@
         <v>5.732</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>17.865385</v>
+        <v>18.831081</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>16.963236</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>8.461</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.423</v>
+        <v>3.336</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>15.604704</v>
@@ -3744,7 +3744,7 @@
         <v>2.8494256</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>3.12</v>
+        <v>2.96</v>
       </c>
       <c r="N9" s="3" t="n">
         <v>3.28593</v>
@@ -3784,13 +3784,13 @@
         <v>26.208576</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>8.691000000000001</v>
+        <v>8.695</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>7.3</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>2.645</v>
+        <v>2.646</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>1.5549644</v>
@@ -3799,7 +3799,7 @@
         <v>0.47783932</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-2.42</v>
+        <v>-2.43</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>1.026</v>
@@ -3937,7 +3937,7 @@
         <v>4.993</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>69.19355</v>
+        <v>71.5</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>28.751812</v>
@@ -3964,7 +3964,7 @@
         <v>4.401539</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.31</v>
+        <v>0.3</v>
       </c>
       <c r="N13" s="3" t="n">
         <v>0.74604</v>
@@ -4004,13 +4004,13 @@
         <v>11.953153</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>6.753</v>
+        <v>6.74</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>5.8</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>2.372</v>
+        <v>2.367</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.7503736</v>
@@ -4057,13 +4057,13 @@
         <v>6.9508166</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>10.592</v>
+        <v>10.64</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>2.474</v>
+        <v>2.485</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>-1.7329991</v>
@@ -4165,13 +4165,13 @@
         <v>16.353237</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>8.893000000000001</v>
+        <v>8.682</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>3.111</v>
+        <v>3.037</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>3.2219791</v>
@@ -4220,7 +4220,7 @@
         <v>4.454545</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-7.324</v>
+        <v>-6.936</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
@@ -4228,7 +4228,7 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1.319</v>
+        <v>1.249</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>1.4994899</v>
@@ -4237,7 +4237,7 @@
         <v>1.694536</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>-0.44</v>
+        <v>-0.42</v>
       </c>
       <c r="N18" s="3" t="n">
         <v>0.99</v>
@@ -4330,13 +4330,13 @@
         <v>21.83471</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>9.455</v>
+        <v>9.462</v>
       </c>
       <c r="I20" s="7" t="n">
         <v>7.2</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1.818</v>
+        <v>1.819</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>1.6436481</v>
@@ -4495,13 +4495,13 @@
         <v>-5.5609756</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12.524</v>
+        <v>12.508</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>9</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>1.909</v>
+        <v>1.906</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>32.571426</v>
@@ -4510,7 +4510,7 @@
         <v>0.27283052</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>-1.12</v>
+        <v>-1.11</v>
       </c>
       <c r="N23" s="3" t="n">
         <v>-0.41</v>
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.825064</v>
+        <v>28.754496</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.1015</v>
+        <v>37.09294</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.904268</v>
+        <v>22.898985</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.601</v>
+        <v>0.597</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>
@@ -7141,7 +7141,7 @@
         <v>0.64763</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>1.21</v>
+        <v>1.24</v>
       </c>
       <c r="P17" s="5" t="n">
         <v>0.221</v>
@@ -7700,7 +7700,7 @@
         <v>35.429</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>22.297874</v>
+        <v>23.083702</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7715,10 +7715,10 @@
         <v>-0.192</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10.795</v>
+        <v>10.532</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="L3" s="7" t="n">
         <v>82</v>
@@ -7761,7 +7761,7 @@
         <v>0.141</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>8.691000000000001</v>
+        <v>8.695</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>7.3</v>
@@ -7790,7 +7790,7 @@
         <v>10.373</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>31.678343</v>
+        <v>32.50654</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7807,10 +7807,10 @@
         <v>-0.187</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>11.398</v>
+        <v>11.256</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>9.199999999999999</v>
+        <v>9</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>41.7</v>
@@ -7853,10 +7853,10 @@
         <v>-0.264</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>10.592</v>
+        <v>10.64</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>8.4</v>
+        <v>8.5</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>40</v>
@@ -7897,7 +7897,7 @@
         <v>0.03</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>16.869</v>
+        <v>16.877</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>11.7</v>
@@ -7944,7 +7944,7 @@
         <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.6764185</v>
+        <v>3.7614515</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7959,10 +7959,10 @@
         <v>-0.035</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>7.297</v>
+        <v>7.176</v>
       </c>
       <c r="K10" s="7" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>69</v>
@@ -7988,7 +7988,7 @@
         <v>6.103</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.553875</v>
+        <v>16.460526</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8003,7 +8003,7 @@
         <v>-0.218</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.623</v>
+        <v>11.652</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>9.800000000000001</v>
@@ -8015,12 +8015,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Monarch Casino &amp; Resort</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -8029,42 +8029,42 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.732</v>
+        <v>1.739</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.865385</v>
+        <v>17.904236</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.032</v>
+        <v>0.041</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.4046</v>
+        <v>0.34986</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>1.113</v>
+        <v>0.19214001</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.09699999999999999</v>
+        <v>0.015</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.461</v>
+        <v>8.682</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>7.4</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>60.3</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>MCRI</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Monarch Casino &amp; Resort</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -8073,31 +8073,31 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.739</v>
+        <v>5.732</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.904236</v>
+        <v>18.831081</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.041</v>
+        <v>0.032</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.34986</v>
+        <v>0.4046</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0.19214001</v>
+        <v>1.113</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.015</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.893000000000001</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>7.6</v>
+        <v>7.2</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>57.1</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="14">
@@ -8183,7 +8183,7 @@
         <v>-0.023</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>9.455</v>
+        <v>9.462</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>7.2</v>
@@ -8275,7 +8275,7 @@
         <v>-0.08800000000000001</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>12.524</v>
+        <v>12.508</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>9</v>
@@ -8366,7 +8366,7 @@
         <v>4.993</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>69.19355</v>
+        <v>71.5</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.888</v>
@@ -8475,10 +8475,10 @@
         <v>-0.404</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>41.491</v>
+        <v>41.22</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>17.8</v>
+        <v>17.7</v>
       </c>
       <c r="L23" s="7" t="n">
         <v>52</v>
@@ -8501,7 +8501,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>18.12</v>
+        <v>18.117</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8521,7 +8521,7 @@
         <v>-0.525</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>13.981</v>
+        <v>13.995</v>
       </c>
       <c r="K24" s="7" t="n">
         <v>9.6</v>
@@ -8567,7 +8567,7 @@
         <v>-0.591</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-7.324</v>
+        <v>-6.936</v>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
@@ -8677,7 +8677,7 @@
         <v>-0.143</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>6.753</v>
+        <v>6.74</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>5.8</v>
@@ -10198,7 +10198,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1298.61</v>
+        <v>1298.62</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1222.04</v>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1291.08</v>
+        <v>1291.09</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1212.98</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1232.9</v>
+        <v>1232.91</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1226.61</v>
@@ -10294,7 +10294,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1258.47</v>
+        <v>1258.48</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1226.48</v>
@@ -10310,7 +10310,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1229.11</v>
+        <v>1229.12</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1234.6</v>
@@ -10326,7 +10326,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1224.81</v>
+        <v>1224.82</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1236.53</v>
@@ -10342,7 +10342,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1216.79</v>
+        <v>1216.8</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1234.06</v>
@@ -10406,7 +10406,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1172.38</v>
+        <v>1172.39</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1205.26</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1179</v>
+        <v>1179.01</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1219.17</v>
@@ -10438,7 +10438,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1184.3</v>
+        <v>1184.31</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1225.54</v>
@@ -10454,7 +10454,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1168.88</v>
+        <v>1168.89</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1225.99</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1174.71</v>
+        <v>1174.72</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1232.21</v>
@@ -10486,7 +10486,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1161.3</v>
+        <v>1161.31</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1237.12</v>
@@ -10502,7 +10502,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1162.87</v>
+        <v>1162.88</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1237</v>
@@ -10518,7 +10518,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1110.39</v>
+        <v>1110.4</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1234.54</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1098.42</v>
+        <v>1098.43</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1230.86</v>
@@ -10550,7 +10550,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1116.63</v>
+        <v>1116.64</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1236.98</v>
@@ -10566,7 +10566,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1112.99</v>
+        <v>1113</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1226.52</v>
@@ -10582,7 +10582,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1134.76</v>
+        <v>1134.77</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1220.58</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1109.5</v>
+        <v>1109.52</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1205.33</v>
@@ -10614,7 +10614,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1136.92</v>
+        <v>1136.93</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1228.46</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1138.88</v>
+        <v>1138.89</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1234.38</v>
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1135.75</v>
+        <v>1135.76</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1231.13</v>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1120.64</v>
+        <v>1120.65</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1230.84</v>
@@ -10678,7 +10678,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1082.78</v>
+        <v>1082.79</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1211.83</v>
@@ -10694,7 +10694,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1073.03</v>
+        <v>1073.04</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1212.68</v>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1088.21</v>
+        <v>1088.22</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1214.64</v>
@@ -10726,7 +10726,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1122.77</v>
+        <v>1122.79</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1220.76</v>
@@ -10742,7 +10742,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1117.65</v>
+        <v>1117.66</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1217.54</v>
@@ -10758,7 +10758,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1117.84</v>
+        <v>1117.85</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1226.34</v>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1073.66</v>
+        <v>1073.67</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1213.82</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1088.67</v>
+        <v>1088.68</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1222.64</v>
@@ -10806,7 +10806,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1092.9</v>
+        <v>1092.91</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1232.96</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1122.74</v>
+        <v>1122.76</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1226.11</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1109.77</v>
+        <v>1109.79</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1220.22</v>
@@ -10854,7 +10854,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1104.46</v>
+        <v>1104.48</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1220.92</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1100.55</v>
+        <v>1100.56</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1210.16</v>
@@ -10886,7 +10886,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1116.45</v>
+        <v>1116.46</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1218.69</v>
@@ -10902,7 +10902,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1114.2</v>
+        <v>1114.21</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1211.9</v>
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1081.79</v>
+        <v>1081.8</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1196.01</v>
@@ -10934,7 +10934,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1083.25</v>
+        <v>1083.26</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1206.49</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1082.17</v>
+        <v>1082.18</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1204.55</v>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1097.55</v>
+        <v>1097.57</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1203.04</v>
@@ -10982,7 +10982,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1082.95</v>
+        <v>1082.97</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1184.77</v>
@@ -10998,7 +10998,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1084.88</v>
+        <v>1084.9</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1178.07</v>
@@ -11014,7 +11014,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1077.11</v>
+        <v>1077.12</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1190.06</v>
@@ -11030,7 +11030,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1089.71</v>
+        <v>1089.73</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1193.19</v>
@@ -11046,7 +11046,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1081.57</v>
+        <v>1081.59</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1176.54</v>
@@ -11062,7 +11062,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1094.48</v>
+        <v>1094.5</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1173.64</v>
@@ -11078,7 +11078,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1065.51</v>
+        <v>1065.53</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1156.81</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1088.04</v>
+        <v>1088.05</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1168.96</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1099.1</v>
+        <v>1099.11</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1165.03</v>
@@ -11126,7 +11126,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1084.84</v>
+        <v>1084.86</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1171.53</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1063.63</v>
+        <v>1063.64</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1063.63</v>
+        <v>1063.64</v>
       </c>
     </row>
     <row r="64">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 19:45
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -1278,7 +1278,7 @@
         <v>49.999996</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>21.844957</v>
+        <v>21.943403</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>10.358</v>
@@ -1516,7 +1516,7 @@
         <v>1.946</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>12.438</v>
+        <v>12.427</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         <v>8.419385999999999</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>17.223</v>
+        <v>17.207</v>
       </c>
       <c r="N16" s="7" t="n">
         <v>10.9</v>
@@ -3887,7 +3887,7 @@
         <v>49.999996</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>21.844957</v>
+        <v>21.943403</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>10.358</v>
@@ -3899,7 +3899,7 @@
         <v>4.075</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.75748</v>
+        <v>4.77892</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>4.1296697</v>
@@ -3908,10 +3908,10 @@
         <v>0.36</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.8239888</v>
+        <v>0.8202921</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>3.7835155</v>
+        <v>3.7665412</v>
       </c>
     </row>
     <row r="13">
@@ -4112,13 +4112,13 @@
         <v>8.419385999999999</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17.223</v>
+        <v>17.207</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>10.9</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>1.787</v>
+        <v>1.785</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>1.00296</v>
@@ -4400,7 +4400,7 @@
         <v>0.20929217</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-12.45</v>
+        <v>-11.81</v>
       </c>
       <c r="N21" s="3" t="n">
         <v>-0.8100000000000001</v>
@@ -8137,7 +8137,7 @@
         <v>-0.019</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.223</v>
+        <v>17.207</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>10.9</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 20:04
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -1272,7 +1272,7 @@
         <v>5.327</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>5.256</v>
+        <v>5.103</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>49.999996</v>
@@ -1281,10 +1281,10 @@
         <v>21.943403</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>10.358</v>
+        <v>10.056</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>2.002</v>
@@ -1699,7 +1699,7 @@
         <v>0.905</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>1.242</v>
+        <v>1.228</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>18.483334</v>
@@ -1708,7 +1708,7 @@
         <v>11.975854</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>6.569</v>
+        <v>6.496</v>
       </c>
       <c r="N19" s="7" t="n">
         <v>4.6</v>
@@ -1816,10 +1816,10 @@
         <v>-0.455</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.556</v>
+        <v>0.549</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>7.795</v>
+        <v>7.765</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -1830,10 +1830,10 @@
         <v>-13.962963</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>22.644</v>
+        <v>22.558</v>
       </c>
       <c r="N21" s="7" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
         <v>0.186</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.512</v>
+        <v>0.517</v>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
@@ -1893,10 +1893,10 @@
         <v>9.170271</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>6.891</v>
+        <v>6.953</v>
       </c>
       <c r="N22" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>1.206</v>
@@ -3890,13 +3890,13 @@
         <v>21.943403</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>10.358</v>
+        <v>10.056</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>4.075</v>
+        <v>3.956</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.77892</v>
@@ -4275,13 +4275,13 @@
         <v>11.975854</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>6.569</v>
+        <v>6.496</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>4.6</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.923</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>3.384193</v>
@@ -4374,7 +4374,7 @@
         <v>11.31</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.556</v>
+        <v>0.549</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4385,19 +4385,19 @@
         <v>-13.962963</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>22.644</v>
+        <v>22.558</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>2.934</v>
+        <v>2.923</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>0.5517612</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.20929217</v>
+        <v>0.20662428</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>-11.81</v>
@@ -4440,13 +4440,13 @@
         <v>9.170271</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>6.891</v>
+        <v>6.953</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1.684</v>
+        <v>1.699</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>-11.393035</v>
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.754496</v>
+        <v>28.764448</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.09294</v>
+        <v>37.105778</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.898985</v>
+        <v>22.90691</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.597</v>
+        <v>0.598</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>
@@ -8209,7 +8209,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.556</v>
+        <v>0.549</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8229,10 +8229,10 @@
         <v>-0.32</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>22.644</v>
+        <v>22.558</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="L16" s="7" t="n">
         <v>28.6</v>
@@ -8429,10 +8429,10 @@
         <v>-0.228</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>10.358</v>
+        <v>10.056</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>9</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L22" s="7" t="n">
         <v>55</v>
@@ -8631,7 +8631,7 @@
         <v>-0.025</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>6.569</v>
+        <v>6.496</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>4.6</v>
@@ -8725,10 +8725,10 @@
         <v>-0.234</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>6.891</v>
+        <v>6.953</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="L30" s="7" t="n">
         <v>29.1</v>
@@ -10278,7 +10278,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1232.91</v>
+        <v>1232.9</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1226.61</v>
@@ -10422,7 +10422,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1179.01</v>
+        <v>1179</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1219.17</v>
@@ -10470,7 +10470,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1174.72</v>
+        <v>1174.71</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1232.21</v>
@@ -10534,7 +10534,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1098.43</v>
+        <v>1098.42</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1230.86</v>
@@ -10598,7 +10598,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1109.52</v>
+        <v>1109.51</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1205.33</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1138.89</v>
+        <v>1138.9</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1234.38</v>
@@ -10790,7 +10790,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1088.68</v>
+        <v>1088.69</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1222.64</v>
@@ -10870,7 +10870,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1100.56</v>
+        <v>1100.57</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1210.16</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1082.18</v>
+        <v>1082.19</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1204.55</v>
@@ -11094,7 +11094,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1088.05</v>
+        <v>1088.06</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1168.96</v>
@@ -11110,7 +11110,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1099.11</v>
+        <v>1099.12</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1165.03</v>
@@ -11142,7 +11142,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1063.64</v>
+        <v>1063.65</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11154,7 +11154,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1063.64</v>
+        <v>1063.65</v>
       </c>
     </row>
     <row r="64">
@@ -11165,7 +11165,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-17.93%</t>
+          <t>-17.92%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 20:09
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.764448</v>
+        <v>28.761131</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.105778</v>
+        <v>37.1015</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.90691</v>
+        <v>22.904268</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.598</v>
@@ -11017,7 +11017,7 @@
         <v>1077.12</v>
       </c>
       <c r="C53" s="13" t="n">
-        <v>1190.06</v>
+        <v>1190.05</v>
       </c>
       <c r="D53" s="13" t="n">
         <v>933.5</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 20:13
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.761131</v>
+        <v>28.767765</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.1015</v>
+        <v>37.110058</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.904268</v>
+        <v>22.909552</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.598</v>
@@ -11017,7 +11017,7 @@
         <v>1077.12</v>
       </c>
       <c r="C53" s="13" t="n">
-        <v>1190.05</v>
+        <v>1190.06</v>
       </c>
       <c r="D53" s="13" t="n">
         <v>933.5</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 20:39
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.767765</v>
+        <v>28.78437</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.110058</v>
+        <v>37.131477</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.909552</v>
+        <v>22.922775</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.598</v>
+        <v>0.599</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 20:43
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6827,13 +6827,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.78437</v>
+        <v>28.781048</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.131477</v>
+        <v>37.127193</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.922775</v>
+        <v>22.920128</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.599</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -679,7 +679,7 @@
         <v>47.743</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>23.083702</v>
+        <v>22.297874</v>
       </c>
       <c r="L2" s="7" t="n">
         <v>13.945294</v>
@@ -860,7 +860,7 @@
         <v>19.694</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>32.50654</v>
+        <v>31.678343</v>
       </c>
       <c r="L5" s="7" t="n">
         <v>16.740803</v>
@@ -978,7 +978,7 @@
         <v>8.618</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.7614515</v>
+        <v>3.6764185</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>10.179922</v>
@@ -1034,16 +1034,16 @@
         <v>6.103</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11.147</v>
+        <v>11.146</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.460526</v>
+        <v>16.553875</v>
       </c>
       <c r="L8" s="7" t="n">
         <v>11.793877</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>11.652</v>
+        <v>11.65</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>9.800000000000001</v>
@@ -1096,7 +1096,7 @@
         <v>6.711</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>18.831081</v>
+        <v>17.865385</v>
       </c>
       <c r="L9" s="7" t="n">
         <v>16.963236</v>
@@ -1336,7 +1336,7 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>71.5</v>
+        <v>69.19355</v>
       </c>
       <c r="L13" s="7" t="n">
         <v>28.751812</v>
@@ -3200,7 +3200,7 @@
         <v>-0.239</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>-275.9</v>
+        <v>-268.2</v>
       </c>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
@@ -3348,7 +3348,7 @@
         <v>35.429</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>23.083702</v>
+        <v>22.297874</v>
       </c>
       <c r="G2" s="7" t="n">
         <v>13.945294</v>
@@ -3369,7 +3369,7 @@
         <v>2.7217827</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>2.27</v>
+        <v>2.35</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>3.75754</v>
@@ -3511,7 +3511,7 @@
         <v>10.373</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>32.50654</v>
+        <v>31.678343</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>16.740803</v>
@@ -3532,7 +3532,7 @@
         <v>1.4532319</v>
       </c>
       <c r="M5" s="3" t="n">
-        <v>3.06</v>
+        <v>3.14</v>
       </c>
       <c r="N5" s="3" t="n">
         <v>5.94177</v>
@@ -3617,7 +3617,7 @@
         <v>6.261</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.7614515</v>
+        <v>3.6764185</v>
       </c>
       <c r="G7" s="7" t="n">
         <v>10.179922</v>
@@ -3638,7 +3638,7 @@
         <v>1.530142</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>22.05</v>
+        <v>22.56</v>
       </c>
       <c r="N7" s="3" t="n">
         <v>8.147410000000001</v>
@@ -3670,19 +3670,19 @@
         <v>6.103</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.460526</v>
+        <v>16.553875</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>11.793877</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>11.652</v>
+        <v>11.65</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>9.800000000000001</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.81</v>
+        <v>3.809</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>6.036396</v>
@@ -3691,7 +3691,7 @@
         <v>2.0859604</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>5.32</v>
+        <v>5.29</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>7.42504</v>
@@ -3723,7 +3723,7 @@
         <v>5.732</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>18.831081</v>
+        <v>17.865385</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>16.963236</v>
@@ -3744,7 +3744,7 @@
         <v>2.8494256</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>2.96</v>
+        <v>3.12</v>
       </c>
       <c r="N9" s="3" t="n">
         <v>3.28593</v>
@@ -3799,7 +3799,7 @@
         <v>0.47783932</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>-2.43</v>
+        <v>-2.42</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>1.026</v>
@@ -3937,7 +3937,7 @@
         <v>4.993</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>71.5</v>
+        <v>69.19355</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>28.751812</v>
@@ -3964,7 +3964,7 @@
         <v>4.401539</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>0.3</v>
+        <v>0.31</v>
       </c>
       <c r="N13" s="3" t="n">
         <v>0.74604</v>
@@ -4237,7 +4237,7 @@
         <v>1.694536</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="N18" s="3" t="n">
         <v>0.99</v>
@@ -4510,7 +4510,7 @@
         <v>0.27283052</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>-1.11</v>
+        <v>-1.12</v>
       </c>
       <c r="N23" s="3" t="n">
         <v>-0.41</v>
@@ -6283,7 +6283,7 @@
         <v>0.41691002</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>1.94</v>
+        <v>2</v>
       </c>
       <c r="P2" s="5" t="n">
         <v>0.4255</v>
@@ -6455,7 +6455,7 @@
         <v>0.68557</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -6569,7 +6569,7 @@
         <v>0.73407</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="P7" s="5" t="n">
         <v>0.0319</v>
@@ -6681,7 +6681,7 @@
         <v>0.88883</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>1.77</v>
+        <v>1.87</v>
       </c>
       <c r="P9" s="5" t="n">
         <v>0.32369998</v>
@@ -6967,7 +6967,7 @@
         <v>0.46130002</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7.11</v>
+        <v>7.14</v>
       </c>
       <c r="P14" s="5" t="n">
         <v>8.8889</v>
@@ -7700,7 +7700,7 @@
         <v>35.429</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>23.083702</v>
+        <v>22.297874</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7790,7 +7790,7 @@
         <v>10.373</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>32.50654</v>
+        <v>31.678343</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.015</v>
@@ -7944,7 +7944,7 @@
         <v>6.261</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.7614515</v>
+        <v>3.6764185</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7988,7 +7988,7 @@
         <v>6.103</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.460526</v>
+        <v>16.553875</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8003,7 +8003,7 @@
         <v>-0.218</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.652</v>
+        <v>11.65</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>9.800000000000001</v>
@@ -8015,12 +8015,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>MCRI</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Monarch Casino &amp; Resort</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -8029,42 +8029,42 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1.739</v>
+        <v>5.732</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>17.904236</v>
+        <v>17.865385</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.041</v>
+        <v>0.032</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>0.34986</v>
+        <v>0.4046</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.19214001</v>
+        <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.015</v>
+        <v>-0.09699999999999999</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.682</v>
+        <v>8.244999999999999</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>62.7</v>
+        <v>60.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>MCRI</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Monarch Casino &amp; Resort</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -8073,31 +8073,31 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>5.732</v>
+        <v>1.739</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>18.831081</v>
+        <v>17.904236</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.032</v>
+        <v>0.041</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.4046</v>
+        <v>0.34986</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>1.113</v>
+        <v>0.19214001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.09699999999999999</v>
+        <v>0.015</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.244999999999999</v>
+        <v>8.682</v>
       </c>
       <c r="K13" s="7" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>54.8</v>
+        <v>57.1</v>
       </c>
     </row>
     <row r="14">
@@ -8366,7 +8366,7 @@
         <v>4.993</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>71.5</v>
+        <v>69.19355</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.888</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-26 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-13.962963</v>
+        <v>-7.024845</v>
       </c>
       <c r="M21" s="7" t="n">
         <v>22.558</v>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-13.962963</v>
+        <v>-7.024845</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>22.558</v>
@@ -4403,7 +4403,7 @@
         <v>-11.81</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>-0.8100000000000001</v>
+        <v>-1.61</v>
       </c>
       <c r="O21" s="3" t="n">
         <v>20.498</v>
@@ -6827,16 +6827,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.781048</v>
+        <v>28.771086</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.127193</v>
+        <v>37.11434</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.920128</v>
+        <v>22.912195</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.599</v>
+        <v>0.598</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-29 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -781,7 +781,7 @@
         <v>20.72</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>-0.0258581</v>
+        <v>-0.02585798</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -842,7 +842,7 @@
         <v>96.59</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>-0.0289535</v>
+        <v>-0.028953428</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -1019,7 +1019,7 @@
         <v>84.52</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-0.0348293</v>
+        <v>-0.034829314</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1078,7 +1078,7 @@
         <v>53.89</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.0331898</v>
+        <v>-0.033189785</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1137,7 +1137,7 @@
         <v>25.85</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-0.0386761</v>
+        <v>-0.038676052</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>31.58</v>
@@ -1257,7 +1257,7 @@
         <v>17.15</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.0472222</v>
+        <v>-0.04722224</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>32.22</v>
@@ -1278,7 +1278,7 @@
         <v>47.638885</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>20.939608</v>
+        <v>20.941422</v>
       </c>
       <c r="M12" s="7" t="n">
         <v>12.004</v>
@@ -1442,7 +1442,7 @@
         <v>5.62</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>0.0162748</v>
+        <v>0.016274893</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1501,7 +1501,7 @@
         <v>13.77</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-0.0549073</v>
+        <v>-0.054907355</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1562,7 +1562,7 @@
         <v>93.98</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-0.0333265</v>
+        <v>-0.033326454</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1743,7 +1743,7 @@
         <v>25.91</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-0.0193036</v>
+        <v>-0.019303566</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1867,7 +1867,7 @@
         <v>6.68</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>-0.0276565</v>
+        <v>-0.027656486</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1928,7 +1928,7 @@
         <v>2.15</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-0.0570175</v>
+        <v>-0.05701759</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -2249,7 +2249,7 @@
         <v>20.72</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>-0.0258581</v>
+        <v>-0.02585798</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.419</v>
@@ -2296,7 +2296,7 @@
         <v>96.59</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.0289535</v>
+        <v>-0.028953428</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.21</v>
@@ -2437,7 +2437,7 @@
         <v>84.52</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>-0.0348293</v>
+        <v>-0.034829314</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.245</v>
@@ -2484,7 +2484,7 @@
         <v>53.89</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.0331898</v>
+        <v>-0.033189785</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.127</v>
@@ -2531,7 +2531,7 @@
         <v>25.85</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.0386761</v>
+        <v>-0.038676052</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.09699999999999999</v>
@@ -2625,7 +2625,7 @@
         <v>17.15</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.0472222</v>
+        <v>-0.04722224</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>-0.265</v>
@@ -2766,7 +2766,7 @@
         <v>5.62</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.0162748</v>
+        <v>0.016274893</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.252</v>
@@ -2813,7 +2813,7 @@
         <v>13.77</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.0549073</v>
+        <v>-0.054907355</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-0.073</v>
@@ -2860,7 +2860,7 @@
         <v>93.98</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>-0.0333265</v>
+        <v>-0.033326454</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>-0.018</v>
@@ -3001,7 +3001,7 @@
         <v>25.91</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>-0.0193036</v>
+        <v>-0.019303566</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>-0.042</v>
@@ -3097,7 +3097,7 @@
         <v>6.68</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.0276565</v>
+        <v>-0.027656486</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-0.255</v>
@@ -3144,7 +3144,7 @@
         <v>2.15</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>-0.0570175</v>
+        <v>-0.05701759</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>-0.14</v>
@@ -3887,7 +3887,7 @@
         <v>47.638885</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>20.939608</v>
+        <v>20.941422</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>12.004</v>
@@ -3899,7 +3899,7 @@
         <v>3.758</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.56031</v>
+        <v>4.5607047</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>3.9346576</v>
@@ -3908,10 +3908,10 @@
         <v>0.36</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.819022</v>
+        <v>0.8189511</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>3.7607093</v>
+        <v>3.7603836</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-29 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6829,16 +6829,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.70983</v>
+        <v>28.73629</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>37.02463</v>
+        <v>37.058754</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.856813</v>
+        <v>22.87788</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.674</v>
+        <v>0.6759999999999999</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-30 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -658,10 +658,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>51.65</v>
+        <v>51.62</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>-0.0773788</v>
+        <v>-0.135422</v>
       </c>
       <c r="F2" s="3" t="n">
         <v>70.45</v>
@@ -673,19 +673,19 @@
         <v>-0.267</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>34.922</v>
+        <v>34.902</v>
       </c>
       <c r="J2" s="6" t="n">
-        <v>47.266</v>
+        <v>47.219</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>21.978725</v>
+        <v>21.965958</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>13.745696</v>
+        <v>13.737711</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>10.427</v>
+        <v>10.417</v>
       </c>
       <c r="N2" s="7" t="n">
         <v>8.9</v>
@@ -694,7 +694,7 @@
         <v>0.888</v>
       </c>
       <c r="P2" s="9" t="n">
-        <v>0.365</v>
+        <v>0.364</v>
       </c>
       <c r="Q2" s="4" t="n">
         <v>-0.204</v>
@@ -717,25 +717,25 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>100.18</v>
+        <v>99.5</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>-0.31840765</v>
+        <v>-0.9950249999999999</v>
       </c>
       <c r="F3" s="3" t="n">
         <v>313.685</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>99.90000000000001</v>
+        <v>98.875</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>-0.6809999999999999</v>
+        <v>-0.6829999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>17.51</v>
+        <v>17.391</v>
       </c>
       <c r="J3" s="6" t="n">
-        <v>29.299</v>
+        <v>29.124</v>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
@@ -743,22 +743,22 @@
         </is>
       </c>
       <c r="L3" s="7" t="n">
-        <v>9.792441</v>
+        <v>9.725972000000001</v>
       </c>
       <c r="M3" s="7" t="n">
-        <v>13.742</v>
+        <v>13.66</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O3" s="8" t="n">
         <v>1.177</v>
       </c>
       <c r="P3" s="4" t="n">
-        <v>-0.5479999999999999</v>
+        <v>-0.551</v>
       </c>
       <c r="Q3" s="4" t="n">
-        <v>-0.541</v>
+        <v>-0.544</v>
       </c>
     </row>
     <row r="4">
@@ -778,10 +778,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>20.84</v>
+        <v>20.93</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>0.6032818599999999</v>
+        <v>0.0101352</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -790,13 +790,13 @@
         <v>20.46</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>-0.573</v>
+        <v>-0.5710000000000001</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>10.334</v>
+        <v>10.376</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>10.977</v>
+        <v>11.081</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
@@ -804,22 +804,22 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>10.841299</v>
+        <v>10.885508</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>40.226</v>
+        <v>40.605</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.682</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>-0.3720000000000001</v>
+        <v>-0.37</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>-0.415</v>
+        <v>-0.413</v>
       </c>
     </row>
     <row r="5">
@@ -839,10 +839,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>97.13</v>
+        <v>96.77</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>0.55916774</v>
+        <v>0.186355</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -851,22 +851,22 @@
         <v>65.25</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>-0.279</v>
+        <v>-0.282</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>10.129</v>
+        <v>10.091</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>19.398</v>
+        <v>19.416</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>30.933151</v>
+        <v>30.81847</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>16.346996</v>
+        <v>16.286392</v>
       </c>
       <c r="M5" s="7" t="n">
-        <v>11.087</v>
+        <v>11.098</v>
       </c>
       <c r="N5" s="7" t="n">
         <v>8.9</v>
@@ -875,10 +875,10 @@
         <v>1.034</v>
       </c>
       <c r="P5" s="9" t="n">
-        <v>0.174</v>
+        <v>0.17</v>
       </c>
       <c r="Q5" s="4" t="n">
-        <v>-0.206</v>
+        <v>-0.209</v>
       </c>
     </row>
     <row r="6">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.05</v>
+        <v>35.62</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>-0.72962385</v>
+        <v>-0.0192731</v>
       </c>
       <c r="F6" s="3" t="n">
         <v>40.16</v>
@@ -910,34 +910,34 @@
         <v>25.3</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>-0.102</v>
+        <v>-0.113</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>9.861000000000001</v>
+        <v>9.742000000000001</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>39.419</v>
+        <v>39.24</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>47.440792</v>
+        <v>46.86842</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>15.387668</v>
+        <v>15.202017</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>16.742</v>
+        <v>16.665</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>1.396</v>
       </c>
       <c r="P6" s="9" t="n">
-        <v>0.216</v>
+        <v>0.202</v>
       </c>
       <c r="Q6" s="4" t="n">
-        <v>-0.012</v>
+        <v>-0.024</v>
       </c>
     </row>
     <row r="7">
@@ -957,10 +957,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>80.73999999999999</v>
+        <v>80.17</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>0.7235456</v>
+        <v>0.0124682</v>
       </c>
       <c r="F7" s="3" t="n">
         <v>89.95999999999999</v>
@@ -969,22 +969,22 @@
         <v>58.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>-0.102</v>
+        <v>-0.109</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>6.095</v>
+        <v>6.052</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8.407999999999999</v>
+        <v>8.409000000000001</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>3.5789008</v>
+        <v>3.5536346</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>9.909897000000001</v>
+        <v>9.839936</v>
       </c>
       <c r="M7" s="7" t="n">
-        <v>7.001</v>
+        <v>7.002</v>
       </c>
       <c r="N7" s="7" t="n">
         <v>5.8</v>
@@ -993,10 +993,10 @@
         <v>1.22</v>
       </c>
       <c r="P7" s="9" t="n">
-        <v>0.238</v>
+        <v>0.229</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>-0.061</v>
+        <v>-0.068</v>
       </c>
     </row>
     <row r="8">
@@ -1016,10 +1016,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>85.87</v>
+        <v>85.86</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>0.015972624</v>
+        <v>0.0158543</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1031,19 +1031,19 @@
         <v>-0.275</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>5.985</v>
+        <v>5.984</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.933</v>
+        <v>11.027</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>16.232515</v>
+        <v>16.230623</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>11.564921</v>
+        <v>11.563575</v>
       </c>
       <c r="M8" s="7" t="n">
-        <v>11.428</v>
+        <v>11.526</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>9.699999999999999</v>
@@ -1075,10 +1075,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>52.88</v>
+        <v>52.19</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>-0.018741851</v>
+        <v>-0.0315458</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1087,34 +1087,34 @@
         <v>35.09</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.244</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>5.437</v>
+        <v>5.367</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6.603</v>
+        <v>6.503</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>16.948719</v>
+        <v>16.727564</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>16.092857</v>
+        <v>15.882871</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>8.113</v>
+        <v>7.991</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>1.453</v>
       </c>
       <c r="P9" s="9" t="n">
-        <v>0.287</v>
+        <v>0.271</v>
       </c>
       <c r="Q9" s="4" t="n">
-        <v>-0.143</v>
+        <v>-0.155</v>
       </c>
     </row>
     <row r="10">
@@ -1137,7 +1137,7 @@
         <v>10.37</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-0.5752677</v>
+        <v>-0.575268</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>14.38</v>
@@ -1152,7 +1152,7 @@
         <v>5.243</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>4.867</v>
+        <v>4.836</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>24.690477</v>
@@ -1161,7 +1161,7 @@
         <v>11.955131</v>
       </c>
       <c r="M10" s="7" t="n">
-        <v>9.917</v>
+        <v>9.855</v>
       </c>
       <c r="N10" s="7" t="n">
         <v>7.7</v>
@@ -1193,10 +1193,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>25.12</v>
+        <v>25.5</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-0.028046436</v>
+        <v>-0.0135397</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>31.58</v>
@@ -1205,13 +1205,13 @@
         <v>17.86</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-0.205</v>
+        <v>-0.193</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>5.128</v>
+        <v>5.205</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>30.178</v>
+        <v>30.107</v>
       </c>
       <c r="K11" s="7" t="inlineStr">
         <is>
@@ -1219,10 +1219,10 @@
         </is>
       </c>
       <c r="L11" s="7" t="n">
-        <v>24.488304</v>
+        <v>24.8538</v>
       </c>
       <c r="M11" s="7" t="n">
-        <v>8.635</v>
+        <v>8.614000000000001</v>
       </c>
       <c r="N11" s="7" t="n">
         <v>7.2</v>
@@ -1231,10 +1231,10 @@
         <v>1.977</v>
       </c>
       <c r="P11" s="9" t="n">
-        <v>0.005</v>
+        <v>0.02</v>
       </c>
       <c r="Q11" s="9" t="n">
-        <v>0.066</v>
+        <v>0.08199999999999999</v>
       </c>
     </row>
     <row r="12">
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>16.52</v>
+        <v>16.77</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-0.03644315</v>
+        <v>-0.0221574</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>32.22</v>
@@ -1266,34 +1266,34 @@
         <v>15.725</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-0.487</v>
+        <v>-0.48</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>4.891</v>
+        <v>4.963</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>4.848</v>
+        <v>4.734</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>45.902775</v>
+        <v>46.583332</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>20.17825</v>
+        <v>20.567583</v>
       </c>
       <c r="M12" s="7" t="n">
-        <v>12.004</v>
+        <v>11.722</v>
       </c>
       <c r="N12" s="7" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="O12" s="8" t="n">
         <v>2.002</v>
       </c>
       <c r="P12" s="4" t="n">
-        <v>-0.236</v>
+        <v>-0.224</v>
       </c>
       <c r="Q12" s="4" t="n">
-        <v>-0.291</v>
+        <v>-0.281</v>
       </c>
     </row>
     <row r="13">
@@ -1313,10 +1313,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-0.018112448</v>
+        <v>-0.013346</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>22.65</v>
@@ -1325,10 +1325,10 @@
         <v>9.66</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-0.091</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>4.795</v>
+        <v>4.819</v>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
@@ -1336,10 +1336,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>66.45161400000001</v>
+        <v>66.77419</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>27.612461</v>
+        <v>27.746504</v>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
@@ -1355,10 +1355,10 @@
         <v>1.552</v>
       </c>
       <c r="P13" s="9" t="n">
-        <v>0.922</v>
+        <v>0.9309999999999999</v>
       </c>
       <c r="Q13" s="9" t="n">
-        <v>0.067</v>
+        <v>0.07200000000000001</v>
       </c>
     </row>
     <row r="14">
@@ -1378,25 +1378,25 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.59</v>
+        <v>12.48</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-0.15860036</v>
+        <v>-0.0103093</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>18.57</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>12.52</v>
+        <v>12.43</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-0.322</v>
+        <v>-0.328</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>2.323</v>
+        <v>2.303</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>5.895</v>
+        <v>5.871</v>
       </c>
       <c r="K14" s="7" t="inlineStr">
         <is>
@@ -1404,10 +1404,10 @@
         </is>
       </c>
       <c r="L14" s="7" t="n">
-        <v>11.110621</v>
+        <v>11.013546</v>
       </c>
       <c r="M14" s="7" t="n">
-        <v>6.684</v>
+        <v>6.656</v>
       </c>
       <c r="N14" s="7" t="n">
         <v>5.7</v>
@@ -1416,10 +1416,10 @@
         <v>1.082</v>
       </c>
       <c r="P14" s="4" t="n">
-        <v>-0.017</v>
+        <v>-0.026</v>
       </c>
       <c r="Q14" s="4" t="n">
-        <v>-0.163</v>
+        <v>-0.17</v>
       </c>
     </row>
     <row r="15">
@@ -1439,10 +1439,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-0.013345162</v>
+        <v>-0.0106761</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1451,22 +1451,22 @@
         <v>4.55</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.452</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>2.256</v>
+        <v>2.262</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>12.938</v>
+        <v>12.868</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.086956</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>6.969671</v>
+        <v>6.9885244</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>10.728</v>
+        <v>10.669</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>8.5</v>
@@ -1475,10 +1475,10 @@
         <v>0.603</v>
       </c>
       <c r="P15" s="9" t="n">
-        <v>0.052</v>
+        <v>0.055</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>-0.262</v>
+        <v>-0.26</v>
       </c>
     </row>
     <row r="16">
@@ -1498,10 +1498,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>13.89</v>
+        <v>13.99</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>0.8714587999999999</v>
+        <v>0.0159767</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1510,13 +1510,13 @@
         <v>11.65</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>-0.326</v>
+        <v>-0.321</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1.855</v>
+        <v>1.868</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>12.326</v>
+        <v>12.353</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
@@ -1524,10 +1524,10 @@
         </is>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.026443</v>
+        <v>8.0842285</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>17.067</v>
+        <v>17.105</v>
       </c>
       <c r="N16" s="7" t="n">
         <v>10.8</v>
@@ -1536,10 +1536,10 @@
         <v>1.364</v>
       </c>
       <c r="P16" s="4" t="n">
-        <v>-0.148</v>
+        <v>-0.142</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>-0.065</v>
+        <v>-0.058</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>94.5</v>
+        <v>94.23</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>0.54798824</v>
+        <v>0.266014</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1571,22 +1571,22 @@
         <v>69.98999999999999</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.173</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>1.69</v>
+        <v>1.685</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1.598</v>
+        <v>1.602</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>17.402395</v>
+        <v>17.353592</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>15.89487</v>
+        <v>15.850294</v>
       </c>
       <c r="M17" s="7" t="n">
-        <v>8.378</v>
+        <v>8.401</v>
       </c>
       <c r="N17" s="7" t="n">
         <v>7.2</v>
@@ -1595,10 +1595,10 @@
         <v>1.376</v>
       </c>
       <c r="P17" s="9" t="n">
-        <v>0.231</v>
+        <v>0.227</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>-0.013</v>
+        <v>-0.016</v>
       </c>
     </row>
     <row r="18">
@@ -1618,25 +1618,25 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.22</v>
+        <v>4.24</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>-0.025404189</v>
+        <v>-0.0207853</v>
       </c>
       <c r="F18" s="3" t="n">
         <v>13.73</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>4.22</v>
+        <v>4.19</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>-0.6929999999999999</v>
+        <v>-0.6909999999999999</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>1.086</v>
+        <v>1.091</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.794</v>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
@@ -1644,10 +1644,10 @@
         </is>
       </c>
       <c r="L18" s="7" t="n">
-        <v>4.262626</v>
+        <v>4.282828</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>-6.772</v>
+        <v>-6.588</v>
       </c>
       <c r="N18" s="7" t="inlineStr">
         <is>
@@ -1658,10 +1658,10 @@
         <v>1.993</v>
       </c>
       <c r="P18" s="4" t="n">
-        <v>-0.578</v>
+        <v>-0.5760000000000001</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>-0.609</v>
+        <v>-0.607</v>
       </c>
     </row>
     <row r="19">
@@ -1681,10 +1681,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>-0.46511805</v>
+        <v>10.76</v>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>0.09302539999999998</v>
       </c>
       <c r="F19" s="3" t="n">
         <v>13.31</v>
@@ -1693,22 +1693,22 @@
         <v>9.015000000000001</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>-0.196</v>
+        <v>-0.192</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.873</v>
+        <v>0.878</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>1.201</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>17.833332</v>
+        <v>17.933332</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>11.554701</v>
+        <v>11.619494</v>
       </c>
       <c r="M19" s="7" t="n">
-        <v>6.349</v>
+        <v>6.353</v>
       </c>
       <c r="N19" s="7" t="n">
         <v>4.5</v>
@@ -1717,10 +1717,10 @@
         <v>1.07</v>
       </c>
       <c r="P19" s="9" t="n">
-        <v>0.079</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="Q19" s="4" t="n">
-        <v>-0.059</v>
+        <v>-0.05400000000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1740,10 +1740,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.29</v>
       </c>
       <c r="E20" s="9" t="n">
-        <v>0.017753801</v>
+        <v>0.0146662</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1752,13 +1752,13 @@
         <v>19.57</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>-0.195</v>
+        <v>-0.197</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.696</v>
+        <v>0.694</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>1.141</v>
+        <v>1.151</v>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
@@ -1766,22 +1766,22 @@
         </is>
       </c>
       <c r="L20" s="7" t="n">
-        <v>21.793388</v>
+        <v>21.727272</v>
       </c>
       <c r="M20" s="7" t="n">
-        <v>9.352</v>
+        <v>9.433999999999999</v>
       </c>
       <c r="N20" s="7" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="O20" s="8" t="n">
         <v>1.412</v>
       </c>
       <c r="P20" s="9" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.034</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>-0.025</v>
+        <v>-0.028</v>
       </c>
     </row>
     <row r="21">
@@ -1801,10 +1801,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>9.42</v>
+        <v>9.74</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-0.10541307</v>
+        <v>-0.0750237</v>
       </c>
       <c r="F21" s="3" t="n">
         <v>20.74</v>
@@ -1813,13 +1813,13 @@
         <v>8.455</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>-0.546</v>
+        <v>-0.53</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.457</v>
+        <v>0.473</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>7.727</v>
+        <v>7.689</v>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
@@ -1827,10 +1827,10 @@
         </is>
       </c>
       <c r="L21" s="7" t="n">
-        <v>-4.291572</v>
+        <v>-4.4373574</v>
       </c>
       <c r="M21" s="7" t="n">
-        <v>22.448</v>
+        <v>22.336</v>
       </c>
       <c r="N21" s="7" t="n">
         <v>15.3</v>
@@ -1841,10 +1841,10 @@
         </is>
       </c>
       <c r="P21" s="4" t="n">
-        <v>-0.234</v>
+        <v>-0.208</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>-0.434</v>
+        <v>-0.415</v>
       </c>
     </row>
     <row r="22">
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.82</v>
+        <v>6.95</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>0.020958135</v>
+        <v>0.0404192</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1876,13 +1876,13 @@
         <v>6.1</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>-0.315</v>
+        <v>-0.302</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.185</v>
+        <v>0.188</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.511</v>
+        <v>0.519</v>
       </c>
       <c r="K22" s="7" t="inlineStr">
         <is>
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="L22" s="7" t="n">
-        <v>9.103529999999999</v>
+        <v>9.277056999999999</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>6.884</v>
+        <v>6.982</v>
       </c>
       <c r="N22" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="O22" s="8" t="n">
         <v>1.206</v>
       </c>
       <c r="P22" s="4" t="n">
-        <v>-0.201</v>
+        <v>-0.186</v>
       </c>
       <c r="Q22" s="4" t="n">
-        <v>-0.24</v>
+        <v>-0.225</v>
       </c>
     </row>
     <row r="23">
@@ -1925,10 +1925,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
       <c r="E23" s="9" t="n">
-        <v>0.01162784</v>
+        <v>0.4651159999999999</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -1937,10 +1937,10 @@
         <v>2.02</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0.572</v>
@@ -1951,10 +1951,10 @@
         </is>
       </c>
       <c r="L23" s="7" t="n">
-        <v>-5.3048778</v>
+        <v>-5.268293</v>
       </c>
       <c r="M23" s="7" t="n">
-        <v>12.406</v>
+        <v>12.414</v>
       </c>
       <c r="N23" s="7" t="n">
         <v>8.9</v>
@@ -1963,10 +1963,10 @@
         <v>1.327</v>
       </c>
       <c r="P23" s="4" t="n">
-        <v>-0.48</v>
+        <v>-0.483</v>
       </c>
       <c r="Q23" s="4" t="n">
-        <v>-0.13</v>
+        <v>-0.136</v>
       </c>
     </row>
     <row r="24">
@@ -2152,16 +2152,16 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>51.65</v>
+        <v>51.62</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>-0.0773788</v>
+        <v>-0.135422</v>
       </c>
       <c r="F2" s="5" t="n">
         <v>-0.204</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>0.365</v>
+        <v>0.364</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>50.8</v>
@@ -2199,28 +2199,28 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>100.18</v>
+        <v>99.5</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>-0.31840765</v>
+        <v>-0.9950249999999999</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.544</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>-0.5479999999999999</v>
+        <v>-0.551</v>
       </c>
       <c r="H3" s="7" t="n">
         <v>-62.9</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.304</v>
+        <v>-0.308</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.5639999999999999</v>
+        <v>-0.5670000000000001</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>-0.6809999999999999</v>
+        <v>-0.6829999999999999</v>
       </c>
       <c r="L3" s="8" t="n">
         <v>1.177</v>
@@ -2246,28 +2246,28 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>20.84</v>
+        <v>20.93</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.6032818599999999</v>
+        <v>0.0101352</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>-0.415</v>
+        <v>-0.413</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>-0.3720000000000001</v>
+        <v>-0.37</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>-39.8</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.233</v>
+        <v>-0.229</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.417</v>
+        <v>-0.414</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>-0.573</v>
+        <v>-0.5710000000000001</v>
       </c>
       <c r="L4" s="8" t="n">
         <v>1.682</v>
@@ -2293,28 +2293,28 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>97.13</v>
+        <v>96.77</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.55916774</v>
+        <v>0.186355</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>-0.206</v>
+        <v>-0.209</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0.174</v>
+        <v>0.17</v>
       </c>
       <c r="H5" s="7" t="n">
         <v>31.6</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.116</v>
+        <v>-0.119</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.15</v>
+        <v>-0.154</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>-0.279</v>
+        <v>-0.282</v>
       </c>
       <c r="L5" s="8" t="n">
         <v>1.034</v>
@@ -2340,28 +2340,28 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.05</v>
+        <v>35.62</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>-0.72962385</v>
+        <v>-0.0192731</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.024</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.216</v>
+        <v>0.202</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>11.8</v>
+        <v>11.7</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.017</v>
+        <v>0.005</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.025</v>
+        <v>0.013</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>-0.102</v>
+        <v>-0.113</v>
       </c>
       <c r="L6" s="8" t="n">
         <v>1.396</v>
@@ -2387,28 +2387,28 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>80.73999999999999</v>
+        <v>80.17</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.7235456</v>
+        <v>0.0124682</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.068</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.238</v>
+        <v>0.229</v>
       </c>
       <c r="H7" s="7" t="n">
         <v>19.1</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.038</v>
+        <v>-0.045</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.032</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>-0.102</v>
+        <v>-0.109</v>
       </c>
       <c r="L7" s="8" t="n">
         <v>1.22</v>
@@ -2434,10 +2434,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>85.87</v>
+        <v>85.86</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.015972624</v>
+        <v>0.0158543</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.233</v>
@@ -2452,7 +2452,7 @@
         <v>-0.094</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.149</v>
+        <v>-0.15</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>-0.275</v>
@@ -2481,28 +2481,28 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>52.88</v>
+        <v>52.19</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>-0.018741851</v>
+        <v>-0.0315458</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>-0.143</v>
+        <v>-0.155</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.287</v>
+        <v>0.271</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>36.8</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.142</v>
+        <v>-0.153</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>-0.099</v>
+        <v>-0.111</v>
       </c>
       <c r="K9" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.244</v>
       </c>
       <c r="L9" s="8" t="n">
         <v>1.453</v>
@@ -2531,7 +2531,7 @@
         <v>10.37</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-0.5752677</v>
+        <v>-0.575268</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>-0.105</v>
@@ -2575,28 +2575,28 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>25.12</v>
+        <v>25.5</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>-0.028046436</v>
+        <v>-0.0135397</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.066</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>0.005</v>
+        <v>0.02</v>
       </c>
       <c r="H11" s="7" t="n">
         <v>-21.6</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.08800000000000001</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.018</v>
+        <v>0.034</v>
       </c>
       <c r="K11" s="5" t="n">
-        <v>-0.205</v>
+        <v>-0.193</v>
       </c>
       <c r="L11" s="8" t="n">
         <v>1.977</v>
@@ -2622,28 +2622,28 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>16.52</v>
+        <v>16.77</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-0.03644315</v>
+        <v>-0.0221574</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-0.291</v>
+        <v>-0.281</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-0.236</v>
+        <v>-0.224</v>
       </c>
       <c r="H12" s="7" t="n">
         <v>-31.9</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.101</v>
+        <v>-0.08699999999999999</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-0.326</v>
+        <v>-0.316</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-0.487</v>
+        <v>-0.48</v>
       </c>
       <c r="L12" s="8" t="n">
         <v>2.002</v>
@@ -2669,28 +2669,28 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-0.018112448</v>
+        <v>-0.013346</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.067</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>0.922</v>
+        <v>0.9309999999999999</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>49.4</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>0.095</v>
+        <v>0.1</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.127</v>
+        <v>0.132</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>-0.091</v>
+        <v>-0.08599999999999999</v>
       </c>
       <c r="L13" s="8" t="n">
         <v>1.552</v>
@@ -2716,28 +2716,28 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.59</v>
+        <v>12.48</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>-0.15860036</v>
+        <v>-0.0103093</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>-0.163</v>
+        <v>-0.17</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.026</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>11.6</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.08699999999999999</v>
+        <v>-0.095</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.185</v>
+        <v>-0.192</v>
       </c>
       <c r="K14" s="5" t="n">
-        <v>-0.322</v>
+        <v>-0.328</v>
       </c>
       <c r="L14" s="8" t="n">
         <v>1.082</v>
@@ -2763,28 +2763,28 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-0.013345162</v>
+        <v>-0.0106761</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.26</v>
       </c>
       <c r="G15" s="5" t="n">
-        <v>0.052</v>
+        <v>0.055</v>
       </c>
       <c r="H15" s="7" t="n">
         <v>3.1</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.076</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>-0.294</v>
+        <v>-0.292</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>-0.454</v>
+        <v>-0.452</v>
       </c>
       <c r="L15" s="8" t="n">
         <v>0.603</v>
@@ -2810,28 +2810,28 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>13.89</v>
+        <v>13.99</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.8714587999999999</v>
+        <v>0.0159767</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.058</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>-0.148</v>
+        <v>-0.142</v>
       </c>
       <c r="H16" s="7" t="n">
         <v>-19.8</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.008</v>
+        <v>0.015</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>-0.145</v>
+        <v>-0.139</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>-0.326</v>
+        <v>-0.321</v>
       </c>
       <c r="L16" s="8" t="n">
         <v>1.364</v>
@@ -2857,28 +2857,28 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>94.5</v>
+        <v>94.23</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.54798824</v>
+        <v>0.266014</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>-0.013</v>
+        <v>-0.016</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>0.231</v>
+        <v>0.227</v>
       </c>
       <c r="H17" s="7" t="n">
         <v>19.5</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-0.004</v>
+        <v>-0.006999999999999999</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>-0.017</v>
+        <v>-0.02</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.173</v>
       </c>
       <c r="L17" s="8" t="n">
         <v>1.376</v>
@@ -2904,28 +2904,28 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.22</v>
+        <v>4.24</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>-0.025404189</v>
+        <v>-0.0207853</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>-0.609</v>
+        <v>-0.607</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>-0.578</v>
+        <v>-0.5760000000000001</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>-37.5</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.414</v>
+        <v>-0.411</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.5870000000000001</v>
+        <v>-0.585</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>-0.6929999999999999</v>
+        <v>-0.6909999999999999</v>
       </c>
       <c r="L18" s="8" t="n">
         <v>1.993</v>
@@ -2951,28 +2951,28 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>10.7</v>
+        <v>10.76</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>-0.46511805</v>
+        <v>0.09302539999999998</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>-0.059</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0.079</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>-2.5</v>
+        <v>-2.4</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>-0.053</v>
+        <v>-0.047</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>-0.045</v>
+        <v>-0.039</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>-0.196</v>
+        <v>-0.192</v>
       </c>
       <c r="L19" s="8" t="n">
         <v>1.07</v>
@@ -2998,28 +2998,28 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.29</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.017753801</v>
+        <v>0.0146662</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.028</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>0.03700000000000001</v>
+        <v>0.034</v>
       </c>
       <c r="H20" s="7" t="n">
         <v>5.4</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.059</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>-0.019</v>
+        <v>-0.022</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>-0.195</v>
+        <v>-0.197</v>
       </c>
       <c r="L20" s="8" t="n">
         <v>1.412</v>
@@ -3045,28 +3045,28 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>9.42</v>
+        <v>9.74</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>-0.10541307</v>
+        <v>-0.0750237</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>-0.434</v>
+        <v>-0.415</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>-0.234</v>
+        <v>-0.208</v>
       </c>
       <c r="H21" s="7" t="n">
         <v>38.1</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.351</v>
+        <v>-0.329</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>-0.291</v>
+        <v>-0.267</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>-0.546</v>
+        <v>-0.53</v>
       </c>
       <c r="L21" s="8" t="inlineStr">
         <is>
@@ -3094,28 +3094,28 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.82</v>
+        <v>6.95</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.020958135</v>
+        <v>0.0404192</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>-0.24</v>
+        <v>-0.225</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>-0.201</v>
+        <v>-0.186</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.186</v>
+        <v>-0.17</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.204</v>
+        <v>-0.188</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>-0.315</v>
+        <v>-0.302</v>
       </c>
       <c r="L22" s="8" t="n">
         <v>1.206</v>
@@ -3141,28 +3141,28 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.01162784</v>
+        <v>0.4651159999999999</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>-0.13</v>
+        <v>-0.136</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>-0.48</v>
+        <v>-0.483</v>
       </c>
       <c r="H23" s="7" t="n">
         <v>-52.5</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.101</v>
+        <v>-0.106</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.296</v>
+        <v>-0.299</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>-0.5620000000000001</v>
+        <v>-0.5639999999999999</v>
       </c>
       <c r="L23" s="8" t="n">
         <v>1.327</v>
@@ -3200,7 +3200,7 @@
         <v>-0.239</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>-262.5</v>
+        <v>-259.8</v>
       </c>
       <c r="I24" s="5" t="n"/>
       <c r="J24" s="5" t="n"/>
@@ -3342,31 +3342,31 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>51.65</v>
+        <v>51.62</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>34.922</v>
+        <v>34.902</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>21.978725</v>
+        <v>21.965958</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>13.745696</v>
+        <v>13.737711</v>
       </c>
       <c r="H2" s="7" t="n">
-        <v>10.427</v>
+        <v>10.417</v>
       </c>
       <c r="I2" s="7" t="n">
         <v>8.9</v>
       </c>
       <c r="J2" s="7" t="n">
-        <v>3.631</v>
+        <v>3.628</v>
       </c>
       <c r="K2" s="7" t="n">
-        <v>21.922752</v>
+        <v>21.910017</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>2.6828258</v>
+        <v>2.6812677</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>2.35</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>100.18</v>
+        <v>99.5</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>17.51</v>
+        <v>17.391</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3406,22 +3406,22 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>9.792441</v>
+        <v>9.725972000000001</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>13.742</v>
+        <v>13.66</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>1.788</v>
+        <v>1.778</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>1.9422256</v>
+        <v>1.9290422</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.0687815</v>
+        <v>1.0615268</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -3450,10 +3450,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>20.84</v>
+        <v>20.93</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>10.334</v>
+        <v>10.376</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -3461,22 +3461,22 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>10.841299</v>
+        <v>10.885508</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>40.226</v>
+        <v>40.605</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1.813</v>
+        <v>1.83</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>16.336206</v>
+        <v>16.40282</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>1.7067827</v>
+        <v>1.7137426</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>-0.01</v>
@@ -3505,31 +3505,31 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>97.13</v>
+        <v>96.77</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>10.129</v>
+        <v>10.091</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>30.933151</v>
+        <v>30.81847</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>16.346996</v>
+        <v>16.286392</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>11.087</v>
+        <v>11.098</v>
       </c>
       <c r="I5" s="7" t="n">
         <v>8.9</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2.718</v>
+        <v>2.72</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>-36.13471</v>
+        <v>-36.000744</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>1.4190465</v>
+        <v>1.4137856</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>3.14</v>
@@ -3558,31 +3558,31 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>36.05</v>
+        <v>35.62</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>9.861000000000001</v>
+        <v>9.742000000000001</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>47.440792</v>
+        <v>46.86842</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>15.387668</v>
+        <v>15.202017</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>16.742</v>
+        <v>16.665</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>2.248</v>
+        <v>2.237</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>3.8327844</v>
+        <v>3.786542</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>0.5622906</v>
+        <v>0.5555066</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0.76</v>
@@ -3611,19 +3611,19 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>80.73999999999999</v>
+        <v>80.17</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>6.095</v>
+        <v>6.052</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>3.5789008</v>
+        <v>3.5536346</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>9.909897000000001</v>
+        <v>9.839936</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>7.001</v>
+        <v>7.002</v>
       </c>
       <c r="I7" s="7" t="n">
         <v>5.8</v>
@@ -3632,10 +3632,10 @@
         <v>2.055</v>
       </c>
       <c r="K7" s="7" t="n">
-        <v>2.3637905</v>
+        <v>2.3471029</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>1.4895545</v>
+        <v>1.4790387</v>
       </c>
       <c r="M7" s="3" t="n">
         <v>22.56</v>
@@ -3664,31 +3664,31 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>85.87</v>
+        <v>85.86</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>5.985</v>
+        <v>5.984</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>16.232515</v>
+        <v>16.230623</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>11.564921</v>
+        <v>11.563575</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>11.428</v>
+        <v>11.526</v>
       </c>
       <c r="I8" s="7" t="n">
         <v>9.699999999999999</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>3.737</v>
+        <v>3.769</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>5.9192114</v>
+        <v>5.9185224</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>2.0454657</v>
+        <v>2.0452275</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>5.29</v>
@@ -3717,31 +3717,31 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>52.88</v>
+        <v>52.19</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>5.437</v>
+        <v>5.367</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>16.948719</v>
+        <v>16.727564</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>16.092857</v>
+        <v>15.882871</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>8.113</v>
+        <v>7.991</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.282</v>
+        <v>3.233</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>14.804031</v>
+        <v>14.610862</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>2.7032228</v>
+        <v>2.6679497</v>
       </c>
       <c r="M9" s="3" t="n">
         <v>3.12</v>
@@ -3782,13 +3782,13 @@
         <v>11.955131</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>9.917</v>
+        <v>9.855</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>7.7</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>2.077</v>
+        <v>2.064</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>7.040054</v>
@@ -3823,10 +3823,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>25.12</v>
+        <v>25.5</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>5.128</v>
+        <v>5.205</v>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
@@ -3834,22 +3834,22 @@
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>24.488304</v>
+        <v>24.8538</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>8.635</v>
+        <v>8.614000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>7.2</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>2.627</v>
+        <v>2.621</v>
       </c>
       <c r="K11" s="7" t="n">
-        <v>1.4529</v>
+        <v>1.4745852</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>0.446475</v>
+        <v>0.4531388</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>-2.42</v>
@@ -3878,40 +3878,40 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>16.52</v>
+        <v>16.77</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>4.891</v>
+        <v>4.963</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>45.902775</v>
+        <v>46.583332</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>20.17825</v>
+        <v>20.567583</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>12.004</v>
+        <v>11.722</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>3.758</v>
+        <v>3.67</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>4.3944983</v>
+        <v>4.4792886</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>3.7912662</v>
+        <v>3.8474758</v>
       </c>
       <c r="M12" s="3" t="n">
         <v>0.36</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>0.8189511</v>
+        <v>0.8153608</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>3.7603836</v>
+        <v>3.7438982</v>
       </c>
     </row>
     <row r="13">
@@ -3931,16 +3931,16 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>4.795</v>
+        <v>4.819</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>66.45161400000001</v>
+        <v>66.77419</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>27.612461</v>
+        <v>27.746504</v>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
@@ -3958,10 +3958,10 @@
         </is>
       </c>
       <c r="K13" s="7" t="n">
-        <v>13.9850645</v>
+        <v>14.052953</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>4.2271185</v>
+        <v>4.2476387</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>0.31</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12.59</v>
+        <v>12.48</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>2.323</v>
+        <v>2.303</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -4001,22 +4001,22 @@
         </is>
       </c>
       <c r="G14" s="7" t="n">
-        <v>11.110621</v>
+        <v>11.013546</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>6.684</v>
+        <v>6.656</v>
       </c>
       <c r="I14" s="7" t="n">
         <v>5.7</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>2.348</v>
+        <v>2.338</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>2.6884475</v>
+        <v>2.6649582</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>0.92521507</v>
+        <v>0.91713136</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>-0.01</v>
@@ -4045,31 +4045,31 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.56</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.256</v>
+        <v>2.262</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.086956</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>6.969671</v>
+        <v>6.9885244</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>10.728</v>
+        <v>10.669</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>8.5</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>2.506</v>
+        <v>2.492</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>-1.7376999</v>
+        <v>-1.7424005</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>0.43686444</v>
+        <v>0.43804622</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>0.46</v>
@@ -4098,10 +4098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>13.89</v>
+        <v>13.99</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1.855</v>
+        <v>1.868</v>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
@@ -4109,22 +4109,22 @@
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.026443</v>
+        <v>8.0842285</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17.067</v>
+        <v>17.105</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>10.8</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>1.771</v>
+        <v>1.775</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>0.9561506</v>
+        <v>0.96303433</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>0.26647866</v>
+        <v>0.26839712</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>-5.83</v>
@@ -4153,31 +4153,31 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>94.5</v>
+        <v>94.23</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1.69</v>
+        <v>1.685</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>17.402395</v>
+        <v>17.353592</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>15.89487</v>
+        <v>15.850294</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>8.378</v>
+        <v>8.401</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>7.2</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>2.931</v>
+        <v>2.939</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>3.1316698</v>
+        <v>3.1228874</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>3.1004798</v>
+        <v>3.0917847</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.43</v>
@@ -4206,10 +4206,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>4.22</v>
+        <v>4.24</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1.086</v>
+        <v>1.091</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
@@ -4217,10 +4217,10 @@
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>4.262626</v>
+        <v>4.282828</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>-6.772</v>
+        <v>-6.588</v>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
@@ -4228,13 +4228,13 @@
         </is>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1.22</v>
+        <v>1.186</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>1.434886</v>
+        <v>1.4416864</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>1.6215286</v>
+        <v>1.6292138</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>-0.44</v>
@@ -4263,31 +4263,31 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>10.7</v>
+        <v>10.76</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>0.873</v>
+        <v>0.878</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>17.833332</v>
+        <v>17.933332</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>11.554701</v>
+        <v>11.619494</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>6.349</v>
+        <v>6.353</v>
       </c>
       <c r="I19" s="7" t="n">
         <v>4.5</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0.902</v>
+        <v>0.903</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>3.2651815</v>
+        <v>3.2834911</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>0.6557925999999999</v>
+        <v>0.65947</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>0.6</v>
@@ -4316,10 +4316,10 @@
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.29</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0.696</v>
+        <v>0.694</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -4327,22 +4327,22 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>21.793388</v>
+        <v>21.727272</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>9.352</v>
+        <v>9.433999999999999</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>1.798</v>
+        <v>1.813</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>1.6405376</v>
+        <v>1.6355606</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>1.096432</v>
+        <v>1.0931057</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>-0.23</v>
@@ -4371,10 +4371,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>9.42</v>
+        <v>9.74</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>0.457</v>
+        <v>0.473</v>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
@@ -4382,25 +4382,25 @@
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>-4.291572</v>
+        <v>-4.4373574</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>22.448</v>
+        <v>22.336</v>
       </c>
       <c r="I21" s="7" t="n">
         <v>15.3</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>2.909</v>
+        <v>2.894</v>
       </c>
       <c r="K21" s="7" t="n">
-        <v>0.45955706</v>
+        <v>0.47516832</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>0.17209555</v>
+        <v>0.17794168</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-11</v>
+        <v>-10.17</v>
       </c>
       <c r="N21" s="3" t="n">
         <v>-2.195</v>
@@ -4426,10 +4426,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6.82</v>
+        <v>6.95</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.185</v>
+        <v>0.188</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -4437,22 +4437,22 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9.103529999999999</v>
+        <v>9.277056999999999</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>6.884</v>
+        <v>6.982</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1.682</v>
+        <v>1.706</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>-11.310117</v>
+        <v>-11.525704</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>0.6068605</v>
+        <v>0.61842823</v>
       </c>
       <c r="M22" s="3" t="n">
         <v>-0.58</v>
@@ -4481,10 +4481,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -4492,22 +4492,22 @@
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>-5.3048778</v>
+        <v>-5.268293</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12.406</v>
+        <v>12.414</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>8.9</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>1.891</v>
+        <v>1.892</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>31.071428</v>
+        <v>30.857143</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>0.26026595</v>
+        <v>0.25847104</v>
       </c>
       <c r="M23" s="3" t="n">
         <v>-1.12</v>
@@ -6245,7 +6245,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>51.65</v>
+        <v>51.62</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -6270,7 +6270,7 @@
         <v>58</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>0.353</v>
+        <v>0.354</v>
       </c>
       <c r="K2" s="7" t="n">
         <v>2.49</v>
@@ -6303,7 +6303,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>100.18</v>
+        <v>99.5</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -6317,7 +6317,7 @@
         <v>27</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>204.7037</v>
+        <v>200.07407</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>354</v>
@@ -6326,7 +6326,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>1.043</v>
+        <v>1.011</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6361,7 +6361,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>20.84</v>
+        <v>20.93</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -6384,7 +6384,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>0.725</v>
+        <v>0.718</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6419,7 +6419,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>97.13</v>
+        <v>96.77</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -6427,7 +6427,7 @@
         </is>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1.26316</v>
+        <v>1.21053</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>18</v>
@@ -6442,7 +6442,7 @@
         <v>118</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.46</v>
+        <v>0.466</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>3.38</v>
@@ -6457,7 +6457,7 @@
         <v>0.6871699999999999</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>1.04</v>
+        <v>1.03</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -6475,7 +6475,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>36.05</v>
+        <v>35.62</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -6498,7 +6498,7 @@
         <v>31</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>0.184</v>
+        <v>0.198</v>
       </c>
       <c r="K6" s="7" t="n">
         <v>4.85</v>
@@ -6533,7 +6533,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>80.73999999999999</v>
+        <v>80.17</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -6556,7 +6556,7 @@
         <v>84</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.17</v>
+        <v>0.178</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>3.91</v>
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>85.87</v>
+        <v>85.86</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -6627,7 +6627,7 @@
         <v>0.81711</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="P8" s="5" t="n">
         <v>0.0828</v>
@@ -6645,7 +6645,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>52.88</v>
+        <v>52.19</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -6668,7 +6668,7 @@
         <v>59</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>0.379</v>
+        <v>0.398</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>4.01</v>
@@ -6683,7 +6683,7 @@
         <v>0.88883</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>1.93</v>
+        <v>1.99</v>
       </c>
       <c r="P9" s="5" t="n">
         <v>0.32369998</v>
@@ -6739,7 +6739,7 @@
         <v>0.19124001</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>1.63</v>
+        <v>1.64</v>
       </c>
       <c r="P10" s="5" t="n">
         <v>0.2831</v>
@@ -6757,7 +6757,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>25.12</v>
+        <v>25.5</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -6780,7 +6780,7 @@
         <v>22</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.272</v>
+        <v>0.253</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>3.37</v>
@@ -6815,7 +6815,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>16.52</v>
+        <v>16.77</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -6829,16 +6829,16 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.584803</v>
+        <v>28.634026</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>36.863396</v>
+        <v>36.926872</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.757275</v>
+        <v>22.796463</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.73</v>
+        <v>0.7070000000000001</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>4.54</v>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>20.6</v>
+        <v>20.7</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -6896,7 +6896,7 @@
         <v>20</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.209</v>
+        <v>0.203</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>1.89</v>
@@ -6931,7 +6931,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>12.59</v>
+        <v>12.48</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -6954,7 +6954,7 @@
         <v>15</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>0.436</v>
+        <v>0.449</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>2.58</v>
@@ -6969,7 +6969,7 @@
         <v>0.46130002</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7.3</v>
+        <v>7.37</v>
       </c>
       <c r="P14" s="5" t="n">
         <v>8.8889</v>
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>5.54</v>
+        <v>5.56</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -7010,7 +7010,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>0.6679999999999999</v>
+        <v>0.662</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.37</v>
@@ -7045,7 +7045,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>13.89</v>
+        <v>13.99</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -7068,7 +7068,7 @@
         <v>15</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.376</v>
+        <v>0.366</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>4.3</v>
@@ -7103,7 +7103,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>94.5</v>
+        <v>94.23</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -7128,7 +7128,7 @@
         <v>93</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>0.139</v>
+        <v>0.143</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>2.64</v>
@@ -7143,7 +7143,7 @@
         <v>0.64763</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="P17" s="5" t="n">
         <v>0.221</v>
@@ -7161,7 +7161,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>4.22</v>
+        <v>4.24</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -7184,7 +7184,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>1.788</v>
+        <v>1.775</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>2.41</v>
@@ -7219,7 +7219,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>10.7</v>
+        <v>10.76</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -7242,7 +7242,7 @@
         <v>14</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>0.449</v>
+        <v>0.441</v>
       </c>
       <c r="K19" s="7" t="n">
         <v>2.55</v>
@@ -7277,7 +7277,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>26.37</v>
+        <v>26.29</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -7302,7 +7302,7 @@
         <v>30</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0.157</v>
+        <v>0.16</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>4.41</v>
@@ -7317,7 +7317,7 @@
         <v>0.68551004</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>3.86</v>
+        <v>3.8</v>
       </c>
       <c r="P20" s="5" t="n">
         <v>4.5455</v>
@@ -7335,7 +7335,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>9.42</v>
+        <v>9.74</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -7346,10 +7346,10 @@
         <v>3.2</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="H21" s="3" t="n">
         <v>18</v>
@@ -7358,7 +7358,7 @@
         <v>11</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.486</v>
+        <v>0.386</v>
       </c>
       <c r="K21" s="7" t="n">
         <v>8.01</v>
@@ -7393,7 +7393,7 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>6.82</v>
+        <v>6.95</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
         <v>10</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.955</v>
+        <v>0.9179999999999999</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>9.81</v>
@@ -7451,7 +7451,7 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2.17</v>
+        <v>2.16</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -7474,7 +7474,7 @@
         <v>2.5</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>0.498</v>
+        <v>0.505</v>
       </c>
       <c r="K23" s="7" t="n">
         <v>5.74</v>
@@ -7699,10 +7699,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>34.922</v>
+        <v>34.902</v>
       </c>
       <c r="E3" s="7" t="n">
-        <v>21.978725</v>
+        <v>21.965958</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0.26</v>
@@ -7717,7 +7717,7 @@
         <v>-0.204</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>10.427</v>
+        <v>10.417</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>8.9</v>
@@ -7743,7 +7743,7 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>5.128</v>
+        <v>5.205</v>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
@@ -7760,10 +7760,10 @@
         <v>-0.10840999</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>0.066</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>8.635</v>
+        <v>8.614000000000001</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>7.2</v>
@@ -7789,10 +7789,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>2.256</v>
+        <v>2.262</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>12.054348</v>
+        <v>12.086956</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>0.08599999999999999</v>
@@ -7806,10 +7806,10 @@
         </is>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.262</v>
+        <v>-0.26</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>10.728</v>
+        <v>10.669</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>8.5</v>
@@ -7835,10 +7835,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>9.861000000000001</v>
+        <v>9.742000000000001</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>47.440792</v>
+        <v>46.86842</v>
       </c>
       <c r="F6" s="5" t="n">
         <v>0.06</v>
@@ -7850,13 +7850,13 @@
         <v>0.1489</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>-0.012</v>
+        <v>-0.024</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>16.742</v>
+        <v>16.665</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="L6" s="7" t="n">
         <v>37.5</v>
@@ -7879,10 +7879,10 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10.129</v>
+        <v>10.091</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>30.933151</v>
+        <v>30.81847</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.015</v>
@@ -7896,10 +7896,10 @@
         </is>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-0.206</v>
+        <v>-0.209</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>11.087</v>
+        <v>11.098</v>
       </c>
       <c r="K7" s="7" t="n">
         <v>8.9</v>
@@ -7943,10 +7943,10 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>6.095</v>
+        <v>6.052</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>3.5789008</v>
+        <v>3.5536346</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>0.02</v>
@@ -7958,16 +7958,16 @@
         <v>0.87788004</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-0.061</v>
+        <v>-0.068</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>7.001</v>
+        <v>7.002</v>
       </c>
       <c r="K10" s="7" t="n">
         <v>5.8</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>71.40000000000001</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11">
@@ -7987,10 +7987,10 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>5.985</v>
+        <v>5.984</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>16.232515</v>
+        <v>16.230623</v>
       </c>
       <c r="F11" s="5" t="n">
         <v>0.067</v>
@@ -8005,7 +8005,7 @@
         <v>-0.233</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>11.428</v>
+        <v>11.526</v>
       </c>
       <c r="K11" s="7" t="n">
         <v>9.699999999999999</v>
@@ -8031,10 +8031,10 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>5.437</v>
+        <v>5.367</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>16.948719</v>
+        <v>16.727564</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>0.032</v>
@@ -8046,13 +8046,13 @@
         <v>1.113</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-0.143</v>
+        <v>-0.155</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>8.113</v>
+        <v>7.991</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>60.3</v>
@@ -8075,10 +8075,10 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>1.69</v>
+        <v>1.685</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>17.402395</v>
+        <v>17.353592</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.041</v>
@@ -8090,10 +8090,10 @@
         <v>0.19214001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.013</v>
+        <v>-0.016</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>8.378</v>
+        <v>8.401</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>7.2</v>
@@ -8119,7 +8119,7 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>1.855</v>
+        <v>1.868</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
@@ -8136,16 +8136,16 @@
         <v>-0.36078</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.065</v>
+        <v>-0.058</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.067</v>
+        <v>17.105</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>10.8</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>45.7</v>
+        <v>48.6</v>
       </c>
     </row>
     <row r="15">
@@ -8165,7 +8165,7 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>0.696</v>
+        <v>0.694</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
@@ -8182,13 +8182,13 @@
         <v>-0.0135</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.025</v>
+        <v>-0.028</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>9.352</v>
+        <v>9.433999999999999</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="L15" s="7" t="n">
         <v>40</v>
@@ -8211,7 +8211,7 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>0.457</v>
+        <v>0.473</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
@@ -8228,10 +8228,10 @@
         <v>-0.5564</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>-0.434</v>
+        <v>-0.415</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>22.448</v>
+        <v>22.336</v>
       </c>
       <c r="K16" s="7" t="n">
         <v>15.3</v>
@@ -8257,7 +8257,7 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
@@ -8274,10 +8274,10 @@
         <v>-1.8681101</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>-0.13</v>
+        <v>-0.136</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>12.406</v>
+        <v>12.414</v>
       </c>
       <c r="K17" s="7" t="n">
         <v>8.9</v>
@@ -8339,7 +8339,7 @@
         <v>-0.105</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>9.917</v>
+        <v>9.855</v>
       </c>
       <c r="K20" s="7" t="n">
         <v>7.7</v>
@@ -8365,10 +8365,10 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>4.795</v>
+        <v>4.819</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>66.45161400000001</v>
+        <v>66.77419</v>
       </c>
       <c r="F21" s="5" t="n">
         <v>0.888</v>
@@ -8380,7 +8380,7 @@
         <v>0.29505</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>0.067</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -8413,10 +8413,10 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>4.891</v>
+        <v>4.963</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>45.902775</v>
+        <v>46.583332</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.201</v>
@@ -8428,13 +8428,13 @@
         <v>0.10515001</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.291</v>
+        <v>-0.281</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>12.004</v>
+        <v>11.722</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>10.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L22" s="7" t="n">
         <v>55</v>
@@ -8457,7 +8457,7 @@
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10.334</v>
+        <v>10.376</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
@@ -8474,13 +8474,13 @@
         <v>0.00452</v>
       </c>
       <c r="I23" s="5" t="n">
-        <v>-0.415</v>
+        <v>-0.413</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>40.226</v>
+        <v>40.605</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="L23" s="7" t="n">
         <v>52</v>
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>17.51</v>
+        <v>17.391</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -8520,13 +8520,13 @@
         <v>-0.038829997</v>
       </c>
       <c r="I24" s="5" t="n">
-        <v>-0.541</v>
+        <v>-0.544</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>13.742</v>
+        <v>13.66</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L24" s="7" t="n">
         <v>48</v>
@@ -8549,7 +8549,7 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1.086</v>
+        <v>1.091</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
@@ -8566,10 +8566,10 @@
         <v>-0.17208</v>
       </c>
       <c r="I25" s="5" t="n">
-        <v>-0.609</v>
+        <v>-0.607</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-6.772</v>
+        <v>-6.588</v>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
@@ -8615,10 +8615,10 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>0.873</v>
+        <v>0.878</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>17.833332</v>
+        <v>17.933332</v>
       </c>
       <c r="F28" s="5" t="n">
         <v>0.075</v>
@@ -8630,10 +8630,10 @@
         <v>0.19236</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>-0.059</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>6.349</v>
+        <v>6.353</v>
       </c>
       <c r="K28" s="7" t="n">
         <v>4.5</v>
@@ -8659,7 +8659,7 @@
         </is>
       </c>
       <c r="D29" s="6" t="n">
-        <v>2.323</v>
+        <v>2.303</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
@@ -8676,10 +8676,10 @@
         <v>0.07395</v>
       </c>
       <c r="I29" s="5" t="n">
-        <v>-0.163</v>
+        <v>-0.17</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>6.684</v>
+        <v>6.656</v>
       </c>
       <c r="K29" s="7" t="n">
         <v>5.7</v>
@@ -8705,7 +8705,7 @@
         </is>
       </c>
       <c r="D30" s="6" t="n">
-        <v>0.185</v>
+        <v>0.188</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
@@ -8724,16 +8724,16 @@
         </is>
       </c>
       <c r="I30" s="5" t="n">
-        <v>-0.24</v>
+        <v>-0.225</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>6.884</v>
+        <v>6.982</v>
       </c>
       <c r="K30" s="7" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
       <c r="L30" s="7" t="n">
-        <v>20.8</v>
+        <v>29.1</v>
       </c>
     </row>
     <row r="31">
@@ -8789,7 +8789,7 @@
         </is>
       </c>
       <c r="L31" s="7" t="n">
-        <v>16.6</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -8925,12 +8925,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BYD</t>
+          <t>PENN</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Boyd Gaming</t>
+          <t>Penn Entertainment</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -8952,17 +8952,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>CZR</t>
+          <t>BYD</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Caesars Entertainment</t>
+          <t>Boyd Gaming</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -8972,24 +8972,24 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Regional Operators</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MGM</t>
+          <t>CZR</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>MGM Resorts International</t>
+          <t>Caesars Entertainment</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -9006,12 +9006,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>RSI</t>
+          <t>MGM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Rush Street Interactive</t>
+          <t>MGM Resorts International</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -9021,51 +9021,51 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2021-08-11</t>
+          <t>2025-12-30</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>MLCO</t>
+          <t>RSI</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Melco Resorts</t>
+          <t>Rush Street Interactive</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-04-30</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2025-12-30</t>
+          <t>2021-08-11</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>RRR</t>
+          <t>MLCO</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Red Rock Resorts</t>
+          <t>Melco Resorts</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -9080,24 +9080,24 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Regional Operators</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GENI</t>
+          <t>RRR</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Genius Sports</t>
+          <t>Red Rock Resorts</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-04-30</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -9107,19 +9107,19 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Regional Operators</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ACEL</t>
+          <t>GENI</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Accel Entertainment</t>
+          <t>Genius Sports</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -9134,24 +9134,24 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Gaming Equipment</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>WYNN</t>
+          <t>ACEL</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Wynn Resorts</t>
+          <t>Accel Entertainment</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -9161,19 +9161,19 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Integrated Resorts</t>
+          <t>Gaming Equipment</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>FLUT</t>
+          <t>WYNN</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Flutter Entertainment</t>
+          <t>Wynn Resorts</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -9188,19 +9188,19 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Online &amp; iGaming</t>
+          <t>Integrated Resorts</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>LNW</t>
+          <t>FLUT</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Light &amp; Wonder</t>
+          <t>Flutter Entertainment</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -9208,37 +9208,37 @@
           <t>2026-05-06</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Gaming Equipment</t>
+          <t>Online &amp; iGaming</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PENN</t>
+          <t>LNW</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Penn Entertainment</t>
+          <t>Light &amp; Wonder</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>2025-12-30</t>
-        </is>
-      </c>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Regional Operators</t>
+          <t>Gaming Equipment</t>
         </is>
       </c>
     </row>
@@ -10200,7 +10200,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1360.62</v>
+        <v>1360.48</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1231.91</v>
@@ -10216,7 +10216,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1361.67</v>
+        <v>1361.57</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1240.12</v>
@@ -10232,7 +10232,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1345.63</v>
+        <v>1345.48</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1247.49</v>
@@ -10248,7 +10248,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1294.39</v>
+        <v>1294.22</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1243.47</v>
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1321.23</v>
+        <v>1321.07</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1243.34</v>
@@ -10280,7 +10280,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1290.19</v>
+        <v>1290.02</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1251.57</v>
@@ -10296,7 +10296,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1285.77</v>
+        <v>1285.61</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1253.53</v>
@@ -10312,7 +10312,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1277.2</v>
+        <v>1277.03</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1251.03</v>
@@ -10328,7 +10328,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1274.7</v>
+        <v>1274.54</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1244.88</v>
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1295.23</v>
+        <v>1295.09</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1248.27</v>
@@ -10360,7 +10360,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1255.69</v>
+        <v>1255.5</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1247.22</v>
@@ -10376,7 +10376,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1230.37</v>
+        <v>1230.19</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1221.83</v>
@@ -10392,7 +10392,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1237.28</v>
+        <v>1237.08</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1235.93</v>
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1242.93</v>
+        <v>1242.74</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1242.39</v>
@@ -10424,7 +10424,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1226.58</v>
+        <v>1226.37</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1242.84</v>
@@ -10440,7 +10440,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1232.87</v>
+        <v>1232.65</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1249.15</v>
@@ -10456,7 +10456,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1218.71</v>
+        <v>1218.52</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1254.13</v>
@@ -10472,7 +10472,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1220.47</v>
+        <v>1220.27</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1254</v>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1164.66</v>
+        <v>1164.39</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1251.51</v>
@@ -10504,7 +10504,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1151.65</v>
+        <v>1151.31</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1247.78</v>
@@ -10520,7 +10520,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1170.91</v>
+        <v>1170.6</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1253.98</v>
@@ -10536,7 +10536,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1167.13</v>
+        <v>1166.8</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1243.38</v>
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1190.01</v>
+        <v>1189.62</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1237.36</v>
@@ -10568,7 +10568,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1163.4</v>
+        <v>1162.95</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1221.9</v>
@@ -10584,7 +10584,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1192.15</v>
+        <v>1191.67</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1245.35</v>
@@ -10600,7 +10600,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1194.34</v>
+        <v>1193.85</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1251.35</v>
@@ -10616,7 +10616,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1190.82</v>
+        <v>1190.34</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1248.05</v>
@@ -10632,7 +10632,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1175.03</v>
+        <v>1174.57</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1247.76</v>
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1135.58</v>
+        <v>1135.14</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1228.49</v>
@@ -10664,7 +10664,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1124.68</v>
+        <v>1124.24</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1229.35</v>
@@ -10680,7 +10680,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1140.55</v>
+        <v>1140.15</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1231.34</v>
@@ -10696,7 +10696,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1176.63</v>
+        <v>1176.24</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1237.54</v>
@@ -10712,7 +10712,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1170.93</v>
+        <v>1170.59</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1234.27</v>
@@ -10728,7 +10728,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1171.14</v>
+        <v>1170.79</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1243.2</v>
@@ -10744,7 +10744,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1124.83</v>
+        <v>1124.56</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1230.51</v>
@@ -10760,7 +10760,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1140.5</v>
+        <v>1140.2</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1239.45</v>
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1145.04</v>
+        <v>1144.75</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1249.91</v>
@@ -10792,7 +10792,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1176.3</v>
+        <v>1176.08</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1242.97</v>
@@ -10808,7 +10808,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1162.72</v>
+        <v>1162.65</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1237</v>
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1153.29</v>
+        <v>1153.24</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1226.79</v>
@@ -10856,7 +10856,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1169.93</v>
+        <v>1169.94</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1235.45</v>
@@ -10872,7 +10872,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1167.4</v>
+        <v>1167.42</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1228.56</v>
@@ -10888,7 +10888,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1133.51</v>
+        <v>1133.56</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1212.46</v>
@@ -10904,7 +10904,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1135.07</v>
+        <v>1135.11</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1223.08</v>
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1134.02</v>
+        <v>1134.07</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1221.11</v>
@@ -10936,7 +10936,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1150.13</v>
+        <v>1150.21</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1219.58</v>
@@ -10952,7 +10952,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1134.75</v>
+        <v>1134.86</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1201.06</v>
@@ -10968,7 +10968,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1136.94</v>
+        <v>1136.99</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1194.26</v>
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1128.69</v>
+        <v>1128.71</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1206.41</v>
@@ -11000,7 +11000,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1141.9</v>
+        <v>1141.89</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1209.59</v>
@@ -11016,7 +11016,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1133.37</v>
+        <v>1133.39</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1192.71</v>
@@ -11032,7 +11032,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1146.5</v>
+        <v>1146.52</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1189.77</v>
@@ -11048,7 +11048,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1116.08</v>
+        <v>1116.14</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1172.71</v>
@@ -11064,7 +11064,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1139.74</v>
+        <v>1139.75</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1185.03</v>
@@ -11080,7 +11080,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1151.23</v>
+        <v>1151.22</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1181.05</v>
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1135.94</v>
+        <v>1135.89</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1187.63</v>
@@ -11112,7 +11112,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1113.87</v>
+        <v>1113.82</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1166.42</v>
@@ -11128,7 +11128,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1087.51</v>
+        <v>1087.47</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1146.53</v>
@@ -11144,7 +11144,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1082.8</v>
+        <v>1081.31</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1082.8</v>
+        <v>1081.31</v>
       </c>
     </row>
     <row r="64">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>-20.42%</t>
+          <t>-20.52%</t>
         </is>
       </c>
     </row>
@@ -11188,7 +11188,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>131.8</v>
+        <v>131.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-30 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6829,13 +6829,13 @@
         <v>21</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>28.634026</v>
+        <v>28.624168</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>36.926872</v>
+        <v>36.91416</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>22.796463</v>
+        <v>22.788616</v>
       </c>
       <c r="J12" s="9" t="n">
         <v>0.7070000000000001</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-03-31 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -796,7 +796,7 @@
         <v>10.718</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>11.411</v>
+        <v>11.421</v>
       </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
@@ -807,10 +807,10 @@
         <v>11.24437</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>41.816</v>
+        <v>41.852</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>1.682</v>
@@ -1093,7 +1093,7 @@
         <v>5.487</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>6.503</v>
+        <v>6.572</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>17.102566</v>
@@ -1102,7 +1102,7 @@
         <v>16.238934</v>
       </c>
       <c r="M9" s="7" t="n">
-        <v>7.991</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="N9" s="7" t="n">
         <v>7</v>
@@ -1457,7 +1457,7 @@
         <v>2.311</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>13.014</v>
+        <v>13.009</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>12.347825</v>
@@ -1466,7 +1466,7 @@
         <v>7.1393557</v>
       </c>
       <c r="M15" s="7" t="n">
-        <v>10.791</v>
+        <v>10.786</v>
       </c>
       <c r="N15" s="7" t="n">
         <v>8.6</v>
@@ -1516,7 +1516,7 @@
         <v>2.007</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>12.487</v>
+        <v>12.485</v>
       </c>
       <c r="K16" s="7" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         <v>8.685200999999999</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>17.29</v>
+        <v>17.288</v>
       </c>
       <c r="N16" s="7" t="n">
         <v>11</v>
@@ -1893,7 +1893,7 @@
         <v>9.517326000000001</v>
       </c>
       <c r="M22" s="7" t="n">
-        <v>7.051</v>
+        <v>7.048</v>
       </c>
       <c r="N22" s="7" t="n">
         <v>5.7</v>
@@ -3464,13 +3464,13 @@
         <v>11.24437</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>41.816</v>
+        <v>41.852</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1.885</v>
+        <v>1.886</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>16.943575</v>
@@ -3729,13 +3729,13 @@
         <v>16.238934</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>7.991</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>7</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>3.233</v>
+        <v>3.267</v>
       </c>
       <c r="K9" s="7" t="n">
         <v>14.93841</v>
@@ -4057,13 +4057,13 @@
         <v>7.1393557</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>10.791</v>
+        <v>10.786</v>
       </c>
       <c r="I15" s="7" t="n">
         <v>8.6</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>2.521</v>
+        <v>2.519</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>-1.7800062</v>
@@ -4112,7 +4112,7 @@
         <v>8.685200999999999</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>17.29</v>
+        <v>17.288</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>11</v>
@@ -4440,13 +4440,13 @@
         <v>9.517326000000001</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>7.051</v>
+        <v>7.048</v>
       </c>
       <c r="I22" s="7" t="n">
         <v>5.7</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1.723</v>
+        <v>1.722</v>
       </c>
       <c r="K22" s="7" t="n">
         <v>-11.824213</v>
@@ -6683,7 +6683,7 @@
         <v>0.88883</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>1.99</v>
+        <v>1.95</v>
       </c>
       <c r="P9" s="5" t="n">
         <v>0.32369998</v>
@@ -6739,7 +6739,7 @@
         <v>0.19124001</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>1.64</v>
+        <v>1.57</v>
       </c>
       <c r="P10" s="5" t="n">
         <v>0.2831</v>
@@ -7809,7 +7809,7 @@
         <v>-0.244</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>10.791</v>
+        <v>10.786</v>
       </c>
       <c r="K5" s="7" t="n">
         <v>8.6</v>
@@ -8049,7 +8049,7 @@
         <v>-0.136</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>7.991</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="K12" s="7" t="n">
         <v>7</v>
@@ -8139,7 +8139,7 @@
         <v>0.012</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>17.29</v>
+        <v>17.288</v>
       </c>
       <c r="K14" s="7" t="n">
         <v>11</v>
@@ -8433,10 +8433,10 @@
         <v>-0.394</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>41.816</v>
+        <v>41.852</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>17.9</v>
+        <v>18</v>
       </c>
       <c r="L22" s="7" t="n">
         <v>52</v>
@@ -8727,7 +8727,7 @@
         <v>-0.205</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>7.051</v>
+        <v>7.048</v>
       </c>
       <c r="K30" s="7" t="n">
         <v>5.7</v>
@@ -10811,7 +10811,7 @@
         <v>1152.65</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>1234.21</v>
+        <v>1234.22</v>
       </c>
       <c r="D40" s="13" t="n">
         <v>997.29</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-01 04:49
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="L4" s="7" t="n">
-        <v>11.24437</v>
+        <v>11.670464</v>
       </c>
       <c r="M4" s="7" t="n">
         <v>41.852</v>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>11.24437</v>
+        <v>11.670464</v>
       </c>
       <c r="H4" s="7" t="n">
         <v>41.852</v>
@@ -3482,7 +3482,7 @@
         <v>-0.01</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>1.92274</v>
+        <v>1.85254</v>
       </c>
       <c r="O4" s="3" t="n">
         <v>1.276</v>
@@ -4237,7 +4237,7 @@
         <v>1.7022208</v>
       </c>
       <c r="M18" s="3" t="n">
-        <v>-0.42</v>
+        <v>-0.44</v>
       </c>
       <c r="N18" s="3" t="n">
         <v>0.99</v>
@@ -4400,7 +4400,7 @@
         <v>0.17611478</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-10.17</v>
+        <v>-10.07</v>
       </c>
       <c r="N21" s="3" t="n">
         <v>-2.195</v>
@@ -6285,7 +6285,7 @@
         <v>0.41682</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2.03</v>
+        <v>1.95</v>
       </c>
       <c r="P2" s="5" t="n">
         <v>0.4255</v>
@@ -6338,7 +6338,7 @@
         <v>0.1886</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>0.91337997</v>
+        <v>0.91329</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -6396,7 +6396,7 @@
         <v>0.02949</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>0.87776</v>
+        <v>0.87717</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -6457,7 +6457,7 @@
         <v>0.68716</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>1.03</v>
+        <v>0.98</v>
       </c>
       <c r="P5" s="5" t="n">
         <v>0.3185</v>
@@ -6507,10 +6507,10 @@
         <v>0.1559</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>0.27407</v>
+        <v>0.27405</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>0.73341006</v>
+        <v>0.73188</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -6571,7 +6571,7 @@
         <v>0.81711</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>0.51</v>
+        <v>0.49</v>
       </c>
       <c r="P7" s="5" t="n">
         <v>0.0828</v>
@@ -6627,7 +6627,7 @@
         <v>0.73407</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="P8" s="5" t="n">
         <v>0.0319</v>
@@ -6680,7 +6680,7 @@
         <v>0.07914</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.88883</v>
+        <v>0.88878</v>
       </c>
       <c r="O9" s="5" t="n">
         <v>1.95</v>
@@ -6887,16 +6887,16 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.855968</v>
+        <v>28.912832</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.213097</v>
+        <v>37.286427</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.97316</v>
+        <v>23.01843</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.7240000000000001</v>
+        <v>0.727</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>4.54</v>
@@ -6905,10 +6905,10 @@
         <v>0.1046</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.01332</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>0.91643</v>
+        <v>0.91309</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
@@ -6969,7 +6969,7 @@
         <v>0.46130002</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>7.37</v>
+        <v>7.22</v>
       </c>
       <c r="P14" s="5" t="n">
         <v>8.8889</v>
@@ -7080,7 +7080,7 @@
         <v>0.01867</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>0.98657995</v>
+        <v>0.98630995</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
@@ -7254,7 +7254,7 @@
         <v>0.13798</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0.76087</v>
+        <v>0.76071</v>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
@@ -7317,7 +7317,7 @@
         <v>0.68551004</v>
       </c>
       <c r="O20" s="5" t="n">
-        <v>3.8</v>
+        <v>3.75</v>
       </c>
       <c r="P20" s="5" t="n">
         <v>4.5455</v>
@@ -7425,7 +7425,7 @@
         <v>0.044099998</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>0.07194</v>
+        <v>0.03882</v>
       </c>
       <c r="N22" s="5" t="n">
         <v>0.80921996</v>
@@ -9561,7 +9561,7 @@
         <v>0.1886</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.91337997</v>
+        <v>0.91329</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>2.02</v>
@@ -9588,7 +9588,7 @@
         <v>0.02949</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.87776</v>
+        <v>0.87717</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>2.13</v>
@@ -9639,10 +9639,10 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>0.27407</v>
+        <v>0.27405</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.73341006</v>
+        <v>0.73188</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>4.85</v>
@@ -9723,7 +9723,7 @@
         <v>0.07914</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.88883</v>
+        <v>0.88878</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>4.01</v>
@@ -9828,10 +9828,10 @@
         </is>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.01337</v>
+        <v>0.01332</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.91643</v>
+        <v>0.91309</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>4.54</v>
@@ -9912,7 +9912,7 @@
         <v>0.01867</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.98657995</v>
+        <v>0.98630995</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>4.3</v>
@@ -9993,7 +9993,7 @@
         <v>0.13798</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.76087</v>
+        <v>0.76071</v>
       </c>
       <c r="E19" s="7" t="n">
         <v>2.55</v>
@@ -10071,7 +10071,7 @@
         </is>
       </c>
       <c r="C22" s="5" t="n">
-        <v>0.07194</v>
+        <v>0.03882</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>0.80921996</v>
@@ -10811,7 +10811,7 @@
         <v>1152.65</v>
       </c>
       <c r="C40" s="13" t="n">
-        <v>1234.22</v>
+        <v>1234.21</v>
       </c>
       <c r="D40" s="13" t="n">
         <v>997.29</v>
@@ -11146,8 +11146,12 @@
       <c r="B61" s="13" t="n">
         <v>1118.11</v>
       </c>
-      <c r="C61" s="13" t="n"/>
-      <c r="D61" s="13" t="n"/>
+      <c r="C61" s="13" t="n">
+        <v>1172.6</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <v>947.37</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-01 22:32
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -732,7 +732,7 @@
         <v>-0.6729999999999999</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>17.951</v>
+        <v>17.943</v>
       </c>
       <c r="J3" s="6" t="n">
         <v>29.69</v>
@@ -3398,7 +3398,7 @@
         <v>102.73</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>17.951</v>
+        <v>17.943</v>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
@@ -3421,7 +3421,7 @@
         <v>1.9916635</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>1.0957019</v>
+        <v>1.0952275</v>
       </c>
       <c r="M3" s="3" t="n">
         <v>-1.75</v>
@@ -6887,16 +6887,16 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.812637</v>
+        <v>28.809309</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.15721</v>
+        <v>37.152924</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.938662</v>
+        <v>22.936012</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.733</v>
+        <v>0.732</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>4.54</v>
@@ -8503,7 +8503,7 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>17.951</v>
+        <v>17.943</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
@@ -10200,7 +10200,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>1321.21</v>
+        <v>1321.23</v>
       </c>
       <c r="C2" s="13" t="n">
         <v>1236.16</v>
@@ -10216,7 +10216,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>1271.06</v>
+        <v>1271.08</v>
       </c>
       <c r="C3" s="13" t="n">
         <v>1232.17</v>
@@ -10232,7 +10232,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>1297.26</v>
+        <v>1297.28</v>
       </c>
       <c r="C4" s="13" t="n">
         <v>1232.05</v>
@@ -10248,7 +10248,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>1266.57</v>
+        <v>1266.59</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1240.19</v>
@@ -10264,7 +10264,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>1262.46</v>
+        <v>1262.48</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>1242.14</v>
@@ -10280,7 +10280,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>1254.19</v>
+        <v>1254.21</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>1239.66</v>
@@ -10296,7 +10296,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>1251.88</v>
+        <v>1251.9</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>1233.57</v>
@@ -10312,7 +10312,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>1271.94</v>
+        <v>1271.96</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>1236.92</v>
@@ -10328,7 +10328,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>1233.2</v>
+        <v>1233.22</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>1235.89</v>
@@ -10344,7 +10344,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>1208.51</v>
+        <v>1208.53</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>1210.73</v>
@@ -10360,7 +10360,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>1215.6</v>
+        <v>1215.62</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>1224.7</v>
@@ -10376,7 +10376,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>1221.15</v>
+        <v>1221.17</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>1231.1</v>
@@ -10392,7 +10392,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>1205.29</v>
+        <v>1205.32</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>1231.55</v>
@@ -10408,7 +10408,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>1211.63</v>
+        <v>1211.66</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>1237.8</v>
@@ -10424,7 +10424,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>1197.82</v>
+        <v>1197.85</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>1242.73</v>
@@ -10440,7 +10440,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>1199.75</v>
+        <v>1199.78</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>1242.61</v>
@@ -10456,7 +10456,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>1143.65</v>
+        <v>1143.68</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>1240.14</v>
@@ -10472,7 +10472,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>1130.96</v>
+        <v>1130.98</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>1236.44</v>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>1150.32</v>
+        <v>1150.34</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>1242.59</v>
@@ -10504,7 +10504,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>1146.98</v>
+        <v>1147</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>1232.08</v>
@@ -10520,7 +10520,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>1169.45</v>
+        <v>1169.48</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>1226.11</v>
@@ -10536,7 +10536,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1143.45</v>
+        <v>1143.48</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1210.8</v>
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>1171.76</v>
+        <v>1171.79</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>1234.03</v>
@@ -10568,7 +10568,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>1173.73</v>
+        <v>1173.76</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>1239.98</v>
@@ -10584,7 +10584,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>1170.41</v>
+        <v>1170.44</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>1236.71</v>
@@ -10600,7 +10600,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>1155.26</v>
+        <v>1155.29</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>1236.42</v>
@@ -10616,7 +10616,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1116.43</v>
+        <v>1116.46</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>1217.32</v>
@@ -10632,7 +10632,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>1106.32</v>
+        <v>1106.35</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>1218.18</v>
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>1121.85</v>
+        <v>1121.88</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>1220.15</v>
@@ -10664,7 +10664,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>1157.05</v>
+        <v>1157.09</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>1226.29</v>
@@ -10680,7 +10680,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>1151.41</v>
+        <v>1151.44</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>1223.06</v>
@@ -10696,7 +10696,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>1151.5</v>
+        <v>1151.54</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>1231.9</v>
@@ -10712,7 +10712,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1105.84</v>
+        <v>1105.88</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>1219.32</v>
@@ -10728,7 +10728,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>1120.97</v>
+        <v>1121</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>1228.19</v>
@@ -10744,7 +10744,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>1125.17</v>
+        <v>1125.21</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>1238.55</v>
@@ -10760,7 +10760,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>1155.59</v>
+        <v>1155.63</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>1231.67</v>
@@ -10776,7 +10776,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>1142.68</v>
+        <v>1142.72</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>1225.76</v>
@@ -10792,7 +10792,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>1136.85</v>
+        <v>1136.89</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>1226.45</v>
@@ -10808,7 +10808,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>1133.05</v>
+        <v>1133.08</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>1215.64</v>
@@ -10824,7 +10824,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>1149.05</v>
+        <v>1149.09</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>1224.22</v>
@@ -10840,7 +10840,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>1146.46</v>
+        <v>1146.5</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>1217.39</v>
@@ -10856,7 +10856,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>1113.13</v>
+        <v>1113.17</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>1201.44</v>
@@ -10872,7 +10872,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>1114.77</v>
+        <v>1114.81</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>1211.96</v>
@@ -10888,7 +10888,7 @@
         </is>
       </c>
       <c r="B45" s="13" t="n">
-        <v>1113.99</v>
+        <v>1114.02</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>1210.01</v>
@@ -10904,7 +10904,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>1129.46</v>
+        <v>1129.49</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>1208.5</v>
@@ -10920,7 +10920,7 @@
         </is>
       </c>
       <c r="B47" s="13" t="n">
-        <v>1114.19</v>
+        <v>1114.22</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>1190.14</v>
@@ -10936,7 +10936,7 @@
         </is>
       </c>
       <c r="B48" s="13" t="n">
-        <v>1116.45</v>
+        <v>1116.48</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>1183.41</v>
@@ -10952,7 +10952,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>1108.51</v>
+        <v>1108.55</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>1195.45</v>
@@ -10968,7 +10968,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>1121.55</v>
+        <v>1121.59</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>1198.6</v>
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="B51" s="13" t="n">
-        <v>1113.17</v>
+        <v>1113.21</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>1181.87</v>
@@ -11000,7 +11000,7 @@
         </is>
       </c>
       <c r="B52" s="13" t="n">
-        <v>1125.93</v>
+        <v>1125.97</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>1178.96</v>
@@ -11016,7 +11016,7 @@
         </is>
       </c>
       <c r="B53" s="13" t="n">
-        <v>1096.04</v>
+        <v>1096.08</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>1162.06</v>
@@ -11032,7 +11032,7 @@
         </is>
       </c>
       <c r="B54" s="13" t="n">
-        <v>1119.1</v>
+        <v>1119.14</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>1174.26</v>
@@ -11048,7 +11048,7 @@
         </is>
       </c>
       <c r="B55" s="13" t="n">
-        <v>1130.55</v>
+        <v>1130.59</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>1170.32</v>
@@ -11064,7 +11064,7 @@
         </is>
       </c>
       <c r="B56" s="13" t="n">
-        <v>1115.57</v>
+        <v>1115.61</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>1176.84</v>
@@ -11080,7 +11080,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>1093.6</v>
+        <v>1093.64</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>1155.82</v>
@@ -11096,7 +11096,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>1067.84</v>
+        <v>1067.88</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>1136.11</v>
@@ -11112,7 +11112,7 @@
         </is>
       </c>
       <c r="B59" s="13" t="n">
-        <v>1061.92</v>
+        <v>1061.95</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>1132.32</v>
@@ -11128,7 +11128,7 @@
         </is>
       </c>
       <c r="B60" s="13" t="n">
-        <v>1102.31</v>
+        <v>1102.35</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>1165.23</v>
@@ -11144,7 +11144,7 @@
         </is>
       </c>
       <c r="B61" s="13" t="n">
-        <v>1112.19</v>
+        <v>1112.23</v>
       </c>
       <c r="C61" s="13" t="n"/>
       <c r="D61" s="13" t="n"/>
@@ -11156,7 +11156,7 @@
         </is>
       </c>
       <c r="B63" s="15" t="n">
-        <v>1112.19</v>
+        <v>1112.23</v>
       </c>
     </row>
     <row r="64">
@@ -11188,7 +11188,7 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>137.6</v>
+        <v>137.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-02 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6869,13 +6869,13 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.772755</v>
+        <v>28.782715</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.105778</v>
+        <v>37.118626</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.90691</v>
+        <v>22.91484</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0.698</v>
@@ -10549,7 +10549,7 @@
         <v>1254.6</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>1300.81</v>
+        <v>1300.82</v>
       </c>
       <c r="D25" s="13" t="n">
         <v>1081.02</v>
@@ -10597,7 +10597,7 @@
         <v>1185.28</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>1281.32</v>
+        <v>1281.33</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>1022.18</v>
@@ -10725,7 +10725,7 @@
         <v>1237.97</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>1295.51</v>
+        <v>1295.52</v>
       </c>
       <c r="D36" s="13" t="n">
         <v>1033.49</v>
@@ -11045,7 +11045,7 @@
         <v>1171.44</v>
       </c>
       <c r="C56" s="13" t="n">
-        <v>1215.73</v>
+        <v>1215.74</v>
       </c>
       <c r="D56" s="13" t="n">
         <v>968.99</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-03 21:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -691,7 +691,7 @@
         <v>9.199999999999999</v>
       </c>
       <c r="O2" s="8" t="n">
-        <v>0.888</v>
+        <v>0.887</v>
       </c>
       <c r="P2" s="4" t="n">
         <v>0.523</v>
@@ -752,7 +752,7 @@
         <v>9.699999999999999</v>
       </c>
       <c r="O3" s="8" t="n">
-        <v>1.177</v>
+        <v>1.157</v>
       </c>
       <c r="P3" s="9" t="n">
         <v>-0.511</v>
@@ -813,7 +813,7 @@
         <v>19.1</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1.682</v>
+        <v>1.674</v>
       </c>
       <c r="P4" s="9" t="n">
         <v>-0.285</v>
@@ -931,7 +931,7 @@
         <v>11.6</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>1.396</v>
+        <v>1.351</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>0.315</v>
@@ -990,7 +990,7 @@
         <v>6</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>1.22</v>
+        <v>1.192</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>0.334</v>
@@ -1049,7 +1049,7 @@
         <v>9.9</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="P8" s="9" t="n">
         <v>-0.18</v>
@@ -1108,7 +1108,7 @@
         <v>7.1</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>1.453</v>
+        <v>1.476</v>
       </c>
       <c r="P9" s="4" t="n">
         <v>0.49</v>
@@ -1169,7 +1169,7 @@
         <v>7.2</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>1.977</v>
+        <v>1.878</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>0.116</v>
@@ -1228,7 +1228,7 @@
         <v>7.9</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>1.1</v>
+        <v>1.066</v>
       </c>
       <c r="P11" s="4" t="n">
         <v>0.6940000000000001</v>
@@ -1275,7 +1275,7 @@
         <v>2.143</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>70.875</v>
+        <v>73.16128999999999</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>30.400517</v>
@@ -1287,7 +1287,7 @@
         <v>11</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>1.552</v>
+        <v>1.457</v>
       </c>
       <c r="P12" s="4" t="n">
         <v>1.104</v>
@@ -1337,7 +1337,7 @@
         <v>47.083332</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>20.641054</v>
+        <v>20.611313</v>
       </c>
       <c r="M13" s="7" t="n">
         <v>12.336</v>
@@ -1346,7 +1346,7 @@
         <v>10.4</v>
       </c>
       <c r="O13" s="8" t="n">
-        <v>2.002</v>
+        <v>1.985</v>
       </c>
       <c r="P13" s="9" t="n">
         <v>-0.2</v>
@@ -1381,7 +1381,7 @@
         <v>18.57</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>12.42</v>
+        <v>12.41</v>
       </c>
       <c r="H14" s="5" t="n">
         <v>-0.314</v>
@@ -1407,7 +1407,7 @@
         <v>5.7</v>
       </c>
       <c r="O14" s="8" t="n">
-        <v>1.082</v>
+        <v>1.08</v>
       </c>
       <c r="P14" s="4" t="n">
         <v>0.055</v>
@@ -1527,7 +1527,7 @@
         <v>10.9</v>
       </c>
       <c r="O16" s="8" t="n">
-        <v>1.364</v>
+        <v>1.327</v>
       </c>
       <c r="P16" s="9" t="n">
         <v>-0.044</v>
@@ -1586,7 +1586,7 @@
         <v>7.4</v>
       </c>
       <c r="O17" s="8" t="n">
-        <v>1.376</v>
+        <v>1.341</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>0.31</v>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="O18" s="8" t="n">
-        <v>1.993</v>
+        <v>2.084</v>
       </c>
       <c r="P18" s="9" t="n">
         <v>-0.519</v>
@@ -1684,7 +1684,7 @@
         <v>13.31</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>9.015000000000001</v>
+        <v>9.17</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>-0.171</v>
@@ -1708,7 +1708,7 @@
         <v>4.6</v>
       </c>
       <c r="O19" s="8" t="n">
-        <v>1.07</v>
+        <v>1.058</v>
       </c>
       <c r="P19" s="4" t="n">
         <v>0.139</v>
@@ -1769,7 +1769,7 @@
         <v>7.3</v>
       </c>
       <c r="O20" s="8" t="n">
-        <v>1.412</v>
+        <v>1.411</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>0.124</v>
@@ -1954,7 +1954,7 @@
         <v>9.1</v>
       </c>
       <c r="O23" s="8" t="n">
-        <v>1.327</v>
+        <v>1.276</v>
       </c>
       <c r="P23" s="9" t="n">
         <v>-0.299</v>
@@ -2161,19 +2161,19 @@
         <v>49</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.025</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>-0.033</v>
+        <v>-0.034</v>
       </c>
       <c r="K2" s="5" t="n">
         <v>-0.229</v>
       </c>
       <c r="L2" s="8" t="n">
-        <v>0.888</v>
+        <v>0.887</v>
       </c>
       <c r="M2" s="10" t="n">
-        <v>3865860</v>
+        <v>3726550</v>
       </c>
     </row>
     <row r="3">
@@ -2208,19 +2208,19 @@
         <v>-67.3</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-0.17</v>
+        <v>-0.16</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>-0.525</v>
+        <v>-0.523</v>
       </c>
       <c r="K3" s="5" t="n">
         <v>-0.6609999999999999</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>1.177</v>
+        <v>1.157</v>
       </c>
       <c r="M3" s="10" t="n">
-        <v>2910820</v>
+        <v>2985900</v>
       </c>
     </row>
     <row r="4">
@@ -2255,19 +2255,19 @@
         <v>-42.9</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>-0.08</v>
+        <v>-0.07400000000000001</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>-0.341</v>
+        <v>-0.34</v>
       </c>
       <c r="K4" s="5" t="n">
         <v>-0.525</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>1.682</v>
+        <v>1.674</v>
       </c>
       <c r="M4" s="10" t="n">
-        <v>15324380</v>
+        <v>15184690</v>
       </c>
     </row>
     <row r="5">
@@ -2302,10 +2302,10 @@
         <v>29.4</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>-0.05</v>
+        <v>-0.048</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>-0.112</v>
+        <v>-0.113</v>
       </c>
       <c r="K5" s="5" t="n">
         <v>-0.243</v>
@@ -2314,7 +2314,7 @@
         <v>1.034</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>1537660</v>
+        <v>1569690</v>
       </c>
     </row>
     <row r="6">
@@ -2349,19 +2349,19 @@
         <v>11.3</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>0.025</v>
+        <v>0.023</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.038</v>
+        <v>0.03700000000000001</v>
       </c>
       <c r="K6" s="5" t="n">
         <v>-0.08699999999999999</v>
       </c>
       <c r="L6" s="8" t="n">
-        <v>1.396</v>
+        <v>1.351</v>
       </c>
       <c r="M6" s="10" t="n">
-        <v>5039480</v>
+        <v>4967730</v>
       </c>
     </row>
     <row r="7">
@@ -2405,10 +2405,10 @@
         <v>-0.06900000000000001</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>1.22</v>
+        <v>1.192</v>
       </c>
       <c r="M7" s="10" t="n">
-        <v>965670</v>
+        <v>935690</v>
       </c>
     </row>
     <row r="8">
@@ -2443,19 +2443,19 @@
         <v>-3</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-0.027</v>
+        <v>-0.024</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>-0.114</v>
+        <v>-0.113</v>
       </c>
       <c r="K8" s="5" t="n">
         <v>-0.248</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="M8" s="10" t="n">
-        <v>980050</v>
+        <v>962470</v>
       </c>
     </row>
     <row r="9">
@@ -2490,7 +2490,7 @@
         <v>34.8</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>-0.091</v>
+        <v>-0.08900000000000001</v>
       </c>
       <c r="J9" s="5" t="n">
         <v>-0.067</v>
@@ -2499,10 +2499,10 @@
         <v>-0.202</v>
       </c>
       <c r="L9" s="8" t="n">
-        <v>1.453</v>
+        <v>1.476</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>1213880</v>
+        <v>1180650</v>
       </c>
     </row>
     <row r="10">
@@ -2537,7 +2537,7 @@
         <v>-21.1</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>0.117</v>
+        <v>0.115</v>
       </c>
       <c r="J10" s="5" t="n">
         <v>0.076</v>
@@ -2546,10 +2546,10 @@
         <v>-0.16</v>
       </c>
       <c r="L10" s="8" t="n">
-        <v>1.977</v>
+        <v>1.878</v>
       </c>
       <c r="M10" s="10" t="n">
-        <v>5025290</v>
+        <v>4883010</v>
       </c>
     </row>
     <row r="11">
@@ -2584,19 +2584,19 @@
         <v>20.7</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>0.049</v>
+        <v>0.047</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>-0.058</v>
+        <v>-0.059</v>
       </c>
       <c r="K11" s="5" t="n">
         <v>-0.261</v>
       </c>
       <c r="L11" s="8" t="n">
-        <v>1.1</v>
+        <v>1.066</v>
       </c>
       <c r="M11" s="10" t="n">
-        <v>2218260</v>
+        <v>2279150</v>
       </c>
     </row>
     <row r="12">
@@ -2631,19 +2631,19 @@
         <v>48.4</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>0.181</v>
+        <v>0.176</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>0.218</v>
+        <v>0.216</v>
       </c>
       <c r="K12" s="5" t="n">
         <v>-0.005</v>
       </c>
       <c r="L12" s="8" t="n">
-        <v>1.552</v>
+        <v>1.457</v>
       </c>
       <c r="M12" s="10" t="n">
-        <v>1859580</v>
+        <v>1855440</v>
       </c>
     </row>
     <row r="13">
@@ -2678,19 +2678,19 @@
         <v>-34.8</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-0.06</v>
+        <v>-0.059</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>-0.301</v>
+        <v>-0.3</v>
       </c>
       <c r="K13" s="5" t="n">
         <v>-0.474</v>
       </c>
       <c r="L13" s="8" t="n">
-        <v>2.002</v>
+        <v>1.985</v>
       </c>
       <c r="M13" s="10" t="n">
-        <v>2411130</v>
+        <v>2216830</v>
       </c>
     </row>
     <row r="14">
@@ -2725,19 +2725,19 @@
         <v>10.1</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-0.05599999999999999</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>-0.172</v>
+        <v>-0.171</v>
       </c>
       <c r="K14" s="5" t="n">
         <v>-0.314</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>1.082</v>
+        <v>1.08</v>
       </c>
       <c r="M14" s="10" t="n">
-        <v>1070360</v>
+        <v>1046980</v>
       </c>
     </row>
     <row r="15">
@@ -2772,7 +2772,7 @@
         <v>-0.6</v>
       </c>
       <c r="I15" s="5" t="n">
-        <v>-0.031</v>
+        <v>-0.029</v>
       </c>
       <c r="J15" s="5" t="n">
         <v>-0.274</v>
@@ -2784,7 +2784,7 @@
         <v>0.603</v>
       </c>
       <c r="M15" s="10" t="n">
-        <v>1568540</v>
+        <v>1570980</v>
       </c>
     </row>
     <row r="16">
@@ -2819,7 +2819,7 @@
         <v>-20</v>
       </c>
       <c r="I16" s="5" t="n">
-        <v>0.068</v>
+        <v>0.067</v>
       </c>
       <c r="J16" s="5" t="n">
         <v>-0.08699999999999999</v>
@@ -2828,10 +2828,10 @@
         <v>-0.283</v>
       </c>
       <c r="L16" s="8" t="n">
-        <v>1.364</v>
+        <v>1.327</v>
       </c>
       <c r="M16" s="10" t="n">
-        <v>3878270</v>
+        <v>3739710</v>
       </c>
     </row>
     <row r="17">
@@ -2866,19 +2866,19 @@
         <v>18.6</v>
       </c>
       <c r="I17" s="5" t="n">
-        <v>0.011</v>
+        <v>0.009000000000000001</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.001</v>
+        <v>-0</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>-0.151</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>1.376</v>
+        <v>1.341</v>
       </c>
       <c r="M17" s="10" t="n">
-        <v>126240</v>
+        <v>138380</v>
       </c>
     </row>
     <row r="18">
@@ -2913,19 +2913,19 @@
         <v>-41.7</v>
       </c>
       <c r="I18" s="5" t="n">
-        <v>-0.275</v>
+        <v>-0.263</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>-0.545</v>
+        <v>-0.5429999999999999</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>-0.6679999999999999</v>
       </c>
       <c r="L18" s="8" t="n">
-        <v>1.993</v>
+        <v>2.084</v>
       </c>
       <c r="M18" s="10" t="n">
-        <v>5607160</v>
+        <v>5629540</v>
       </c>
     </row>
     <row r="19">
@@ -2969,10 +2969,10 @@
         <v>-0.171</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>1.07</v>
+        <v>1.058</v>
       </c>
       <c r="M19" s="10" t="n">
-        <v>337570</v>
+        <v>337420</v>
       </c>
     </row>
     <row r="20">
@@ -3007,7 +3007,7 @@
         <v>5.4</v>
       </c>
       <c r="I20" s="5" t="n">
-        <v>-0.026</v>
+        <v>-0.025</v>
       </c>
       <c r="J20" s="5" t="n">
         <v>0.006999999999999999</v>
@@ -3016,10 +3016,10 @@
         <v>-0.174</v>
       </c>
       <c r="L20" s="8" t="n">
-        <v>1.412</v>
+        <v>1.411</v>
       </c>
       <c r="M20" s="10" t="n">
-        <v>156040</v>
+        <v>159460</v>
       </c>
     </row>
     <row r="21">
@@ -3054,7 +3054,7 @@
         <v>36</v>
       </c>
       <c r="I21" s="5" t="n">
-        <v>-0.291</v>
+        <v>-0.285</v>
       </c>
       <c r="J21" s="5" t="n">
         <v>-0.277</v>
@@ -3068,7 +3068,7 @@
         </is>
       </c>
       <c r="M21" s="10" t="n">
-        <v>89560</v>
+        <v>88650</v>
       </c>
     </row>
     <row r="22">
@@ -3103,10 +3103,10 @@
         <v>2.5</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>-0.13</v>
+        <v>-0.125</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>-0.188</v>
+        <v>-0.187</v>
       </c>
       <c r="K22" s="5" t="n">
         <v>-0.305</v>
@@ -3115,7 +3115,7 @@
         <v>1.254</v>
       </c>
       <c r="M22" s="10" t="n">
-        <v>176300</v>
+        <v>175090</v>
       </c>
     </row>
     <row r="23">
@@ -3153,16 +3153,16 @@
         <v>0.07400000000000001</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>-0.163</v>
+        <v>-0.162</v>
       </c>
       <c r="K23" s="5" t="n">
         <v>-0.485</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>1.327</v>
+        <v>1.276</v>
       </c>
       <c r="M23" s="10" t="n">
-        <v>114240</v>
+        <v>114740</v>
       </c>
     </row>
     <row r="24">
@@ -3878,7 +3878,7 @@
         <v>5.28</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>70.875</v>
+        <v>73.16128999999999</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>30.400517</v>
@@ -3899,7 +3899,7 @@
         <v>4.653935</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0.32</v>
+        <v>0.31</v>
       </c>
       <c r="N12" s="3" t="n">
         <v>0.74604</v>
@@ -3934,7 +3934,7 @@
         <v>47.083332</v>
       </c>
       <c r="G13" s="7" t="n">
-        <v>20.641054</v>
+        <v>20.611313</v>
       </c>
       <c r="H13" s="7" t="n">
         <v>12.336</v>
@@ -3955,7 +3955,7 @@
         <v>0.36</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>0.82117903</v>
+        <v>0.822364</v>
       </c>
       <c r="O13" s="3" t="n">
         <v>3.631733</v>
@@ -4388,7 +4388,7 @@
         <v>0.17629746</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>-9.83</v>
+        <v>-10.08</v>
       </c>
       <c r="N21" s="3" t="n">
         <v>-2.195</v>
@@ -6231,13 +6231,11 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>1.6</v>
       </c>
       <c r="F2" s="10" t="n">
         <v>19</v>
@@ -6261,10 +6259,10 @@
         <v>0.0312</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>0.57722</v>
+        <v>0.58443</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>0.41657</v>
+        <v>0.42181998</v>
       </c>
       <c r="O2" s="5" t="n">
         <v>1.93</v>
@@ -6320,7 +6318,7 @@
         <v>0.1886</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>0.91232</v>
+        <v>0.91231</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -6357,7 +6355,7 @@
         <v>34</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>35.80294</v>
+        <v>36.12647</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>76</v>
@@ -6366,7 +6364,7 @@
         <v>24</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>0.546</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="K4" s="7" t="n">
         <v>2.13</v>
@@ -6378,7 +6376,7 @@
         <v>0.02949</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>0.87719</v>
+        <v>0.87735003</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -6430,13 +6428,13 @@
         <v>3.38</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>0.083500005</v>
+        <v>0.077</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>0.27119</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.68648005</v>
+        <v>0.68651</v>
       </c>
       <c r="O5" s="5" t="n">
         <v>0.98</v>
@@ -6492,7 +6490,7 @@
         <v>0.27405</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>0.7318699400000001</v>
+        <v>0.73197997</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -6544,13 +6542,13 @@
         <v>3.91</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>0.065</v>
+        <v>0.0643</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>0.30977</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>0.73263</v>
+        <v>0.73286</v>
       </c>
       <c r="O7" s="5" t="n">
         <v>0.88</v>
@@ -6585,7 +6583,7 @@
         <v>12</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>135.5</v>
+        <v>135.08333</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>152</v>
@@ -6594,7 +6592,7 @@
         <v>110</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>0.521</v>
+        <v>0.517</v>
       </c>
       <c r="K8" s="7" t="n">
         <v>2.17</v>
@@ -6606,7 +6604,7 @@
         <v>0.05964</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>0.81574994</v>
+        <v>0.81599</v>
       </c>
       <c r="O8" s="5" t="n">
         <v>0.49</v>
@@ -6662,7 +6660,7 @@
         <v>0.07914</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.88878</v>
+        <v>0.88912004</v>
       </c>
       <c r="O9" s="5" t="n">
         <v>1.89</v>
@@ -6718,7 +6716,7 @@
         <v>0.010570001</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>1.1194301</v>
+        <v>1.11946</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
@@ -6745,11 +6743,13 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>strong_buy</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>1.25</v>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
       </c>
       <c r="F11" s="10" t="n">
         <v>8</v>
@@ -6776,7 +6776,7 @@
         <v>0.68889</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>0.19124001</v>
+        <v>0.19118999</v>
       </c>
       <c r="O11" s="5" t="n">
         <v>1.6</v>
@@ -6832,7 +6832,7 @@
         <v>0.07084</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.93137</v>
+        <v>0.93138003</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
@@ -6869,22 +6869,22 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.782715</v>
+        <v>28.7396</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.118626</v>
+        <v>37.063023</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.91484</v>
+        <v>22.880514</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>0.698</v>
+        <v>0.696</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>4.54</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.0917</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>0.01332</v>
@@ -6983,7 +6983,7 @@
         <v>13</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>9.24231</v>
+        <v>9.13462</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>12.3</v>
@@ -6992,7 +6992,7 @@
         <v>6</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.627</v>
+        <v>0.608</v>
       </c>
       <c r="K15" s="7" t="n">
         <v>2.37</v>
@@ -7062,7 +7062,7 @@
         <v>0.01867</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>0.98630995</v>
+        <v>0.9857900000000001</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
@@ -7120,7 +7120,7 @@
         <v>0.32022998</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>0.64682996</v>
+        <v>0.64678</v>
       </c>
       <c r="O17" s="5" t="n">
         <v>1.24</v>
@@ -7155,7 +7155,7 @@
         <v>17</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>11.76471</v>
+        <v>11.64706</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>21</v>
@@ -7164,7 +7164,7 @@
         <v>6</v>
       </c>
       <c r="J18" s="4" t="n">
-        <v>1.58</v>
+        <v>1.554</v>
       </c>
       <c r="K18" s="7" t="n">
         <v>2.41</v>
@@ -7176,7 +7176,7 @@
         <v>0.09823</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.94935995</v>
+        <v>0.94938004</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
@@ -7292,7 +7292,7 @@
         <v>0.27324</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>0.68483</v>
+        <v>0.68468004</v>
       </c>
       <c r="O20" s="5" t="n">
         <v>3.7</v>
@@ -7342,7 +7342,7 @@
         <v>8.01</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>0.105500005</v>
+        <v>0.1148</v>
       </c>
       <c r="M21" s="5" t="n">
         <v>0.12769</v>
@@ -8396,7 +8396,7 @@
         <v>5.28</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>70.875</v>
+        <v>73.16128999999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.278</v>
@@ -9509,10 +9509,10 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>0.57722</v>
+        <v>0.58443</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>0.41657</v>
+        <v>0.42181998</v>
       </c>
       <c r="E2" s="7" t="n">
         <v>2.49</v>
@@ -9539,7 +9539,7 @@
         <v>0.1886</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>0.91232</v>
+        <v>0.91231</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>2.02</v>
@@ -9566,7 +9566,7 @@
         <v>0.02949</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.87719</v>
+        <v>0.87735003</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>2.13</v>
@@ -9593,13 +9593,13 @@
         <v>0.27119</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.68648005</v>
+        <v>0.68651</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>3.38</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.083500005</v>
+        <v>0.077</v>
       </c>
       <c r="G5" s="10" t="n">
         <v>6833602</v>
@@ -9620,7 +9620,7 @@
         <v>0.27405</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.7318699400000001</v>
+        <v>0.73197997</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>4.85</v>
@@ -9647,13 +9647,13 @@
         <v>0.30977</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.73263</v>
+        <v>0.73286</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>3.91</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.065</v>
+        <v>0.0643</v>
       </c>
       <c r="G7" s="10" t="n">
         <v>3749544</v>
@@ -9674,7 +9674,7 @@
         <v>0.05964</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.81574994</v>
+        <v>0.81599</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>2.17</v>
@@ -9701,7 +9701,7 @@
         <v>0.07914</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.88878</v>
+        <v>0.88912004</v>
       </c>
       <c r="E9" s="7" t="n">
         <v>4.01</v>
@@ -9728,7 +9728,7 @@
         <v>0.010570001</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>1.1194301</v>
+        <v>1.11946</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>3.37</v>
@@ -9755,7 +9755,7 @@
         <v>0.68889</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.19124001</v>
+        <v>0.19118999</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>4.72</v>
@@ -9782,7 +9782,7 @@
         <v>0.07084</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.93137</v>
+        <v>0.93138003</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>1.89</v>
@@ -9815,7 +9815,7 @@
         <v>4.54</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.1046</v>
+        <v>0.0917</v>
       </c>
       <c r="G13" s="10" t="n">
         <v>10753999</v>
@@ -9890,7 +9890,7 @@
         <v>0.01867</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.98630995</v>
+        <v>0.9857900000000001</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>4.3</v>
@@ -9917,7 +9917,7 @@
         <v>0.32022998</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.64682996</v>
+        <v>0.64678</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>2.64</v>
@@ -9944,7 +9944,7 @@
         <v>0.09823</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.94935995</v>
+        <v>0.94938004</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>2.41</v>
@@ -9998,7 +9998,7 @@
         <v>0.27324</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.68483</v>
+        <v>0.68468004</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>4.41</v>
@@ -10031,7 +10031,7 @@
         <v>8.01</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.105500005</v>
+        <v>0.1148</v>
       </c>
       <c r="G21" s="10" t="n">
         <v>814259</v>
@@ -10549,7 +10549,7 @@
         <v>1254.6</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>1300.82</v>
+        <v>1300.81</v>
       </c>
       <c r="D25" s="13" t="n">
         <v>1081.02</v>
@@ -10597,7 +10597,7 @@
         <v>1185.28</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>1281.33</v>
+        <v>1281.32</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>1022.18</v>
@@ -10725,7 +10725,7 @@
         <v>1237.97</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>1295.52</v>
+        <v>1295.51</v>
       </c>
       <c r="D36" s="13" t="n">
         <v>1033.49</v>
@@ -11045,7 +11045,7 @@
         <v>1171.44</v>
       </c>
       <c r="C56" s="13" t="n">
-        <v>1215.74</v>
+        <v>1215.73</v>
       </c>
       <c r="D56" s="13" t="n">
         <v>968.99</v>
@@ -11124,8 +11124,12 @@
       <c r="B61" s="13" t="n">
         <v>1195.97</v>
       </c>
-      <c r="C61" s="13" t="n"/>
-      <c r="D61" s="13" t="n"/>
+      <c r="C61" s="13" t="n">
+        <v>1235.98</v>
+      </c>
+      <c r="D61" s="13" t="n">
+        <v>993.04</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="14" t="inlineStr">

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-05 21:32
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -781,7 +781,7 @@
         <v>23.16</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>0.0451264</v>
+        <v>0.04512635</v>
       </c>
       <c r="F4" s="3" t="n">
         <v>48.78</v>
@@ -842,7 +842,7 @@
         <v>102.03</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>-0.555555</v>
+        <v>-0.5555553</v>
       </c>
       <c r="F5" s="3" t="n">
         <v>134.72</v>
@@ -1019,7 +1019,7 @@
         <v>89.06999999999999</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>-0.0448894</v>
+        <v>-0.04488936800000001</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>118.46</v>
@@ -1078,7 +1078,7 @@
         <v>55.04</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>0.145564</v>
+        <v>0.14556374</v>
       </c>
       <c r="F9" s="3" t="n">
         <v>68.98999999999999</v>
@@ -1316,7 +1316,7 @@
         <v>16.95</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.0192424</v>
+        <v>0.019242313</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>32.22</v>
@@ -1436,7 +1436,7 @@
         <v>5.68</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>-0.0155979</v>
+        <v>-0.015597947</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>10.15</v>
@@ -1495,7 +1495,7 @@
         <v>14.77</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>-0.0153333</v>
+        <v>-0.015333303</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>20.61</v>
@@ -1556,7 +1556,7 @@
         <v>96.68000000000001</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>0.259255</v>
+        <v>0.2592554</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>113.88</v>
@@ -1737,7 +1737,7 @@
         <v>27.04</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>0.0127341</v>
+        <v>0.012734088</v>
       </c>
       <c r="F20" s="3" t="n">
         <v>32.74</v>
@@ -1861,7 +1861,7 @@
         <v>6.92</v>
       </c>
       <c r="E22" s="9" t="n">
-        <v>-0.574712</v>
+        <v>-0.5747120999999999</v>
       </c>
       <c r="F22" s="3" t="n">
         <v>9.949999999999999</v>
@@ -1922,7 +1922,7 @@
         <v>2.55</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>0.0580912</v>
+        <v>0.05809133499999999</v>
       </c>
       <c r="F23" s="3" t="n">
         <v>4.95</v>
@@ -2243,7 +2243,7 @@
         <v>23.16</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.0451264</v>
+        <v>0.04512635</v>
       </c>
       <c r="F4" s="5" t="n">
         <v>-0.351</v>
@@ -2290,7 +2290,7 @@
         <v>102.03</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>-0.555555</v>
+        <v>-0.5555553</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>-0.166</v>
@@ -2431,7 +2431,7 @@
         <v>89.06999999999999</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>-0.0448894</v>
+        <v>-0.04488936800000001</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>-0.204</v>
@@ -2478,7 +2478,7 @@
         <v>55.04</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.145564</v>
+        <v>0.14556374</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>-0.108</v>
@@ -2666,7 +2666,7 @@
         <v>16.95</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.0192424</v>
+        <v>0.019242313</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>-0.273</v>
@@ -2760,7 +2760,7 @@
         <v>5.68</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>-0.0155979</v>
+        <v>-0.015597947</v>
       </c>
       <c r="F15" s="5" t="n">
         <v>-0.244</v>
@@ -2807,7 +2807,7 @@
         <v>14.77</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>-0.0153333</v>
+        <v>-0.015333303</v>
       </c>
       <c r="F16" s="5" t="n">
         <v>-0.005</v>
@@ -2854,7 +2854,7 @@
         <v>96.68000000000001</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.259255</v>
+        <v>0.2592554</v>
       </c>
       <c r="F17" s="5" t="n">
         <v>0.01</v>
@@ -2995,7 +2995,7 @@
         <v>27.04</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.0127341</v>
+        <v>0.012734088</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>-0</v>
@@ -3091,7 +3091,7 @@
         <v>6.92</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>-0.574712</v>
+        <v>-0.5747120999999999</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>-0.229</v>
@@ -3138,7 +3138,7 @@
         <v>2.55</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.0580912</v>
+        <v>0.05809133499999999</v>
       </c>
       <c r="F23" s="5" t="n">
         <v>0.02</v>
@@ -6291,13 +6291,13 @@
         </is>
       </c>
       <c r="E3" s="7" t="n">
-        <v>1.66667</v>
+        <v>1.69231</v>
       </c>
       <c r="F3" s="10" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>199.44444</v>
+        <v>198.65385</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>354</v>
@@ -6306,7 +6306,7 @@
         <v>125</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>0.875</v>
+        <v>0.867</v>
       </c>
       <c r="K3" s="7" t="n">
         <v>2.02</v>
@@ -6869,13 +6869,13 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.7396</v>
+        <v>28.752853</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.063023</v>
+        <v>37.080116</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.880514</v>
+        <v>22.891066</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0.696</v>
@@ -10549,7 +10549,7 @@
         <v>1254.6</v>
       </c>
       <c r="C25" s="13" t="n">
-        <v>1300.81</v>
+        <v>1300.82</v>
       </c>
       <c r="D25" s="13" t="n">
         <v>1081.02</v>
@@ -10597,7 +10597,7 @@
         <v>1185.28</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>1281.32</v>
+        <v>1281.33</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>1022.18</v>
@@ -10725,7 +10725,7 @@
         <v>1237.97</v>
       </c>
       <c r="C36" s="13" t="n">
-        <v>1295.51</v>
+        <v>1295.52</v>
       </c>
       <c r="D36" s="13" t="n">
         <v>1033.49</v>
@@ -11045,7 +11045,7 @@
         <v>1171.44</v>
       </c>
       <c r="C56" s="13" t="n">
-        <v>1215.73</v>
+        <v>1215.74</v>
       </c>
       <c r="D56" s="13" t="n">
         <v>968.99</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-05 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6869,13 +6869,13 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.752853</v>
+        <v>28.746225</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.080116</v>
+        <v>37.071568</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.891066</v>
+        <v>22.88579</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0.696</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-06 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6869,13 +6869,13 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>28.766117</v>
+        <v>28.769436</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.09722</v>
+        <v>37.1015</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>22.901627</v>
+        <v>22.904268</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0.6929999999999999</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-07 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6869,16 +6869,16 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>29.134367</v>
+        <v>29.120764</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.565105</v>
+        <v>37.547565</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>23.19047</v>
+        <v>23.179642</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.758</v>
+        <v>0.757</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>4.54</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-08 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6869,13 +6869,13 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>29.107176</v>
+        <v>29.103779</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.530045</v>
+        <v>37.525665</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>23.168825</v>
+        <v>23.166122</v>
       </c>
       <c r="J13" s="4" t="n">
         <v>0.75</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-09 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -6867,16 +6867,16 @@
         <v>21</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>29.04828</v>
+        <v>29.068672</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>37.604626</v>
+        <v>37.631023</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>23.214869</v>
+        <v>23.231165</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.9059999999999999</v>
+        <v>0.907</v>
       </c>
       <c r="K13" s="7" t="n">
         <v>4.54</v>
@@ -10324,7 +10324,7 @@
         <v>4001.52</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>1451.79</v>
+        <v>1451.8</v>
       </c>
     </row>
     <row r="12">
@@ -10385,7 +10385,7 @@
         <v>1905.82</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>4001.06</v>
+        <v>4001.05</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1399.91</v>
@@ -10401,7 +10401,7 @@
         <v>1892.86</v>
       </c>
       <c r="C16" s="13" t="n">
-        <v>3967.23</v>
+        <v>3967.22</v>
       </c>
       <c r="D16" s="13" t="n">
         <v>1384.23</v>
@@ -10609,7 +10609,7 @@
         <v>1805.19</v>
       </c>
       <c r="C29" s="13" t="n">
-        <v>3926.15</v>
+        <v>3926.14</v>
       </c>
       <c r="D29" s="13" t="n">
         <v>1346.9</v>
@@ -10977,7 +10977,7 @@
         <v>1781.56</v>
       </c>
       <c r="C52" s="13" t="n">
-        <v>3721.68</v>
+        <v>3721.67</v>
       </c>
       <c r="D52" s="13" t="n">
         <v>1278.58</v>

</xml_diff>

<commit_message>
Auto-refresh: casino gaming market data update 2026-04-11 22:31
</commit_message>
<xml_diff>
--- a/Gaming_Equities.xlsx
+++ b/Gaming_Equities.xlsx
@@ -10385,7 +10385,7 @@
         <v>1897.9</v>
       </c>
       <c r="C15" s="13" t="n">
-        <v>3967.22</v>
+        <v>3967.23</v>
       </c>
       <c r="D15" s="13" t="n">
         <v>1384.28</v>
@@ -10593,7 +10593,7 @@
         <v>1810.32</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>3926.14</v>
+        <v>3926.15</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>1346.71</v>
@@ -10961,7 +10961,7 @@
         <v>1787.61</v>
       </c>
       <c r="C51" s="13" t="n">
-        <v>3721.67</v>
+        <v>3721.68</v>
       </c>
       <c r="D51" s="13" t="n">
         <v>1278.59</v>

</xml_diff>